<commit_message>
Add upcoming meeting time zones
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -8159,7 +8159,6 @@
           <t>setup</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -8172,7 +8171,6 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -8185,7 +8183,6 @@
           <t>fullText</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -8198,7 +8195,6 @@
           <t>extraction</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -8211,7 +8207,6 @@
           <t>analysis</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13186,7 +13181,6 @@
           <t>setup</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13199,7 +13193,6 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13212,7 +13205,6 @@
           <t>fullText</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13225,7 +13217,6 @@
           <t>extraction</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13238,7 +13229,6 @@
           <t>analysis</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -26565,14 +26555,46 @@
           <t>mtg-01</t>
         </is>
       </c>
-      <c r="B2" s="25" t="n"/>
-      <c r="C2" s="25" t="n"/>
-      <c r="D2" s="25" t="n"/>
-      <c r="E2" s="25" t="n"/>
-      <c r="F2" s="25" t="n"/>
-      <c r="G2" s="25" t="n"/>
-      <c r="H2" s="25" t="n"/>
-      <c r="I2" s="25" t="n"/>
+      <c r="B2" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C2" s="25" t="inlineStr">
+        <is>
+          <t>2:00-3:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="D2" s="25" t="inlineStr">
+        <is>
+          <t>7:00-8:00 AM BST</t>
+        </is>
+      </c>
+      <c r="E2" s="25" t="inlineStr">
+        <is>
+          <t>NK Training - Medication Adherence</t>
+        </is>
+      </c>
+      <c r="F2" s="25" t="inlineStr">
+        <is>
+          <t>CDT calendar time: Jun 8, 1:00-2:00 AM. Nested Knowledge training for Medication Adherence.</t>
+        </is>
+      </c>
+      <c r="G2" s="25" t="inlineStr">
+        <is>
+          <t>Amanda Cross / Rehan Sarwar / Krishna / Nested Knowledge</t>
+        </is>
+      </c>
+      <c r="H2" s="25" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I2" s="25" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
       <c r="J2" s="25" t="inlineStr">
         <is>
           <t>Scheduled</t>
@@ -26583,10 +26605,10 @@
           <t>phase1-04</t>
         </is>
       </c>
-      <c r="L2" s="25" t="n"/>
+      <c r="L2" s="25" t="inlineStr"/>
       <c r="M2" s="25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -26596,14 +26618,46 @@
           <t>mtg-02</t>
         </is>
       </c>
-      <c r="B3" s="25" t="n"/>
-      <c r="C3" s="25" t="n"/>
-      <c r="D3" s="25" t="n"/>
-      <c r="E3" s="25" t="n"/>
-      <c r="F3" s="25" t="n"/>
-      <c r="G3" s="25" t="n"/>
-      <c r="H3" s="25" t="n"/>
-      <c r="I3" s="25" t="n"/>
+      <c r="B3" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C3" s="25" t="inlineStr">
+        <is>
+          <t>3:00-4:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="D3" s="25" t="inlineStr">
+        <is>
+          <t>8:00-9:00 AM BST</t>
+        </is>
+      </c>
+      <c r="E3" s="25" t="inlineStr">
+        <is>
+          <t>Onboarding - Medication Adherence</t>
+        </is>
+      </c>
+      <c r="F3" s="25" t="inlineStr">
+        <is>
+          <t>CDT calendar time: Jun 8, 2:00-3:00 AM. Onboarding and split-team workflow confirmation.</t>
+        </is>
+      </c>
+      <c r="G3" s="25" t="inlineStr">
+        <is>
+          <t>Amanda Cross / Rehan Sarwar / Krishna</t>
+        </is>
+      </c>
+      <c r="H3" s="25" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I3" s="25" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
       <c r="J3" s="25" t="inlineStr">
         <is>
           <t>Scheduled</t>
@@ -26614,10 +26668,10 @@
           <t>phase1-04</t>
         </is>
       </c>
-      <c r="L3" s="25" t="n"/>
+      <c r="L3" s="25" t="inlineStr"/>
       <c r="M3" s="25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -26627,14 +26681,46 @@
           <t>mtg-03</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n"/>
-      <c r="C4" s="25" t="n"/>
-      <c r="D4" s="25" t="n"/>
-      <c r="E4" s="25" t="n"/>
-      <c r="F4" s="25" t="n"/>
-      <c r="G4" s="25" t="n"/>
-      <c r="H4" s="25" t="n"/>
-      <c r="I4" s="25" t="n"/>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>5:00-6:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>10:00-11:00 AM BST</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Vitamin C Onboarding</t>
+        </is>
+      </c>
+      <c r="F4" s="25" t="inlineStr">
+        <is>
+          <t>CDT calendar time: Jun 12, 4:00-5:00 AM. Review onboarding for Vitamin C.</t>
+        </is>
+      </c>
+      <c r="G4" s="25" t="inlineStr">
+        <is>
+          <t>Jai Das / Krishna / Core Team</t>
+        </is>
+      </c>
+      <c r="H4" s="25" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I4" s="25" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
       <c r="J4" s="25" t="inlineStr">
         <is>
           <t>Scheduled</t>
@@ -26645,10 +26731,10 @@
           <t>phase1-05</t>
         </is>
       </c>
-      <c r="L4" s="25" t="n"/>
+      <c r="L4" s="25" t="inlineStr"/>
       <c r="M4" s="25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -26658,28 +26744,56 @@
           <t>mtg-04</t>
         </is>
       </c>
-      <c r="B5" s="25" t="n"/>
-      <c r="C5" s="25" t="n"/>
-      <c r="D5" s="25" t="n"/>
-      <c r="E5" s="25" t="n"/>
-      <c r="F5" s="25" t="n"/>
-      <c r="G5" s="25" t="n"/>
-      <c r="H5" s="25" t="n"/>
-      <c r="I5" s="25" t="n"/>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>10:00-11:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="inlineStr">
+        <is>
+          <t>3:00-4:00 PM BST</t>
+        </is>
+      </c>
+      <c r="E5" s="25" t="inlineStr">
+        <is>
+          <t>AI Pilot Core Project Team Catch-up</t>
+        </is>
+      </c>
+      <c r="F5" s="25" t="inlineStr">
+        <is>
+          <t>CDT calendar time: 9:00-10:00 AM. Core project team catch-up.</t>
+        </is>
+      </c>
+      <c r="G5" s="25" t="inlineStr">
+        <is>
+          <t>Core Project Team</t>
+        </is>
+      </c>
+      <c r="H5" s="25" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I5" s="25" t="inlineStr">
+        <is>
+          <t>Project coordination</t>
+        </is>
+      </c>
       <c r="J5" s="25" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
-      <c r="K5" s="25" t="inlineStr">
-        <is>
-          <t>new-01</t>
-        </is>
-      </c>
-      <c r="L5" s="25" t="n"/>
+      <c r="K5" s="25" t="inlineStr"/>
+      <c r="L5" s="25" t="inlineStr"/>
       <c r="M5" s="25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore pilot dashboard visibility
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -36460,6 +36460,7 @@
           <t>Pilot closeout / lessons learned</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>2026-05-10</t>
@@ -36472,7 +36473,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -36540,7 +36541,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -41461,6 +41462,7 @@
           <t>NextAction</t>
         </is>
       </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>No</t>
@@ -46007,7 +46009,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -46319,7 +46320,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -46440,7 +46440,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -46626,7 +46625,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -46777,7 +46775,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -50192,7 +50189,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -50380,7 +50376,6 @@
         </is>
       </c>
     </row>
-    <row r="117"/>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
@@ -50526,7 +50521,6 @@
         </is>
       </c>
     </row>
-    <row r="121"/>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Close pilot follow-up actions
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -36437,7 +36437,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Wrapping Up</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -36457,10 +36457,9 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Pilot closeout / lessons learned</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
+          <t>Pilot closeout closed</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>2026-05-10</t>
@@ -36468,7 +36467,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Wrapping Up</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -36505,7 +36504,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Wrapping Up</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -36525,10 +36524,9 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Pilot completion check</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
+          <t>Pilot closeout closed</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>2026-05-13</t>
@@ -36536,7 +36534,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -40618,6 +40616,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -40677,7 +40676,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Wrapping Up</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -40794,6 +40793,8 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -40985,6 +40986,8 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
@@ -41248,6 +41251,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -41362,7 +41366,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Wrapping Up</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -41430,7 +41434,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Pilot closeout / lessons learned</t>
+          <t>Pilot closeout closed</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -41447,7 +41451,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Time-on-task values and survey receipt still need verification for pilot closeout.</t>
+          <t>Pilot closeout record closed; no active follow-up required.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -41462,7 +41466,6 @@
           <t>NextAction</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>No</t>
@@ -41494,7 +41497,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Full-text time not reported.</t>
+          <t>Closed.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -41511,7 +41514,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Wrapping Up</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -41550,7 +41553,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -41559,6 +41562,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -45539,7 +45543,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Check whether reported title/abstract and data extraction times are sufficiently reliable for pilot note.</t>
+          <t>Closed; no active follow-up required.</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -45581,7 +45585,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -45601,7 +45605,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Matteo said all surveys were submitted; confirm in survey system.</t>
+          <t>Closed; no active follow-up required.</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -45638,7 +45642,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -45658,7 +45662,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Include review retention, tool support, workload clarity, and volunteer usability points.</t>
+          <t>Closed; no active follow-up required.</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -45793,12 +45797,12 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Matteo reported title/abstract and data extraction timing values; full-text time was not reported and needs to be documented as a limitation.</t>
+          <t>Closed; no active follow-up required.</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -45855,12 +45859,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Matteo indicated survey completion, but receipt should be confirmed in the survey system.</t>
+          <t>Closed; no active follow-up required.</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -45950,12 +45954,17 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Closed; no active follow-up required.</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -46009,6 +46018,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -46123,7 +46133,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -46191,7 +46201,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Pilot completion check</t>
+          <t>Pilot closeout closed</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -46208,7 +46218,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>No fresh completion update found in the latest email batch.</t>
+          <t>Pilot closeout record closed; no active follow-up required.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -46223,7 +46233,6 @@
           <t>NextAction</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>No</t>
@@ -46255,7 +46264,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Pilot output status still unclear.</t>
+          <t>Closed.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -46272,7 +46281,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -46311,7 +46320,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -46320,6 +46329,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -50280,7 +50290,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -50300,7 +50310,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Clarify whether remaining pilot outputs are ready for closeout and adjudication preparation.</t>
+          <t>Closed; no active follow-up required.</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -50337,7 +50347,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -50357,7 +50367,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Confirm whether outputs are complete enough to share with Sean/data manager.</t>
+          <t>Closed; no active follow-up required.</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -50492,12 +50502,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>Latest Laser AI completion status and availability of outputs for adjudication preparation remain unclear.</t>
+          <t>Closed; no active follow-up required.</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -50587,12 +50597,17 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Closed; no active follow-up required.</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update upcoming meeting list
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -26581,7 +26581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="14" customWidth="1" style="29" min="1" max="2"/>
@@ -26723,7 +26723,7 @@
       <c r="L2" s="25" t="inlineStr"/>
       <c r="M2" s="25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -26786,7 +26786,7 @@
       <c r="L3" s="25" t="inlineStr"/>
       <c r="M3" s="25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -26849,44 +26849,32 @@
       <c r="L4" s="25" t="inlineStr"/>
       <c r="M4" s="25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
         <is>
-          <t>mtg-04</t>
-        </is>
-      </c>
-      <c r="B5" s="25" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C5" s="25" t="inlineStr">
-        <is>
-          <t>10:00-11:00 AM EDT</t>
-        </is>
-      </c>
-      <c r="D5" s="25" t="inlineStr">
-        <is>
-          <t>3:00-4:00 PM BST</t>
-        </is>
-      </c>
+          <t>mtg-05</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="n"/>
+      <c r="C5" s="25" t="n"/>
+      <c r="D5" s="25" t="n"/>
       <c r="E5" s="25" t="inlineStr">
         <is>
-          <t>AI Pilot Core Project Team Catch-up</t>
+          <t>Fruit &amp; Veg Re-onboarding</t>
         </is>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>CDT calendar time: 9:00-10:00 AM. Core project team catch-up.</t>
+          <t>Re-onboarding meeting for Fruit &amp; Veg; time TBD.</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>Core Project Team</t>
+          <t>Rebecca K. Hodder / Krishna / Core Team</t>
         </is>
       </c>
       <c r="H5" s="25" t="inlineStr">
@@ -26896,7 +26884,7 @@
       </c>
       <c r="I5" s="25" t="inlineStr">
         <is>
-          <t>Project coordination</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="J5" s="25" t="inlineStr">
@@ -26904,8 +26892,12 @@
           <t>Scheduled</t>
         </is>
       </c>
-      <c r="K5" s="25" t="inlineStr"/>
-      <c r="L5" s="25" t="inlineStr"/>
+      <c r="K5" s="25" t="inlineStr">
+        <is>
+          <t>phase1-03</t>
+        </is>
+      </c>
+      <c r="L5" s="25" t="n"/>
       <c r="M5" s="25" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -26915,25 +26907,159 @@
     <row r="6">
       <c r="A6" s="25" t="inlineStr">
         <is>
-          <t>mtg-05</t>
+          <t>mtg-06</t>
         </is>
       </c>
       <c r="B6" s="25" t="n"/>
       <c r="C6" s="25" t="n"/>
       <c r="D6" s="25" t="n"/>
-      <c r="E6" s="25" t="n"/>
-      <c r="F6" s="25" t="n"/>
-      <c r="G6" s="25" t="n"/>
-      <c r="H6" s="25" t="n"/>
-      <c r="I6" s="25" t="n"/>
+      <c r="E6" s="25" t="inlineStr">
+        <is>
+          <t>NK Training - Human Milk Fortifier</t>
+        </is>
+      </c>
+      <c r="F6" s="25" t="inlineStr">
+        <is>
+          <t>Nested Knowledge training for Human Milk Fortifier; time TBD.</t>
+        </is>
+      </c>
+      <c r="G6" s="25" t="inlineStr">
+        <is>
+          <t>Mohan Pammi / Krishna / Nested Knowledge</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I6" s="25" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
       <c r="J6" s="25" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
-      <c r="K6" s="25" t="n"/>
+      <c r="K6" s="25" t="inlineStr">
+        <is>
+          <t>phase1-07</t>
+        </is>
+      </c>
       <c r="L6" s="25" t="n"/>
       <c r="M6" s="25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>mtg-07</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="n"/>
+      <c r="C7" s="25" t="n"/>
+      <c r="D7" s="25" t="n"/>
+      <c r="E7" s="25" t="inlineStr">
+        <is>
+          <t>Human Milk Fortifier Onboarding</t>
+        </is>
+      </c>
+      <c r="F7" s="25" t="inlineStr">
+        <is>
+          <t>Onboarding meeting for Human Milk Fortifier; time TBD.</t>
+        </is>
+      </c>
+      <c r="G7" s="25" t="inlineStr">
+        <is>
+          <t>Mohan Pammi / Krishna / Core Team</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I7" s="25" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="J7" s="25" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="K7" s="25" t="inlineStr">
+        <is>
+          <t>phase1-07</t>
+        </is>
+      </c>
+      <c r="L7" s="25" t="n"/>
+      <c r="M7" s="25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>mtg-04</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>10:00-11:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>3:00-4:00 PM BST</t>
+        </is>
+      </c>
+      <c r="E8" s="25" t="inlineStr">
+        <is>
+          <t>AI Pilot Core Project Team Catch-up</t>
+        </is>
+      </c>
+      <c r="F8" s="25" t="inlineStr">
+        <is>
+          <t>CDT calendar time: 9:00-10:00 AM. Core project team catch-up.</t>
+        </is>
+      </c>
+      <c r="G8" s="25" t="inlineStr">
+        <is>
+          <t>Core Project Team</t>
+        </is>
+      </c>
+      <c r="H8" s="25" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I8" s="25" t="inlineStr">
+        <is>
+          <t>Project coordination</t>
+        </is>
+      </c>
+      <c r="J8" s="25" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="K8" s="25" t="n"/>
+      <c r="L8" s="25" t="n"/>
+      <c r="M8" s="25" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -40616,7 +40742,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -40793,8 +40918,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -40986,8 +41109,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
@@ -41251,7 +41372,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -41562,7 +41682,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -46018,7 +46137,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -46329,7 +46447,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update Phase 1 onboarding workflow statuses
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -13723,7 +13723,7 @@
       </c>
       <c r="I49" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J49" s="18" t="n"/>
@@ -13776,7 +13776,7 @@
       </c>
       <c r="I50" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J50" s="18" t="n"/>
@@ -13829,7 +13829,7 @@
       </c>
       <c r="I51" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J51" s="18" t="n"/>
@@ -13882,7 +13882,7 @@
       </c>
       <c r="I52" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J52" s="18" t="n"/>
@@ -13988,7 +13988,7 @@
       </c>
       <c r="I54" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J54" s="18" t="n"/>
@@ -14041,7 +14041,7 @@
       </c>
       <c r="I55" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J55" s="18" t="n"/>
@@ -14094,7 +14094,7 @@
       </c>
       <c r="I56" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J56" s="18" t="n"/>
@@ -28007,7 +28007,7 @@
       </c>
       <c r="I49" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J49" s="18" t="n"/>
@@ -28060,7 +28060,7 @@
       </c>
       <c r="I50" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J50" s="18" t="n"/>
@@ -28113,7 +28113,7 @@
       </c>
       <c r="I51" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J51" s="18" t="n"/>
@@ -28166,7 +28166,7 @@
       </c>
       <c r="I52" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J52" s="18" t="n"/>
@@ -28219,7 +28219,7 @@
       </c>
       <c r="I53" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J53" s="18" t="n"/>
@@ -28272,7 +28272,7 @@
       </c>
       <c r="I54" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J54" s="18" t="n"/>
@@ -28325,7 +28325,7 @@
       </c>
       <c r="I55" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J55" s="18" t="n"/>
@@ -28378,7 +28378,7 @@
       </c>
       <c r="I56" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J56" s="18" t="n"/>
@@ -32600,7 +32600,7 @@
       </c>
       <c r="I49" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J49" s="18" t="n"/>
@@ -32653,7 +32653,7 @@
       </c>
       <c r="I50" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J50" s="18" t="n"/>
@@ -32706,7 +32706,7 @@
       </c>
       <c r="I51" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J51" s="18" t="n"/>
@@ -32759,7 +32759,7 @@
       </c>
       <c r="I52" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J52" s="18" t="n"/>
@@ -32812,7 +32812,7 @@
       </c>
       <c r="I53" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J53" s="18" t="n"/>
@@ -32865,7 +32865,7 @@
       </c>
       <c r="I54" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J54" s="18" t="n"/>
@@ -32971,7 +32971,7 @@
       </c>
       <c r="I56" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J56" s="18" t="n"/>

</xml_diff>

<commit_message>
Correct Fruit and Probiotics workflow counts
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -3403,7 +3403,7 @@
       </c>
       <c r="I53" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J53" s="18" t="n"/>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="I56" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J56" s="18" t="n"/>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="I58" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J58" s="18" t="n"/>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="I59" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J59" s="18" t="n"/>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="I60" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J60" s="18" t="n"/>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="I61" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J61" s="18" t="n"/>
@@ -3880,7 +3880,7 @@
       </c>
       <c r="I62" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J62" s="18" t="n"/>
@@ -3933,7 +3933,7 @@
       </c>
       <c r="I63" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
@@ -3986,7 +3986,7 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
@@ -28484,7 +28484,7 @@
       </c>
       <c r="I58" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J58" s="18" t="n"/>
@@ -28537,7 +28537,7 @@
       </c>
       <c r="I59" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J59" s="18" t="n"/>
@@ -28590,7 +28590,7 @@
       </c>
       <c r="I60" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J60" s="18" t="n"/>
@@ -28643,7 +28643,7 @@
       </c>
       <c r="I61" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J61" s="18" t="n"/>
@@ -28696,7 +28696,7 @@
       </c>
       <c r="I62" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J62" s="18" t="n"/>
@@ -28749,7 +28749,7 @@
       </c>
       <c r="I63" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>

</xml_diff>

<commit_message>
Update dashboard review pipeline
# Conflicts:
#	AI-Platform-Study/dashboard/app.js
#	AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
#	AI-Platform-Study/dashboard/data.js
#	AI-Platform-Study/dashboard/data/cochrane_dashboard_backend_template.xlsx
#	AI-Platform-Study/dashboard/export-data-js.js
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Resources" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup complete / awaiting abstract screening</t>
+          <t>Abstract Screening</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Project setup and workflow configuration complete; internal team meeting scheduled for 2026-07-08 before abstract screening starts</t>
+          <t>Abstract screening commenced on 2026-07-08; high preparation effort (&gt;30 hours) and Laser AI data extraction constraints under discussion</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Project setup and workflow configuration are complete; internal team meeting scheduled for 2026-07-08 prior to commencing abstract screening</t>
+          <t>Abstract screening commenced on 2026-07-08. Team reported &gt;30 hours of preparation effort before active testing; Laser AI DE constraints/data item preparation remain under discussion.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm readiness at 2026-07-08 internal meeting and commence abstract screening</t>
+          <t>Monitor abstract screening progress; document preparation effort; discuss Laser AI DE constraints with core/Laser AI team</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abstract screening not yet commenced pending internal meeting</t>
+          <t>Abstract screening has commenced; preparation effort was higher than expected and DE setup constraints may need core/Laser AI discussion</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Pending start</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3986,7 +3986,7 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
@@ -4039,12 +4039,16 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
       <c r="K65" s="18" t="n"/>
-      <c r="L65" s="18" t="n"/>
+      <c r="L65" s="18" t="inlineStr">
+        <is>
+          <t>Screening commenced on 2026-07-08.</t>
+        </is>
+      </c>
       <c r="M65" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4092,12 +4096,16 @@
       </c>
       <c r="I66" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
       <c r="K66" s="18" t="n"/>
-      <c r="L66" s="18" t="n"/>
+      <c r="L66" s="18" t="inlineStr">
+        <is>
+          <t>AI-assisted screening commenced / active testing underway.</t>
+        </is>
+      </c>
       <c r="M66" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13000,7 +13008,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Setup phase underway; Laser AI allocated; search/LILACS clarification and remaining setup materials are being finalized; abstract screening has not yet commenced</t>
+          <t>RIS/search results received and uploaded to SharePoint; Laser AI access email resent; other required setup files still missing; abstract screening has not yet commenced</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13017,7 +13025,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Vitamin C is in the setup phase with Laser AI allocated. Search/LILACS clarification and remaining setup materials are being finalized; abstract screening has not yet commenced.</t>
+          <t>Search results received; RIS files uploaded to SharePoint; Laser AI account email resent. Other required setup files were not found in SharePoint/email.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13034,7 +13042,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete setup materials and Laser AI configuration before commencing abstract screening</t>
+          <t>Request/locate protocol, eligibility criteria, data items, and remaining setup files; confirm Laser AI login before configuration/screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13068,7 +13076,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Screening start depends on completion of setup materials and Laser AI configuration</t>
+          <t>Screening start depends on remaining setup files and Laser AI configuration</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -13124,7 +13132,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13206,7 +13214,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>RIS uploaded / remaining files pending</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -13329,12 +13337,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LILACS/search support ongoing</t>
+          <t>RIS files uploaded to SharePoint</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -13373,12 +13381,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Awaiting final materials</t>
+          <t>Required setup file not found in SharePoint/email</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -13395,12 +13403,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Required setup file not found in SharePoint/email</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -13417,12 +13425,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Required setup file not found in SharePoint/email</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -14046,7 +14054,11 @@
       </c>
       <c r="J55" s="18" t="n"/>
       <c r="K55" s="18" t="n"/>
-      <c r="L55" s="18" t="n"/>
+      <c r="L55" s="18" t="inlineStr">
+        <is>
+          <t>Laser AI activation/reset email resent; login confirmation pending.</t>
+        </is>
+      </c>
       <c r="M55" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14200,12 +14212,16 @@
       </c>
       <c r="I58" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J58" s="18" t="n"/>
       <c r="K58" s="18" t="n"/>
-      <c r="L58" s="18" t="n"/>
+      <c r="L58" s="18" t="inlineStr">
+        <is>
+          <t>RIS/search results received and uploaded to SharePoint.</t>
+        </is>
+      </c>
       <c r="M58" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14258,7 +14274,11 @@
       </c>
       <c r="J59" s="18" t="n"/>
       <c r="K59" s="18" t="n"/>
-      <c r="L59" s="18" t="n"/>
+      <c r="L59" s="18" t="inlineStr">
+        <is>
+          <t>Protocol/criteria not found in SharePoint/email.</t>
+        </is>
+      </c>
       <c r="M59" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14311,7 +14331,11 @@
       </c>
       <c r="J60" s="18" t="n"/>
       <c r="K60" s="18" t="n"/>
-      <c r="L60" s="18" t="n"/>
+      <c r="L60" s="18" t="inlineStr">
+        <is>
+          <t>Data items not found in SharePoint/email.</t>
+        </is>
+      </c>
       <c r="M60" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14465,12 +14489,16 @@
       </c>
       <c r="I63" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
-      <c r="L63" s="18" t="n"/>
+      <c r="L63" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup cannot complete until remaining setup files are located/provided.</t>
+        </is>
+      </c>
       <c r="M63" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -22076,7 +22104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="22" customWidth="1" style="29" min="1" max="1"/>
@@ -22267,27 +22295,27 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>Amanda Cross ? Interventions for improving medication-taking ability and adherence in older adults prescribed multiple medications</t>
+          <t>Medication-Taking Ability and Adherence (Amanda Cross)</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
+          <t>Withdrawn &amp; Reason</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
           <t>Withdrawn</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
-        <is>
-          <t>Team has withdrawn from the platform study due to capacity constraints</t>
-        </is>
-      </c>
       <c r="E13" s="17" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>Amanda Cross / Rehan Sarwar</t>
+          <t>Amanda Cross</t>
         </is>
       </c>
       <c r="G13" s="17" t="inlineStr">
@@ -22297,7 +22325,7 @@
       </c>
       <c r="H13" s="17" t="inlineStr">
         <is>
-          <t>Withdrawn due to capacity constraints; retain as historical record</t>
+          <t>Team has withdrawn from the platform study due to capacity constraints.</t>
         </is>
       </c>
       <c r="I13" s="17" t="inlineStr">
@@ -22826,15 +22854,56 @@
       </c>
     </row>
     <row r="30" ht="24" customHeight="1" s="29">
-      <c r="A30" s="17" t="n"/>
-      <c r="B30" s="17" t="n"/>
-      <c r="C30" s="17" t="n"/>
-      <c r="D30" s="17" t="n"/>
-      <c r="E30" s="17" t="n"/>
-      <c r="F30" s="17" t="n"/>
-      <c r="G30" s="17" t="n"/>
-      <c r="H30" s="17" t="n"/>
-      <c r="I30" s="17" t="n"/>
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>new-19</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong — Oral galactagogues</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>Future Phase</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>Potential later-phase candidate; rerun search expected in 10–14 days; prior update work substantially completed; written consent received</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>Later phase / Phase 2</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong; Cochrane Malaysia / Jacqueline J Ho</t>
+        </is>
+      </c>
+      <c r="G30" s="17" t="inlineStr">
+        <is>
+          <t>Rerun search expected July 2026; screening/additional DE August–September 2026; submission October 2026</t>
+        </is>
+      </c>
+      <c r="H30" s="17" t="inlineStr">
+        <is>
+          <t>Initial search completed; 26 new eligible studies; DE and ROB 1 completed; INSPECT-SR and ROB 2 underway; students available in August</t>
+        </is>
+      </c>
+      <c r="I30" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="24" customHeight="1" s="29">
       <c r="A31" s="17" t="n"/>
@@ -23119,6 +23188,100 @@
       <c r="B58" s="18" t="inlineStr">
         <is>
           <t>Not suitable for the current validation phase. Keep brief reason in Remarks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>withdrawn-med-adherence</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Medication-Taking Ability and Adherence (Amanda Cross)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Withdrawn &amp; Reason</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Amanda Cross</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Duplicate hidden; use new-02 withdrawn row.</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>withdrawn-abdominal-irrigation</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Abdominal Irrigation at Caesarean Section (Anna Rogers)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Withdrawn &amp; Reason</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Anna Rogers</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Team has withdrawn from the platform study and will not be participating.</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -26961,9 +27124,21 @@
           <t>mtg-07</t>
         </is>
       </c>
-      <c r="B7" s="25" t="n"/>
-      <c r="C7" s="25" t="n"/>
-      <c r="D7" s="25" t="n"/>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>9:00-10:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>2:00-3:00 PM BST</t>
+        </is>
+      </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
           <t>Human Milk Fortifier Onboarding</t>
@@ -26971,12 +27146,12 @@
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>Onboarding meeting for Human Milk Fortifier; time TBD.</t>
+          <t>Onboarding meeting for Human Milk Fortifier; invite accepted by review team members.</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>Mohan Pammi / Krishna / Core Team</t>
+          <t>Mohan Pammi / Murali Premkumar / Gautham KS / Michelle Fiander / Krishna / Core Team</t>
         </is>
       </c>
       <c r="H7" s="25" t="inlineStr">
@@ -27230,7 +27405,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Onboarded / awaiting template revisions</t>
+          <t>Ready for abstract screening</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -27298,7 +27473,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Onboarding and tool training completed; RIS file, protocol, eligibility criteria, and draft data extraction template received</t>
+          <t>Nested Knowledge project ready for screening with 1,077 citations; screening planned to start on 2026-07-13; Bradley NK access still needs confirmation</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27315,7 +27490,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RIS file, protocol, eligibility criteria, and draft data extraction template received; awaiting final template revisions before project configuration and screening begin</t>
+          <t>Nested Knowledge project is ready for screening with 1,077 citations after 11 duplicates were removed; screening planned to start on 2026-07-13</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27332,7 +27507,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Await final template revisions before project configuration and screening begin</t>
+          <t>Confirm Bradley NK access and begin human/AI-assisted abstract screening on 2026-07-13</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27349,7 +27524,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -27366,7 +27541,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Project configuration and screening depend on final data extraction template revisions</t>
+          <t>Bradley NK user recognition/access still needs confirmation, but project is ready for screening</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -27422,7 +27597,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27504,7 +27679,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Awaiting final template revisions</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -27521,7 +27696,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready to start</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -28330,7 +28505,11 @@
       </c>
       <c r="J55" s="18" t="n"/>
       <c r="K55" s="18" t="n"/>
-      <c r="L55" s="18" t="n"/>
+      <c r="L55" s="18" t="inlineStr">
+        <is>
+          <t>Bradley NK user recognition still needs confirmation.</t>
+        </is>
+      </c>
       <c r="M55" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -28749,12 +28928,16 @@
       </c>
       <c r="I63" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
-      <c r="L63" s="18" t="n"/>
+      <c r="L63" s="18" t="inlineStr">
+        <is>
+          <t>1,077 citations uploaded; 11 duplicates removed.</t>
+        </is>
+      </c>
       <c r="M63" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -28802,12 +28985,16 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
       <c r="K64" s="18" t="n"/>
-      <c r="L64" s="18" t="n"/>
+      <c r="L64" s="18" t="inlineStr">
+        <is>
+          <t>Screening forms reviewed; minor edits made; screening planned for 2026-07-13.</t>
+        </is>
+      </c>
       <c r="M64" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -31891,7 +32078,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Participation confirmed; team roles agreed; onboarding and study material collection underway; tool training pending</t>
+          <t>Participation confirmed; team roles agreed; onboarding meeting scheduled/accepted for 2026-07-14; study material collection underway; tool training pending</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -31908,7 +32095,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Participation confirmed; team roles agreed; study material collection and onboarding are underway</t>
+          <t>Participation confirmed; roles agreed; onboarding meeting scheduled/accepted for 2026-07-14; study materials still pending</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -31925,7 +32112,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Collect study materials, complete Nested Knowledge tool training, and configure project for screening</t>
+          <t>Complete onboarding on 2026-07-14, collect study materials, then complete Nested Knowledge tool training</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -31942,7 +32129,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -31959,7 +32146,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tool training and project configuration pending</t>
+          <t>Onboarding scheduled; tool training and project configuration still pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32015,7 +32202,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32080,7 +32267,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Underway</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -36697,7 +36884,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Full-text screening</t>
+          <t>Full-text complete / DE setup</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -36717,17 +36904,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Full-text screening nearing completion; data extraction setup underway</t>
+          <t>Full-text screening completed; data extraction setup pending improved Laser AI form</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Complete full-text screening by 2026-07-08 and continue data extraction setup</t>
+          <t>Complete post-full-text survey and finalise improved Laser AI data extraction form before data extraction</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -36841,7 +37028,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Setup complete / awaiting abstract screening</t>
+          <t>Abstract Screening</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -36861,17 +37048,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Project setup and workflow configuration complete; internal team meeting scheduled for 2026-07-08 before abstract screening starts</t>
+          <t>Abstract screening commenced on 2026-07-08; high preparation effort (&gt;30 hours) and Laser AI data extraction constraints under discussion</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Confirm readiness at 2026-07-08 internal meeting and commence abstract screening</t>
+          <t>Monitor abstract screening progress; document preparation effort; discuss Laser AI DE constraints with core/Laser AI team</t>
         </is>
       </c>
       <c r="K6" s="22" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -37000,12 +37187,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Setup phase underway; Laser AI allocated; search/LILACS clarification and remaining setup materials are being finalized; abstract screening has not yet commenced</t>
+          <t>RIS/search results received and uploaded to SharePoint; Laser AI access email resent; other required setup files still missing; abstract screening has not yet commenced</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Complete setup materials and Laser AI configuration before commencing abstract screening</t>
+          <t>Request/locate protocol, eligibility criteria, data items, and remaining setup files; confirm Laser AI login before configuration/screening</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -37124,7 +37311,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Onboarded / awaiting template revisions</t>
+          <t>Ready for abstract screening</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -37144,17 +37331,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Onboarding and tool training completed; RIS file, protocol, eligibility criteria, and draft data extraction template received</t>
+          <t>Nested Knowledge project ready for screening with 1,077 citations; screening planned to start on 2026-07-13; Bradley NK access still needs confirmation</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Await final template revisions before project configuration and screening begin</t>
+          <t>Confirm Bradley NK access and begin human/AI-assisted abstract screening on 2026-07-13</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -37216,17 +37403,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Participation confirmed; team roles agreed; onboarding and study material collection underway; tool training pending</t>
+          <t>Participation confirmed; team roles agreed; onboarding meeting scheduled/accepted for 2026-07-14; study material collection underway; tool training pending</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Collect study materials, complete Nested Knowledge tool training, and configure project for screening</t>
+          <t>Complete onboarding on 2026-07-14, collect study materials, complete Nested Knowledge tool training, and configure project for screening</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -50892,7 +51079,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text screening</t>
+          <t>Full-text complete / DE setup</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -50960,7 +51147,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text screening nearing completion; data extraction setup underway</t>
+          <t>Full-text screening completed; data extraction setup pending improved Laser AI form</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -50977,7 +51164,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Full-text screening nearing completion; expected completion 2026-07-08; data extraction setup underway</t>
+          <t>Full-text screening completed; post-full-text survey shared; Laser AI working on improved DE form expected 2026-07-13</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -50994,7 +51181,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete full-text screening by 2026-07-08 and continue data extraction setup</t>
+          <t>Complete post-full-text survey and finalise improved Laser AI data extraction form before data extraction</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -51011,7 +51198,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -51028,7 +51215,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>On track for full-text completion; data extraction setup next dependency</t>
+          <t>Full-text screening complete; data extraction depends on improved Laser AI DE form</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -51084,7 +51271,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -51200,7 +51387,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -51217,7 +51404,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Setup underway</t>
+          <t>DE setup pending improved Laser AI form</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -51365,12 +51552,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Improved Laser AI DE form pending</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -52541,7 +52728,7 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
@@ -53018,7 +53205,7 @@
       </c>
       <c r="I74" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
@@ -53230,7 +53417,7 @@
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
@@ -53283,7 +53470,7 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
@@ -53336,7 +53523,7 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
@@ -53389,7 +53576,7 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
@@ -53548,7 +53735,7 @@
       </c>
       <c r="I84" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J84" s="18" t="n"/>
@@ -53813,7 +54000,7 @@
       </c>
       <c r="I89" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J89" s="18" t="n"/>
@@ -54025,7 +54212,7 @@
       </c>
       <c r="I93" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J93" s="18" t="n"/>

</xml_diff>

<commit_message>
Update review status snapshot
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2286,6 +2286,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2400,7 +2401,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract Screening</t>
+          <t>AI screening paused</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2468,7 +2469,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abstract screening commenced on 2026-07-08; high preparation effort (&gt;30 hours) and Laser AI data extraction constraints under discussion</t>
+          <t>Conventional abstract screening may continue, but AI-assisted screening is paused until 2026-07-20 while workflow and Laser AI updates are addressed.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2485,7 +2486,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abstract screening commenced on 2026-07-08. Team reported &gt;30 hours of preparation effort before active testing; Laser AI DE constraints/data item preparation remain under discussion.</t>
+          <t>Conventional abstract screening may continue, but AI-assisted screening is paused until 2026-07-20 while workflow and Laser AI updates are addressed.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2502,7 +2503,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Monitor abstract screening progress; document preparation effort; discuss Laser AI DE constraints with core/Laser AI team</t>
+          <t>Confirm the restart decision on 2026-07-20; resume AI-assisted screening only after guidance and continue documenting preparation effort.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2519,7 +2520,7 @@
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2592,7 +2593,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2601,6 +2602,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -2736,6 +2738,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -2921,6 +2924,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -3071,6 +3075,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -6493,6 +6498,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -12826,6 +12832,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -12940,7 +12947,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Setup blocked - missing files</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -13008,7 +13015,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RIS/search results received and uploaded to SharePoint; Laser AI access email resent; other required setup files still missing; abstract screening has not yet commenced</t>
+          <t>RIS/search files are uploaded, but the protocol, eligibility criteria and selected data-extraction items are still missing. Screening has not been approved to start.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13025,7 +13032,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Search results received; RIS files uploaded to SharePoint; Laser AI account email resent. Other required setup files were not found in SharePoint/email.</t>
+          <t>RIS/search files are uploaded, but the protocol, eligibility criteria and selected data-extraction items are still missing. Screening has not been approved to start.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13042,7 +13049,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Request/locate protocol, eligibility criteria, data items, and remaining setup files; confirm Laser AI login before configuration/screening</t>
+          <t>Obtain the protocol, inclusion/exclusion criteria and approximately 35 data items; then allow 2-3 working days for Laser AI setup and confirm the screening start.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13132,7 +13139,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13141,6 +13148,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -13276,6 +13284,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -13461,6 +13470,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -13611,6 +13621,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -17045,6 +17056,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -17346,6 +17358,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -17491,6 +17504,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -22866,7 +22880,7 @@
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>Future Phase</t>
+          <t>Under Shortlisting</t>
         </is>
       </c>
       <c r="D30" s="17" t="inlineStr">
@@ -27291,6 +27305,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -27405,7 +27420,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ready for abstract screening</t>
+          <t>Ready / calibration before screening</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -27473,7 +27488,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nested Knowledge project ready for screening with 1,077 citations; screening planned to start on 2026-07-13; Bradley NK access still needs confirmation</t>
+          <t>Nested Knowledge is ready with 1,077 citations. Screening had not started as of 2026-07-15; the team is completing a 100-record calibration and has agreed screening milestones.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27490,7 +27505,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nested Knowledge project is ready for screening with 1,077 citations after 11 duplicates were removed; screening planned to start on 2026-07-13</t>
+          <t>Nested Knowledge is ready with 1,077 citations. Screening had not started as of 2026-07-15; the team is completing a 100-record calibration and has agreed screening milestones.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27507,7 +27522,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm Bradley NK access and begin human/AI-assisted abstract screening on 2026-07-13</t>
+          <t>Complete calibration, start conventional and AI-assisted abstract screening, and finish title/abstract screening by 2026-07-28.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27524,7 +27539,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -27597,7 +27612,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27606,6 +27621,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -27751,6 +27767,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -27936,6 +27953,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -28062,6 +28080,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -31488,6 +31507,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -31729,6 +31749,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -31820,6 +31841,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -31896,6 +31918,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -32010,7 +32033,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Onboarding / materials collection</t>
+          <t>Onboarding and training complete</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32078,7 +32101,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Participation confirmed; team roles agreed; onboarding meeting scheduled/accepted for 2026-07-14; study material collection underway; tool training pending</t>
+          <t>Onboarding and Nested Knowledge training were completed on 2026-07-14. Project setup is waiting for RIS/search results, eligibility criteria, the protocol and approximately 35 data-extraction items.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32095,7 +32118,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Participation confirmed; roles agreed; onboarding meeting scheduled/accepted for 2026-07-14; study materials still pending</t>
+          <t>Onboarding and Nested Knowledge training were completed on 2026-07-14. Project setup is waiting for RIS/search results, eligibility criteria, the protocol and approximately 35 data-extraction items.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32112,7 +32135,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete onboarding on 2026-07-14, collect study materials, then complete Nested Knowledge tool training</t>
+          <t>Collect the missing study files; finalise a comparable 35-item data-extraction list with Sean; then configure the Nested Knowledge project.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32129,7 +32152,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -32202,7 +32225,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32211,6 +32234,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -32356,6 +32380,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -32541,6 +32566,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -32667,6 +32693,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -36081,6 +36108,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -36322,6 +36350,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -36413,6 +36442,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -36884,7 +36914,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Full-text complete / DE setup</t>
+          <t>Data extraction ready</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -36904,17 +36934,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Full-text screening completed; data extraction setup pending improved Laser AI form</t>
+          <t>Laser AI data-extraction template is uploaded and ready. The AI-assisted team will extract only studies included by the conventional team; if more than 10 are included, a random sample of 10 will be used.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Complete post-full-text survey and finalise improved Laser AI data extraction form before data extraction</t>
+          <t>Begin data extraction using the conventional included-study set; randomly select 10 studies if the conventional set exceeds 10.</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -36956,7 +36986,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Abstract Screening</t>
+          <t>DE setup / Laser AI comparison</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -36976,17 +37006,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Conventional title/abstract screening nearing completion; AI-assisted full-text selection almost complete; data extraction preparation/sample planning underway</t>
+          <t>Nested Knowledge screening is complete and the DE workflow is being finalised. A separate Laser AI abstract-screening comparison is set up with 2,225 citations and is ready to begin.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Complete conventional title/abstract screening; prepare common sample of up to 10 studies for later data extraction</t>
+          <t>Finalise the Nested Knowledge DE workflow; run the Laser AI comparison and provide preliminary output for the interim snapshot.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -37028,7 +37058,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Abstract Screening</t>
+          <t>AI screening paused</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -37048,17 +37078,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Abstract screening commenced on 2026-07-08; high preparation effort (&gt;30 hours) and Laser AI data extraction constraints under discussion</t>
+          <t>Conventional abstract screening may continue, but AI-assisted screening is paused until 2026-07-20 while workflow and Laser AI updates are addressed.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Monitor abstract screening progress; document preparation effort; discuss Laser AI DE constraints with core/Laser AI team</t>
+          <t>Confirm the restart decision on 2026-07-20; resume AI-assisted screening only after guidance and continue documenting preparation effort.</t>
         </is>
       </c>
       <c r="K6" s="22" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -37167,7 +37197,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Setup blocked - missing files</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -37187,12 +37217,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>RIS/search results received and uploaded to SharePoint; Laser AI access email resent; other required setup files still missing; abstract screening has not yet commenced</t>
+          <t>RIS/search files are uploaded, but the protocol, eligibility criteria and selected data-extraction items are still missing. Screening has not been approved to start.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Request/locate protocol, eligibility criteria, data items, and remaining setup files; confirm Laser AI login before configuration/screening</t>
+          <t>Obtain the protocol, inclusion/exclusion criteria and approximately 35 data items; then allow 2-3 working days for Laser AI setup and confirm the screening start.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -37311,7 +37341,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Ready for abstract screening</t>
+          <t>Ready / calibration before screening</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -37331,17 +37361,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Nested Knowledge project ready for screening with 1,077 citations; screening planned to start on 2026-07-13; Bradley NK access still needs confirmation</t>
+          <t>Nested Knowledge is ready with 1,077 citations. Screening had not started as of 2026-07-15; the team is completing a 100-record calibration and has agreed screening milestones.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Confirm Bradley NK access and begin human/AI-assisted abstract screening on 2026-07-13</t>
+          <t>Complete calibration, start conventional and AI-assisted abstract screening, and finish title/abstract screening by 2026-07-28.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -37383,7 +37413,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Onboarding / materials collection</t>
+          <t>Onboarding and training complete</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -37403,17 +37433,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Participation confirmed; team roles agreed; onboarding meeting scheduled/accepted for 2026-07-14; study material collection underway; tool training pending</t>
+          <t>Onboarding and Nested Knowledge training were completed on 2026-07-14. Project setup is waiting for RIS/search results, eligibility criteria, the protocol and approximately 35 data-extraction items.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Complete onboarding on 2026-07-14, collect study materials, complete Nested Knowledge tool training, and configure project for screening</t>
+          <t>Collect the missing study files; finalise a comparable 35-item data-extraction list with Sean; then configure the Nested Knowledge project.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -50965,6 +50995,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -51079,7 +51110,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text complete / DE setup</t>
+          <t>Data extraction ready</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -51147,7 +51178,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text screening completed; data extraction setup pending improved Laser AI form</t>
+          <t>Laser AI data-extraction template is uploaded and ready. The AI-assisted team will extract only studies included by the conventional team; if more than 10 are included, a random sample of 10 will be used.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -51164,7 +51195,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Full-text screening completed; post-full-text survey shared; Laser AI working on improved DE form expected 2026-07-13</t>
+          <t>Laser AI data-extraction template is uploaded and ready. The AI-assisted team will extract only studies included by the conventional team; if more than 10 are included, a random sample of 10 will be used.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -51181,7 +51212,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete post-full-text survey and finalise improved Laser AI data extraction form before data extraction</t>
+          <t>Begin data extraction using the conventional included-study set; randomly select 10 studies if the conventional set exceeds 10.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -51198,7 +51229,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -51271,7 +51302,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -51280,6 +51311,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -51425,6 +51457,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -51610,6 +51643,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -51760,6 +51794,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -55174,6 +55209,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -55695,6 +55731,7 @@
     <row r="124" s="29"/>
     <row r="125" s="29"/>
     <row r="126" s="29"/>
+    <row r="127"/>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
@@ -56150,6 +56187,7 @@
     <row r="138" s="29"/>
     <row r="139" s="29"/>
     <row r="140" s="29"/>
+    <row r="141"/>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
         <is>
@@ -56349,6 +56387,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -56463,7 +56502,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract Screening</t>
+          <t>DE setup / Laser AI comparison</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56531,7 +56570,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Conventional title/abstract screening nearing completion; AI-assisted full-text selection almost complete; data extraction preparation/sample planning underway</t>
+          <t>Nested Knowledge screening is complete and the DE workflow is being finalised. A separate Laser AI abstract-screening comparison is set up with 2,225 citations and is ready to begin.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56548,7 +56587,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Conventional title/abstract screening is nearing completion; AI-assisted full-text selection is almost complete. The team is preparing a common sample of up to 10 studies for later data extraction.</t>
+          <t>Nested Knowledge screening is complete and the DE workflow is being finalised. A separate Laser AI abstract-screening comparison is set up with 2,225 citations and is ready to begin.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56565,7 +56604,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete conventional title/abstract screening; prepare common sample of up to 10 studies for later data extraction</t>
+          <t>Finalise the Nested Knowledge DE workflow; run the Laser AI comparison and provide preliminary output for the interim snapshot.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56582,7 +56621,7 @@
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56655,7 +56694,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56664,6 +56703,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -56809,6 +56849,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -56994,6 +57035,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -57144,6 +57186,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -60558,6 +60601,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -61129,6 +61173,7 @@
     <row r="124" s="29"/>
     <row r="125" s="29"/>
     <row r="126" s="29"/>
+    <row r="127"/>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
@@ -61697,6 +61742,7 @@
     </row>
     <row r="138" s="29"/>
     <row r="139" s="29"/>
+    <row r="140"/>
     <row r="141">
       <c r="A141" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Hold Fruit and Veg AI screening
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AI screening paused</t>
+          <t>AI screening on hold</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Conventional abstract screening may continue, but AI-assisted screening is paused until 2026-07-20 while workflow and Laser AI updates are addressed.</t>
+          <t>The review team has been asked to hold AI-assisted abstract screening while workflow guidance and Laser AI updates are addressed. Conventional abstract screening may continue.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Conventional abstract screening may continue, but AI-assisted screening is paused until 2026-07-20 while workflow and Laser AI updates are addressed.</t>
+          <t>The review team has been asked to hold AI-assisted abstract screening while workflow guidance and Laser AI updates are addressed. Conventional abstract screening may continue.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm the restart decision on 2026-07-20; resume AI-assisted screening only after guidance and continue documenting preparation effort.</t>
+          <t>Confirm the restart decision on 2026-07-20; resume AI-assisted screening only after guidance is agreed and continue documenting preparation effort.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -12832,7 +12832,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -13148,7 +13147,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -13284,7 +13282,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -13470,7 +13467,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -13621,7 +13617,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -17056,7 +17051,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -17358,7 +17352,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -17504,7 +17497,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -27305,7 +27297,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -27621,7 +27612,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -27767,7 +27757,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -27953,7 +27942,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -28080,7 +28068,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -31507,7 +31494,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -31749,7 +31735,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -31841,7 +31826,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -31918,7 +31902,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -32234,7 +32217,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -32380,7 +32362,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -32566,7 +32547,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -32693,7 +32673,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -36108,7 +36087,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -36350,7 +36328,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -36442,7 +36419,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -37058,7 +37034,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AI screening paused</t>
+          <t>AI screening on hold</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -37078,12 +37054,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Conventional abstract screening may continue, but AI-assisted screening is paused until 2026-07-20 while workflow and Laser AI updates are addressed.</t>
+          <t>The review team has been asked to hold AI-assisted abstract screening while workflow guidance and Laser AI updates are addressed. Conventional abstract screening may continue.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Confirm the restart decision on 2026-07-20; resume AI-assisted screening only after guidance and continue documenting preparation effort.</t>
+          <t>Confirm the restart decision on 2026-07-20; resume AI-assisted screening only after guidance is agreed and continue documenting preparation effort.</t>
         </is>
       </c>
       <c r="K6" s="22" t="inlineStr">
@@ -50995,7 +50971,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -51311,7 +51286,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -51457,7 +51431,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -51643,7 +51616,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -51794,7 +51766,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -55209,7 +55180,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -55731,7 +55701,6 @@
     <row r="124" s="29"/>
     <row r="125" s="29"/>
     <row r="126" s="29"/>
-    <row r="127"/>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
@@ -56187,7 +56156,6 @@
     <row r="138" s="29"/>
     <row r="139" s="29"/>
     <row r="140" s="29"/>
-    <row r="141"/>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
         <is>
@@ -56387,7 +56355,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -56703,7 +56670,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -56849,7 +56815,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -57035,7 +57000,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -57186,7 +57150,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -60601,7 +60564,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -61173,7 +61135,6 @@
     <row r="124" s="29"/>
     <row r="125" s="29"/>
     <row r="126" s="29"/>
-    <row r="127"/>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
@@ -61742,7 +61703,6 @@
     </row>
     <row r="138" s="29"/>
     <row r="139" s="29"/>
-    <row r="140"/>
     <row r="141">
       <c r="A141" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update dashboard date to July 17
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2593,7 +2593,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2602,7 +2602,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -2738,7 +2737,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -2924,7 +2922,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -3075,7 +3072,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -6498,7 +6494,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -7815,6 +7810,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -8116,7 +8112,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -12832,6 +12828,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -13138,7 +13135,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -17622,6 +17619,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -17928,7 +17926,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27297,6 +27295,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -27603,7 +27602,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -31902,6 +31901,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -32208,7 +32208,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -41565,6 +41565,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -41866,7 +41867,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -46330,6 +46331,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -46631,7 +46633,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -50971,6 +50973,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -51277,7 +51280,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56355,6 +56358,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -56661,7 +56665,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">

</xml_diff>

<commit_message>
Update Global Dashboard timeline and meetings
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -1,37 +1,21 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
+  <dc:creator xmlns:dc="http://purl.org/dc/elements/1.1/">Krishna Kishore Pandalaneni</dc:creator>
+  <dcterms:created xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-05-27T01:47:03Z</dcterms:created>
+  <dcterms:modified xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-07-16T17:29:25Z</dcterms:modified>
+  <cp:lastModifiedBy>Krishna Kishore Pandalaneni</cp:lastModifiedBy>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="9">
@@ -324,7 +308,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewIndexTable" displayName="ReviewIndexTable" ref="A1:N11" headerRowCount="1">
   <tableColumns count="14">
     <tableColumn id="1" name="ReviewID"/>
@@ -346,7 +330,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table10.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Workflow_Caffeine_5" displayName="Workflow_Caffeine_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -364,7 +348,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Tasks_Caffeine_6" displayName="Tasks_Caffeine_6" ref="A114:K117" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -383,7 +367,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Comms_Caffeine_7" displayName="Comms_Caffeine_7" ref="A120:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -404,7 +388,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="Critical_Caffeine_8" displayName="Critical_Caffeine_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -419,7 +403,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="Executive_DMARDsRA_1" displayName="Executive_DMARDsRA_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -431,7 +415,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table15.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="Milestones_DMARDsRA_2" displayName="Milestones_DMARDsRA_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -445,7 +429,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table16.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="Files_DMARDsRA_3" displayName="Files_DMARDsRA_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -460,7 +444,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table17.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="Stages_DMARDsRA_4" displayName="Stages_DMARDsRA_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -476,7 +460,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table18.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="Workflow_DMARDsRA_5" displayName="Workflow_DMARDsRA_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -494,7 +478,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table19.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="Tasks_DMARDsRA_6" displayName="Tasks_DMARDsRA_6" ref="A114:K116" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -513,7 +497,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Workflow63ActionsTable" displayName="Workflow63ActionsTable" ref="A1:G64" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="Workflow Master"/>
@@ -528,7 +512,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table20.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="Comms_DMARDsRA_7" displayName="Comms_DMARDsRA_7" ref="A119:M120" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -549,7 +533,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table21.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Critical_DMARDsRA_8" displayName="Critical_DMARDsRA_8" ref="A123:G124" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -564,7 +548,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table22.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="Executive_BPTargets_1" displayName="Executive_BPTargets_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -576,7 +560,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table23.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="Milestones_BPTargets_2" displayName="Milestones_BPTargets_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -590,7 +574,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table24.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="Files_BPTargets_3" displayName="Files_BPTargets_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -605,7 +589,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table25.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="Stages_BPTargets_4" displayName="Stages_BPTargets_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -621,7 +605,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table26.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="Workflow_BPTargets_5" displayName="Workflow_BPTargets_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -639,7 +623,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table27.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="Tasks_BPTargets_6" displayName="Tasks_BPTargets_6" ref="A114:K122" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -658,7 +642,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table28.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="Comms_BPTargets_7" displayName="Comms_BPTargets_7" ref="A129:M135" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -679,7 +663,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table29.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="Critical_BPTargets_8" displayName="Critical_BPTargets_8" ref="A143:G146" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -694,7 +678,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="GlobalPhaseCards" displayName="GlobalPhaseCards" ref="A4:E9" headerRowCount="1">
   <tableColumns count="5">
     <tableColumn id="1" name="PhaseKey"/>
@@ -707,7 +691,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table30.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="Executive_Psoriasis_1" displayName="Executive_Psoriasis_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -719,7 +703,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table31.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="Milestones_Psoriasis_2" displayName="Milestones_Psoriasis_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -733,7 +717,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table32.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="Files_Psoriasis_3" displayName="Files_Psoriasis_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -748,7 +732,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table33.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="Stages_Psoriasis_4" displayName="Stages_Psoriasis_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -764,7 +748,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table34.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="Workflow_Psoriasis_5" displayName="Workflow_Psoriasis_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -782,7 +766,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table35.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="Tasks_Psoriasis_6" displayName="Tasks_Psoriasis_6" ref="A114:K123" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -801,7 +785,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table36.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="Comms_Psoriasis_7" displayName="Comms_Psoriasis_7" ref="A129:M132" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -822,7 +806,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table37.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="Critical_Psoriasis_8" displayName="Critical_Psoriasis_8" ref="A142:G146" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -837,7 +821,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table38.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="Executive_FruitVeg_1" displayName="Executive_FruitVeg_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -849,7 +833,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table39.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="Milestones_FruitVeg_2" displayName="Milestones_FruitVeg_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -863,7 +847,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="GlobalResources" displayName="GlobalResources" ref="A13:H18" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="ResourceID"/>
@@ -879,7 +863,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table40.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table40.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="Files_FruitVeg_3" displayName="Files_FruitVeg_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -894,7 +878,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table41.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="Stages_FruitVeg_4" displayName="Stages_FruitVeg_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -910,7 +894,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table42.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="Workflow_FruitVeg_5" displayName="Workflow_FruitVeg_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -928,7 +912,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table43.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="Tasks_FruitVeg_6" displayName="Tasks_FruitVeg_6" ref="A114:K123" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -947,7 +931,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table44.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="Comms_FruitVeg_7" displayName="Comms_FruitVeg_7" ref="A125:M132" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -968,7 +952,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table45.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="Critical_FruitVeg_8" displayName="Critical_FruitVeg_8" ref="A135:G139" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -983,7 +967,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table46.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="Executive_Chlamydia_1" displayName="Executive_Chlamydia_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -995,7 +979,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table47.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="Milestones_Chlamydia_2" displayName="Milestones_Chlamydia_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1009,7 +993,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table48.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="Files_Chlamydia_3" displayName="Files_Chlamydia_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1024,7 +1008,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table49.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="Stages_Chlamydia_4" displayName="Stages_Chlamydia_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1040,7 +1024,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GlobalUpcomingMeetings" displayName="GlobalUpcomingMeetings" ref="A22:H28" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="MeetingID"/>
@@ -1056,7 +1040,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table50.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table50.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="Workflow_Chlamydia_5" displayName="Workflow_Chlamydia_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1074,7 +1058,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table51.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="Tasks_Chlamydia_6" displayName="Tasks_Chlamydia_6" ref="A114:K118" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1093,7 +1077,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table52.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="Comms_Chlamydia_7" displayName="Comms_Chlamydia_7" ref="A121:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1114,7 +1098,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table53.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="Critical_Chlamydia_8" displayName="Critical_Chlamydia_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1129,7 +1113,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table54.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="Executive_Review5TBD_1" displayName="Executive_Review5TBD_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1141,7 +1125,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table55.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="Milestones_Review5TBD_2" displayName="Milestones_Review5TBD_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1155,7 +1139,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table56.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="Files_Review5TBD_3" displayName="Files_Review5TBD_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1170,7 +1154,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table57.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="Stages_Review5TBD_4" displayName="Stages_Review5TBD_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1186,7 +1170,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table58.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="Workflow_Review5TBD_5" displayName="Workflow_Review5TBD_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1204,7 +1188,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table59.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table59.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="Tasks_Review5TBD_6" displayName="Tasks_Review5TBD_6" ref="A114:K118" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1223,7 +1207,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Executive_Caffeine_1" displayName="Executive_Caffeine_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1235,7 +1219,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table60.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table60.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="Comms_Review5TBD_7" displayName="Comms_Review5TBD_7" ref="A121:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1256,7 +1240,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table61.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="Critical_Review5TBD_8" displayName="Critical_Review5TBD_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1271,7 +1255,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table62.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="Executive_Phase2Batch_1" displayName="Executive_Phase2Batch_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1283,7 +1267,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table63.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="Milestones_Phase2Batch_2" displayName="Milestones_Phase2Batch_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1297,7 +1281,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table64.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="64" name="Files_Phase2Batch_3" displayName="Files_Phase2Batch_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1312,7 +1296,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table65.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="65" name="Stages_Phase2Batch_4" displayName="Stages_Phase2Batch_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1328,7 +1312,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table66.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="66" name="Workflow_Phase2Batch_5" displayName="Workflow_Phase2Batch_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1346,7 +1330,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table67.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="67" name="Tasks_Phase2Batch_6" displayName="Tasks_Phase2Batch_6" ref="A114:K115" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1365,7 +1349,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table68.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="68" name="Comms_Phase2Batch_7" displayName="Comms_Phase2Batch_7" ref="A118:M119" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1386,7 +1370,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table69.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table69.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="Critical_Phase2Batch_8" displayName="Critical_Phase2Batch_8" ref="A122:G123" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1401,7 +1385,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Milestones_Caffeine_2" displayName="Milestones_Caffeine_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1415,7 +1399,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table70.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table70.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="CandidatePipeline" displayName="CandidatePipeline" ref="A11:J29" headerRowCount="1">
   <tableColumns count="9">
     <tableColumn id="1" name="CandidateID"/>
@@ -1432,7 +1416,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table71.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="71" name="UpcomingMeetingsTable" displayName="UpcomingMeetingsTable" ref="A1:M6" headerRowCount="1">
   <autoFilter ref="A1:M6"/>
   <tableColumns count="13">
@@ -1454,7 +1438,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Files_Caffeine_3" displayName="Files_Caffeine_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1469,7 +1453,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table9.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Stages_Caffeine_4" displayName="Stages_Caffeine_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1485,7 +1469,7 @@
 </table>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
     <a:clrScheme name="ChatGPT">
@@ -1632,7 +1616,39 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2254,7 +2270,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2591,9 +2607,9 @@
           <t>LastUpdated</t>
         </is>
       </c>
-      <c r="B20" s="22" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -7778,7 +7794,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8112,7 +8128,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -12534,7 +12550,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12796,7 +12812,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13135,7 +13151,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -17587,7 +17603,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17926,7 +17942,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -22102,7 +22118,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23303,7 +23319,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26742,7 +26758,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27263,7 +27279,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27602,7 +27618,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -31869,7 +31885,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -32208,7 +32224,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -36463,7 +36479,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -36645,7 +36661,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -37446,7 +37462,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40912,7 +40928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41016,7 +41032,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mid April to End June</t>
+          <t>Mid April onward</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -41043,12 +41059,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>End June</t>
+          <t>July 2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Decision Gate</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -41070,12 +41086,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Start July to End September</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Pending decision</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -41097,12 +41113,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>Q3 2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Interim snapshot ready</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -41361,17 +41377,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>meet-001</t>
+          <t>mtg-05</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>15 May 2026</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Usability survey tracking discussion</t>
+          <t>Fruit &amp; Veg Re-onboarding</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Rebecca K. Hodder / Krishna / Core Team</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Re-onboarding meeting for Fruit &amp; Veg; time TBD.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -41379,6 +41405,11 @@
           <t>Scheduled</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Time TBD</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -41386,137 +41417,37 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>meet-002</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>18 May 2026</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Core team discussion with Meghan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Sent</t>
-        </is>
-      </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>meet-003</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>19 May 2026</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>BP Targets review team check-in</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Sent</t>
-        </is>
-      </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>meet-004</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>19 May 2026</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Psoriasis review team check-in</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Sent</t>
-        </is>
-      </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>meet-005</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>19 May 2026</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Adjudication pilot deadline</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>meet-006</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>21 May 2026</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>PM + PI meeting</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Sent</t>
-        </is>
-      </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -41533,7 +41464,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41867,7 +41798,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -46299,7 +46230,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -46633,7 +46564,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -50941,7 +50872,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -51280,7 +51211,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56326,7 +56257,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -56663,9 +56594,9 @@
           <t>LastUpdated</t>
         </is>
       </c>
-      <c r="B20" s="22" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">

</xml_diff>

<commit_message>
Update Phase 1 milestone states
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>RIS uploaded / remaining files pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -13246,11 +13246,6 @@
       <c r="A26" t="inlineStr">
         <is>
           <t>abstract</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Not Started</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -32289,7 +32284,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -32321,11 +32316,6 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32338,11 +32328,6 @@
           <t>fullText</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32353,11 +32338,6 @@
       <c r="A28" t="inlineStr">
         <is>
           <t>extraction</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Not Started</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -56695,7 +56675,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Active / nearing completion</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -56710,11 +56690,6 @@
           <t>fullText</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>AI-assisted full-text selection almost complete</t>
-        </is>
-      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -56725,11 +56700,6 @@
       <c r="A28" t="inlineStr">
         <is>
           <t>extraction</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Preparation only</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">

</xml_diff>

<commit_message>
Update July review dashboard snapshot
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -1,21 +1,37 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
-  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
-  <AppVersion>3.1</AppVersion>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
-  <dc:creator xmlns:dc="http://purl.org/dc/elements/1.1/">Krishna Kishore Pandalaneni</dc:creator>
-  <dcterms:created xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-05-27T01:47:03Z</dcterms:created>
-  <dcterms:modified xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-07-16T17:29:25Z</dcterms:modified>
-  <cp:lastModifiedBy>Krishna Kishore Pandalaneni</cp:lastModifiedBy>
-</cp:coreProperties>
-</file>
-
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="9">
@@ -308,7 +324,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\tables\table1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewIndexTable" displayName="ReviewIndexTable" ref="A1:N11" headerRowCount="1">
   <tableColumns count="14">
     <tableColumn id="1" name="ReviewID"/>
@@ -330,7 +346,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Workflow_Caffeine_5" displayName="Workflow_Caffeine_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -348,7 +364,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Tasks_Caffeine_6" displayName="Tasks_Caffeine_6" ref="A114:K117" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -367,7 +383,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Comms_Caffeine_7" displayName="Comms_Caffeine_7" ref="A120:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -388,7 +404,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="Critical_Caffeine_8" displayName="Critical_Caffeine_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -403,7 +419,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="Executive_DMARDsRA_1" displayName="Executive_DMARDsRA_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -415,7 +431,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="Milestones_DMARDsRA_2" displayName="Milestones_DMARDsRA_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -429,7 +445,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="Files_DMARDsRA_3" displayName="Files_DMARDsRA_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -444,7 +460,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="Stages_DMARDsRA_4" displayName="Stages_DMARDsRA_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -460,7 +476,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="Workflow_DMARDsRA_5" displayName="Workflow_DMARDsRA_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -478,7 +494,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="Tasks_DMARDsRA_6" displayName="Tasks_DMARDsRA_6" ref="A114:K116" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -497,7 +513,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Workflow63ActionsTable" displayName="Workflow63ActionsTable" ref="A1:G64" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="Workflow Master"/>
@@ -512,7 +528,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="Comms_DMARDsRA_7" displayName="Comms_DMARDsRA_7" ref="A119:M120" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -533,7 +549,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Critical_DMARDsRA_8" displayName="Critical_DMARDsRA_8" ref="A123:G124" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -548,7 +564,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="Executive_BPTargets_1" displayName="Executive_BPTargets_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -560,7 +576,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="Milestones_BPTargets_2" displayName="Milestones_BPTargets_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -574,7 +590,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="Files_BPTargets_3" displayName="Files_BPTargets_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -589,7 +605,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="Stages_BPTargets_4" displayName="Stages_BPTargets_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -605,7 +621,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="Workflow_BPTargets_5" displayName="Workflow_BPTargets_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -623,7 +639,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="Tasks_BPTargets_6" displayName="Tasks_BPTargets_6" ref="A114:K122" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -642,7 +658,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="Comms_BPTargets_7" displayName="Comms_BPTargets_7" ref="A129:M135" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -663,7 +679,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="Critical_BPTargets_8" displayName="Critical_BPTargets_8" ref="A143:G146" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -678,7 +694,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="GlobalPhaseCards" displayName="GlobalPhaseCards" ref="A4:E9" headerRowCount="1">
   <tableColumns count="5">
     <tableColumn id="1" name="PhaseKey"/>
@@ -691,7 +707,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="Executive_Psoriasis_1" displayName="Executive_Psoriasis_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -703,7 +719,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="Milestones_Psoriasis_2" displayName="Milestones_Psoriasis_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -717,7 +733,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="Files_Psoriasis_3" displayName="Files_Psoriasis_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -732,7 +748,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="Stages_Psoriasis_4" displayName="Stages_Psoriasis_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -748,7 +764,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="Workflow_Psoriasis_5" displayName="Workflow_Psoriasis_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -766,7 +782,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="Tasks_Psoriasis_6" displayName="Tasks_Psoriasis_6" ref="A114:K123" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -785,7 +801,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="Comms_Psoriasis_7" displayName="Comms_Psoriasis_7" ref="A129:M132" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -806,7 +822,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="Critical_Psoriasis_8" displayName="Critical_Psoriasis_8" ref="A142:G146" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -821,7 +837,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="Executive_FruitVeg_1" displayName="Executive_FruitVeg_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -833,7 +849,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="Milestones_FruitVeg_2" displayName="Milestones_FruitVeg_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -847,7 +863,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="GlobalResources" displayName="GlobalResources" ref="A13:H18" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="ResourceID"/>
@@ -863,7 +879,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table40.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table40.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="Files_FruitVeg_3" displayName="Files_FruitVeg_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -878,7 +894,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table41.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="Stages_FruitVeg_4" displayName="Stages_FruitVeg_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -894,7 +910,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table42.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="Workflow_FruitVeg_5" displayName="Workflow_FruitVeg_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -912,7 +928,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table43.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="Tasks_FruitVeg_6" displayName="Tasks_FruitVeg_6" ref="A114:K123" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -931,7 +947,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table44.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="Comms_FruitVeg_7" displayName="Comms_FruitVeg_7" ref="A125:M132" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -952,7 +968,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table45.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="Critical_FruitVeg_8" displayName="Critical_FruitVeg_8" ref="A135:G139" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -967,7 +983,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table46.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="Executive_Chlamydia_1" displayName="Executive_Chlamydia_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -979,7 +995,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table47.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="Milestones_Chlamydia_2" displayName="Milestones_Chlamydia_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -993,7 +1009,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table48.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="Files_Chlamydia_3" displayName="Files_Chlamydia_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1008,7 +1024,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table49.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="Stages_Chlamydia_4" displayName="Stages_Chlamydia_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1024,7 +1040,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GlobalUpcomingMeetings" displayName="GlobalUpcomingMeetings" ref="A22:H28" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="MeetingID"/>
@@ -1040,7 +1056,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table50.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table50.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="Workflow_Chlamydia_5" displayName="Workflow_Chlamydia_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1058,7 +1074,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table51.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="Tasks_Chlamydia_6" displayName="Tasks_Chlamydia_6" ref="A114:K118" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1077,7 +1093,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table52.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="Comms_Chlamydia_7" displayName="Comms_Chlamydia_7" ref="A121:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1098,7 +1114,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table53.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="Critical_Chlamydia_8" displayName="Critical_Chlamydia_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1113,7 +1129,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table54.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="Executive_Review5TBD_1" displayName="Executive_Review5TBD_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1125,7 +1141,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table55.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="Milestones_Review5TBD_2" displayName="Milestones_Review5TBD_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1139,7 +1155,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table56.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="Files_Review5TBD_3" displayName="Files_Review5TBD_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1154,7 +1170,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table57.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="Stages_Review5TBD_4" displayName="Stages_Review5TBD_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1170,7 +1186,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table58.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="Workflow_Review5TBD_5" displayName="Workflow_Review5TBD_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1188,7 +1204,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table59.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table59.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="Tasks_Review5TBD_6" displayName="Tasks_Review5TBD_6" ref="A114:K118" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1207,7 +1223,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Executive_Caffeine_1" displayName="Executive_Caffeine_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1219,7 +1235,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table60.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table60.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="Comms_Review5TBD_7" displayName="Comms_Review5TBD_7" ref="A121:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1240,7 +1256,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table61.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="Critical_Review5TBD_8" displayName="Critical_Review5TBD_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1255,7 +1271,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table62.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="Executive_Phase2Batch_1" displayName="Executive_Phase2Batch_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1267,7 +1283,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table63.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="Milestones_Phase2Batch_2" displayName="Milestones_Phase2Batch_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1281,7 +1297,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table64.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="64" name="Files_Phase2Batch_3" displayName="Files_Phase2Batch_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1296,7 +1312,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table65.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="65" name="Stages_Phase2Batch_4" displayName="Stages_Phase2Batch_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1312,7 +1328,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table66.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="66" name="Workflow_Phase2Batch_5" displayName="Workflow_Phase2Batch_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1330,7 +1346,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table67.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="67" name="Tasks_Phase2Batch_6" displayName="Tasks_Phase2Batch_6" ref="A114:K115" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1349,7 +1365,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table68.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="68" name="Comms_Phase2Batch_7" displayName="Comms_Phase2Batch_7" ref="A118:M119" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1370,7 +1386,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table69.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table69.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="Critical_Phase2Batch_8" displayName="Critical_Phase2Batch_8" ref="A122:G123" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1385,7 +1401,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Milestones_Caffeine_2" displayName="Milestones_Caffeine_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1399,7 +1415,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table70.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table70.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="CandidatePipeline" displayName="CandidatePipeline" ref="A11:J29" headerRowCount="1">
   <tableColumns count="9">
     <tableColumn id="1" name="CandidateID"/>
@@ -1416,7 +1432,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table71.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="71" name="UpcomingMeetingsTable" displayName="UpcomingMeetingsTable" ref="A1:M6" headerRowCount="1">
   <autoFilter ref="A1:M6"/>
   <tableColumns count="13">
@@ -1438,7 +1454,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Files_Caffeine_3" displayName="Files_Caffeine_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1453,7 +1469,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Stages_Caffeine_4" displayName="Stages_Caffeine_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1469,7 +1485,7 @@
 </table>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
     <a:clrScheme name="ChatGPT">
@@ -1616,39 +1632,7 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2270,7 +2254,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2485,7 +2469,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The review team has been asked to hold AI-assisted abstract screening while workflow guidance and Laser AI updates are addressed. Conventional abstract screening may continue.</t>
+          <t>AI-assisted abstract screening remains paused as of 2026-07-21 while Laser AI workflow guidance and platform updates are reviewed. Conventional abstract screening may continue.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2502,7 +2486,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The review team has been asked to hold AI-assisted abstract screening while workflow guidance and Laser AI updates are addressed. Conventional abstract screening may continue.</t>
+          <t>AI-assisted abstract screening remains paused as of 2026-07-21 while Laser AI workflow guidance and platform updates are reviewed. Conventional abstract screening may continue.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2519,7 +2503,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm the restart decision on 2026-07-20; resume AI-assisted screening only after guidance is agreed and continue documenting preparation effort.</t>
+          <t>Obtain the core-team restart decision and revised Laser AI guidance before resuming AI-assisted screening; continue recording preparation and screening time separately.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2536,7 +2520,7 @@
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2553,7 +2537,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abstract screening has commenced; preparation effort was higher than expected and DE setup constraints may need core/Laser AI discussion</t>
+          <t>AI-assisted screening remains paused; the team reported more than 30 hours of preparation before active testing, approximate and not formally tracked.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2607,9 +2591,9 @@
           <t>LastUpdated</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2708,7 +2692,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Paused - conventional may continue</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -7794,7 +7778,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8128,7 +8112,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -12550,7 +12534,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12812,7 +12796,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12959,7 +12943,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup blocked - missing files</t>
+          <t>Setup in progress - search access issue</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -13027,7 +13011,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RIS/search files are uploaded, but the protocol, eligibility criteria and selected data-extraction items are still missing. Screening has not been approved to start.</t>
+          <t>The protocol and 35 selected data-extraction items have been received, and the live extraction document has been updated. Search/RIS files are available, but LILACS and IBECS remain inaccessible; screening has not yet been approved to start.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13044,7 +13028,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RIS/search files are uploaded, but the protocol, eligibility criteria and selected data-extraction items are still missing. Screening has not been approved to start.</t>
+          <t>The protocol and 35 selected data-extraction items have been received, and the live extraction document has been updated. Search/RIS files are available, but LILACS and IBECS remain inaccessible; screening has not yet been approved to start.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13061,7 +13045,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Obtain the protocol, inclusion/exclusion criteria and approximately 35 data items; then allow 2-3 working days for Laser AI setup and confirm the screening start.</t>
+          <t>Resolve or document the inaccessible LILACS/IBECS searches, review the “Vit C” search-term concern, finalise Laser AI setup, and confirm when screening may start.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13095,7 +13079,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Screening start depends on remaining setup files and Laser AI configuration</t>
+          <t>Most setup materials are now available; database-access and search-strategy issues remain before screening can start.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -13151,7 +13135,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13233,7 +13217,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Protocol/data items received; search access issue pending</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -13246,6 +13230,11 @@
       <c r="A26" t="inlineStr">
         <is>
           <t>abstract</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -13356,7 +13345,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>RIS files uploaded to SharePoint</t>
+          <t>Search/RIS files received; some database searches unavailable</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -13395,12 +13384,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Required setup file not found in SharePoint/email</t>
+          <t>Eligibility criteria provided in protocol</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -13417,12 +13406,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Required setup file not found in SharePoint/email</t>
+          <t>35 selected data items received; live document updated</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -13439,12 +13428,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Required setup file not found in SharePoint/email</t>
+          <t>Protocol received</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -17598,7 +17587,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17937,7 +17926,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -22113,7 +22102,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22268,7 +22257,7 @@
       </c>
       <c r="D12" s="17" t="inlineStr">
         <is>
-          <t>Participation confirmed; team roles agreed; onboarding and study material collection underway; tool training pending</t>
+          <t>Onboarding and Nested Knowledge training completed; study materials and setup inputs pending</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22283,12 +22272,12 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>Onboarding and study material collection underway</t>
+          <t>Training complete; study material collection underway</t>
         </is>
       </c>
       <c r="H12" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-07 Human Milk; Nested Knowledge allocated; tool training pending</t>
+          <t>Converted to phase1-07 Human Milk; Nested Knowledge allocated; training complete; awaiting study files and setup inputs</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -22412,7 +22401,7 @@
       </c>
       <c r="D15" s="17" t="inlineStr">
         <is>
-          <t>Tracked as phase1-05</t>
+          <t>Protocol and 35 data items received; search files uploaded; LILACS/IBECS access issue remains</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
@@ -22427,12 +22416,12 @@
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>Search update in progress</t>
+          <t>Setup in progress; database-access issue unresolved</t>
         </is>
       </c>
       <c r="H15" s="17" t="inlineStr">
         <is>
-          <t>Final updated search/RIS and remaining study materials pending; Sean supporting LILACS/search issue</t>
+          <t>Converted to phase1-05 Vitamin C; protocol and data items received; screening awaits resolution or documentation of inaccessible databases</t>
         </is>
       </c>
       <c r="I15" s="17" t="inlineStr">
@@ -23314,7 +23303,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26753,7 +26742,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27088,7 +27077,11 @@
           <t>mtg-06</t>
         </is>
       </c>
-      <c r="B6" s="25" t="n"/>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
       <c r="C6" s="25" t="n"/>
       <c r="D6" s="25" t="n"/>
       <c r="E6" s="25" t="inlineStr">
@@ -27098,7 +27091,7 @@
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>Nested Knowledge training for Human Milk Fortifier; time TBD.</t>
+          <t>Nested Knowledge training completed for Human Milk Fortifier.</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
@@ -27118,7 +27111,7 @@
       </c>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="K6" s="25" t="inlineStr">
@@ -27181,7 +27174,7 @@
       </c>
       <c r="J7" s="25" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="K7" s="25" t="inlineStr">
@@ -27274,7 +27267,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27613,7 +27606,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -31880,7 +31873,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -32163,7 +32156,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Onboarding scheduled; tool training and project configuration still pending</t>
+          <t>Training is complete; project configuration is pending the RIS/search files, eligibility criteria, protocol and selected data-extraction items.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32219,7 +32212,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32316,6 +32309,11 @@
           <t>abstract</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32328,6 +32326,11 @@
           <t>fullText</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32338,6 +32341,11 @@
       <c r="A28" t="inlineStr">
         <is>
           <t>extraction</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -36459,7 +36467,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -36641,7 +36649,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -36886,7 +36894,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Data extraction ready</t>
+          <t>Data extraction underway</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -36906,17 +36914,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Laser AI data-extraction template is uploaded and ready. The AI-assisted team will extract only studies included by the conventional team; if more than 10 are included, a random sample of 10 will be used.</t>
+          <t>Data extraction is underway in both workflows. The team expects to complete extraction during the week of 2026-08-03. The AI-assisted team is using the conventional included-study set, capped at 10 studies if needed.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Begin data extraction using the conventional included-study set; randomly select 10 studies if the conventional set exceeds 10.</t>
+          <t>Complete conventional and Laser AI data extraction, notify the project team when both workflows are finished, and submit the extraction outputs and time logs.</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Week of 2026-08-03</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -36958,7 +36966,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>DE setup / Laser AI comparison</t>
+          <t>DE preparation / validation analysis</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -36978,17 +36986,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Nested Knowledge screening is complete and the DE workflow is being finalised. A separate Laser AI abstract-screening comparison is set up with 2,225 citations and is ready to begin.</t>
+          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete. Ten studies have been selected for data extraction. Ten repeated Laser AI abstract-screening outputs were received; Run 10 appears incomplete, and 44 citations in Runs 3–5 remain unevaluated, so the comparison results are provisional.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Finalise the Nested Knowledge DE workflow; run the Laser AI comparison and provide preliminary output for the interim snapshot.</t>
+          <t>Finalise the Nested Knowledge data-extraction workflow; obtain conventional workflow timing/results; correct Run 10 and resolve the 44 unevaluated citations; complete the interim comparison.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -37050,17 +37058,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>The review team has been asked to hold AI-assisted abstract screening while workflow guidance and Laser AI updates are addressed. Conventional abstract screening may continue.</t>
+          <t>AI-assisted abstract screening remains paused as of 2026-07-21 while Laser AI workflow guidance and platform updates are reviewed. Conventional abstract screening may continue.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Confirm the restart decision on 2026-07-20; resume AI-assisted screening only after guidance is agreed and continue documenting preparation effort.</t>
+          <t>Obtain the core-team restart decision and revised Laser AI guidance before resuming AI-assisted screening; continue recording preparation and screening time separately.</t>
         </is>
       </c>
       <c r="K6" s="22" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -37169,7 +37177,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Setup blocked - missing files</t>
+          <t>Setup in progress - search access issue</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -37189,12 +37197,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>RIS/search files are uploaded, but the protocol, eligibility criteria and selected data-extraction items are still missing. Screening has not been approved to start.</t>
+          <t>The protocol and 35 selected data-extraction items have been received, and the live extraction document has been updated. Search/RIS files are available, but LILACS and IBECS remain inaccessible; screening has not yet been approved to start.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Obtain the protocol, inclusion/exclusion criteria and approximately 35 data items; then allow 2-3 working days for Laser AI setup and confirm the screening start.</t>
+          <t>Resolve or document the inaccessible LILACS/IBECS searches, review the “Vit C” search-term concern, finalise Laser AI setup, and confirm when screening may start.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -37442,7 +37450,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40908,7 +40916,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41444,7 +41452,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41778,7 +41786,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -46210,7 +46218,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -46544,7 +46552,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -50852,7 +50860,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -50999,7 +51007,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data extraction ready</t>
+          <t>Data extraction underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -51067,7 +51075,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Laser AI data-extraction template is uploaded and ready. The AI-assisted team will extract only studies included by the conventional team; if more than 10 are included, a random sample of 10 will be used.</t>
+          <t>Data extraction is underway in both workflows. The team expects to complete extraction during the week of 2026-08-03. The AI-assisted team is using the conventional included-study set, capped at 10 studies if needed.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -51084,7 +51092,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Laser AI data-extraction template is uploaded and ready. The AI-assisted team will extract only studies included by the conventional team; if more than 10 are included, a random sample of 10 will be used.</t>
+          <t>Data extraction is underway in both workflows. The team expects to complete extraction during the week of 2026-08-03. The AI-assisted team is using the conventional included-study set, capped at 10 studies if needed.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -51101,7 +51109,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Begin data extraction using the conventional included-study set; randomly select 10 studies if the conventional set exceeds 10.</t>
+          <t>Complete conventional and Laser AI data extraction, notify the project team when both workflows are finished, and submit the extraction outputs and time logs.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -51118,7 +51126,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Week of 2026-08-03</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -51135,7 +51143,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Full-text screening complete; data extraction depends on improved Laser AI DE form</t>
+          <t>Data extraction has started; completion is expected during the week of 2026-08-03.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -51191,7 +51199,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -51324,7 +51332,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DE setup pending improved Laser AI form</t>
+          <t>Active - expected week of 2026-08-03</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -51472,12 +51480,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Improved Laser AI DE form pending</t>
+          <t>Template ready; extraction underway</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -56237,7 +56245,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -56384,7 +56392,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DE setup / Laser AI comparison</t>
+          <t>DE preparation / validation analysis</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56452,7 +56460,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nested Knowledge screening is complete and the DE workflow is being finalised. A separate Laser AI abstract-screening comparison is set up with 2,225 citations and is ready to begin.</t>
+          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete. Ten studies have been selected for data extraction. Ten repeated Laser AI abstract-screening outputs were received; Run 10 appears incomplete, and 44 citations in Runs 3–5 remain unevaluated, so the comparison results are provisional.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56469,7 +56477,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nested Knowledge screening is complete and the DE workflow is being finalised. A separate Laser AI abstract-screening comparison is set up with 2,225 citations and is ready to begin.</t>
+          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete. Ten studies have been selected for data extraction. Ten repeated Laser AI abstract-screening outputs were received; Run 10 appears incomplete, and 44 citations in Runs 3–5 remain unevaluated, so the comparison results are provisional.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56486,7 +56494,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Finalise the Nested Knowledge DE workflow; run the Laser AI comparison and provide preliminary output for the interim snapshot.</t>
+          <t>Finalise the Nested Knowledge data-extraction workflow; obtain conventional workflow timing/results; correct Run 10 and resolve the 44 unevaluated citations; complete the interim comparison.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56503,7 +56511,7 @@
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56520,7 +56528,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Main workflow remains in abstract screening; data extraction is only in preparation/sample planning stage</t>
+          <t>Conventional workflow timing is pending, and the repeated Laser AI outputs require validation before final reporting.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56574,9 +56582,9 @@
           <t>LastUpdated</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56675,7 +56683,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Complete - NK semi-automated</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -56690,6 +56698,11 @@
           <t>fullText</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Complete - AI-assisted</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -56702,6 +56715,11 @@
           <t>extraction</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10 studies selected / setup in progress</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -56712,6 +56730,11 @@
       <c r="A29" t="inlineStr">
         <is>
           <t>analysis</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Preliminary Laser AI comparison underway</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -56803,12 +56826,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>10 extraction-study PDFs received</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -56847,12 +56870,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>10 studies selected; NK extraction workflow being finalised</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">

</xml_diff>

<commit_message>
Refresh phase 1 dashboard statuses
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2286,7 +2286,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2401,7 +2400,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AI screening on hold</t>
+          <t>Abstract Screening</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2469,7 +2468,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AI-assisted abstract screening remains paused as of 2026-07-21 while Laser AI workflow guidance and platform updates are reviewed. Conventional abstract screening may continue.</t>
+          <t>Laser AI abstract screening is complete. Fifteen studies have advanced to full-text screening. The conventional team is consolidating its abstract-screening results.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2486,7 +2485,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AI-assisted abstract screening remains paused as of 2026-07-21 while Laser AI workflow guidance and platform updates are reviewed. Conventional abstract screening may continue.</t>
+          <t>Laser AI abstract screening is complete. Fifteen studies have advanced to full-text screening. The conventional team is consolidating its abstract-screening results.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2503,7 +2502,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Obtain the core-team restart decision and revised Laser AI guidance before resuming AI-assisted screening; continue recording preparation and screening time separately.</t>
+          <t>Complete the usability survey, await conventional-team consolidation, retrieve the PDFs for the 15 studies, and proceed with full-text screening setup.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2537,7 +2536,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AI-assisted screening remains paused; the team reported more than 30 hours of preparation before active testing, approximate and not formally tracked.</t>
+          <t>The agreed decision-flow changes were initially not saved in Laser AI. Version 2 was subsequently applied, but earlier screened records may not include the comparator assessment; document this during the comparison.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2593,7 +2592,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2692,7 +2691,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Paused - conventional may continue</t>
+          <t>AI complete; conventional consolidation pending</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2705,6 +2704,11 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>fullText</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>15 studies identified; PDF retrieval and full-text setup pending</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2820,12 +2824,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>15 full-text records identified; PDFs to be retrieved and uploaded</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2842,12 +2846,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Revised title/abstract decision flow saved as Version 2; full-text decision flow prepared</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2994,7 +2998,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3017,7 +3021,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>AI complete; conventional consolidation pending</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3040,7 +3044,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Setup pending for 15 studies</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3987,7 +3991,7 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
@@ -4040,16 +4044,12 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
       <c r="K65" s="18" t="n"/>
-      <c r="L65" s="18" t="inlineStr">
-        <is>
-          <t>Screening commenced on 2026-07-08.</t>
-        </is>
-      </c>
+      <c r="L65" s="18" t="n"/>
       <c r="M65" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4097,16 +4097,12 @@
       </c>
       <c r="I66" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
       <c r="K66" s="18" t="n"/>
-      <c r="L66" s="18" t="inlineStr">
-        <is>
-          <t>AI-assisted screening commenced / active testing underway.</t>
-        </is>
-      </c>
+      <c r="L66" s="18" t="n"/>
       <c r="M66" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -7810,7 +7806,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -8112,7 +8107,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -12828,7 +12823,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -12943,7 +12937,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup in progress - search access issue</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -13011,7 +13005,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The protocol and 35 selected data-extraction items have been received, and the live extraction document has been updated. Search/RIS files are available, but LILACS and IBECS remain inaccessible; screening has not yet been approved to start.</t>
+          <t>Setup phase underway; Laser AI allocated; search/LILACS clarification and remaining setup materials are being finalized; abstract screening has not yet commenced</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13028,7 +13022,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The protocol and 35 selected data-extraction items have been received, and the live extraction document has been updated. Search/RIS files are available, but LILACS and IBECS remain inaccessible; screening has not yet been approved to start.</t>
+          <t>Vitamin C is in the setup phase with Laser AI allocated. Search/LILACS clarification and remaining setup materials are being finalized; abstract screening has not yet commenced.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13045,7 +13039,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Resolve or document the inaccessible LILACS/IBECS searches, review the “Vit C” search-term concern, finalise Laser AI setup, and confirm when screening may start.</t>
+          <t>Complete setup materials and Laser AI configuration before commencing abstract screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13079,7 +13073,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Most setup materials are now available; database-access and search-strategy issues remain before screening can start.</t>
+          <t>Screening start depends on completion of setup materials and Laser AI configuration</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -13135,7 +13129,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13217,7 +13211,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Protocol/data items received; search access issue pending</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -13340,12 +13334,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Search/RIS files received; some database searches unavailable</t>
+          <t>LILACS/search support ongoing</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -13384,12 +13378,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Eligibility criteria provided in protocol</t>
+          <t>Awaiting final materials</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -13406,12 +13400,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>35 selected data items received; live document updated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -13428,12 +13422,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Protocol received</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -14057,11 +14051,7 @@
       </c>
       <c r="J55" s="18" t="n"/>
       <c r="K55" s="18" t="n"/>
-      <c r="L55" s="18" t="inlineStr">
-        <is>
-          <t>Laser AI activation/reset email resent; login confirmation pending.</t>
-        </is>
-      </c>
+      <c r="L55" s="18" t="n"/>
       <c r="M55" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14215,16 +14205,12 @@
       </c>
       <c r="I58" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J58" s="18" t="n"/>
       <c r="K58" s="18" t="n"/>
-      <c r="L58" s="18" t="inlineStr">
-        <is>
-          <t>RIS/search results received and uploaded to SharePoint.</t>
-        </is>
-      </c>
+      <c r="L58" s="18" t="n"/>
       <c r="M58" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14277,11 +14263,7 @@
       </c>
       <c r="J59" s="18" t="n"/>
       <c r="K59" s="18" t="n"/>
-      <c r="L59" s="18" t="inlineStr">
-        <is>
-          <t>Protocol/criteria not found in SharePoint/email.</t>
-        </is>
-      </c>
+      <c r="L59" s="18" t="n"/>
       <c r="M59" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14334,11 +14316,7 @@
       </c>
       <c r="J60" s="18" t="n"/>
       <c r="K60" s="18" t="n"/>
-      <c r="L60" s="18" t="inlineStr">
-        <is>
-          <t>Data items not found in SharePoint/email.</t>
-        </is>
-      </c>
+      <c r="L60" s="18" t="n"/>
       <c r="M60" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14492,16 +14470,12 @@
       </c>
       <c r="I63" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
-      <c r="L63" s="18" t="inlineStr">
-        <is>
-          <t>Tool setup cannot complete until remaining setup files are located/provided.</t>
-        </is>
-      </c>
+      <c r="L63" s="18" t="n"/>
       <c r="M63" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -17619,7 +17593,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -17926,7 +17899,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -22108,7 +22081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="22" customWidth="1" style="29" min="1" max="1"/>
@@ -22257,7 +22230,7 @@
       </c>
       <c r="D12" s="17" t="inlineStr">
         <is>
-          <t>Onboarding and Nested Knowledge training completed; study materials and setup inputs pending</t>
+          <t>Participation confirmed; team roles agreed; onboarding and study material collection underway; tool training pending</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22272,12 +22245,12 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>Training complete; study material collection underway</t>
+          <t>Onboarding and study material collection underway</t>
         </is>
       </c>
       <c r="H12" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-07 Human Milk; Nested Knowledge allocated; training complete; awaiting study files and setup inputs</t>
+          <t>Converted to phase1-07 Human Milk; Nested Knowledge allocated; tool training pending</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -22299,27 +22272,27 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>Medication-Taking Ability and Adherence (Amanda Cross)</t>
+          <t>Amanda Cross ? Interventions for improving medication-taking ability and adherence in older adults prescribed multiple medications</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>Withdrawn &amp; Reason</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Team has withdrawn from the platform study due to capacity constraints</t>
         </is>
       </c>
       <c r="E13" s="17" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>Amanda Cross</t>
+          <t>Amanda Cross / Rehan Sarwar</t>
         </is>
       </c>
       <c r="G13" s="17" t="inlineStr">
@@ -22329,7 +22302,7 @@
       </c>
       <c r="H13" s="17" t="inlineStr">
         <is>
-          <t>Team has withdrawn from the platform study due to capacity constraints.</t>
+          <t>Withdrawn due to capacity constraints; retain as historical record</t>
         </is>
       </c>
       <c r="I13" s="17" t="inlineStr">
@@ -22401,7 +22374,7 @@
       </c>
       <c r="D15" s="17" t="inlineStr">
         <is>
-          <t>Protocol and 35 data items received; search files uploaded; LILACS/IBECS access issue remains</t>
+          <t>Tracked as phase1-05</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
@@ -22416,12 +22389,12 @@
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>Setup in progress; database-access issue unresolved</t>
+          <t>Search update in progress</t>
         </is>
       </c>
       <c r="H15" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-05 Vitamin C; protocol and data items received; screening awaits resolution or documentation of inaccessible databases</t>
+          <t>Final updated search/RIS and remaining study materials pending; Sean supporting LILACS/search issue</t>
         </is>
       </c>
       <c r="I15" s="17" t="inlineStr">
@@ -22858,56 +22831,15 @@
       </c>
     </row>
     <row r="30" ht="24" customHeight="1" s="29">
-      <c r="A30" s="17" t="inlineStr">
-        <is>
-          <t>new-19</t>
-        </is>
-      </c>
-      <c r="B30" s="17" t="inlineStr">
-        <is>
-          <t>Siew Cheng Foong — Oral galactagogues</t>
-        </is>
-      </c>
-      <c r="C30" s="17" t="inlineStr">
-        <is>
-          <t>Under Shortlisting</t>
-        </is>
-      </c>
-      <c r="D30" s="17" t="inlineStr">
-        <is>
-          <t>Potential later-phase candidate; rerun search expected in 10–14 days; prior update work substantially completed; written consent received</t>
-        </is>
-      </c>
-      <c r="E30" s="17" t="inlineStr">
-        <is>
-          <t>Later phase / Phase 2</t>
-        </is>
-      </c>
-      <c r="F30" s="17" t="inlineStr">
-        <is>
-          <t>Siew Cheng Foong; Cochrane Malaysia / Jacqueline J Ho</t>
-        </is>
-      </c>
-      <c r="G30" s="17" t="inlineStr">
-        <is>
-          <t>Rerun search expected July 2026; screening/additional DE August–September 2026; submission October 2026</t>
-        </is>
-      </c>
-      <c r="H30" s="17" t="inlineStr">
-        <is>
-          <t>Initial search completed; 26 new eligible studies; DE and ROB 1 completed; INSPECT-SR and ROB 2 underway; students available in August</t>
-        </is>
-      </c>
-      <c r="I30" s="17" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A30" s="17" t="n"/>
+      <c r="B30" s="17" t="n"/>
+      <c r="C30" s="17" t="n"/>
+      <c r="D30" s="17" t="n"/>
+      <c r="E30" s="17" t="n"/>
+      <c r="F30" s="17" t="n"/>
+      <c r="G30" s="17" t="n"/>
+      <c r="H30" s="17" t="n"/>
+      <c r="I30" s="17" t="n"/>
     </row>
     <row r="31" ht="24" customHeight="1" s="29">
       <c r="A31" s="17" t="n"/>
@@ -23192,100 +23124,6 @@
       <c r="B58" s="18" t="inlineStr">
         <is>
           <t>Not suitable for the current validation phase. Keep brief reason in Remarks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>withdrawn-med-adherence</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Medication-Taking Ability and Adherence (Amanda Cross)</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Withdrawn &amp; Reason</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Amanda Cross</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Duplicate hidden; use new-02 withdrawn row.</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>withdrawn-abdominal-irrigation</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Abdominal Irrigation at Caesarean Section (Anna Rogers)</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Withdrawn &amp; Reason</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>Anna Rogers</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Team has withdrawn from the platform study and will not be participating.</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -27077,11 +26915,7 @@
           <t>mtg-06</t>
         </is>
       </c>
-      <c r="B6" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
+      <c r="B6" s="25" t="n"/>
       <c r="C6" s="25" t="n"/>
       <c r="D6" s="25" t="n"/>
       <c r="E6" s="25" t="inlineStr">
@@ -27091,7 +26925,7 @@
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>Nested Knowledge training completed for Human Milk Fortifier.</t>
+          <t>Nested Knowledge training for Human Milk Fortifier; time TBD.</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
@@ -27111,7 +26945,7 @@
       </c>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="K6" s="25" t="inlineStr">
@@ -27132,21 +26966,9 @@
           <t>mtg-07</t>
         </is>
       </c>
-      <c r="B7" s="25" t="inlineStr">
-        <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-      <c r="C7" s="25" t="inlineStr">
-        <is>
-          <t>9:00-10:00 AM EDT</t>
-        </is>
-      </c>
-      <c r="D7" s="25" t="inlineStr">
-        <is>
-          <t>2:00-3:00 PM BST</t>
-        </is>
-      </c>
+      <c r="B7" s="25" t="n"/>
+      <c r="C7" s="25" t="n"/>
+      <c r="D7" s="25" t="n"/>
       <c r="E7" s="25" t="inlineStr">
         <is>
           <t>Human Milk Fortifier Onboarding</t>
@@ -27154,12 +26976,12 @@
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>Onboarding meeting for Human Milk Fortifier; invite accepted by review team members.</t>
+          <t>Onboarding meeting for Human Milk Fortifier; time TBD.</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>Mohan Pammi / Murali Premkumar / Gautham KS / Michelle Fiander / Krishna / Core Team</t>
+          <t>Mohan Pammi / Krishna / Core Team</t>
         </is>
       </c>
       <c r="H7" s="25" t="inlineStr">
@@ -27174,7 +26996,7 @@
       </c>
       <c r="J7" s="25" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="K7" s="25" t="inlineStr">
@@ -27299,7 +27121,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -27414,7 +27235,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ready / calibration before screening</t>
+          <t>Onboarded / awaiting template revisions</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -27482,7 +27303,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nested Knowledge is ready with 1,077 citations. Screening had not started as of 2026-07-15; the team is completing a 100-record calibration and has agreed screening milestones.</t>
+          <t>Onboarding and tool training completed; RIS file, protocol, eligibility criteria, and draft data extraction template received</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27499,7 +27320,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nested Knowledge is ready with 1,077 citations. Screening had not started as of 2026-07-15; the team is completing a 100-record calibration and has agreed screening milestones.</t>
+          <t>RIS file, protocol, eligibility criteria, and draft data extraction template received; awaiting final template revisions before project configuration and screening begin</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27516,7 +27337,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete calibration, start conventional and AI-assisted abstract screening, and finish title/abstract screening by 2026-07-28.</t>
+          <t>Await final template revisions before project configuration and screening begin</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27533,7 +27354,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -27550,7 +27371,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bradley NK user recognition/access still needs confirmation, but project is ready for screening</t>
+          <t>Project configuration and screening depend on final data extraction template revisions</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -27606,7 +27427,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27688,7 +27509,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Awaiting final template revisions</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -27705,7 +27526,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ready to start</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -28514,11 +28335,7 @@
       </c>
       <c r="J55" s="18" t="n"/>
       <c r="K55" s="18" t="n"/>
-      <c r="L55" s="18" t="inlineStr">
-        <is>
-          <t>Bradley NK user recognition still needs confirmation.</t>
-        </is>
-      </c>
+      <c r="L55" s="18" t="n"/>
       <c r="M55" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -28937,16 +28754,12 @@
       </c>
       <c r="I63" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
-      <c r="L63" s="18" t="inlineStr">
-        <is>
-          <t>1,077 citations uploaded; 11 duplicates removed.</t>
-        </is>
-      </c>
+      <c r="L63" s="18" t="n"/>
       <c r="M63" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -28994,16 +28807,12 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
       <c r="K64" s="18" t="n"/>
-      <c r="L64" s="18" t="inlineStr">
-        <is>
-          <t>Screening forms reviewed; minor edits made; screening planned for 2026-07-13.</t>
-        </is>
-      </c>
+      <c r="L64" s="18" t="n"/>
       <c r="M64" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -31905,7 +31714,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -32020,7 +31828,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Onboarding and training complete</t>
+          <t>Onboarding / materials collection</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32088,7 +31896,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Onboarding and Nested Knowledge training were completed on 2026-07-14. Project setup is waiting for RIS/search results, eligibility criteria, the protocol and approximately 35 data-extraction items.</t>
+          <t>Participation confirmed; team roles agreed; onboarding and study material collection underway; tool training pending</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32105,7 +31913,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Onboarding and Nested Knowledge training were completed on 2026-07-14. Project setup is waiting for RIS/search results, eligibility criteria, the protocol and approximately 35 data-extraction items.</t>
+          <t>Participation confirmed; team roles agreed; study material collection and onboarding are underway</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32122,7 +31930,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Collect the missing study files; finalise a comparable 35-item data-extraction list with Sean; then configure the Nested Knowledge project.</t>
+          <t>Collect study materials, complete Nested Knowledge tool training, and configure project for screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32156,7 +31964,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Training is complete; project configuration is pending the RIS/search files, eligibility criteria, protocol and selected data-extraction items.</t>
+          <t>Tool training and project configuration pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32212,7 +32020,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32277,7 +32085,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Underway</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -36580,7 +36388,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>v4 adds full old Workflow_Master columns, including DependsOn and Blocks.</t>
+          <t>Updated 2026-07-30: Corrected review status labels: Psoriasis and Fruit &amp; Vegetable in Abstract Screening; Vitamin C in Setup phase.</t>
         </is>
       </c>
     </row>
@@ -36894,7 +36702,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Data extraction underway</t>
+          <t>Full-text screening</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -36914,17 +36722,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Data extraction is underway in both workflows. The team expects to complete extraction during the week of 2026-08-03. The AI-assisted team is using the conventional included-study set, capped at 10 studies if needed.</t>
+          <t>Full-text screening nearing completion; data extraction setup underway</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Complete conventional and Laser AI data extraction, notify the project team when both workflows are finished, and submit the extraction outputs and time logs.</t>
+          <t>Complete full-text screening by 2026-07-08 and continue data extraction setup</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>Week of 2026-08-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -36966,7 +36774,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>DE preparation / validation analysis</t>
+          <t>Abstract Screening</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -36986,17 +36794,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete. Ten studies have been selected for data extraction. Ten repeated Laser AI abstract-screening outputs were received; Run 10 appears incomplete, and 44 citations in Runs 3–5 remain unevaluated, so the comparison results are provisional.</t>
+          <t>Conventional title/abstract screening nearing completion; AI-assisted full-text selection almost complete; data extraction preparation/sample planning underway</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Finalise the Nested Knowledge data-extraction workflow; obtain conventional workflow timing/results; correct Run 10 and resolve the 44 unevaluated citations; complete the interim comparison.</t>
+          <t>Complete conventional title/abstract screening; prepare common sample of up to 10 studies for later data extraction</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -37038,7 +36846,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AI screening on hold</t>
+          <t>Abstract Screening</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -37058,12 +36866,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>AI-assisted abstract screening remains paused as of 2026-07-21 while Laser AI workflow guidance and platform updates are reviewed. Conventional abstract screening may continue.</t>
+          <t>Laser AI abstract screening is complete. Fifteen studies have advanced to full-text screening. The conventional team is consolidating its abstract-screening results.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Obtain the core-team restart decision and revised Laser AI guidance before resuming AI-assisted screening; continue recording preparation and screening time separately.</t>
+          <t>Complete the usability survey, await conventional-team consolidation, retrieve the PDFs for the 15 studies, and proceed with full-text screening setup.</t>
         </is>
       </c>
       <c r="K6" s="22" t="inlineStr">
@@ -37177,7 +36985,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Setup in progress - search access issue</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -37197,12 +37005,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>The protocol and 35 selected data-extraction items have been received, and the live extraction document has been updated. Search/RIS files are available, but LILACS and IBECS remain inaccessible; screening has not yet been approved to start.</t>
+          <t>Setup phase underway; Laser AI allocated; search/LILACS clarification and remaining setup materials are being finalized; abstract screening has not yet commenced</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Resolve or document the inaccessible LILACS/IBECS searches, review the “Vit C” search-term concern, finalise Laser AI setup, and confirm when screening may start.</t>
+          <t>Complete setup materials and Laser AI configuration before commencing abstract screening</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -37321,7 +37129,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Ready / calibration before screening</t>
+          <t>Onboarded / awaiting template revisions</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -37341,17 +37149,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Nested Knowledge is ready with 1,077 citations. Screening had not started as of 2026-07-15; the team is completing a 100-record calibration and has agreed screening milestones.</t>
+          <t>Onboarding and tool training completed; RIS file, protocol, eligibility criteria, and draft data extraction template received</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Complete calibration, start conventional and AI-assisted abstract screening, and finish title/abstract screening by 2026-07-28.</t>
+          <t>Await final template revisions before project configuration and screening begin</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -37393,7 +37201,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Onboarding and training complete</t>
+          <t>Onboarding / materials collection</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -37413,12 +37221,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Onboarding and Nested Knowledge training were completed on 2026-07-14. Project setup is waiting for RIS/search results, eligibility criteria, the protocol and approximately 35 data-extraction items.</t>
+          <t>Participation confirmed; team roles agreed; onboarding and study material collection underway; tool training pending</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Collect the missing study files; finalise a comparable 35-item data-extraction list with Sean; then configure the Nested Knowledge project.</t>
+          <t>Collect study materials, complete Nested Knowledge tool training, and configure project for screening</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -41020,7 +40828,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mid April onward</t>
+          <t>Mid April to End June</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -41047,12 +40855,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>July 2026</t>
+          <t>End June</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Decision Gate</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -41074,12 +40882,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Start July to End September</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Pending decision</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -41101,12 +40909,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>October</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Interim snapshot ready</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -41365,77 +41173,167 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>mtg-05</t>
+          <t>meet-001</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>15 May 2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Fruit &amp; Veg Re-onboarding</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Rebecca K. Hodder / Krishna / Core Team</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Re-onboarding meeting for Fruit &amp; Veg; time TBD.</t>
+          <t>Usability survey tracking discussion</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Completed / No longer required</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Time TBD</t>
+          <t>AI abstract screening completed; conventional consolidation and full-text setup are the next steps.</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>meet-002</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>18 May 2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Core team discussion with Meghan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>meet-003</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>19 May 2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BP Targets review team check-in</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>meet-004</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>19 May 2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Psoriasis review team check-in</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>meet-005</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>19 May 2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Adjudication pilot deadline</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>meet-006</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>21 May 2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PM + PI meeting</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -41484,7 +41382,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -41786,7 +41683,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -46250,7 +46147,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -46552,7 +46448,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -50892,7 +50788,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -51007,7 +50902,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data extraction underway</t>
+          <t>Full-text screening</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -51075,7 +50970,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Data extraction is underway in both workflows. The team expects to complete extraction during the week of 2026-08-03. The AI-assisted team is using the conventional included-study set, capped at 10 studies if needed.</t>
+          <t>Full-text screening nearing completion; data extraction setup underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -51092,7 +50987,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Data extraction is underway in both workflows. The team expects to complete extraction during the week of 2026-08-03. The AI-assisted team is using the conventional included-study set, capped at 10 studies if needed.</t>
+          <t>Full-text screening nearing completion; expected completion 2026-07-08; data extraction setup underway</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -51109,7 +51004,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete conventional and Laser AI data extraction, notify the project team when both workflows are finished, and submit the extraction outputs and time logs.</t>
+          <t>Complete full-text screening by 2026-07-08 and continue data extraction setup</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -51126,7 +51021,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Week of 2026-08-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -51143,7 +51038,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Data extraction has started; completion is expected during the week of 2026-08-03.</t>
+          <t>On track for full-text completion; data extraction setup next dependency</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -51199,7 +51094,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -51315,7 +51210,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -51332,7 +51227,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Active - expected week of 2026-08-03</t>
+          <t>Setup underway</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -51485,7 +51380,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Template ready; extraction underway</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -52656,7 +52551,7 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
@@ -53133,7 +53028,7 @@
       </c>
       <c r="I74" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
@@ -53345,7 +53240,7 @@
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
@@ -53398,7 +53293,7 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
@@ -53451,7 +53346,7 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
@@ -53504,7 +53399,7 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
@@ -53663,7 +53558,7 @@
       </c>
       <c r="I84" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J84" s="18" t="n"/>
@@ -53928,7 +53823,7 @@
       </c>
       <c r="I89" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J89" s="18" t="n"/>
@@ -54140,7 +54035,7 @@
       </c>
       <c r="I93" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J93" s="18" t="n"/>
@@ -56277,7 +56172,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -56392,7 +56286,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DE preparation / validation analysis</t>
+          <t>Abstract Screening</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56460,7 +56354,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete. Ten studies have been selected for data extraction. Ten repeated Laser AI abstract-screening outputs were received; Run 10 appears incomplete, and 44 citations in Runs 3–5 remain unevaluated, so the comparison results are provisional.</t>
+          <t>Conventional title/abstract screening nearing completion; AI-assisted full-text selection almost complete; data extraction preparation/sample planning underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56477,7 +56371,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete. Ten studies have been selected for data extraction. Ten repeated Laser AI abstract-screening outputs were received; Run 10 appears incomplete, and 44 citations in Runs 3–5 remain unevaluated, so the comparison results are provisional.</t>
+          <t>Conventional title/abstract screening is nearing completion; AI-assisted full-text selection is almost complete. The team is preparing a common sample of up to 10 studies for later data extraction.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56494,7 +56388,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Finalise the Nested Knowledge data-extraction workflow; obtain conventional workflow timing/results; correct Run 10 and resolve the 44 unevaluated citations; complete the interim comparison.</t>
+          <t>Complete conventional title/abstract screening; prepare common sample of up to 10 studies for later data extraction</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56511,7 +56405,7 @@
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56528,7 +56422,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Conventional workflow timing is pending, and the repeated Laser AI outputs require validation before final reporting.</t>
+          <t>Main workflow remains in abstract screening; data extraction is only in preparation/sample planning stage</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56584,7 +56478,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56683,7 +56577,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Complete - NK semi-automated</t>
+          <t>Active / nearing completion</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -56700,7 +56594,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Complete - AI-assisted</t>
+          <t>AI-assisted full-text selection almost complete</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -56717,7 +56611,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10 studies selected / setup in progress</t>
+          <t>Preparation only</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -56730,11 +56624,6 @@
       <c r="A29" t="inlineStr">
         <is>
           <t>analysis</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Preliminary Laser AI comparison underway</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -56826,12 +56715,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>10 extraction-study PDFs received</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -56870,12 +56759,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>10 studies selected; NK extraction workflow being finalised</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">

</xml_diff>

<commit_message>
Correct review phase status cards
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2400,7 +2400,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract Screening</t>
+          <t>Abstract Screening Complete</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Laser AI abstract screening is complete. Fifteen studies have advanced to full-text screening. The conventional team is consolidating its abstract-screening results.</t>
+          <t>Abstract screening completed; fifteen studies identified for full-text screening setup</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Laser AI abstract screening is complete. Fifteen studies have advanced to full-text screening. The conventional team is consolidating its abstract-screening results.</t>
+          <t>Abstract screening completed; fifteen studies identified for full-text screening setup</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete the usability survey, await conventional-team consolidation, retrieve the PDFs for the 15 studies, and proceed with full-text screening setup.</t>
+          <t>Complete usability survey, retrieve PDFs for the 15 studies, and prepare full-text screening setup.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AI complete; conventional consolidation pending</t>
+          <t>Abstract screening complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>AI complete; conventional consolidation pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Setup phase underway; Laser AI allocated; search/LILACS clarification and remaining setup materials are being finalized; abstract screening has not yet commenced</t>
+          <t>Setup phase underway; configuration and source materials are being finalized before screening starts</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13022,7 +13022,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Vitamin C is in the setup phase with Laser AI allocated. Search/LILACS clarification and remaining setup materials are being finalized; abstract screening has not yet commenced.</t>
+          <t>Setup phase underway; configuration and source materials are being finalized before screening starts</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13039,7 +13039,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete setup materials and Laser AI configuration before commencing abstract screening</t>
+          <t>Complete setup materials and Laser AI configuration before commencing abstract screening.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13129,7 +13129,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13228,7 +13228,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -13241,6 +13241,11 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>fullText</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Screening not yet started</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -13530,7 +13535,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -27235,7 +27240,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Onboarded / awaiting template revisions</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -27303,7 +27308,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Onboarding and tool training completed; RIS file, protocol, eligibility criteria, and draft data extraction template received</t>
+          <t>Setup phase underway; template revisions and project configuration remain before screening begins</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27320,7 +27325,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RIS file, protocol, eligibility criteria, and draft data extraction template received; awaiting final template revisions before project configuration and screening begin</t>
+          <t>Setup phase underway; template revisions and project configuration remain before screening begins</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27337,7 +27342,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Await final template revisions before project configuration and screening begin</t>
+          <t>Finalize template revisions, complete project configuration, and then begin screening.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27427,7 +27432,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27526,7 +27531,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -27543,7 +27548,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Template revisions/configuration pending</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -27832,7 +27837,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -31828,7 +31833,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Onboarding / materials collection</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -31896,7 +31901,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Participation confirmed; team roles agreed; onboarding and study material collection underway; tool training pending</t>
+          <t>Setup phase underway; study materials, training, and configuration are still being completed</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -31913,7 +31918,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Participation confirmed; team roles agreed; study material collection and onboarding are underway</t>
+          <t>Setup phase underway; study materials, training, and configuration are still being completed</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -31930,7 +31935,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Collect study materials, complete Nested Knowledge tool training, and configure project for screening</t>
+          <t>Collect study materials, complete Nested Knowledge tool training, and configure the project for screening.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32020,7 +32025,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32119,7 +32124,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -32136,7 +32141,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Materials/training/configuration pending</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -32425,7 +32430,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -36388,7 +36393,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Updated 2026-07-30: Corrected review status labels: Psoriasis and Fruit &amp; Vegetable in Abstract Screening; Vitamin C in Setup phase.</t>
+          <t>2026-07-30 phase status recheck: BP Targets moved to Data Extraction / Analysis; Psoriasis moved to Full-text Screening; Fruit &amp; Veg marked Abstract Screening Complete; Probiotics AAD and Human Milk set to Setup phase.</t>
         </is>
       </c>
     </row>
@@ -36702,7 +36707,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Full-text screening</t>
+          <t>Data Extraction / Analysis</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -36722,12 +36727,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Full-text screening nearing completion; data extraction setup underway</t>
+          <t>Data extraction phase; full-text screening outputs are feeding extraction and analysis setup</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Complete full-text screening by 2026-07-08 and continue data extraction setup</t>
+          <t>Continue data extraction and analysis preparation; reconcile full-text decisions and submit extraction outputs/time logs.</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
@@ -36774,7 +36779,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Abstract Screening</t>
+          <t>Full-text Screening</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -36794,12 +36799,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Conventional title/abstract screening nearing completion; AI-assisted full-text selection almost complete; data extraction preparation/sample planning underway</t>
+          <t>Full-text screening phase; abstract screening has moved forward into full-text review preparation</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Complete conventional title/abstract screening; prepare common sample of up to 10 studies for later data extraction</t>
+          <t>Complete full-text screening and prepare the agreed common sample for later data extraction.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -36846,7 +36851,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Abstract Screening</t>
+          <t>Abstract Screening Complete</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -36866,12 +36871,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Laser AI abstract screening is complete. Fifteen studies have advanced to full-text screening. The conventional team is consolidating its abstract-screening results.</t>
+          <t>Abstract screening completed; fifteen studies identified for full-text screening setup</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Complete the usability survey, await conventional-team consolidation, retrieve the PDFs for the 15 studies, and proceed with full-text screening setup.</t>
+          <t>Complete usability survey, retrieve PDFs for the 15 studies, and prepare full-text screening setup.</t>
         </is>
       </c>
       <c r="K6" s="22" t="inlineStr">
@@ -37005,12 +37010,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Setup phase underway; Laser AI allocated; search/LILACS clarification and remaining setup materials are being finalized; abstract screening has not yet commenced</t>
+          <t>Setup phase underway; configuration and source materials are being finalized before screening starts</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Complete setup materials and Laser AI configuration before commencing abstract screening</t>
+          <t>Complete setup materials and Laser AI configuration before commencing abstract screening.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -37129,7 +37134,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Onboarded / awaiting template revisions</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -37149,12 +37154,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Onboarding and tool training completed; RIS file, protocol, eligibility criteria, and draft data extraction template received</t>
+          <t>Setup phase underway; template revisions and project configuration remain before screening begins</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Await final template revisions before project configuration and screening begin</t>
+          <t>Finalize template revisions, complete project configuration, and then begin screening.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -37201,7 +37206,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Onboarding / materials collection</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -37221,12 +37226,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Participation confirmed; team roles agreed; onboarding and study material collection underway; tool training pending</t>
+          <t>Setup phase underway; study materials, training, and configuration are still being completed</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Collect study materials, complete Nested Knowledge tool training, and configure project for screening</t>
+          <t>Collect study materials, complete Nested Knowledge tool training, and configure the project for screening.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -50902,7 +50907,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text screening</t>
+          <t>Data Extraction / Analysis</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -50970,7 +50975,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text screening nearing completion; data extraction setup underway</t>
+          <t>Data extraction phase; full-text screening outputs are feeding extraction and analysis setup</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -50987,7 +50992,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Full-text screening nearing completion; expected completion 2026-07-08; data extraction setup underway</t>
+          <t>Data extraction phase; full-text screening outputs are feeding extraction and analysis setup</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -51004,7 +51009,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete full-text screening by 2026-07-08 and continue data extraction setup</t>
+          <t>Continue data extraction and analysis preparation; reconcile full-text decisions and submit extraction outputs/time logs.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -51094,7 +51099,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -51193,7 +51198,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Data extraction phase</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -51210,7 +51215,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Full-text decisions feeding extraction setup</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -51505,7 +51510,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -51528,7 +51533,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -51551,7 +51556,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -51574,7 +51579,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -56286,7 +56291,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract Screening</t>
+          <t>Full-text Screening</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56354,7 +56359,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Conventional title/abstract screening nearing completion; AI-assisted full-text selection almost complete; data extraction preparation/sample planning underway</t>
+          <t>Full-text screening phase; abstract screening has moved forward into full-text review preparation</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56371,7 +56376,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Conventional title/abstract screening is nearing completion; AI-assisted full-text selection is almost complete. The team is preparing a common sample of up to 10 studies for later data extraction.</t>
+          <t>Full-text screening phase; abstract screening has moved forward into full-text review preparation</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56388,7 +56393,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete conventional title/abstract screening; prepare common sample of up to 10 studies for later data extraction</t>
+          <t>Complete full-text screening and prepare the agreed common sample for later data extraction.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56478,7 +56483,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56577,7 +56582,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Active / nearing completion</t>
+          <t>Full-text screening in progress</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -56594,7 +56599,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AI-assisted full-text selection almost complete</t>
+          <t>Abstract screening completed; full-text phase active</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -56889,7 +56894,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -56912,7 +56917,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -56935,7 +56940,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">

</xml_diff>

<commit_message>
Correct live review phase status cards
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2400,7 +2400,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract Screening</t>
+          <t>Abstract Screening Complete</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Laser AI abstract screening is complete. Fifteen studies have advanced to full-text screening. The conventional team is consolidating its abstract-screening results.</t>
+          <t>Abstract screening completed; fifteen studies identified for full-text screening setup</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Laser AI abstract screening is complete. Fifteen studies have advanced to full-text screening. The conventional team is consolidating its abstract-screening results.</t>
+          <t>Abstract screening completed; fifteen studies identified for full-text screening setup</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete the usability survey, await conventional-team consolidation, retrieve the PDFs for the 15 studies, and proceed with full-text screening setup.</t>
+          <t>Complete usability survey, retrieve PDFs for the 15 studies, and prepare full-text screening setup.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AI complete; conventional consolidation pending</t>
+          <t>Abstract screening complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>AI complete; conventional consolidation pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Setup phase underway; Laser AI allocated; search/LILACS clarification and remaining setup materials are being finalized; abstract screening has not yet commenced</t>
+          <t>Setup phase underway; configuration and source materials are being finalized before screening starts</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13022,7 +13022,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Vitamin C is in the setup phase with Laser AI allocated. Search/LILACS clarification and remaining setup materials are being finalized; abstract screening has not yet commenced.</t>
+          <t>Setup phase underway; configuration and source materials are being finalized before screening starts</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13039,7 +13039,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete setup materials and Laser AI configuration before commencing abstract screening</t>
+          <t>Complete setup materials and Laser AI configuration before commencing abstract screening.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13129,7 +13129,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13228,7 +13228,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -13241,6 +13241,11 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>fullText</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Screening not yet started</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -13530,7 +13535,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -27235,7 +27240,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Onboarded / awaiting template revisions</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -27303,7 +27308,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Onboarding and tool training completed; RIS file, protocol, eligibility criteria, and draft data extraction template received</t>
+          <t>Setup phase underway; template revisions and project configuration remain before screening begins</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27320,7 +27325,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RIS file, protocol, eligibility criteria, and draft data extraction template received; awaiting final template revisions before project configuration and screening begin</t>
+          <t>Setup phase underway; template revisions and project configuration remain before screening begins</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27337,7 +27342,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Await final template revisions before project configuration and screening begin</t>
+          <t>Finalize template revisions, complete project configuration, and then begin screening.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27427,7 +27432,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27526,7 +27531,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -27543,7 +27548,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Template revisions/configuration pending</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -27832,7 +27837,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -31828,7 +31833,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Onboarding / materials collection</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -31896,7 +31901,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Participation confirmed; team roles agreed; onboarding and study material collection underway; tool training pending</t>
+          <t>Setup phase underway; study materials, training, and configuration are still being completed</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -31913,7 +31918,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Participation confirmed; team roles agreed; study material collection and onboarding are underway</t>
+          <t>Setup phase underway; study materials, training, and configuration are still being completed</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -31930,7 +31935,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Collect study materials, complete Nested Knowledge tool training, and configure project for screening</t>
+          <t>Collect study materials, complete Nested Knowledge tool training, and configure the project for screening.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32020,7 +32025,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32119,7 +32124,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -32136,7 +32141,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Materials/training/configuration pending</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -32425,7 +32430,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -36388,7 +36393,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Updated 2026-07-30: Corrected review status labels: Psoriasis and Fruit &amp; Vegetable in Abstract Screening; Vitamin C in Setup phase.</t>
+          <t>2026-07-30 phase status recheck: BP Targets moved to Data Extraction / Analysis; Psoriasis moved to Full-text Screening; Fruit &amp; Veg marked Abstract Screening Complete; Probiotics AAD and Human Milk set to Setup phase.</t>
         </is>
       </c>
     </row>
@@ -36702,7 +36707,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Full-text screening</t>
+          <t>Data Extraction / Analysis</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -36722,12 +36727,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Full-text screening nearing completion; data extraction setup underway</t>
+          <t>Data extraction phase; full-text screening outputs are feeding extraction and analysis setup</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Complete full-text screening by 2026-07-08 and continue data extraction setup</t>
+          <t>Continue data extraction and analysis preparation; reconcile full-text decisions and submit extraction outputs/time logs.</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
@@ -36774,7 +36779,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Abstract Screening</t>
+          <t>Full-text Screening</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -36794,12 +36799,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Conventional title/abstract screening nearing completion; AI-assisted full-text selection almost complete; data extraction preparation/sample planning underway</t>
+          <t>Full-text screening phase; abstract screening has moved forward into full-text review preparation</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Complete conventional title/abstract screening; prepare common sample of up to 10 studies for later data extraction</t>
+          <t>Complete full-text screening and prepare the agreed common sample for later data extraction.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -36846,7 +36851,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Abstract Screening</t>
+          <t>Abstract Screening Complete</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -36866,12 +36871,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Laser AI abstract screening is complete. Fifteen studies have advanced to full-text screening. The conventional team is consolidating its abstract-screening results.</t>
+          <t>Abstract screening completed; fifteen studies identified for full-text screening setup</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Complete the usability survey, await conventional-team consolidation, retrieve the PDFs for the 15 studies, and proceed with full-text screening setup.</t>
+          <t>Complete usability survey, retrieve PDFs for the 15 studies, and prepare full-text screening setup.</t>
         </is>
       </c>
       <c r="K6" s="22" t="inlineStr">
@@ -37005,12 +37010,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Setup phase underway; Laser AI allocated; search/LILACS clarification and remaining setup materials are being finalized; abstract screening has not yet commenced</t>
+          <t>Setup phase underway; configuration and source materials are being finalized before screening starts</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Complete setup materials and Laser AI configuration before commencing abstract screening</t>
+          <t>Complete setup materials and Laser AI configuration before commencing abstract screening.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -37129,7 +37134,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Onboarded / awaiting template revisions</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -37149,12 +37154,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Onboarding and tool training completed; RIS file, protocol, eligibility criteria, and draft data extraction template received</t>
+          <t>Setup phase underway; template revisions and project configuration remain before screening begins</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Await final template revisions before project configuration and screening begin</t>
+          <t>Finalize template revisions, complete project configuration, and then begin screening.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -37201,7 +37206,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Onboarding / materials collection</t>
+          <t>Setup phase</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -37221,12 +37226,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Participation confirmed; team roles agreed; onboarding and study material collection underway; tool training pending</t>
+          <t>Setup phase underway; study materials, training, and configuration are still being completed</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Collect study materials, complete Nested Knowledge tool training, and configure project for screening</t>
+          <t>Collect study materials, complete Nested Knowledge tool training, and configure the project for screening.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -50902,7 +50907,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text screening</t>
+          <t>Data Extraction / Analysis</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -50970,7 +50975,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text screening nearing completion; data extraction setup underway</t>
+          <t>Data extraction phase; full-text screening outputs are feeding extraction and analysis setup</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -50987,7 +50992,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Full-text screening nearing completion; expected completion 2026-07-08; data extraction setup underway</t>
+          <t>Data extraction phase; full-text screening outputs are feeding extraction and analysis setup</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -51004,7 +51009,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete full-text screening by 2026-07-08 and continue data extraction setup</t>
+          <t>Continue data extraction and analysis preparation; reconcile full-text decisions and submit extraction outputs/time logs.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -51094,7 +51099,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -51193,7 +51198,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Data extraction phase</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -51210,7 +51215,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Full-text decisions feeding extraction setup</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -51505,7 +51510,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -51528,7 +51533,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -51551,7 +51556,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -51574,7 +51579,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -56286,7 +56291,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract Screening</t>
+          <t>Full-text Screening</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56354,7 +56359,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Conventional title/abstract screening nearing completion; AI-assisted full-text selection almost complete; data extraction preparation/sample planning underway</t>
+          <t>Full-text screening phase; abstract screening has moved forward into full-text review preparation</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56371,7 +56376,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Conventional title/abstract screening is nearing completion; AI-assisted full-text selection is almost complete. The team is preparing a common sample of up to 10 studies for later data extraction.</t>
+          <t>Full-text screening phase; abstract screening has moved forward into full-text review preparation</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56388,7 +56393,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete conventional title/abstract screening; prepare common sample of up to 10 studies for later data extraction</t>
+          <t>Complete full-text screening and prepare the agreed common sample for later data extraction.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56478,7 +56483,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56577,7 +56582,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Active / nearing completion</t>
+          <t>Full-text screening in progress</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -56594,7 +56599,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AI-assisted full-text selection almost complete</t>
+          <t>Abstract screening completed; full-text phase active</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -56889,7 +56894,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -56912,7 +56917,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -56935,7 +56940,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">

</xml_diff>

<commit_message>
Update August dashboard review snapshot
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -1,37 +1,21 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
+  <dc:creator xmlns:dc="http://purl.org/dc/elements/1.1/">Krishna Kishore Pandalaneni</dc:creator>
+  <dcterms:created xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-05-27T01:47:03Z</dcterms:created>
+  <dcterms:modified xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-07-30T14:56:52Z</dcterms:modified>
+  <cp:lastModifiedBy>Krishna Kishore Pandalaneni</cp:lastModifiedBy>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="9">
@@ -324,7 +308,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewIndexTable" displayName="ReviewIndexTable" ref="A1:N11" headerRowCount="1">
   <tableColumns count="14">
     <tableColumn id="1" name="ReviewID"/>
@@ -346,7 +330,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table10.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Workflow_Caffeine_5" displayName="Workflow_Caffeine_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -364,7 +348,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Tasks_Caffeine_6" displayName="Tasks_Caffeine_6" ref="A114:K117" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -383,7 +367,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Comms_Caffeine_7" displayName="Comms_Caffeine_7" ref="A120:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -404,7 +388,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="Critical_Caffeine_8" displayName="Critical_Caffeine_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -419,7 +403,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="Executive_DMARDsRA_1" displayName="Executive_DMARDsRA_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -431,7 +415,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table15.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="Milestones_DMARDsRA_2" displayName="Milestones_DMARDsRA_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -445,7 +429,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table16.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="Files_DMARDsRA_3" displayName="Files_DMARDsRA_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -460,7 +444,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table17.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="Stages_DMARDsRA_4" displayName="Stages_DMARDsRA_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -476,7 +460,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table18.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="Workflow_DMARDsRA_5" displayName="Workflow_DMARDsRA_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -494,7 +478,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table19.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="Tasks_DMARDsRA_6" displayName="Tasks_DMARDsRA_6" ref="A114:K116" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -513,7 +497,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Workflow63ActionsTable" displayName="Workflow63ActionsTable" ref="A1:G64" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="Workflow Master"/>
@@ -528,7 +512,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table20.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="Comms_DMARDsRA_7" displayName="Comms_DMARDsRA_7" ref="A119:M120" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -549,7 +533,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table21.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Critical_DMARDsRA_8" displayName="Critical_DMARDsRA_8" ref="A123:G124" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -564,7 +548,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table22.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="Executive_BPTargets_1" displayName="Executive_BPTargets_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -576,7 +560,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table23.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="Milestones_BPTargets_2" displayName="Milestones_BPTargets_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -590,7 +574,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table24.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="Files_BPTargets_3" displayName="Files_BPTargets_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -605,7 +589,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table25.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="Stages_BPTargets_4" displayName="Stages_BPTargets_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -621,7 +605,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table26.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="Workflow_BPTargets_5" displayName="Workflow_BPTargets_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -639,7 +623,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table27.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="Tasks_BPTargets_6" displayName="Tasks_BPTargets_6" ref="A114:K122" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -658,7 +642,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table28.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="Comms_BPTargets_7" displayName="Comms_BPTargets_7" ref="A129:M135" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -679,7 +663,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table29.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="Critical_BPTargets_8" displayName="Critical_BPTargets_8" ref="A143:G146" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -694,7 +678,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="GlobalPhaseCards" displayName="GlobalPhaseCards" ref="A4:E9" headerRowCount="1">
   <tableColumns count="5">
     <tableColumn id="1" name="PhaseKey"/>
@@ -707,7 +691,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table30.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="Executive_Psoriasis_1" displayName="Executive_Psoriasis_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -719,7 +703,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table31.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="Milestones_Psoriasis_2" displayName="Milestones_Psoriasis_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -733,7 +717,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table32.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="Files_Psoriasis_3" displayName="Files_Psoriasis_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -748,7 +732,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table33.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="Stages_Psoriasis_4" displayName="Stages_Psoriasis_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -764,7 +748,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table34.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="Workflow_Psoriasis_5" displayName="Workflow_Psoriasis_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -782,7 +766,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table35.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="Tasks_Psoriasis_6" displayName="Tasks_Psoriasis_6" ref="A114:K123" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -801,7 +785,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table36.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="Comms_Psoriasis_7" displayName="Comms_Psoriasis_7" ref="A129:M132" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -822,7 +806,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table37.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="Critical_Psoriasis_8" displayName="Critical_Psoriasis_8" ref="A142:G146" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -837,7 +821,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table38.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="Executive_FruitVeg_1" displayName="Executive_FruitVeg_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -849,7 +833,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table39.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="Milestones_FruitVeg_2" displayName="Milestones_FruitVeg_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -863,7 +847,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="GlobalResources" displayName="GlobalResources" ref="A13:H18" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="ResourceID"/>
@@ -879,7 +863,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table40.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table40.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="Files_FruitVeg_3" displayName="Files_FruitVeg_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -894,7 +878,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table41.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="Stages_FruitVeg_4" displayName="Stages_FruitVeg_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -910,7 +894,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table42.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="Workflow_FruitVeg_5" displayName="Workflow_FruitVeg_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -928,7 +912,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table43.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="Tasks_FruitVeg_6" displayName="Tasks_FruitVeg_6" ref="A114:K123" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -947,7 +931,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table44.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="Comms_FruitVeg_7" displayName="Comms_FruitVeg_7" ref="A125:M132" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -968,7 +952,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table45.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="Critical_FruitVeg_8" displayName="Critical_FruitVeg_8" ref="A135:G139" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -983,7 +967,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table46.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="Executive_Chlamydia_1" displayName="Executive_Chlamydia_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -995,7 +979,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table47.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="Milestones_Chlamydia_2" displayName="Milestones_Chlamydia_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1009,7 +993,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table48.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="Files_Chlamydia_3" displayName="Files_Chlamydia_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1024,7 +1008,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table49.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="Stages_Chlamydia_4" displayName="Stages_Chlamydia_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1040,7 +1024,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GlobalUpcomingMeetings" displayName="GlobalUpcomingMeetings" ref="A22:H28" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="MeetingID"/>
@@ -1056,7 +1040,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table50.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table50.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="Workflow_Chlamydia_5" displayName="Workflow_Chlamydia_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1074,7 +1058,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table51.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="Tasks_Chlamydia_6" displayName="Tasks_Chlamydia_6" ref="A114:K118" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1093,7 +1077,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table52.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="Comms_Chlamydia_7" displayName="Comms_Chlamydia_7" ref="A121:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1114,7 +1098,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table53.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="Critical_Chlamydia_8" displayName="Critical_Chlamydia_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1129,7 +1113,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table54.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="Executive_Review5TBD_1" displayName="Executive_Review5TBD_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1141,7 +1125,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table55.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="Milestones_Review5TBD_2" displayName="Milestones_Review5TBD_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1155,7 +1139,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table56.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="Files_Review5TBD_3" displayName="Files_Review5TBD_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1170,7 +1154,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table57.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="Stages_Review5TBD_4" displayName="Stages_Review5TBD_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1186,7 +1170,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table58.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="Workflow_Review5TBD_5" displayName="Workflow_Review5TBD_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1204,7 +1188,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table59.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table59.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="Tasks_Review5TBD_6" displayName="Tasks_Review5TBD_6" ref="A114:K118" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1223,7 +1207,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Executive_Caffeine_1" displayName="Executive_Caffeine_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1235,7 +1219,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table60.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table60.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="Comms_Review5TBD_7" displayName="Comms_Review5TBD_7" ref="A121:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1256,7 +1240,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table61.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="Critical_Review5TBD_8" displayName="Critical_Review5TBD_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1271,7 +1255,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table62.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="Executive_Phase2Batch_1" displayName="Executive_Phase2Batch_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1283,7 +1267,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table63.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="Milestones_Phase2Batch_2" displayName="Milestones_Phase2Batch_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1297,7 +1281,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table64.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="64" name="Files_Phase2Batch_3" displayName="Files_Phase2Batch_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1312,7 +1296,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table65.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="65" name="Stages_Phase2Batch_4" displayName="Stages_Phase2Batch_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1328,7 +1312,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table66.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="66" name="Workflow_Phase2Batch_5" displayName="Workflow_Phase2Batch_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1346,7 +1330,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table67.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="67" name="Tasks_Phase2Batch_6" displayName="Tasks_Phase2Batch_6" ref="A114:K115" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1365,7 +1349,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table68.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="68" name="Comms_Phase2Batch_7" displayName="Comms_Phase2Batch_7" ref="A118:M119" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1386,7 +1370,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table69.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table69.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="Critical_Phase2Batch_8" displayName="Critical_Phase2Batch_8" ref="A122:G123" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1401,7 +1385,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Milestones_Caffeine_2" displayName="Milestones_Caffeine_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1415,7 +1399,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table70.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table70.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="CandidatePipeline" displayName="CandidatePipeline" ref="A11:J29" headerRowCount="1">
   <tableColumns count="9">
     <tableColumn id="1" name="CandidateID"/>
@@ -1432,7 +1416,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table71.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="71" name="UpcomingMeetingsTable" displayName="UpcomingMeetingsTable" ref="A1:M6" headerRowCount="1">
   <autoFilter ref="A1:M6"/>
   <tableColumns count="13">
@@ -1454,7 +1438,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Files_Caffeine_3" displayName="Files_Caffeine_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1469,7 +1453,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table9.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Stages_Caffeine_4" displayName="Stages_Caffeine_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1485,7 +1469,7 @@
 </table>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
     <a:clrScheme name="ChatGPT">
@@ -1632,7 +1616,39 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2254,7 +2270,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2400,7 +2416,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract Screening Complete</t>
+          <t>Abstract screening complete / full-text preparation</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2468,7 +2484,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abstract screening completed; fifteen studies identified for full-text screening setup</t>
+          <t>Laser AI and conventional abstract screening are complete. The AI workflow advanced 15 records to full text. The conventional export and DOIs are still awaited. Before full-text screening, the team must confirm whether 128 records from prior monthly searches should be added to both arms, agree a PDF-sharing method, and finalise amendments to the full-text decision flow.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2485,7 +2501,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abstract screening completed; fifteen studies identified for full-text screening setup</t>
+          <t>Laser AI and conventional abstract screening are complete. The AI workflow advanced 15 records to full text. The conventional export and DOIs are still awaited. Before full-text screening, the team must confirm whether 128 records from prior monthly searches should be added to both arms, agree a PDF-sharing method, and finalise amendments to the full-text decision flow.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2502,7 +2518,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete usability survey, retrieve PDFs for the 15 studies, and prepare full-text screening setup.</t>
+          <t>Receive and reconcile the conventional full-text export; confirm inclusion of the 128 prior records and the PDF-sharing method; finalise the full-text decision flow; then start parallel full-text screening.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2517,9 +2533,9 @@
           <t>TargetDate</t>
         </is>
       </c>
-      <c r="B16" s="22" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TBD - after full-text set reconciliation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2536,7 +2552,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>The agreed decision-flow changes were initially not saved in Laser AI. Version 2 was subsequently applied, but earlier screened records may not include the comparator assessment; document this during the comparison.</t>
+          <t>The earlier AI-screening pause is resolved. Full-text start now depends on reconciling records and PDFs and confirming the full-text workflow.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2590,9 +2606,9 @@
           <t>LastUpdated</t>
         </is>
       </c>
-      <c r="B20" s="22" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2691,7 +2707,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Abstract screening complete</t>
+          <t>Complete - both workflows</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2708,7 +2724,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>15 studies identified; PDF retrieval and full-text setup pending</t>
+          <t>Preparation - awaiting record/PDF reconciliation</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2829,7 +2845,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>15 full-text records identified; PDFs to be retrieved and uploaded</t>
+          <t>Awaiting PDF-sharing method and reconciled full-text set</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2846,12 +2862,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Revised title/abstract decision flow saved as Version 2; full-text decision flow prepared</t>
+          <t>Full-text decision flow under amendment</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2990,15 +3006,20 @@
           <t>Setup / Coordination</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>0</v>
-      </c>
-      <c r="C42" t="n">
-        <v>0</v>
+      <c r="B42">
+        <v>100</v>
+      </c>
+      <c r="C42">
+        <v>100</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
           <t>Complete</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Abstract-screening setup completed for both workflows.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3013,15 +3034,20 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43" t="n">
-        <v>0</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0</v>
+      <c r="B43">
+        <v>100</v>
+      </c>
+      <c r="C43">
+        <v>100</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>Complete</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Conventional and Laser AI abstract screening complete; AI workflow moved 15 records to full text.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3044,7 +3070,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Setup pending for 15 studies</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Awaiting conventional export/DOIs, decision on 128 prior records, PDF-sharing method and final decision flow.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4042,14 +4073,18 @@
           <t>w21,w24,w25</t>
         </is>
       </c>
-      <c r="I65" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
       <c r="K65" s="18" t="n"/>
-      <c r="L65" s="18" t="n"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Conventional abstract screening complete; export and DOIs awaited.</t>
+        </is>
+      </c>
       <c r="M65" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4095,14 +4130,18 @@
           <t>w19,w21,w24,w25</t>
         </is>
       </c>
-      <c r="I66" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
       <c r="K66" s="18" t="n"/>
-      <c r="L66" s="18" t="n"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Laser AI abstract screening complete.</t>
+        </is>
+      </c>
       <c r="M66" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4148,14 +4187,18 @@
           <t>w20</t>
         </is>
       </c>
-      <c r="I67" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J67" s="18" t="n"/>
       <c r="K67" s="18" t="n"/>
-      <c r="L67" s="18" t="n"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>AI workflow identified 15 records for full-text screening.</t>
+        </is>
+      </c>
       <c r="M67" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4201,14 +4244,18 @@
           <t>w24,w25</t>
         </is>
       </c>
-      <c r="I68" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J68" s="18" t="n"/>
       <c r="K68" s="18" t="n"/>
-      <c r="L68" s="18" t="n"/>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>RIS file for 15 AI-selected full-text records shared.</t>
+        </is>
+      </c>
       <c r="M68" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4254,14 +4301,18 @@
           <t>w22</t>
         </is>
       </c>
-      <c r="I69" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J69" s="18" t="n"/>
       <c r="K69" s="18" t="n"/>
-      <c r="L69" s="18" t="n"/>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Usability survey link sent after Laser AI screening.</t>
+        </is>
+      </c>
       <c r="M69" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4413,14 +4464,18 @@
           <t>w25</t>
         </is>
       </c>
-      <c r="I72" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J72" s="18" t="n"/>
       <c r="K72" s="18" t="n"/>
-      <c r="L72" s="18" t="n"/>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Reconcile conventional export with AI output and determine treatment of 128 prior records.</t>
+        </is>
+      </c>
       <c r="M72" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4519,14 +4574,18 @@
           <t>w27,w29</t>
         </is>
       </c>
-      <c r="I74" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
-      <c r="L74" s="18" t="n"/>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>PDF-sharing method and complete full-text record set are being confirmed.</t>
+        </is>
+      </c>
       <c r="M74" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4678,14 +4737,18 @@
           <t>w30</t>
         </is>
       </c>
-      <c r="I77" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J77" s="18" t="n"/>
       <c r="K77" s="18" t="n"/>
-      <c r="L77" s="18" t="n"/>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Full-text decision flow requires final amendments.</t>
+        </is>
+      </c>
       <c r="M77" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4731,14 +4794,18 @@
           <t>w31</t>
         </is>
       </c>
-      <c r="I78" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
-      <c r="L78" s="18" t="n"/>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Full-text workflow setup awaits record/PDF reconciliation and final criteria.</t>
+        </is>
+      </c>
       <c r="M78" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -7774,7 +7841,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12529,7 +12596,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12620,12 +12687,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>General information folder</t>
+          <t>2026 AI platform study shared folder</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Shared folder with onboarding and scope documents.</t>
+          <t>Current shared folder in the AI Methods Group location; use this version going forward.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -12635,7 +12702,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://example.com/general-folder</t>
+          <t>https://cochranecollaboration.sharepoint.com/sites/EPM-EPRI/AI%20Methods%20Group/AI%20Methods%20Group%20%28shared%20folder%29/2026_AI%20platform%20study%20%28Shared%20folder%29</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -12666,8 +12733,15 @@
       <c r="K4" t="n">
         <v>1</v>
       </c>
-      <c r="L4" s="22" t="n">
-        <v>46156</v>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Current source of truth. Sean updated shortcuts; the old folder should be deleted or clearly archived to avoid confusion.</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -12791,7 +12865,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13005,7 +13079,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Setup phase underway; configuration and source materials are being finalized before screening starts</t>
+          <t>The protocol, eligibility criteria and 35 selected data-extraction items are available. Sean is running the accessible Index Medicus searches, while a wildcard inconsistency in the search strategy requires clarification. LILACS and IBECS remain inaccessible and the Native Health Research Database is retired. Screening has not started.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13022,7 +13096,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Setup phase underway; configuration and source materials are being finalized before screening starts</t>
+          <t>The protocol, eligibility criteria and 35 selected data-extraction items are available. Sean is running the accessible Index Medicus searches, while a wildcard inconsistency in the search strategy requires clarification. LILACS and IBECS remain inaccessible and the Native Health Research Database is retired. Screening has not started.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13039,7 +13113,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete setup materials and Laser AI configuration before commencing abstract screening.</t>
+          <t>Resolve the wildcard/search-strategy question; complete the accessible searches; document the unavailable databases; consolidate the final RIS set; then finalise Laser AI setup and approve screening to start.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13073,7 +13147,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Screening start depends on completion of setup materials and Laser AI configuration</t>
+          <t>Core protocol and data-item inputs are complete. Search-strategy clarification and inaccessible database documentation remain the gating issues.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -13129,7 +13203,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13211,7 +13285,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Protocol/data items complete; search strategy/database access under review</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -13344,7 +13418,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LILACS/search support ongoing</t>
+          <t>Search/RIS files received; accessible Index Medicus searches underway; LILACS/IBECS unavailable</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -13388,7 +13462,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Awaiting final materials</t>
+          <t>Eligibility criteria received in protocol</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -13535,7 +13609,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Protocol and data items complete; search strategy/database access issues remain.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -14261,14 +14340,18 @@
           <t>w12,w15,w29</t>
         </is>
       </c>
-      <c r="I59" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J59" s="18" t="n"/>
       <c r="K59" s="18" t="n"/>
-      <c r="L59" s="18" t="n"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Protocol and eligibility criteria received.</t>
+        </is>
+      </c>
       <c r="M59" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14314,14 +14397,18 @@
           <t>w13,w14,w43,w44</t>
         </is>
       </c>
-      <c r="I60" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J60" s="18" t="n"/>
       <c r="K60" s="18" t="n"/>
-      <c r="L60" s="18" t="n"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>35 selected data-extraction items received.</t>
+        </is>
+      </c>
       <c r="M60" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14367,14 +14454,18 @@
           <t>w14,w44</t>
         </is>
       </c>
-      <c r="I61" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J61" s="18" t="n"/>
       <c r="K61" s="18" t="n"/>
-      <c r="L61" s="18" t="n"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Comparable extraction structure requires final review.</t>
+        </is>
+      </c>
       <c r="M61" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14420,14 +14511,18 @@
           <t>w43,w44,w45</t>
         </is>
       </c>
-      <c r="I62" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J62" s="18" t="n"/>
       <c r="K62" s="18" t="n"/>
-      <c r="L62" s="18" t="n"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Final template approval pending.</t>
+        </is>
+      </c>
       <c r="M62" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14480,7 +14575,11 @@
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
-      <c r="L63" s="18" t="n"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Laser AI setup awaits final search set and search-strategy resolution.</t>
+        </is>
+      </c>
       <c r="M63" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -17566,7 +17665,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22080,7 +22179,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22233,9 +22332,9 @@
           <t>Converted to full sheet</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
-        <is>
-          <t>Participation confirmed; team roles agreed; onboarding and study material collection underway; tool training pending</t>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Converted to phase1-07; setup inputs complete and Nested Knowledge configuration underway</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22248,14 +22347,14 @@
           <t>Mohan Pammi</t>
         </is>
       </c>
-      <c r="G12" s="17" t="inlineStr">
-        <is>
-          <t>Onboarding and study material collection underway</t>
-        </is>
-      </c>
-      <c r="H12" s="17" t="inlineStr">
-        <is>
-          <t>Converted to phase1-07 Human Milk; Nested Knowledge allocated; tool training pending</t>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Configuration and setup validation underway</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Converted to phase1-07 Human Milk; RIS, criteria, protocol information and 35 data items received</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -22377,9 +22476,9 @@
           <t>Converted to full sheet</t>
         </is>
       </c>
-      <c r="D15" s="17" t="inlineStr">
-        <is>
-          <t>Tracked as phase1-05</t>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Protocol, criteria and 35 data items received; accessible searches underway; wildcard and LILACS/IBECS issues remain</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
@@ -22392,14 +22491,14 @@
           <t>Syeda Kanza Naqvi / Jai Das</t>
         </is>
       </c>
-      <c r="G15" s="17" t="inlineStr">
-        <is>
-          <t>Search update in progress</t>
-        </is>
-      </c>
-      <c r="H15" s="17" t="inlineStr">
-        <is>
-          <t>Final updated search/RIS and remaining study materials pending; Sean supporting LILACS/search issue</t>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Setup in progress; screening awaits final search resolution</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Converted to phase1-05 Vitamin C; search strategy/database access issues remain before screening</t>
         </is>
       </c>
       <c r="I15" s="17" t="inlineStr">
@@ -22838,46 +22937,185 @@
     <row r="30" ht="24" customHeight="1" s="29">
       <c r="A30" s="17" t="n"/>
       <c r="B30" s="17" t="n"/>
-      <c r="C30" s="17" t="n"/>
-      <c r="D30" s="17" t="n"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Shortlisted</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Onboarding confirmed for 2026-08-10 at 3:00 PM Malaysia time; whole team and two Cochrane elective students will attend</t>
+        </is>
+      </c>
       <c r="E30" s="17" t="n"/>
       <c r="F30" s="17" t="n"/>
-      <c r="G30" s="17" t="n"/>
-      <c r="H30" s="17" t="n"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Onboarding 2026-08-10; screening/additional data extraction August–September 2026; submission October 2026</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Initial search completed; 26 new eligible studies; data extraction and ROB 1 completed; INSPECT-SR and ROB 2 underway. Gerald is unavailable for onboarding; other project team members will conduct it.</t>
+        </is>
+      </c>
       <c r="I30" s="17" t="n"/>
     </row>
     <row r="31" ht="24" customHeight="1" s="29">
-      <c r="A31" s="17" t="n"/>
-      <c r="B31" s="17" t="n"/>
-      <c r="C31" s="17" t="n"/>
-      <c r="D31" s="17" t="n"/>
-      <c r="E31" s="17" t="n"/>
-      <c r="F31" s="17" t="n"/>
-      <c r="G31" s="17" t="n"/>
-      <c r="H31" s="17" t="n"/>
-      <c r="I31" s="17" t="n"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>new-20</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Melissa Moraes — review update details pending</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Under Shortlisting</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Interested and gathering the review topic, scope, eligible designs, search/screening status, expected new studies and timeline for eligibility review</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Melissa Moraes</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>TBD — awaiting review details</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>No separate eligibility form is required; review details are pending.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="24" customHeight="1" s="29">
-      <c r="A32" s="17" t="n"/>
-      <c r="B32" s="17" t="n"/>
-      <c r="C32" s="17" t="n"/>
-      <c r="D32" s="17" t="n"/>
-      <c r="E32" s="17" t="n"/>
-      <c r="F32" s="17" t="n"/>
-      <c r="G32" s="17" t="n"/>
-      <c r="H32" s="17" t="n"/>
-      <c r="I32" s="17" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>new-21</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Prof Iram Manzoor / Akhtar Saeed Medical and Dental College — review details pending</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Under Shortlisting</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Interest received; review title, status, timeline, parallel-workflow capacity and data-access details requested</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Prof Iram Manzoor / Sohail Sabir</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>TBD — awaiting review details</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Eligibility questions sent on 2026-07-31; no review-specific information received yet.</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="24" customHeight="1" s="29">
-      <c r="A33" s="17" t="n"/>
-      <c r="B33" s="17" t="n"/>
-      <c r="C33" s="17" t="n"/>
-      <c r="D33" s="17" t="n"/>
-      <c r="E33" s="17" t="n"/>
-      <c r="F33" s="17" t="n"/>
-      <c r="G33" s="17" t="n"/>
-      <c r="H33" s="17" t="n"/>
-      <c r="I33" s="17" t="n"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>new-22</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Eva Madrid / Cochrane Evidence Synthesis Unit Iberoamérica</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Future Phase</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Interested, but no ongoing Cochrane review updates are currently available</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Future opportunity</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Eva Madrid</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>No current update</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Keep in mind for future calls when an eligible Cochrane review update is available.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="24" customHeight="1" s="29">
       <c r="A34" s="17" t="n"/>
@@ -23146,7 +23384,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26585,7 +26823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27075,6 +27313,68 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>mtg-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>3:00-4:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>8:00-9:00 AM BST</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Oral Galactagogues Onboarding</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Initial onboarding, study workflow explanation and next-step planning before tool training/setup.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong / full review team / two Cochrane elective students / CESAR project team</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Later phase / Phase 2</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>new-19</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="M2:M200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -27094,7 +27394,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31687,7 +31987,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31833,7 +32133,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Setup inputs complete / configuration underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -31901,7 +32201,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Setup phase underway; study materials, training, and configuration are still being completed</t>
+          <t>The deduplicated RIS/search set (2,053 records), eligibility criteria, protocol information and 35 selected data-extraction items have been received. Questions on the selected items and deduplication were addressed; Nested Knowledge configuration and setup validation are next.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -31918,7 +32218,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Setup phase underway; study materials, training, and configuration are still being completed</t>
+          <t>The deduplicated RIS/search set (2,053 records), eligibility criteria, protocol information and 35 selected data-extraction items have been received. Questions on the selected items and deduplication were addressed; Nested Knowledge configuration and setup validation are next.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -31935,7 +32235,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Collect study materials, complete Nested Knowledge tool training, and configure the project for screening.</t>
+          <t>Configure Nested Knowledge using the received RIS, criteria, protocol information and 35-item list; obtain final confirmation on the extraction structure; validate the setup before screening starts.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -31952,7 +32252,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBD - after setup validation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -31969,7 +32269,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tool training and project configuration pending</t>
+          <t>Input collection is complete; tool configuration, final form confirmation and setup validation remain.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32025,7 +32325,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32107,7 +32407,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Inputs complete / configuration underway</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -32240,12 +32540,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Study materials collection underway</t>
+          <t>Deduplicated RIS received (2,053 records)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -32284,12 +32584,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Study materials collection underway</t>
+          <t>Eligibility criteria received</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -32306,12 +32606,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Study materials collection underway</t>
+          <t>35 selected data items received; questions addressed</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -32328,12 +32628,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Study materials collection underway</t>
+          <t>Protocol information / prior review received</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -32430,7 +32730,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Setup inputs are complete; Nested Knowledge configuration and validation are next.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -32873,14 +33178,18 @@
           <t>w10,w11,w12</t>
         </is>
       </c>
-      <c r="I54" s="18" t="inlineStr">
-        <is>
-          <t>Under Review</t>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J54" s="18" t="n"/>
       <c r="K54" s="18" t="n"/>
-      <c r="L54" s="18" t="n"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Shared folder is in use; selected data items were uploaded.</t>
+        </is>
+      </c>
       <c r="M54" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33085,14 +33394,18 @@
           <t>w15</t>
         </is>
       </c>
-      <c r="I58" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J58" s="18" t="n"/>
       <c r="K58" s="18" t="n"/>
-      <c r="L58" s="18" t="n"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Deduplicated RIS received with 2,053 unique records.</t>
+        </is>
+      </c>
       <c r="M58" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33138,14 +33451,18 @@
           <t>w12,w15,w29</t>
         </is>
       </c>
-      <c r="I59" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J59" s="18" t="n"/>
       <c r="K59" s="18" t="n"/>
-      <c r="L59" s="18" t="n"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Eligibility criteria and protocol information received.</t>
+        </is>
+      </c>
       <c r="M59" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33191,14 +33508,18 @@
           <t>w13,w14,w43,w44</t>
         </is>
       </c>
-      <c r="I60" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J60" s="18" t="n"/>
       <c r="K60" s="18" t="n"/>
-      <c r="L60" s="18" t="n"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>35 selected data items received.</t>
+        </is>
+      </c>
       <c r="M60" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33244,14 +33565,18 @@
           <t>w14,w44</t>
         </is>
       </c>
-      <c r="I61" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J61" s="18" t="n"/>
       <c r="K61" s="18" t="n"/>
-      <c r="L61" s="18" t="n"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Questions on the extraction structure were addressed by the review team.</t>
+        </is>
+      </c>
       <c r="M61" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33297,14 +33622,18 @@
           <t>w43,w44,w45</t>
         </is>
       </c>
-      <c r="I62" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J62" s="18" t="n"/>
       <c r="K62" s="18" t="n"/>
-      <c r="L62" s="18" t="n"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Comments addressed; final confirmation remains.</t>
+        </is>
+      </c>
       <c r="M62" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33350,14 +33679,18 @@
           <t>w16</t>
         </is>
       </c>
-      <c r="I63" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
-      <c r="L63" s="18" t="n"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Nested Knowledge configuration is the next operational step.</t>
+        </is>
+      </c>
       <c r="M63" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -36280,7 +36613,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -36462,7 +36795,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -36799,12 +37132,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Full-text screening phase; abstract screening has moved forward into full-text review preparation</t>
+          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete; 10 studies are selected for data extraction. Conventional timing is now available: Emilie—abstract 3h36m10s and full text 12h; Robin—abstract 6h35m and full text 4h12m (corrected from 3h06m). Repeated Laser AI output issues remain: Run 10 appears incomplete and 44 citations in Runs 3–5 remain unevaluated.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Complete full-text screening and prepare the agreed common sample for later data extraction.</t>
+          <t>Finalise the Nested Knowledge data-extraction workflow; validate and consolidate conventional and AI-assisted time logs; correct Run 10 and resolve the 44 unevaluated citations; complete the interim comparison.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -36851,7 +37184,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Abstract Screening Complete</t>
+          <t>Abstract screening complete / full-text preparation</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -36871,17 +37204,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Abstract screening completed; fifteen studies identified for full-text screening setup</t>
+          <t>Laser AI and conventional abstract screening are complete. The AI workflow advanced 15 records to full text. The conventional export and DOIs are still awaited. Before full-text screening, the team must confirm whether 128 records from prior monthly searches should be added to both arms, agree a PDF-sharing method, and finalise amendments to the full-text decision flow.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Complete usability survey, retrieve PDFs for the 15 studies, and prepare full-text screening setup.</t>
-        </is>
-      </c>
-      <c r="K6" s="22" t="inlineStr">
-        <is>
-          <t>TBD</t>
+          <t>Receive and reconcile the conventional full-text export; confirm inclusion of the 128 prior records and the PDF-sharing method; finalise the full-text decision flow; then start parallel full-text screening.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>TBD - after full-text set reconciliation</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -37010,12 +37343,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Setup phase underway; configuration and source materials are being finalized before screening starts</t>
+          <t>The protocol, eligibility criteria and 35 selected data-extraction items are available. Sean is running the accessible Index Medicus searches, while a wildcard inconsistency in the search strategy requires clarification. LILACS and IBECS remain inaccessible and the Native Health Research Database is retired. Screening has not started.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Complete setup materials and Laser AI configuration before commencing abstract screening.</t>
+          <t>Resolve the wildcard/search-strategy question; complete the accessible searches; document the unavailable databases; consolidate the final RIS set; then finalise Laser AI setup and approve screening to start.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -37206,7 +37539,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Setup inputs complete / configuration underway</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -37226,17 +37559,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Setup phase underway; study materials, training, and configuration are still being completed</t>
+          <t>The deduplicated RIS/search set (2,053 records), eligibility criteria, protocol information and 35 selected data-extraction items have been received. Questions on the selected items and deduplication were addressed; Nested Knowledge configuration and setup validation are next.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Collect study materials, complete Nested Knowledge tool training, and configure the project for screening.</t>
+          <t>Configure Nested Knowledge using the received RIS, criteria, protocol information and 35-item list; obtain final confirmation on the extraction structure; validate the setup before screening starts.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBD - after setup validation</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -37263,7 +37596,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40729,7 +41062,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40990,6 +41323,11 @@
           <t>res-001</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026 AI platform study shared folder</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>Folder</t>
@@ -41003,6 +41341,16 @@
       <c r="E14" t="inlineStr">
         <is>
           <t>Active</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://cochranecollaboration.sharepoint.com/sites/EPM-EPRI/AI%20Methods%20Group/AI%20Methods%20Group%20%28shared%20folder%29/2026_AI%20platform%20study%20%28Shared%20folder%29</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>AI Methods Group folder is the current source of truth; old folder should be archived or deleted.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -41210,22 +41558,37 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>meet-002</t>
+          <t>mtg-08</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>18 May 2026</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Core team discussion with Meghan</t>
+          <t>Oral Galactagogues Onboarding</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong / full review team / two elective students / CESAR project team</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Initial onboarding and workflow planning before tool training/setup.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sent</t>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>3:00 PM Malaysia / 8:00 AM BST / 3:00 AM EDT</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -41355,7 +41718,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -46120,7 +46483,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -50761,7 +51124,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -56145,7 +56508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -56359,7 +56722,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text screening phase; abstract screening has moved forward into full-text review preparation</t>
+          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete; 10 studies are selected for data extraction. Conventional timing is now available: Emilie—abstract 3h36m10s and full text 12h; Robin—abstract 6h35m and full text 4h12m (corrected from 3h06m). Repeated Laser AI output issues remain: Run 10 appears incomplete and 44 citations in Runs 3–5 remain unevaluated.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56376,7 +56739,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Full-text screening phase; abstract screening has moved forward into full-text review preparation</t>
+          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete; 10 studies are selected for data extraction. Conventional timing is now available: Emilie—abstract 3h36m10s and full text 12h; Robin—abstract 6h35m and full text 4h12m (corrected from 3h06m). Repeated Laser AI output issues remain: Run 10 appears incomplete and 44 citations in Runs 3–5 remain unevaluated.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56393,7 +56756,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete full-text screening and prepare the agreed common sample for later data extraction.</t>
+          <t>Finalise the Nested Knowledge data-extraction workflow; validate and consolidate conventional and AI-assisted time logs; correct Run 10 and resolve the 44 unevaluated citations; complete the interim comparison.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56408,7 +56771,7 @@
           <t>TargetDate</t>
         </is>
       </c>
-      <c r="B16" s="22" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
@@ -56427,7 +56790,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Main workflow remains in abstract screening; data extraction is only in preparation/sample planning stage</t>
+          <t>Conventional timing has been received; repeated Laser AI output validation issues remain before final reporting.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56481,9 +56844,9 @@
           <t>LastUpdated</t>
         </is>
       </c>
-      <c r="B20" s="22" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56813,7 +57176,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Conventional timing received: Emilie abstract 3h36m10s, full text 12h; Robin abstract 6h35m, full text 4h12m (corrected from 3h06m).</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -56886,15 +57249,20 @@
           <t>Setup / Coordination</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>0</v>
-      </c>
-      <c r="C42" t="n">
-        <v>0</v>
+      <c r="B42">
+        <v>100</v>
+      </c>
+      <c r="C42">
+        <v>100</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
           <t>Complete</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Onboarding and setup complete.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -56909,15 +57277,20 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43" t="n">
-        <v>0</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0</v>
+      <c r="B43">
+        <v>100</v>
+      </c>
+      <c r="C43">
+        <v>100</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>Complete</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Conventional and Nested Knowledge abstract screening complete.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -56932,15 +57305,20 @@
           <t>Full-text Screening</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>0</v>
-      </c>
-      <c r="C44" t="n">
-        <v>0</v>
+      <c r="B44">
+        <v>100</v>
+      </c>
+      <c r="C44">
+        <v>100</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Conventional and AI-assisted full-text screening complete; 10 studies selected.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -56963,7 +57341,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Nested Knowledge data-extraction setup and repeated-run validation analysis are underway.</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">

</xml_diff>

<commit_message>
Correct Phase 1 review status labels
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -27540,7 +27540,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Abstract screening underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -37112,7 +37112,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Full-text Screening</t>
+          <t>Data extraction / analysis</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -37467,7 +37467,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Abstract screening underway</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -56654,7 +56654,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text Screening</t>
+          <t>Data extraction / analysis</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">

</xml_diff>

<commit_message>
Sync live dashboard review statuses
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -1,37 +1,21 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
+  <dc:creator xmlns:dc="http://purl.org/dc/elements/1.1/">Krishna Kishore Pandalaneni</dc:creator>
+  <dcterms:created xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-05-27T01:47:03Z</dcterms:created>
+  <dcterms:modified xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-07-30T14:56:52Z</dcterms:modified>
+  <cp:lastModifiedBy>Krishna Kishore Pandalaneni</cp:lastModifiedBy>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="9">
@@ -324,7 +308,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewIndexTable" displayName="ReviewIndexTable" ref="A1:N11" headerRowCount="1">
   <tableColumns count="14">
     <tableColumn id="1" name="ReviewID"/>
@@ -346,7 +330,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table10.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Workflow_Caffeine_5" displayName="Workflow_Caffeine_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -364,7 +348,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Tasks_Caffeine_6" displayName="Tasks_Caffeine_6" ref="A114:K117" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -383,7 +367,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Comms_Caffeine_7" displayName="Comms_Caffeine_7" ref="A120:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -404,7 +388,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="Critical_Caffeine_8" displayName="Critical_Caffeine_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -419,7 +403,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="Executive_DMARDsRA_1" displayName="Executive_DMARDsRA_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -431,7 +415,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table15.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="Milestones_DMARDsRA_2" displayName="Milestones_DMARDsRA_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -445,7 +429,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table16.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="Files_DMARDsRA_3" displayName="Files_DMARDsRA_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -460,7 +444,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table17.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="Stages_DMARDsRA_4" displayName="Stages_DMARDsRA_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -476,7 +460,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table18.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="Workflow_DMARDsRA_5" displayName="Workflow_DMARDsRA_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -494,7 +478,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table19.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="Tasks_DMARDsRA_6" displayName="Tasks_DMARDsRA_6" ref="A114:K116" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -513,7 +497,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Workflow63ActionsTable" displayName="Workflow63ActionsTable" ref="A1:G64" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="Workflow Master"/>
@@ -528,7 +512,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table20.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="Comms_DMARDsRA_7" displayName="Comms_DMARDsRA_7" ref="A119:M120" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -549,7 +533,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table21.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Critical_DMARDsRA_8" displayName="Critical_DMARDsRA_8" ref="A123:G124" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -564,7 +548,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table22.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="Executive_BPTargets_1" displayName="Executive_BPTargets_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -576,7 +560,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table23.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="Milestones_BPTargets_2" displayName="Milestones_BPTargets_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -590,7 +574,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table24.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="Files_BPTargets_3" displayName="Files_BPTargets_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -605,7 +589,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table25.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="Stages_BPTargets_4" displayName="Stages_BPTargets_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -621,7 +605,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table26.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="Workflow_BPTargets_5" displayName="Workflow_BPTargets_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -639,7 +623,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table27.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="Tasks_BPTargets_6" displayName="Tasks_BPTargets_6" ref="A114:K122" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -658,7 +642,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table28.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="Comms_BPTargets_7" displayName="Comms_BPTargets_7" ref="A129:M135" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -679,7 +663,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table29.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="Critical_BPTargets_8" displayName="Critical_BPTargets_8" ref="A143:G146" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -694,7 +678,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="GlobalPhaseCards" displayName="GlobalPhaseCards" ref="A4:E9" headerRowCount="1">
   <tableColumns count="5">
     <tableColumn id="1" name="PhaseKey"/>
@@ -707,7 +691,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table30.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="Executive_Psoriasis_1" displayName="Executive_Psoriasis_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -719,7 +703,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table31.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="Milestones_Psoriasis_2" displayName="Milestones_Psoriasis_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -733,7 +717,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table32.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="Files_Psoriasis_3" displayName="Files_Psoriasis_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -748,7 +732,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table33.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="Stages_Psoriasis_4" displayName="Stages_Psoriasis_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -764,7 +748,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table34.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="Workflow_Psoriasis_5" displayName="Workflow_Psoriasis_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -782,7 +766,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table35.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="Tasks_Psoriasis_6" displayName="Tasks_Psoriasis_6" ref="A114:K123" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -801,7 +785,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table36.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="Comms_Psoriasis_7" displayName="Comms_Psoriasis_7" ref="A129:M132" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -822,7 +806,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table37.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="Critical_Psoriasis_8" displayName="Critical_Psoriasis_8" ref="A142:G146" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -837,7 +821,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table38.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="Executive_FruitVeg_1" displayName="Executive_FruitVeg_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -849,7 +833,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table39.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="Milestones_FruitVeg_2" displayName="Milestones_FruitVeg_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -863,7 +847,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="GlobalResources" displayName="GlobalResources" ref="A13:H18" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="ResourceID"/>
@@ -879,7 +863,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table40.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table40.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="Files_FruitVeg_3" displayName="Files_FruitVeg_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -894,7 +878,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table41.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="Stages_FruitVeg_4" displayName="Stages_FruitVeg_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -910,7 +894,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table42.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="Workflow_FruitVeg_5" displayName="Workflow_FruitVeg_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -928,7 +912,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table43.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="Tasks_FruitVeg_6" displayName="Tasks_FruitVeg_6" ref="A114:K123" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -947,7 +931,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table44.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="Comms_FruitVeg_7" displayName="Comms_FruitVeg_7" ref="A125:M132" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -968,7 +952,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table45.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="Critical_FruitVeg_8" displayName="Critical_FruitVeg_8" ref="A135:G139" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -983,7 +967,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table46.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="Executive_Chlamydia_1" displayName="Executive_Chlamydia_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -995,7 +979,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table47.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="Milestones_Chlamydia_2" displayName="Milestones_Chlamydia_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1009,7 +993,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table48.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="Files_Chlamydia_3" displayName="Files_Chlamydia_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1024,7 +1008,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table49.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="Stages_Chlamydia_4" displayName="Stages_Chlamydia_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1040,7 +1024,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GlobalUpcomingMeetings" displayName="GlobalUpcomingMeetings" ref="A22:H28" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="MeetingID"/>
@@ -1056,7 +1040,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table50.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table50.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="Workflow_Chlamydia_5" displayName="Workflow_Chlamydia_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1074,7 +1058,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table51.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="Tasks_Chlamydia_6" displayName="Tasks_Chlamydia_6" ref="A114:K118" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1093,7 +1077,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table52.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="Comms_Chlamydia_7" displayName="Comms_Chlamydia_7" ref="A121:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1114,7 +1098,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table53.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="Critical_Chlamydia_8" displayName="Critical_Chlamydia_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1129,7 +1113,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table54.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="Executive_Review5TBD_1" displayName="Executive_Review5TBD_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1141,7 +1125,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table55.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="Milestones_Review5TBD_2" displayName="Milestones_Review5TBD_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1155,7 +1139,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table56.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="Files_Review5TBD_3" displayName="Files_Review5TBD_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1170,7 +1154,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table57.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="Stages_Review5TBD_4" displayName="Stages_Review5TBD_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1186,7 +1170,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table58.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="Workflow_Review5TBD_5" displayName="Workflow_Review5TBD_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1204,7 +1188,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table59.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table59.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="Tasks_Review5TBD_6" displayName="Tasks_Review5TBD_6" ref="A114:K118" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1223,7 +1207,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Executive_Caffeine_1" displayName="Executive_Caffeine_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1235,7 +1219,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table60.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table60.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="Comms_Review5TBD_7" displayName="Comms_Review5TBD_7" ref="A121:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1256,7 +1240,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table61.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="Critical_Review5TBD_8" displayName="Critical_Review5TBD_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1271,7 +1255,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table62.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="Executive_Phase2Batch_1" displayName="Executive_Phase2Batch_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1283,7 +1267,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table63.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="Milestones_Phase2Batch_2" displayName="Milestones_Phase2Batch_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1297,7 +1281,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table64.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="64" name="Files_Phase2Batch_3" displayName="Files_Phase2Batch_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1312,7 +1296,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table65.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="65" name="Stages_Phase2Batch_4" displayName="Stages_Phase2Batch_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1328,7 +1312,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table66.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="66" name="Workflow_Phase2Batch_5" displayName="Workflow_Phase2Batch_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1346,7 +1330,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table67.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="67" name="Tasks_Phase2Batch_6" displayName="Tasks_Phase2Batch_6" ref="A114:K115" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1365,7 +1349,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table68.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="68" name="Comms_Phase2Batch_7" displayName="Comms_Phase2Batch_7" ref="A118:M119" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1386,7 +1370,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table69.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table69.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="Critical_Phase2Batch_8" displayName="Critical_Phase2Batch_8" ref="A122:G123" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1401,7 +1385,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Milestones_Caffeine_2" displayName="Milestones_Caffeine_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1415,7 +1399,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table70.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table70.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="CandidatePipeline" displayName="CandidatePipeline" ref="A11:J29" headerRowCount="1">
   <tableColumns count="9">
     <tableColumn id="1" name="CandidateID"/>
@@ -1432,7 +1416,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table71.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="71" name="UpcomingMeetingsTable" displayName="UpcomingMeetingsTable" ref="A1:M6" headerRowCount="1">
   <autoFilter ref="A1:M6"/>
   <tableColumns count="13">
@@ -1454,7 +1438,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Files_Caffeine_3" displayName="Files_Caffeine_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1469,7 +1453,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\tables\table9.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Stages_Caffeine_4" displayName="Stages_Caffeine_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1485,7 +1469,7 @@
 </table>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
     <a:clrScheme name="ChatGPT">
@@ -1632,7 +1616,39 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2254,7 +2270,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2400,7 +2416,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract Screening Complete</t>
+          <t>Abstract screening complete / full-text preparation</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2468,7 +2484,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abstract screening completed; fifteen studies identified for full-text screening setup</t>
+          <t>Laser AI and conventional abstract screening are complete. The AI workflow advanced 15 records to full text. The conventional export and DOIs are still awaited. Before full-text screening, the team must confirm whether 128 records from prior monthly searches should be added to both arms, agree a PDF-sharing method, and finalise amendments to the full-text decision flow.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2485,7 +2501,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abstract screening completed; fifteen studies identified for full-text screening setup</t>
+          <t>Laser AI and conventional abstract screening are complete. The AI workflow advanced 15 records to full text. The conventional export and DOIs are still awaited. Before full-text screening, the team must confirm whether 128 records from prior monthly searches should be added to both arms, agree a PDF-sharing method, and finalise amendments to the full-text decision flow.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2502,7 +2518,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete usability survey, retrieve PDFs for the 15 studies, and prepare full-text screening setup.</t>
+          <t>Receive and reconcile the conventional full-text export; confirm inclusion of the 128 prior records and the PDF-sharing method; finalise the full-text decision flow; then start parallel full-text screening.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2517,9 +2533,9 @@
           <t>TargetDate</t>
         </is>
       </c>
-      <c r="B16" s="22" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TBD - after full-text set reconciliation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2536,7 +2552,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>The agreed decision-flow changes were initially not saved in Laser AI. Version 2 was subsequently applied, but earlier screened records may not include the comparator assessment; document this during the comparison.</t>
+          <t>The earlier AI-screening pause is resolved. Full-text start now depends on reconciling records and PDFs and confirming the full-text workflow.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2590,9 +2606,9 @@
           <t>LastUpdated</t>
         </is>
       </c>
-      <c r="B20" s="22" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2691,7 +2707,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Abstract screening complete</t>
+          <t>Complete - both workflows</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2708,7 +2724,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>15 studies identified; PDF retrieval and full-text setup pending</t>
+          <t>Preparation - awaiting record/PDF reconciliation</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2829,7 +2845,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>15 full-text records identified; PDFs to be retrieved and uploaded</t>
+          <t>Awaiting PDF-sharing method and reconciled full-text set</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2846,12 +2862,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Revised title/abstract decision flow saved as Version 2; full-text decision flow prepared</t>
+          <t>Full-text decision flow under amendment</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2990,15 +3006,20 @@
           <t>Setup / Coordination</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>0</v>
-      </c>
-      <c r="C42" t="n">
-        <v>0</v>
+      <c r="B42">
+        <v>100</v>
+      </c>
+      <c r="C42">
+        <v>100</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
           <t>Complete</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Abstract-screening setup completed for both workflows.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3013,15 +3034,20 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43" t="n">
-        <v>0</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0</v>
+      <c r="B43">
+        <v>100</v>
+      </c>
+      <c r="C43">
+        <v>100</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>Complete</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Conventional and Laser AI abstract screening complete; AI workflow moved 15 records to full text.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3044,7 +3070,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Setup pending for 15 studies</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Awaiting conventional export/DOIs, decision on 128 prior records, PDF-sharing method and final decision flow.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4042,14 +4073,18 @@
           <t>w21,w24,w25</t>
         </is>
       </c>
-      <c r="I65" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
       <c r="K65" s="18" t="n"/>
-      <c r="L65" s="18" t="n"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Conventional abstract screening complete; export and DOIs awaited.</t>
+        </is>
+      </c>
       <c r="M65" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4095,14 +4130,18 @@
           <t>w19,w21,w24,w25</t>
         </is>
       </c>
-      <c r="I66" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
       <c r="K66" s="18" t="n"/>
-      <c r="L66" s="18" t="n"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Laser AI abstract screening complete.</t>
+        </is>
+      </c>
       <c r="M66" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4148,14 +4187,18 @@
           <t>w20</t>
         </is>
       </c>
-      <c r="I67" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J67" s="18" t="n"/>
       <c r="K67" s="18" t="n"/>
-      <c r="L67" s="18" t="n"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>AI workflow identified 15 records for full-text screening.</t>
+        </is>
+      </c>
       <c r="M67" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4201,14 +4244,18 @@
           <t>w24,w25</t>
         </is>
       </c>
-      <c r="I68" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J68" s="18" t="n"/>
       <c r="K68" s="18" t="n"/>
-      <c r="L68" s="18" t="n"/>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>RIS file for 15 AI-selected full-text records shared.</t>
+        </is>
+      </c>
       <c r="M68" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4254,14 +4301,18 @@
           <t>w22</t>
         </is>
       </c>
-      <c r="I69" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J69" s="18" t="n"/>
       <c r="K69" s="18" t="n"/>
-      <c r="L69" s="18" t="n"/>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Usability survey link sent after Laser AI screening.</t>
+        </is>
+      </c>
       <c r="M69" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4413,14 +4464,18 @@
           <t>w25</t>
         </is>
       </c>
-      <c r="I72" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J72" s="18" t="n"/>
       <c r="K72" s="18" t="n"/>
-      <c r="L72" s="18" t="n"/>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Reconcile conventional export with AI output and determine treatment of 128 prior records.</t>
+        </is>
+      </c>
       <c r="M72" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4519,14 +4574,18 @@
           <t>w27,w29</t>
         </is>
       </c>
-      <c r="I74" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
-      <c r="L74" s="18" t="n"/>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>PDF-sharing method and complete full-text record set are being confirmed.</t>
+        </is>
+      </c>
       <c r="M74" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4678,14 +4737,18 @@
           <t>w30</t>
         </is>
       </c>
-      <c r="I77" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J77" s="18" t="n"/>
       <c r="K77" s="18" t="n"/>
-      <c r="L77" s="18" t="n"/>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Full-text decision flow requires final amendments.</t>
+        </is>
+      </c>
       <c r="M77" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4731,14 +4794,18 @@
           <t>w31</t>
         </is>
       </c>
-      <c r="I78" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
-      <c r="L78" s="18" t="n"/>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Full-text workflow setup awaits record/PDF reconciliation and final criteria.</t>
+        </is>
+      </c>
       <c r="M78" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -7774,7 +7841,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12529,7 +12596,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12620,12 +12687,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>General information folder</t>
+          <t>2026 AI platform study shared folder</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Shared folder with onboarding and scope documents.</t>
+          <t>Current shared folder in the AI Methods Group location; use this version going forward.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -12635,7 +12702,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://example.com/general-folder</t>
+          <t>https://cochranecollaboration.sharepoint.com/sites/EPM-EPRI/AI%20Methods%20Group/AI%20Methods%20Group%20%28shared%20folder%29/2026_AI%20platform%20study%20%28Shared%20folder%29</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -12666,8 +12733,15 @@
       <c r="K4" t="n">
         <v>1</v>
       </c>
-      <c r="L4" s="22" t="n">
-        <v>46156</v>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Current source of truth. Sean updated shortcuts; the old folder should be deleted or clearly archived to avoid confusion.</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -12791,7 +12865,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13005,7 +13079,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Setup phase underway; configuration and source materials are being finalized before screening starts</t>
+          <t>The protocol, eligibility criteria and 35 selected data-extraction items are available. Sean is running the accessible Index Medicus searches, while a wildcard inconsistency in the search strategy requires clarification. LILACS and IBECS remain inaccessible and the Native Health Research Database is retired. Screening has not started.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13022,7 +13096,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Setup phase underway; configuration and source materials are being finalized before screening starts</t>
+          <t>The protocol, eligibility criteria and 35 selected data-extraction items are available. Sean is running the accessible Index Medicus searches, while a wildcard inconsistency in the search strategy requires clarification. LILACS and IBECS remain inaccessible and the Native Health Research Database is retired. Screening has not started.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13039,7 +13113,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete setup materials and Laser AI configuration before commencing abstract screening.</t>
+          <t>Resolve the wildcard/search-strategy question; complete the accessible searches; document the unavailable databases; consolidate the final RIS set; then finalise Laser AI setup and approve screening to start.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13073,7 +13147,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Screening start depends on completion of setup materials and Laser AI configuration</t>
+          <t>Core protocol and data-item inputs are complete. Search-strategy clarification and inaccessible database documentation remain the gating issues.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -13129,7 +13203,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13211,7 +13285,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Protocol/data items complete; search strategy/database access under review</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -13344,7 +13418,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LILACS/search support ongoing</t>
+          <t>Search/RIS files received; accessible Index Medicus searches underway; LILACS/IBECS unavailable</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -13388,7 +13462,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Awaiting final materials</t>
+          <t>Eligibility criteria received in protocol</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -13535,7 +13609,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Protocol and data items complete; search strategy/database access issues remain.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -14261,14 +14340,18 @@
           <t>w12,w15,w29</t>
         </is>
       </c>
-      <c r="I59" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J59" s="18" t="n"/>
       <c r="K59" s="18" t="n"/>
-      <c r="L59" s="18" t="n"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Protocol and eligibility criteria received.</t>
+        </is>
+      </c>
       <c r="M59" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14314,14 +14397,18 @@
           <t>w13,w14,w43,w44</t>
         </is>
       </c>
-      <c r="I60" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J60" s="18" t="n"/>
       <c r="K60" s="18" t="n"/>
-      <c r="L60" s="18" t="n"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>35 selected data-extraction items received.</t>
+        </is>
+      </c>
       <c r="M60" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14367,14 +14454,18 @@
           <t>w14,w44</t>
         </is>
       </c>
-      <c r="I61" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J61" s="18" t="n"/>
       <c r="K61" s="18" t="n"/>
-      <c r="L61" s="18" t="n"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Comparable extraction structure requires final review.</t>
+        </is>
+      </c>
       <c r="M61" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14420,14 +14511,18 @@
           <t>w43,w44,w45</t>
         </is>
       </c>
-      <c r="I62" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J62" s="18" t="n"/>
       <c r="K62" s="18" t="n"/>
-      <c r="L62" s="18" t="n"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Final template approval pending.</t>
+        </is>
+      </c>
       <c r="M62" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14480,7 +14575,11 @@
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
-      <c r="L63" s="18" t="n"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Laser AI setup awaits final search set and search-strategy resolution.</t>
+        </is>
+      </c>
       <c r="M63" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -17566,7 +17665,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22080,7 +22179,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22233,9 +22332,9 @@
           <t>Converted to full sheet</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
-        <is>
-          <t>Participation confirmed; team roles agreed; onboarding and study material collection underway; tool training pending</t>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Converted to phase1-07; setup inputs complete and Nested Knowledge configuration underway</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22248,14 +22347,14 @@
           <t>Mohan Pammi</t>
         </is>
       </c>
-      <c r="G12" s="17" t="inlineStr">
-        <is>
-          <t>Onboarding and study material collection underway</t>
-        </is>
-      </c>
-      <c r="H12" s="17" t="inlineStr">
-        <is>
-          <t>Converted to phase1-07 Human Milk; Nested Knowledge allocated; tool training pending</t>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Configuration and setup validation underway</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Converted to phase1-07 Human Milk; RIS, criteria, protocol information and 35 data items received</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -22377,9 +22476,9 @@
           <t>Converted to full sheet</t>
         </is>
       </c>
-      <c r="D15" s="17" t="inlineStr">
-        <is>
-          <t>Tracked as phase1-05</t>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Protocol, criteria and 35 data items received; accessible searches underway; wildcard and LILACS/IBECS issues remain</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
@@ -22392,14 +22491,14 @@
           <t>Syeda Kanza Naqvi / Jai Das</t>
         </is>
       </c>
-      <c r="G15" s="17" t="inlineStr">
-        <is>
-          <t>Search update in progress</t>
-        </is>
-      </c>
-      <c r="H15" s="17" t="inlineStr">
-        <is>
-          <t>Final updated search/RIS and remaining study materials pending; Sean supporting LILACS/search issue</t>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Setup in progress; screening awaits final search resolution</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Converted to phase1-05 Vitamin C; search strategy/database access issues remain before screening</t>
         </is>
       </c>
       <c r="I15" s="17" t="inlineStr">
@@ -22838,46 +22937,185 @@
     <row r="30" ht="24" customHeight="1" s="29">
       <c r="A30" s="17" t="n"/>
       <c r="B30" s="17" t="n"/>
-      <c r="C30" s="17" t="n"/>
-      <c r="D30" s="17" t="n"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Shortlisted</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Onboarding confirmed for 2026-08-10 at 3:00 PM Malaysia time; whole team and two Cochrane elective students will attend</t>
+        </is>
+      </c>
       <c r="E30" s="17" t="n"/>
       <c r="F30" s="17" t="n"/>
-      <c r="G30" s="17" t="n"/>
-      <c r="H30" s="17" t="n"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Onboarding 2026-08-10; screening/additional data extraction August–September 2026; submission October 2026</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Initial search completed; 26 new eligible studies; data extraction and ROB 1 completed; INSPECT-SR and ROB 2 underway. Gerald is unavailable for onboarding; other project team members will conduct it.</t>
+        </is>
+      </c>
       <c r="I30" s="17" t="n"/>
     </row>
     <row r="31" ht="24" customHeight="1" s="29">
-      <c r="A31" s="17" t="n"/>
-      <c r="B31" s="17" t="n"/>
-      <c r="C31" s="17" t="n"/>
-      <c r="D31" s="17" t="n"/>
-      <c r="E31" s="17" t="n"/>
-      <c r="F31" s="17" t="n"/>
-      <c r="G31" s="17" t="n"/>
-      <c r="H31" s="17" t="n"/>
-      <c r="I31" s="17" t="n"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>new-20</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Melissa Moraes — review update details pending</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Under Shortlisting</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Interested and gathering the review topic, scope, eligible designs, search/screening status, expected new studies and timeline for eligibility review</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Melissa Moraes</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>TBD — awaiting review details</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>No separate eligibility form is required; review details are pending.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="24" customHeight="1" s="29">
-      <c r="A32" s="17" t="n"/>
-      <c r="B32" s="17" t="n"/>
-      <c r="C32" s="17" t="n"/>
-      <c r="D32" s="17" t="n"/>
-      <c r="E32" s="17" t="n"/>
-      <c r="F32" s="17" t="n"/>
-      <c r="G32" s="17" t="n"/>
-      <c r="H32" s="17" t="n"/>
-      <c r="I32" s="17" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>new-21</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Prof Iram Manzoor / Akhtar Saeed Medical and Dental College — review details pending</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Under Shortlisting</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Interest received; review title, status, timeline, parallel-workflow capacity and data-access details requested</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Prof Iram Manzoor / Sohail Sabir</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>TBD — awaiting review details</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Eligibility questions sent on 2026-07-31; no review-specific information received yet.</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="24" customHeight="1" s="29">
-      <c r="A33" s="17" t="n"/>
-      <c r="B33" s="17" t="n"/>
-      <c r="C33" s="17" t="n"/>
-      <c r="D33" s="17" t="n"/>
-      <c r="E33" s="17" t="n"/>
-      <c r="F33" s="17" t="n"/>
-      <c r="G33" s="17" t="n"/>
-      <c r="H33" s="17" t="n"/>
-      <c r="I33" s="17" t="n"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>new-22</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Eva Madrid / Cochrane Evidence Synthesis Unit Iberoamérica</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Future Phase</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Interested, but no ongoing Cochrane review updates are currently available</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Future opportunity</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Eva Madrid</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>No current update</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Keep in mind for future calls when an eligible Cochrane review update is available.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="24" customHeight="1" s="29">
       <c r="A34" s="17" t="n"/>
@@ -23146,7 +23384,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26585,7 +26823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27075,6 +27313,68 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>mtg-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>3:00-4:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>8:00-9:00 AM BST</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Oral Galactagogues Onboarding</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Initial onboarding, study workflow explanation and next-step planning before tool training/setup.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong / full review team / two Cochrane elective students / CESAR project team</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Later phase / Phase 2</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>new-19</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="M2:M200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -27094,7 +27394,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27240,7 +27540,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Abstract screening underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -31687,7 +31987,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31833,7 +32133,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Setup inputs complete / configuration underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -31901,7 +32201,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Setup phase underway; study materials, training, and configuration are still being completed</t>
+          <t>The deduplicated RIS/search set (2,053 records), eligibility criteria, protocol information and 35 selected data-extraction items have been received. Questions on the selected items and deduplication were addressed; Nested Knowledge configuration and setup validation are next.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -31918,7 +32218,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Setup phase underway; study materials, training, and configuration are still being completed</t>
+          <t>The deduplicated RIS/search set (2,053 records), eligibility criteria, protocol information and 35 selected data-extraction items have been received. Questions on the selected items and deduplication were addressed; Nested Knowledge configuration and setup validation are next.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -31935,7 +32235,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Collect study materials, complete Nested Knowledge tool training, and configure the project for screening.</t>
+          <t>Configure Nested Knowledge using the received RIS, criteria, protocol information and 35-item list; obtain final confirmation on the extraction structure; validate the setup before screening starts.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -31952,7 +32252,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBD - after setup validation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -31969,7 +32269,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tool training and project configuration pending</t>
+          <t>Input collection is complete; tool configuration, final form confirmation and setup validation remain.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32025,7 +32325,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32107,7 +32407,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Inputs complete / configuration underway</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -32240,12 +32540,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Study materials collection underway</t>
+          <t>Deduplicated RIS received (2,053 records)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -32284,12 +32584,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Study materials collection underway</t>
+          <t>Eligibility criteria received</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -32306,12 +32606,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Study materials collection underway</t>
+          <t>35 selected data items received; questions addressed</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -32328,12 +32628,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Study materials collection underway</t>
+          <t>Protocol information / prior review received</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -32430,7 +32730,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Setup inputs are complete; Nested Knowledge configuration and validation are next.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -32873,14 +33178,18 @@
           <t>w10,w11,w12</t>
         </is>
       </c>
-      <c r="I54" s="18" t="inlineStr">
-        <is>
-          <t>Under Review</t>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J54" s="18" t="n"/>
       <c r="K54" s="18" t="n"/>
-      <c r="L54" s="18" t="n"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Shared folder is in use; selected data items were uploaded.</t>
+        </is>
+      </c>
       <c r="M54" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33085,14 +33394,18 @@
           <t>w15</t>
         </is>
       </c>
-      <c r="I58" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J58" s="18" t="n"/>
       <c r="K58" s="18" t="n"/>
-      <c r="L58" s="18" t="n"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Deduplicated RIS received with 2,053 unique records.</t>
+        </is>
+      </c>
       <c r="M58" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33138,14 +33451,18 @@
           <t>w12,w15,w29</t>
         </is>
       </c>
-      <c r="I59" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J59" s="18" t="n"/>
       <c r="K59" s="18" t="n"/>
-      <c r="L59" s="18" t="n"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Eligibility criteria and protocol information received.</t>
+        </is>
+      </c>
       <c r="M59" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33191,14 +33508,18 @@
           <t>w13,w14,w43,w44</t>
         </is>
       </c>
-      <c r="I60" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J60" s="18" t="n"/>
       <c r="K60" s="18" t="n"/>
-      <c r="L60" s="18" t="n"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>35 selected data items received.</t>
+        </is>
+      </c>
       <c r="M60" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33244,14 +33565,18 @@
           <t>w14,w44</t>
         </is>
       </c>
-      <c r="I61" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J61" s="18" t="n"/>
       <c r="K61" s="18" t="n"/>
-      <c r="L61" s="18" t="n"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Questions on the extraction structure were addressed by the review team.</t>
+        </is>
+      </c>
       <c r="M61" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33297,14 +33622,18 @@
           <t>w43,w44,w45</t>
         </is>
       </c>
-      <c r="I62" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J62" s="18" t="n"/>
       <c r="K62" s="18" t="n"/>
-      <c r="L62" s="18" t="n"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Comments addressed; final confirmation remains.</t>
+        </is>
+      </c>
       <c r="M62" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33350,14 +33679,18 @@
           <t>w16</t>
         </is>
       </c>
-      <c r="I63" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
-      <c r="L63" s="18" t="n"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Nested Knowledge configuration is the next operational step.</t>
+        </is>
+      </c>
       <c r="M63" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -36280,7 +36613,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -36462,7 +36795,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -36779,7 +37112,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Full-text Screening</t>
+          <t>Data extraction / analysis</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -36799,12 +37132,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Full-text screening phase; abstract screening has moved forward into full-text review preparation</t>
+          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete; 10 studies are selected for data extraction. Conventional timing is now available: Emilie—abstract 3h36m10s and full text 12h; Robin—abstract 6h35m and full text 4h12m (corrected from 3h06m). Repeated Laser AI output issues remain: Run 10 appears incomplete and 44 citations in Runs 3–5 remain unevaluated.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Complete full-text screening and prepare the agreed common sample for later data extraction.</t>
+          <t>Finalise the Nested Knowledge data-extraction workflow; validate and consolidate conventional and AI-assisted time logs; correct Run 10 and resolve the 44 unevaluated citations; complete the interim comparison.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -36851,7 +37184,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Abstract Screening Complete</t>
+          <t>Abstract screening complete / full-text preparation</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -36871,17 +37204,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Abstract screening completed; fifteen studies identified for full-text screening setup</t>
+          <t>Laser AI and conventional abstract screening are complete. The AI workflow advanced 15 records to full text. The conventional export and DOIs are still awaited. Before full-text screening, the team must confirm whether 128 records from prior monthly searches should be added to both arms, agree a PDF-sharing method, and finalise amendments to the full-text decision flow.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Complete usability survey, retrieve PDFs for the 15 studies, and prepare full-text screening setup.</t>
-        </is>
-      </c>
-      <c r="K6" s="22" t="inlineStr">
-        <is>
-          <t>TBD</t>
+          <t>Receive and reconcile the conventional full-text export; confirm inclusion of the 128 prior records and the PDF-sharing method; finalise the full-text decision flow; then start parallel full-text screening.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>TBD - after full-text set reconciliation</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -37010,12 +37343,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Setup phase underway; configuration and source materials are being finalized before screening starts</t>
+          <t>The protocol, eligibility criteria and 35 selected data-extraction items are available. Sean is running the accessible Index Medicus searches, while a wildcard inconsistency in the search strategy requires clarification. LILACS and IBECS remain inaccessible and the Native Health Research Database is retired. Screening has not started.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Complete setup materials and Laser AI configuration before commencing abstract screening.</t>
+          <t>Resolve the wildcard/search-strategy question; complete the accessible searches; document the unavailable databases; consolidate the final RIS set; then finalise Laser AI setup and approve screening to start.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -37134,7 +37467,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Abstract screening underway</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -37206,7 +37539,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Setup inputs complete / configuration underway</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -37226,17 +37559,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Setup phase underway; study materials, training, and configuration are still being completed</t>
+          <t>The deduplicated RIS/search set (2,053 records), eligibility criteria, protocol information and 35 selected data-extraction items have been received. Questions on the selected items and deduplication were addressed; Nested Knowledge configuration and setup validation are next.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Collect study materials, complete Nested Knowledge tool training, and configure the project for screening.</t>
+          <t>Configure Nested Knowledge using the received RIS, criteria, protocol information and 35-item list; obtain final confirmation on the extraction structure; validate the setup before screening starts.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBD - after setup validation</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -37263,7 +37596,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40729,7 +41062,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40990,6 +41323,11 @@
           <t>res-001</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026 AI platform study shared folder</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>Folder</t>
@@ -41003,6 +41341,16 @@
       <c r="E14" t="inlineStr">
         <is>
           <t>Active</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://cochranecollaboration.sharepoint.com/sites/EPM-EPRI/AI%20Methods%20Group/AI%20Methods%20Group%20%28shared%20folder%29/2026_AI%20platform%20study%20%28Shared%20folder%29</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>AI Methods Group folder is the current source of truth; old folder should be archived or deleted.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -41210,22 +41558,37 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>meet-002</t>
+          <t>mtg-08</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>18 May 2026</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Core team discussion with Meghan</t>
+          <t>Oral Galactagogues Onboarding</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong / full review team / two elective students / CESAR project team</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Initial onboarding and workflow planning before tool training/setup.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sent</t>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>3:00 PM Malaysia / 8:00 AM BST / 3:00 AM EDT</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -41355,7 +41718,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -46120,7 +46483,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -50761,7 +51124,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -56145,7 +56508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -56291,7 +56654,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text Screening</t>
+          <t>Data extraction / analysis</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56359,7 +56722,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text screening phase; abstract screening has moved forward into full-text review preparation</t>
+          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete; 10 studies are selected for data extraction. Conventional timing is now available: Emilie—abstract 3h36m10s and full text 12h; Robin—abstract 6h35m and full text 4h12m (corrected from 3h06m). Repeated Laser AI output issues remain: Run 10 appears incomplete and 44 citations in Runs 3–5 remain unevaluated.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56376,7 +56739,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Full-text screening phase; abstract screening has moved forward into full-text review preparation</t>
+          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete; 10 studies are selected for data extraction. Conventional timing is now available: Emilie—abstract 3h36m10s and full text 12h; Robin—abstract 6h35m and full text 4h12m (corrected from 3h06m). Repeated Laser AI output issues remain: Run 10 appears incomplete and 44 citations in Runs 3–5 remain unevaluated.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56393,7 +56756,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete full-text screening and prepare the agreed common sample for later data extraction.</t>
+          <t>Finalise the Nested Knowledge data-extraction workflow; validate and consolidate conventional and AI-assisted time logs; correct Run 10 and resolve the 44 unevaluated citations; complete the interim comparison.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56408,7 +56771,7 @@
           <t>TargetDate</t>
         </is>
       </c>
-      <c r="B16" s="22" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
@@ -56427,7 +56790,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Main workflow remains in abstract screening; data extraction is only in preparation/sample planning stage</t>
+          <t>Conventional timing has been received; repeated Laser AI output validation issues remain before final reporting.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56481,9 +56844,9 @@
           <t>LastUpdated</t>
         </is>
       </c>
-      <c r="B20" s="22" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56813,7 +57176,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Conventional timing received: Emilie abstract 3h36m10s, full text 12h; Robin abstract 6h35m, full text 4h12m (corrected from 3h06m).</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -56886,15 +57249,20 @@
           <t>Setup / Coordination</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>0</v>
-      </c>
-      <c r="C42" t="n">
-        <v>0</v>
+      <c r="B42">
+        <v>100</v>
+      </c>
+      <c r="C42">
+        <v>100</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
           <t>Complete</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Onboarding and setup complete.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -56909,15 +57277,20 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43" t="n">
-        <v>0</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0</v>
+      <c r="B43">
+        <v>100</v>
+      </c>
+      <c r="C43">
+        <v>100</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>Complete</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Conventional and Nested Knowledge abstract screening complete.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -56932,15 +57305,20 @@
           <t>Full-text Screening</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>0</v>
-      </c>
-      <c r="C44" t="n">
-        <v>0</v>
+      <c r="B44">
+        <v>100</v>
+      </c>
+      <c r="C44">
+        <v>100</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Conventional and AI-assisted full-text screening complete; 10 studies selected.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -56963,7 +57341,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Nested Knowledge data-extraction setup and repeated-run validation analysis are underway.</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">

</xml_diff>

<commit_message>
Update executive milestone status bars
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -27814,7 +27814,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Awaiting final template revisions</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -27831,7 +27831,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -27846,11 +27846,6 @@
           <t>fullText</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Template revisions/configuration pending</t>
-        </is>
-      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -27861,11 +27856,6 @@
       <c r="A28" t="inlineStr">
         <is>
           <t>extraction</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Draft template received</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -56945,7 +56935,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Full-text screening in progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -56962,7 +56952,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Abstract screening completed; full-text phase active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -56979,7 +56969,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Preparation only</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">

</xml_diff>

<commit_message>
Align executive milestone dots with review status
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -51551,7 +51551,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Data extraction phase</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -51568,7 +51568,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Full-text decisions feeding extraction setup</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -51585,7 +51585,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Setup underway</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">

</xml_diff>

<commit_message>
Align Pages milestone dots with review status
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -27814,7 +27814,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Awaiting final template revisions</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -27831,7 +27831,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -27846,11 +27846,6 @@
           <t>fullText</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Template revisions/configuration pending</t>
-        </is>
-      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -27861,11 +27856,6 @@
       <c r="A28" t="inlineStr">
         <is>
           <t>extraction</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Draft template received</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -51561,7 +51551,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Data extraction phase</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -51578,7 +51568,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Full-text decisions feeding extraction setup</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -51595,7 +51585,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Setup underway</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -56945,7 +56935,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Full-text screening in progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -56962,7 +56952,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Abstract screening completed; full-text phase active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -56979,7 +56969,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Preparation only</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">

</xml_diff>

<commit_message>
Update review status wording
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -37030,7 +37030,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Data Extraction / Analysis</t>
+          <t>Data extraction underway</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -37102,7 +37102,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data extraction / analysis</t>
+          <t>Data extraction underway</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -51260,7 +51260,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data Extraction / Analysis</t>
+          <t>Data extraction underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56644,7 +56644,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data extraction / analysis</t>
+          <t>Data extraction underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">

</xml_diff>

<commit_message>
Sync review status wording
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -37030,7 +37030,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Data Extraction / Analysis</t>
+          <t>Data extraction underway</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -37102,7 +37102,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data extraction / analysis</t>
+          <t>Data extraction underway</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -51260,7 +51260,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data Extraction / Analysis</t>
+          <t>Data extraction underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56644,7 +56644,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data extraction / analysis</t>
+          <t>Data extraction underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">

</xml_diff>

<commit_message>
Update next steps and progress trackers
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2724,7 +2724,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Preparation - awaiting record/PDF reconciliation</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -13285,7 +13285,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Protocol/data items complete; search strategy/database access under review</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -27642,7 +27642,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Finalize template revisions, complete project configuration, and then begin screening.</t>
+          <t>Continue conventional and AI-assisted abstract screening; monitor progress and time logs; then prepare the full-text screening stage.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -37482,7 +37482,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Finalize template revisions, complete project configuration, and then begin screening.</t>
+          <t>Continue conventional and AI-assisted abstract screening; monitor progress and time logs; then prepare the full-text screening stage.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">

</xml_diff>

<commit_message>
Sync next steps and progress trackers
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2724,7 +2724,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Preparation - awaiting record/PDF reconciliation</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -13285,7 +13285,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Protocol/data items complete; search strategy/database access under review</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -27642,7 +27642,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Finalize template revisions, complete project configuration, and then begin screening.</t>
+          <t>Continue conventional and AI-assisted abstract screening; monitor progress and time logs; then prepare the full-text screening stage.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -37482,7 +37482,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Finalize template revisions, complete project configuration, and then begin screening.</t>
+          <t>Continue conventional and AI-assisted abstract screening; monitor progress and time logs; then prepare the full-text screening stage.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">

</xml_diff>

<commit_message>
Refresh dashboard workbook updates
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -1,21 +1,37 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
-  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
-  <AppVersion>3.1</AppVersion>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
-  <dc:creator xmlns:dc="http://purl.org/dc/elements/1.1/">Krishna Kishore Pandalaneni</dc:creator>
-  <dcterms:created xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-05-27T01:47:03Z</dcterms:created>
-  <dcterms:modified xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-07-30T14:56:52Z</dcterms:modified>
-  <cp:lastModifiedBy>Krishna Kishore Pandalaneni</cp:lastModifiedBy>
-</cp:coreProperties>
-</file>
-
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="9">
@@ -308,7 +324,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\tables\table1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewIndexTable" displayName="ReviewIndexTable" ref="A1:N11" headerRowCount="1">
   <tableColumns count="14">
     <tableColumn id="1" name="ReviewID"/>
@@ -330,7 +346,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Workflow_Caffeine_5" displayName="Workflow_Caffeine_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -348,7 +364,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Tasks_Caffeine_6" displayName="Tasks_Caffeine_6" ref="A114:K117" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -367,7 +383,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Comms_Caffeine_7" displayName="Comms_Caffeine_7" ref="A120:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -388,7 +404,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="Critical_Caffeine_8" displayName="Critical_Caffeine_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -403,7 +419,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="Executive_DMARDsRA_1" displayName="Executive_DMARDsRA_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -415,7 +431,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="Milestones_DMARDsRA_2" displayName="Milestones_DMARDsRA_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -429,7 +445,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="Files_DMARDsRA_3" displayName="Files_DMARDsRA_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -444,7 +460,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="Stages_DMARDsRA_4" displayName="Stages_DMARDsRA_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -460,7 +476,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="Workflow_DMARDsRA_5" displayName="Workflow_DMARDsRA_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -478,7 +494,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="Tasks_DMARDsRA_6" displayName="Tasks_DMARDsRA_6" ref="A114:K116" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -497,7 +513,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Workflow63ActionsTable" displayName="Workflow63ActionsTable" ref="A1:G64" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="Workflow Master"/>
@@ -512,7 +528,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="Comms_DMARDsRA_7" displayName="Comms_DMARDsRA_7" ref="A119:M120" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -533,7 +549,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Critical_DMARDsRA_8" displayName="Critical_DMARDsRA_8" ref="A123:G124" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -548,7 +564,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="Executive_BPTargets_1" displayName="Executive_BPTargets_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -560,7 +576,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="Milestones_BPTargets_2" displayName="Milestones_BPTargets_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -574,7 +590,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="Files_BPTargets_3" displayName="Files_BPTargets_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -589,7 +605,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="Stages_BPTargets_4" displayName="Stages_BPTargets_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -605,7 +621,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="Workflow_BPTargets_5" displayName="Workflow_BPTargets_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -623,7 +639,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="Tasks_BPTargets_6" displayName="Tasks_BPTargets_6" ref="A114:K122" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -642,7 +658,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="Comms_BPTargets_7" displayName="Comms_BPTargets_7" ref="A129:M135" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -663,7 +679,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="Critical_BPTargets_8" displayName="Critical_BPTargets_8" ref="A143:G146" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -678,7 +694,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="GlobalPhaseCards" displayName="GlobalPhaseCards" ref="A4:E9" headerRowCount="1">
   <tableColumns count="5">
     <tableColumn id="1" name="PhaseKey"/>
@@ -691,7 +707,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="Executive_Psoriasis_1" displayName="Executive_Psoriasis_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -703,7 +719,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="Milestones_Psoriasis_2" displayName="Milestones_Psoriasis_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -717,7 +733,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="Files_Psoriasis_3" displayName="Files_Psoriasis_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -732,7 +748,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="Stages_Psoriasis_4" displayName="Stages_Psoriasis_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -748,7 +764,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="Workflow_Psoriasis_5" displayName="Workflow_Psoriasis_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -766,7 +782,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="Tasks_Psoriasis_6" displayName="Tasks_Psoriasis_6" ref="A114:K123" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -785,7 +801,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="Comms_Psoriasis_7" displayName="Comms_Psoriasis_7" ref="A129:M132" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -806,7 +822,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="Critical_Psoriasis_8" displayName="Critical_Psoriasis_8" ref="A142:G146" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -821,7 +837,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="Executive_FruitVeg_1" displayName="Executive_FruitVeg_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -833,7 +849,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="Milestones_FruitVeg_2" displayName="Milestones_FruitVeg_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -847,7 +863,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="GlobalResources" displayName="GlobalResources" ref="A13:H18" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="ResourceID"/>
@@ -863,7 +879,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table40.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table40.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="Files_FruitVeg_3" displayName="Files_FruitVeg_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -878,7 +894,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table41.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="Stages_FruitVeg_4" displayName="Stages_FruitVeg_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -894,7 +910,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table42.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="Workflow_FruitVeg_5" displayName="Workflow_FruitVeg_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -912,7 +928,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table43.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="Tasks_FruitVeg_6" displayName="Tasks_FruitVeg_6" ref="A114:K123" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -931,7 +947,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table44.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="Comms_FruitVeg_7" displayName="Comms_FruitVeg_7" ref="A125:M132" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -952,7 +968,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table45.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="Critical_FruitVeg_8" displayName="Critical_FruitVeg_8" ref="A135:G139" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -967,7 +983,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table46.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="Executive_Chlamydia_1" displayName="Executive_Chlamydia_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -979,7 +995,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table47.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="Milestones_Chlamydia_2" displayName="Milestones_Chlamydia_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -993,7 +1009,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table48.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="Files_Chlamydia_3" displayName="Files_Chlamydia_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1008,7 +1024,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table49.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="Stages_Chlamydia_4" displayName="Stages_Chlamydia_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1024,7 +1040,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GlobalUpcomingMeetings" displayName="GlobalUpcomingMeetings" ref="A22:H28" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="MeetingID"/>
@@ -1040,7 +1056,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table50.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table50.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="Workflow_Chlamydia_5" displayName="Workflow_Chlamydia_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1058,7 +1074,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table51.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="Tasks_Chlamydia_6" displayName="Tasks_Chlamydia_6" ref="A114:K118" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1077,7 +1093,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table52.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="Comms_Chlamydia_7" displayName="Comms_Chlamydia_7" ref="A121:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1098,7 +1114,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table53.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="Critical_Chlamydia_8" displayName="Critical_Chlamydia_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1113,7 +1129,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table54.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="Executive_Review5TBD_1" displayName="Executive_Review5TBD_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1125,7 +1141,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table55.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="Milestones_Review5TBD_2" displayName="Milestones_Review5TBD_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1139,7 +1155,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table56.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="Files_Review5TBD_3" displayName="Files_Review5TBD_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1154,7 +1170,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table57.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="Stages_Review5TBD_4" displayName="Stages_Review5TBD_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1170,7 +1186,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table58.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="Workflow_Review5TBD_5" displayName="Workflow_Review5TBD_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1188,7 +1204,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table59.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table59.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="Tasks_Review5TBD_6" displayName="Tasks_Review5TBD_6" ref="A114:K118" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1207,7 +1223,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Executive_Caffeine_1" displayName="Executive_Caffeine_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1219,7 +1235,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table60.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table60.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="Comms_Review5TBD_7" displayName="Comms_Review5TBD_7" ref="A121:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1240,7 +1256,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table61.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="Critical_Review5TBD_8" displayName="Critical_Review5TBD_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1255,7 +1271,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table62.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="Executive_Phase2Batch_1" displayName="Executive_Phase2Batch_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1267,7 +1283,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table63.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="Milestones_Phase2Batch_2" displayName="Milestones_Phase2Batch_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1281,7 +1297,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table64.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="64" name="Files_Phase2Batch_3" displayName="Files_Phase2Batch_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1296,7 +1312,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table65.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="65" name="Stages_Phase2Batch_4" displayName="Stages_Phase2Batch_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1312,7 +1328,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table66.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="66" name="Workflow_Phase2Batch_5" displayName="Workflow_Phase2Batch_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1330,7 +1346,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table67.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="67" name="Tasks_Phase2Batch_6" displayName="Tasks_Phase2Batch_6" ref="A114:K115" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1349,7 +1365,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table68.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="68" name="Comms_Phase2Batch_7" displayName="Comms_Phase2Batch_7" ref="A118:M119" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1370,7 +1386,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table69.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table69.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="Critical_Phase2Batch_8" displayName="Critical_Phase2Batch_8" ref="A122:G123" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1385,7 +1401,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Milestones_Caffeine_2" displayName="Milestones_Caffeine_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1399,7 +1415,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table70.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table70.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="CandidatePipeline" displayName="CandidatePipeline" ref="A11:J29" headerRowCount="1">
   <tableColumns count="9">
     <tableColumn id="1" name="CandidateID"/>
@@ -1416,7 +1432,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table71.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="71" name="UpcomingMeetingsTable" displayName="UpcomingMeetingsTable" ref="A1:M6" headerRowCount="1">
   <autoFilter ref="A1:M6"/>
   <tableColumns count="13">
@@ -1438,7 +1454,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Files_Caffeine_3" displayName="Files_Caffeine_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1453,7 +1469,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Stages_Caffeine_4" displayName="Stages_Caffeine_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1469,7 +1485,7 @@
 </table>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
     <a:clrScheme name="ChatGPT">
@@ -1616,39 +1632,7 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2270,7 +2254,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2416,7 +2400,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract screening complete / full-text preparation</t>
+          <t>Full-text screening preparation</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2484,7 +2468,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Laser AI and conventional abstract screening are complete. The AI workflow advanced 15 records to full text. The conventional export and DOIs are still awaited. Before full-text screening, the team must confirm whether 128 records from prior monthly searches should be added to both arms, agree a PDF-sharing method, and finalise amendments to the full-text decision flow.</t>
+          <t>AI-assisted and conventional abstract screening are complete. Fifteen April/May records are moving to full text, and 128 prior-search records will also be added to both arms. Shared-folder access for PDFs is in place.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2501,7 +2485,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Laser AI and conventional abstract screening are complete. The AI workflow advanced 15 records to full text. The conventional export and DOIs are still awaited. Before full-text screening, the team must confirm whether 128 records from prior monthly searches should be added to both arms, agree a PDF-sharing method, and finalise amendments to the full-text decision flow.</t>
+          <t>AI-assisted and conventional abstract screening are complete. Fifteen April/May records are moving to full text, and 128 prior-search records will also be added to both arms. Shared-folder access for PDFs is in place.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2518,7 +2502,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Receive and reconcile the conventional full-text export; confirm inclusion of the 128 prior records and the PDF-sharing method; finalise the full-text decision flow; then start parallel full-text screening.</t>
+          <t>Consolidate the final full-text record set and DOIs, upload PDFs, finalise any full-text decision-flow amendments, and proceed with full-text screening in both arms.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2552,7 +2536,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>The earlier AI-screening pause is resolved. Full-text start now depends on reconciling records and PDFs and confirming the full-text workflow.</t>
+          <t>Abstract screening is complete; the current dependency is consolidating the full-text set and PDFs, including the additional 128 prior-search records.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2608,7 +2592,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2840,12 +2824,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Awaiting PDF-sharing method and reconciled full-text set</t>
+          <t>Shared folder provided; PDFs being collected/uploaded for full-text screening.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2862,12 +2846,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Full-text decision flow under amendment</t>
+          <t>Full-text decision flow and eligibility criteria configured; minor amendments under review.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3006,10 +2990,10 @@
           <t>Setup / Coordination</t>
         </is>
       </c>
-      <c r="B42">
+      <c r="B42" t="n">
         <v>100</v>
       </c>
-      <c r="C42">
+      <c r="C42" t="n">
         <v>100</v>
       </c>
       <c r="D42" t="inlineStr">
@@ -3034,10 +3018,10 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43">
+      <c r="B43" t="n">
         <v>100</v>
       </c>
-      <c r="C43">
+      <c r="C43" t="n">
         <v>100</v>
       </c>
       <c r="D43" t="inlineStr">
@@ -7841,7 +7825,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12596,7 +12580,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12865,7 +12849,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13011,7 +12995,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Setup in progress - search strategy/access issue</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -13079,7 +13063,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The protocol, eligibility criteria and 35 selected data-extraction items are available. Sean is running the accessible Index Medicus searches, while a wildcard inconsistency in the search strategy requires clarification. LILACS and IBECS remain inaccessible and the Native Health Research Database is retired. Screening has not started.</t>
+          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13096,7 +13080,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The protocol, eligibility criteria and 35 selected data-extraction items are available. Sean is running the accessible Index Medicus searches, while a wildcard inconsistency in the search strategy requires clarification. LILACS and IBECS remain inaccessible and the Native Health Research Database is retired. Screening has not started.</t>
+          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13113,7 +13097,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Resolve the wildcard/search-strategy question; complete the accessible searches; document the unavailable databases; consolidate the final RIS set; then finalise Laser AI setup and approve screening to start.</t>
+          <t>Clarify wildcard use, complete accessible searches, document LILACS/IBECS limitations, finalise Laser AI setup, and confirm the screening start.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13147,7 +13131,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Core protocol and data-item inputs are complete. Search-strategy clarification and inaccessible database documentation remain the gating issues.</t>
+          <t>Most setup materials are available; search-strategy clarification and database-access issues remain before screening can start.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -13203,7 +13187,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13300,11 +13284,6 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Setup phase</t>
-        </is>
-      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13315,11 +13294,6 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>fullText</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Screening not yet started</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -13418,7 +13392,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Search/RIS files received; accessible Index Medicus searches underway; LILACS/IBECS unavailable</t>
+          <t>Search/RIS files partly available; additional searches await wildcard clarification; LILACS/IBECS remain inaccessible.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -17665,7 +17639,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22179,7 +22153,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22935,8 +22909,16 @@
       </c>
     </row>
     <row r="30" ht="24" customHeight="1" s="29">
-      <c r="A30" s="17" t="n"/>
-      <c r="B30" s="17" t="n"/>
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>new-19</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong - Oral galactagogues for increasing breast milk production in mothers of non-hospitalised term infants</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
           <t>Shortlisted</t>
@@ -22944,22 +22926,39 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Onboarding confirmed for 2026-08-10 at 3:00 PM Malaysia time; whole team and two Cochrane elective students will attend</t>
-        </is>
-      </c>
-      <c r="E30" s="17" t="n"/>
-      <c r="F30" s="17" t="n"/>
+          <t>Onboarding confirmed for 2026-08-10 at 3:00 PM Malaysia time; full team and two Cochrane elective students will attend.</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Onboarding 2026-08-10; screening/additional data extraction August–September 2026; submission October 2026</t>
+          <t>Onboarding 2026-08-10; tool training and setup to follow.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Initial search completed; 26 new eligible studies; data extraction and ROB 1 completed; INSPECT-SR and ROB 2 underway. Gerald is unavailable for onboarding; other project team members will conduct it.</t>
-        </is>
-      </c>
-      <c r="I30" s="17" t="n"/>
+          <t>Initial onboarding will cover the study and parallel workflow; tool training and setup will be scheduled afterward.</t>
+        </is>
+      </c>
+      <c r="I30" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="24" customHeight="1" s="29">
       <c r="A31" t="inlineStr">
@@ -23384,7 +23383,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26823,13 +26822,13 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="14" customWidth="1" style="29" min="1" max="2"/>
@@ -27336,17 +27335,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Oral Galactagogues Onboarding</t>
+          <t>Oral galactagogues onboarding</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Initial onboarding, study workflow explanation and next-step planning before tool training/setup.</t>
+          <t>Initial onboarding and pilot workflow overview; tool training/setup to follow</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Siew Cheng Foong / full review team / two Cochrane elective students / CESAR project team</t>
+          <t>Siew Cheng Foong / full review team / 2 Cochrane elective students / project team</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -27356,17 +27355,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Later phase / Phase 2</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>Scheduled</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>new-19</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -27394,7 +27388,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31977,7 +31971,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -32123,7 +32117,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup inputs complete / configuration underway</t>
+          <t>Setup in progress</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32191,7 +32185,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The deduplicated RIS/search set (2,053 records), eligibility criteria, protocol information and 35 selected data-extraction items have been received. Questions on the selected items and deduplication were addressed; Nested Knowledge configuration and setup validation are next.</t>
+          <t>Onboarding/training are complete. The team has supplied a deduplicated RIS file with 2,053 records, 35 selected data items, and Study Protocol Info containing inclusion/exclusion/PICOS details. Nested Knowledge configuration can proceed.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32208,7 +32202,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The deduplicated RIS/search set (2,053 records), eligibility criteria, protocol information and 35 selected data-extraction items have been received. Questions on the selected items and deduplication were addressed; Nested Knowledge configuration and setup validation are next.</t>
+          <t>Onboarding/training are complete. The team has supplied a deduplicated RIS file with 2,053 records, 35 selected data items, and Study Protocol Info containing inclusion/exclusion/PICOS details. Nested Knowledge configuration can proceed.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32225,7 +32219,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Configure Nested Knowledge using the received RIS, criteria, protocol information and 35-item list; obtain final confirmation on the extraction structure; validate the setup before screening starts.</t>
+          <t>Configure the Nested Knowledge project, confirm screening instructions/calibration, and begin abstract screening once setup is complete.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32259,7 +32253,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Input collection is complete; tool configuration, final form confirmation and setup validation remain.</t>
+          <t>Key setup inputs are now received; Nested Knowledge configuration is the next step. Full-text PDFs can be assembled later for the full-text stage.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32315,7 +32309,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32380,7 +32374,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Underway</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -32397,7 +32391,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Inputs complete / configuration underway</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -32412,11 +32406,6 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Setup phase</t>
-        </is>
-      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32429,11 +32418,6 @@
           <t>fullText</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Materials/training/configuration pending</t>
-        </is>
-      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32444,11 +32428,6 @@
       <c r="A28" t="inlineStr">
         <is>
           <t>extraction</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Not Started</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -32535,7 +32514,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Deduplicated RIS received (2,053 records)</t>
+          <t>Deduplicated RIS/search file received - 2,053 records.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -32579,7 +32558,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Eligibility criteria received</t>
+          <t>Inclusion/exclusion criteria and PICOS received in Study Protocol Info.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -32601,7 +32580,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>35 selected data items received; questions addressed</t>
+          <t>35 selected data-extraction items received.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -32623,7 +32602,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Protocol information / prior review received</t>
+          <t>Protocol / Study Protocol Info received.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -36603,7 +36582,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -36785,7 +36764,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -37050,17 +37029,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Data extraction phase; full-text screening outputs are feeding extraction and analysis setup</t>
+          <t>Data extraction remains underway. Blood Pressure Targets is expected to complete the Laser AI data-extraction stage during the week of 2026-08-10. Completed outputs will then be collected for analysis.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Continue data extraction and analysis preparation; reconcile full-text decisions and submit extraction outputs/time logs.</t>
+          <t>Complete data extraction, collect extraction outputs and time logs, and send the data-extraction usability survey once the stage is complete.</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>Week of 2026-08-10</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -37122,12 +37101,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete; 10 studies are selected for data extraction. Conventional timing is now available: Emilie—abstract 3h36m10s and full text 12h; Robin—abstract 6h35m and full text 4h12m (corrected from 3h06m). Repeated Laser AI output issues remain: Run 10 appears incomplete and 44 citations in Runs 3–5 remain unevaluated.</t>
+          <t>Abstract and full-text screening are complete in the AI-assisted and conventional workflows. Ten studies are selected for data extraction. Conventional screening time-on-task is now complete; Robin's full-text time was corrected to 4h12. Repeated Laser AI run-validation issues remain provisional.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Finalise the Nested Knowledge data-extraction workflow; validate and consolidate conventional and AI-assisted time logs; correct Run 10 and resolve the 44 unevaluated citations; complete the interim comparison.</t>
+          <t>Finalise the Nested Knowledge data-extraction workflow; correct Run 10 and resolve the 44 unevaluated citations in Runs 3-5; complete the interim comparison.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -37174,7 +37153,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Abstract screening complete / full-text preparation</t>
+          <t>Full-text screening preparation</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -37194,12 +37173,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Laser AI and conventional abstract screening are complete. The AI workflow advanced 15 records to full text. The conventional export and DOIs are still awaited. Before full-text screening, the team must confirm whether 128 records from prior monthly searches should be added to both arms, agree a PDF-sharing method, and finalise amendments to the full-text decision flow.</t>
+          <t>AI-assisted and conventional abstract screening are complete. Fifteen April/May records are moving to full text, and 128 prior-search records will also be added to both arms. Shared-folder access for PDFs is in place.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Receive and reconcile the conventional full-text export; confirm inclusion of the 128 prior records and the PDF-sharing method; finalise the full-text decision flow; then start parallel full-text screening.</t>
+          <t>Consolidate the final full-text record set and DOIs, upload PDFs, finalise any full-text decision-flow amendments, and proceed with full-text screening in both arms.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -37313,7 +37292,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Setup in progress - search strategy/access issue</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -37333,12 +37312,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>The protocol, eligibility criteria and 35 selected data-extraction items are available. Sean is running the accessible Index Medicus searches, while a wildcard inconsistency in the search strategy requires clarification. LILACS and IBECS remain inaccessible and the Native Health Research Database is retired. Screening has not started.</t>
+          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Resolve the wildcard/search-strategy question; complete the accessible searches; document the unavailable databases; consolidate the final RIS set; then finalise Laser AI setup and approve screening to start.</t>
+          <t>Clarify wildcard use, complete accessible searches, document LILACS/IBECS limitations, finalise Laser AI setup, and confirm the screening start.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -37529,7 +37508,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Setup inputs complete / configuration underway</t>
+          <t>Setup in progress</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -37549,12 +37528,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>The deduplicated RIS/search set (2,053 records), eligibility criteria, protocol information and 35 selected data-extraction items have been received. Questions on the selected items and deduplication were addressed; Nested Knowledge configuration and setup validation are next.</t>
+          <t>Onboarding/training are complete. The team has supplied a deduplicated RIS file with 2,053 records, 35 selected data items, and Study Protocol Info containing inclusion/exclusion/PICOS details. Nested Knowledge configuration can proceed.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Configure Nested Knowledge using the received RIS, criteria, protocol information and 35-item list; obtain final confirmation on the extraction structure; validate the setup before screening starts.</t>
+          <t>Configure the Nested Knowledge project, confirm screening instructions/calibration, and begin abstract screening once setup is complete.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -37586,7 +37565,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41052,7 +41031,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41708,7 +41687,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -46473,7 +46452,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -51114,7 +51093,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -51328,7 +51307,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Data extraction phase; full-text screening outputs are feeding extraction and analysis setup</t>
+          <t>Data extraction remains underway. Blood Pressure Targets is expected to complete the Laser AI data-extraction stage during the week of 2026-08-10. Completed outputs will then be collected for analysis.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -51345,7 +51324,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Data extraction phase; full-text screening outputs are feeding extraction and analysis setup</t>
+          <t>Data extraction remains underway. Blood Pressure Targets is expected to complete the Laser AI data-extraction stage during the week of 2026-08-10. Completed outputs will then be collected for analysis.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -51362,7 +51341,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Continue data extraction and analysis preparation; reconcile full-text decisions and submit extraction outputs/time logs.</t>
+          <t>Complete data extraction, collect extraction outputs and time logs, and send the data-extraction usability survey once the stage is complete.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -51379,7 +51358,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>Week of 2026-08-10</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -51396,7 +51375,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>On track for full-text completion; data extraction setup next dependency</t>
+          <t>Data extraction is underway; completion is now expected during the week of 2026-08-10.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -51452,7 +51431,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56498,7 +56477,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -56712,7 +56691,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete; 10 studies are selected for data extraction. Conventional timing is now available: Emilie—abstract 3h36m10s and full text 12h; Robin—abstract 6h35m and full text 4h12m (corrected from 3h06m). Repeated Laser AI output issues remain: Run 10 appears incomplete and 44 citations in Runs 3–5 remain unevaluated.</t>
+          <t>Abstract and full-text screening are complete in the AI-assisted and conventional workflows. Ten studies are selected for data extraction. Conventional screening time-on-task is now complete; Robin's full-text time was corrected to 4h12. Repeated Laser AI run-validation issues remain provisional.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56729,7 +56708,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete; 10 studies are selected for data extraction. Conventional timing is now available: Emilie—abstract 3h36m10s and full text 12h; Robin—abstract 6h35m and full text 4h12m (corrected from 3h06m). Repeated Laser AI output issues remain: Run 10 appears incomplete and 44 citations in Runs 3–5 remain unevaluated.</t>
+          <t>Abstract and full-text screening are complete in the AI-assisted and conventional workflows. Ten studies are selected for data extraction. Conventional screening time-on-task is now complete; Robin's full-text time was corrected to 4h12. Repeated Laser AI run-validation issues remain provisional.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56746,7 +56725,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Finalise the Nested Knowledge data-extraction workflow; validate and consolidate conventional and AI-assisted time logs; correct Run 10 and resolve the 44 unevaluated citations; complete the interim comparison.</t>
+          <t>Finalise the Nested Knowledge data-extraction workflow; correct Run 10 and resolve the 44 unevaluated citations in Runs 3-5; complete the interim comparison.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56780,7 +56759,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Conventional timing has been received; repeated Laser AI output validation issues remain before final reporting.</t>
+          <t>Repeated Laser AI outputs still require validation before final reporting; conventional screening timing has now been received and updated.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -57239,10 +57218,10 @@
           <t>Setup / Coordination</t>
         </is>
       </c>
-      <c r="B42">
+      <c r="B42" t="n">
         <v>100</v>
       </c>
-      <c r="C42">
+      <c r="C42" t="n">
         <v>100</v>
       </c>
       <c r="D42" t="inlineStr">
@@ -57267,10 +57246,10 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43">
+      <c r="B43" t="n">
         <v>100</v>
       </c>
-      <c r="C43">
+      <c r="C43" t="n">
         <v>100</v>
       </c>
       <c r="D43" t="inlineStr">
@@ -57295,10 +57274,10 @@
           <t>Full-text Screening</t>
         </is>
       </c>
-      <c r="B44">
+      <c r="B44" t="n">
         <v>100</v>
       </c>
-      <c r="C44">
+      <c r="C44" t="n">
         <v>100</v>
       </c>
       <c r="D44" t="inlineStr">

</xml_diff>

<commit_message>
Sync dashboard workbook updates
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -1,21 +1,37 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
-  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
-  <AppVersion>3.1</AppVersion>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
-  <dc:creator xmlns:dc="http://purl.org/dc/elements/1.1/">Krishna Kishore Pandalaneni</dc:creator>
-  <dcterms:created xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-05-27T01:47:03Z</dcterms:created>
-  <dcterms:modified xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-07-30T14:56:52Z</dcterms:modified>
-  <cp:lastModifiedBy>Krishna Kishore Pandalaneni</cp:lastModifiedBy>
-</cp:coreProperties>
-</file>
-
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="9">
@@ -308,7 +324,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\tables\table1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReviewIndexTable" displayName="ReviewIndexTable" ref="A1:N11" headerRowCount="1">
   <tableColumns count="14">
     <tableColumn id="1" name="ReviewID"/>
@@ -330,7 +346,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Workflow_Caffeine_5" displayName="Workflow_Caffeine_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -348,7 +364,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Tasks_Caffeine_6" displayName="Tasks_Caffeine_6" ref="A114:K117" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -367,7 +383,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Comms_Caffeine_7" displayName="Comms_Caffeine_7" ref="A120:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -388,7 +404,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="Critical_Caffeine_8" displayName="Critical_Caffeine_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -403,7 +419,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="Executive_DMARDsRA_1" displayName="Executive_DMARDsRA_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -415,7 +431,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="Milestones_DMARDsRA_2" displayName="Milestones_DMARDsRA_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -429,7 +445,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="Files_DMARDsRA_3" displayName="Files_DMARDsRA_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -444,7 +460,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="Stages_DMARDsRA_4" displayName="Stages_DMARDsRA_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -460,7 +476,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="Workflow_DMARDsRA_5" displayName="Workflow_DMARDsRA_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -478,7 +494,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="Tasks_DMARDsRA_6" displayName="Tasks_DMARDsRA_6" ref="A114:K116" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -497,7 +513,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Workflow63ActionsTable" displayName="Workflow63ActionsTable" ref="A1:G64" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="Workflow Master"/>
@@ -512,7 +528,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="Comms_DMARDsRA_7" displayName="Comms_DMARDsRA_7" ref="A119:M120" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -533,7 +549,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Critical_DMARDsRA_8" displayName="Critical_DMARDsRA_8" ref="A123:G124" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -548,7 +564,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="Executive_BPTargets_1" displayName="Executive_BPTargets_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -560,7 +576,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="Milestones_BPTargets_2" displayName="Milestones_BPTargets_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -574,7 +590,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="Files_BPTargets_3" displayName="Files_BPTargets_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -589,7 +605,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="Stages_BPTargets_4" displayName="Stages_BPTargets_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -605,7 +621,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="Workflow_BPTargets_5" displayName="Workflow_BPTargets_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -623,7 +639,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="Tasks_BPTargets_6" displayName="Tasks_BPTargets_6" ref="A114:K122" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -642,7 +658,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="Comms_BPTargets_7" displayName="Comms_BPTargets_7" ref="A129:M135" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -663,7 +679,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="Critical_BPTargets_8" displayName="Critical_BPTargets_8" ref="A143:G146" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -678,7 +694,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="GlobalPhaseCards" displayName="GlobalPhaseCards" ref="A4:E9" headerRowCount="1">
   <tableColumns count="5">
     <tableColumn id="1" name="PhaseKey"/>
@@ -691,7 +707,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="Executive_Psoriasis_1" displayName="Executive_Psoriasis_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -703,7 +719,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="Milestones_Psoriasis_2" displayName="Milestones_Psoriasis_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -717,7 +733,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="Files_Psoriasis_3" displayName="Files_Psoriasis_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -732,7 +748,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="Stages_Psoriasis_4" displayName="Stages_Psoriasis_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -748,7 +764,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="Workflow_Psoriasis_5" displayName="Workflow_Psoriasis_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -766,7 +782,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="Tasks_Psoriasis_6" displayName="Tasks_Psoriasis_6" ref="A114:K123" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -785,7 +801,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="Comms_Psoriasis_7" displayName="Comms_Psoriasis_7" ref="A129:M132" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -806,7 +822,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="Critical_Psoriasis_8" displayName="Critical_Psoriasis_8" ref="A142:G146" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -821,7 +837,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="Executive_FruitVeg_1" displayName="Executive_FruitVeg_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -833,7 +849,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="Milestones_FruitVeg_2" displayName="Milestones_FruitVeg_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -847,7 +863,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="GlobalResources" displayName="GlobalResources" ref="A13:H18" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="ResourceID"/>
@@ -863,7 +879,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table40.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table40.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="Files_FruitVeg_3" displayName="Files_FruitVeg_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -878,7 +894,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table41.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="Stages_FruitVeg_4" displayName="Stages_FruitVeg_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -894,7 +910,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table42.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="Workflow_FruitVeg_5" displayName="Workflow_FruitVeg_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -912,7 +928,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table43.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="Tasks_FruitVeg_6" displayName="Tasks_FruitVeg_6" ref="A114:K123" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -931,7 +947,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table44.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="Comms_FruitVeg_7" displayName="Comms_FruitVeg_7" ref="A125:M132" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -952,7 +968,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table45.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="Critical_FruitVeg_8" displayName="Critical_FruitVeg_8" ref="A135:G139" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -967,7 +983,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table46.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="Executive_Chlamydia_1" displayName="Executive_Chlamydia_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -979,7 +995,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table47.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="Milestones_Chlamydia_2" displayName="Milestones_Chlamydia_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -993,7 +1009,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table48.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="Files_Chlamydia_3" displayName="Files_Chlamydia_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1008,7 +1024,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table49.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="Stages_Chlamydia_4" displayName="Stages_Chlamydia_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1024,7 +1040,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GlobalUpcomingMeetings" displayName="GlobalUpcomingMeetings" ref="A22:H28" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="MeetingID"/>
@@ -1040,7 +1056,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table50.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table50.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="Workflow_Chlamydia_5" displayName="Workflow_Chlamydia_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1058,7 +1074,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table51.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="Tasks_Chlamydia_6" displayName="Tasks_Chlamydia_6" ref="A114:K118" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1077,7 +1093,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table52.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="Comms_Chlamydia_7" displayName="Comms_Chlamydia_7" ref="A121:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1098,7 +1114,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table53.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="Critical_Chlamydia_8" displayName="Critical_Chlamydia_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1113,7 +1129,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table54.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="Executive_Review5TBD_1" displayName="Executive_Review5TBD_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1125,7 +1141,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table55.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="Milestones_Review5TBD_2" displayName="Milestones_Review5TBD_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1139,7 +1155,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table56.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="Files_Review5TBD_3" displayName="Files_Review5TBD_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1154,7 +1170,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table57.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="Stages_Review5TBD_4" displayName="Stages_Review5TBD_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1170,7 +1186,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table58.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="Workflow_Review5TBD_5" displayName="Workflow_Review5TBD_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1188,7 +1204,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table59.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table59.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="Tasks_Review5TBD_6" displayName="Tasks_Review5TBD_6" ref="A114:K118" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1207,7 +1223,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Executive_Caffeine_1" displayName="Executive_Caffeine_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1219,7 +1235,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table60.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table60.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="Comms_Review5TBD_7" displayName="Comms_Review5TBD_7" ref="A121:M122" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1240,7 +1256,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table61.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="Critical_Review5TBD_8" displayName="Critical_Review5TBD_8" ref="A125:G126" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1255,7 +1271,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table62.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="Executive_Phase2Batch_1" displayName="Executive_Phase2Batch_1" ref="A4:D20" headerRowCount="1">
   <tableColumns count="4">
     <tableColumn id="1" name="Card Field"/>
@@ -1267,7 +1283,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table63.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="Milestones_Phase2Batch_2" displayName="Milestones_Phase2Batch_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1281,7 +1297,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table64.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="64" name="Files_Phase2Batch_3" displayName="Files_Phase2Batch_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1296,7 +1312,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table65.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="65" name="Stages_Phase2Batch_4" displayName="Stages_Phase2Batch_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1312,7 +1328,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table66.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="66" name="Workflow_Phase2Batch_5" displayName="Workflow_Phase2Batch_5" ref="A48:J111" headerRowCount="1">
   <tableColumns count="10">
     <tableColumn id="1" name="ActionOrder"/>
@@ -1330,7 +1346,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table67.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="67" name="Tasks_Phase2Batch_6" displayName="Tasks_Phase2Batch_6" ref="A114:K115" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="TaskID"/>
@@ -1349,7 +1365,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table68.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="68" name="Comms_Phase2Batch_7" displayName="Comms_Phase2Batch_7" ref="A118:M119" headerRowCount="1">
   <tableColumns count="13">
     <tableColumn id="1" name="CommunicationID"/>
@@ -1370,7 +1386,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table69.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table69.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="Critical_Phase2Batch_8" displayName="Critical_Phase2Batch_8" ref="A122:G123" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="CriticalItem"/>
@@ -1385,7 +1401,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Milestones_Caffeine_2" displayName="Milestones_Caffeine_2" ref="A23:F29" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Milestone"/>
@@ -1399,7 +1415,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table70.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table70.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="CandidatePipeline" displayName="CandidatePipeline" ref="A11:J29" headerRowCount="1">
   <tableColumns count="9">
     <tableColumn id="1" name="CandidateID"/>
@@ -1416,7 +1432,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table71.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="71" name="UpcomingMeetingsTable" displayName="UpcomingMeetingsTable" ref="A1:M6" headerRowCount="1">
   <autoFilter ref="A1:M6"/>
   <tableColumns count="13">
@@ -1438,7 +1454,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Files_Caffeine_3" displayName="Files_Caffeine_3" ref="A32:G38" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="FileType"/>
@@ -1453,7 +1469,7 @@
 </table>
 </file>
 
-<file path=xl\tables\table9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Stages_Caffeine_4" displayName="Stages_Caffeine_4" ref="A41:H45" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="StageName"/>
@@ -1469,7 +1485,7 @@
 </table>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
     <a:clrScheme name="ChatGPT">
@@ -1616,39 +1632,7 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="850" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Guide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Index" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_63_Actions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global_Dashboard" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-01 Caffeine" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pilot-02 DMARDs RA" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-01 BP Targets" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-02 Psoriasis" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-03 Fruit &amp; Veg" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-04 Med Adherence" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-05 Vitamin C" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase2-01 Phase 2 Batch" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New_Reviews" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_Master" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2270,7 +2254,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2416,7 +2400,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract screening complete / full-text preparation</t>
+          <t>Full-text screening preparation</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2484,7 +2468,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Laser AI and conventional abstract screening are complete. The AI workflow advanced 15 records to full text. The conventional export and DOIs are still awaited. Before full-text screening, the team must confirm whether 128 records from prior monthly searches should be added to both arms, agree a PDF-sharing method, and finalise amendments to the full-text decision flow.</t>
+          <t>AI-assisted and conventional abstract screening are complete. Fifteen April/May records are moving to full text, and 128 prior-search records will also be added to both arms. Shared-folder access for PDFs is in place.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2501,7 +2485,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Laser AI and conventional abstract screening are complete. The AI workflow advanced 15 records to full text. The conventional export and DOIs are still awaited. Before full-text screening, the team must confirm whether 128 records from prior monthly searches should be added to both arms, agree a PDF-sharing method, and finalise amendments to the full-text decision flow.</t>
+          <t>AI-assisted and conventional abstract screening are complete. Fifteen April/May records are moving to full text, and 128 prior-search records will also be added to both arms. Shared-folder access for PDFs is in place.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2518,7 +2502,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Receive and reconcile the conventional full-text export; confirm inclusion of the 128 prior records and the PDF-sharing method; finalise the full-text decision flow; then start parallel full-text screening.</t>
+          <t>Consolidate the final full-text record set and DOIs, upload PDFs, finalise any full-text decision-flow amendments, and proceed with full-text screening in both arms.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2552,7 +2536,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>The earlier AI-screening pause is resolved. Full-text start now depends on reconciling records and PDFs and confirming the full-text workflow.</t>
+          <t>Abstract screening is complete; the current dependency is consolidating the full-text set and PDFs, including the additional 128 prior-search records.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2608,7 +2592,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2840,12 +2824,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Awaiting PDF-sharing method and reconciled full-text set</t>
+          <t>Shared folder provided; PDFs being collected/uploaded for full-text screening.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2862,12 +2846,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Full-text decision flow under amendment</t>
+          <t>Full-text decision flow and eligibility criteria configured; minor amendments under review.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3006,10 +2990,10 @@
           <t>Setup / Coordination</t>
         </is>
       </c>
-      <c r="B42">
+      <c r="B42" t="n">
         <v>100</v>
       </c>
-      <c r="C42">
+      <c r="C42" t="n">
         <v>100</v>
       </c>
       <c r="D42" t="inlineStr">
@@ -3034,10 +3018,10 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43">
+      <c r="B43" t="n">
         <v>100</v>
       </c>
-      <c r="C43">
+      <c r="C43" t="n">
         <v>100</v>
       </c>
       <c r="D43" t="inlineStr">
@@ -7841,7 +7825,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12596,7 +12580,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12865,7 +12849,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13011,7 +12995,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Setup in progress - search strategy/access issue</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -13079,7 +13063,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The protocol, eligibility criteria and 35 selected data-extraction items are available. Sean is running the accessible Index Medicus searches, while a wildcard inconsistency in the search strategy requires clarification. LILACS and IBECS remain inaccessible and the Native Health Research Database is retired. Screening has not started.</t>
+          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13096,7 +13080,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The protocol, eligibility criteria and 35 selected data-extraction items are available. Sean is running the accessible Index Medicus searches, while a wildcard inconsistency in the search strategy requires clarification. LILACS and IBECS remain inaccessible and the Native Health Research Database is retired. Screening has not started.</t>
+          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13113,7 +13097,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Resolve the wildcard/search-strategy question; complete the accessible searches; document the unavailable databases; consolidate the final RIS set; then finalise Laser AI setup and approve screening to start.</t>
+          <t>Clarify wildcard use, complete accessible searches, document LILACS/IBECS limitations, finalise Laser AI setup, and confirm the screening start.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13147,7 +13131,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Core protocol and data-item inputs are complete. Search-strategy clarification and inaccessible database documentation remain the gating issues.</t>
+          <t>Most setup materials are available; search-strategy clarification and database-access issues remain before screening can start.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -13203,7 +13187,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13300,11 +13284,6 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Setup phase</t>
-        </is>
-      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13315,11 +13294,6 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>fullText</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Screening not yet started</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -13418,7 +13392,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Search/RIS files received; accessible Index Medicus searches underway; LILACS/IBECS unavailable</t>
+          <t>Search/RIS files partly available; additional searches await wildcard clarification; LILACS/IBECS remain inaccessible.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -17665,7 +17639,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22179,7 +22153,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22935,8 +22909,16 @@
       </c>
     </row>
     <row r="30" ht="24" customHeight="1" s="29">
-      <c r="A30" s="17" t="n"/>
-      <c r="B30" s="17" t="n"/>
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>new-19</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong - Oral galactagogues for increasing breast milk production in mothers of non-hospitalised term infants</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
           <t>Shortlisted</t>
@@ -22944,22 +22926,39 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Onboarding confirmed for 2026-08-10 at 3:00 PM Malaysia time; whole team and two Cochrane elective students will attend</t>
-        </is>
-      </c>
-      <c r="E30" s="17" t="n"/>
-      <c r="F30" s="17" t="n"/>
+          <t>Onboarding confirmed for 2026-08-10 at 3:00 PM Malaysia time; full team and two Cochrane elective students will attend.</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Onboarding 2026-08-10; screening/additional data extraction August–September 2026; submission October 2026</t>
+          <t>Onboarding 2026-08-10; tool training and setup to follow.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Initial search completed; 26 new eligible studies; data extraction and ROB 1 completed; INSPECT-SR and ROB 2 underway. Gerald is unavailable for onboarding; other project team members will conduct it.</t>
-        </is>
-      </c>
-      <c r="I30" s="17" t="n"/>
+          <t>Initial onboarding will cover the study and parallel workflow; tool training and setup will be scheduled afterward.</t>
+        </is>
+      </c>
+      <c r="I30" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="24" customHeight="1" s="29">
       <c r="A31" t="inlineStr">
@@ -23384,7 +23383,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26823,13 +26822,13 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="14" customWidth="1" style="29" min="1" max="2"/>
@@ -27336,17 +27335,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Oral Galactagogues Onboarding</t>
+          <t>Oral galactagogues onboarding</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Initial onboarding, study workflow explanation and next-step planning before tool training/setup.</t>
+          <t>Initial onboarding and pilot workflow overview; tool training/setup to follow</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Siew Cheng Foong / full review team / two Cochrane elective students / CESAR project team</t>
+          <t>Siew Cheng Foong / full review team / 2 Cochrane elective students / project team</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -27356,17 +27355,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Later phase / Phase 2</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>Scheduled</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>new-19</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -27394,7 +27388,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31977,7 +31971,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -32123,7 +32117,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup inputs complete / configuration underway</t>
+          <t>Setup in progress</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32191,7 +32185,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The deduplicated RIS/search set (2,053 records), eligibility criteria, protocol information and 35 selected data-extraction items have been received. Questions on the selected items and deduplication were addressed; Nested Knowledge configuration and setup validation are next.</t>
+          <t>Onboarding/training are complete. The team has supplied a deduplicated RIS file with 2,053 records, 35 selected data items, and Study Protocol Info containing inclusion/exclusion/PICOS details. Nested Knowledge configuration can proceed.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32208,7 +32202,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The deduplicated RIS/search set (2,053 records), eligibility criteria, protocol information and 35 selected data-extraction items have been received. Questions on the selected items and deduplication were addressed; Nested Knowledge configuration and setup validation are next.</t>
+          <t>Onboarding/training are complete. The team has supplied a deduplicated RIS file with 2,053 records, 35 selected data items, and Study Protocol Info containing inclusion/exclusion/PICOS details. Nested Knowledge configuration can proceed.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32225,7 +32219,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Configure Nested Knowledge using the received RIS, criteria, protocol information and 35-item list; obtain final confirmation on the extraction structure; validate the setup before screening starts.</t>
+          <t>Configure the Nested Knowledge project, confirm screening instructions/calibration, and begin abstract screening once setup is complete.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32259,7 +32253,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Input collection is complete; tool configuration, final form confirmation and setup validation remain.</t>
+          <t>Key setup inputs are now received; Nested Knowledge configuration is the next step. Full-text PDFs can be assembled later for the full-text stage.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32315,7 +32309,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32380,7 +32374,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Underway</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -32397,7 +32391,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Inputs complete / configuration underway</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -32412,11 +32406,6 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Setup phase</t>
-        </is>
-      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32429,11 +32418,6 @@
           <t>fullText</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Materials/training/configuration pending</t>
-        </is>
-      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32444,11 +32428,6 @@
       <c r="A28" t="inlineStr">
         <is>
           <t>extraction</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Not Started</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -32535,7 +32514,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Deduplicated RIS received (2,053 records)</t>
+          <t>Deduplicated RIS/search file received - 2,053 records.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -32579,7 +32558,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Eligibility criteria received</t>
+          <t>Inclusion/exclusion criteria and PICOS received in Study Protocol Info.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -32601,7 +32580,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>35 selected data items received; questions addressed</t>
+          <t>35 selected data-extraction items received.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -32623,7 +32602,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Protocol information / prior review received</t>
+          <t>Protocol / Study Protocol Info received.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -36603,7 +36582,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -36785,7 +36764,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -37050,17 +37029,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Data extraction phase; full-text screening outputs are feeding extraction and analysis setup</t>
+          <t>Data extraction remains underway. Blood Pressure Targets is expected to complete the Laser AI data-extraction stage during the week of 2026-08-10. Completed outputs will then be collected for analysis.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Continue data extraction and analysis preparation; reconcile full-text decisions and submit extraction outputs/time logs.</t>
+          <t>Complete data extraction, collect extraction outputs and time logs, and send the data-extraction usability survey once the stage is complete.</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>Week of 2026-08-10</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -37122,12 +37101,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete; 10 studies are selected for data extraction. Conventional timing is now available: Emilie—abstract 3h36m10s and full text 12h; Robin—abstract 6h35m and full text 4h12m (corrected from 3h06m). Repeated Laser AI output issues remain: Run 10 appears incomplete and 44 citations in Runs 3–5 remain unevaluated.</t>
+          <t>Abstract and full-text screening are complete in the AI-assisted and conventional workflows. Ten studies are selected for data extraction. Conventional screening time-on-task is now complete; Robin's full-text time was corrected to 4h12. Repeated Laser AI run-validation issues remain provisional.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Finalise the Nested Knowledge data-extraction workflow; validate and consolidate conventional and AI-assisted time logs; correct Run 10 and resolve the 44 unevaluated citations; complete the interim comparison.</t>
+          <t>Finalise the Nested Knowledge data-extraction workflow; correct Run 10 and resolve the 44 unevaluated citations in Runs 3-5; complete the interim comparison.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -37174,7 +37153,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Abstract screening complete / full-text preparation</t>
+          <t>Full-text screening preparation</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -37194,12 +37173,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Laser AI and conventional abstract screening are complete. The AI workflow advanced 15 records to full text. The conventional export and DOIs are still awaited. Before full-text screening, the team must confirm whether 128 records from prior monthly searches should be added to both arms, agree a PDF-sharing method, and finalise amendments to the full-text decision flow.</t>
+          <t>AI-assisted and conventional abstract screening are complete. Fifteen April/May records are moving to full text, and 128 prior-search records will also be added to both arms. Shared-folder access for PDFs is in place.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Receive and reconcile the conventional full-text export; confirm inclusion of the 128 prior records and the PDF-sharing method; finalise the full-text decision flow; then start parallel full-text screening.</t>
+          <t>Consolidate the final full-text record set and DOIs, upload PDFs, finalise any full-text decision-flow amendments, and proceed with full-text screening in both arms.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -37313,7 +37292,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Setup phase</t>
+          <t>Setup in progress - search strategy/access issue</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -37333,12 +37312,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>The protocol, eligibility criteria and 35 selected data-extraction items are available. Sean is running the accessible Index Medicus searches, while a wildcard inconsistency in the search strategy requires clarification. LILACS and IBECS remain inaccessible and the Native Health Research Database is retired. Screening has not started.</t>
+          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Resolve the wildcard/search-strategy question; complete the accessible searches; document the unavailable databases; consolidate the final RIS set; then finalise Laser AI setup and approve screening to start.</t>
+          <t>Clarify wildcard use, complete accessible searches, document LILACS/IBECS limitations, finalise Laser AI setup, and confirm the screening start.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -37529,7 +37508,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Setup inputs complete / configuration underway</t>
+          <t>Setup in progress</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -37549,12 +37528,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>The deduplicated RIS/search set (2,053 records), eligibility criteria, protocol information and 35 selected data-extraction items have been received. Questions on the selected items and deduplication were addressed; Nested Knowledge configuration and setup validation are next.</t>
+          <t>Onboarding/training are complete. The team has supplied a deduplicated RIS file with 2,053 records, 35 selected data items, and Study Protocol Info containing inclusion/exclusion/PICOS details. Nested Knowledge configuration can proceed.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Configure Nested Knowledge using the received RIS, criteria, protocol information and 35-item list; obtain final confirmation on the extraction structure; validate the setup before screening starts.</t>
+          <t>Configure the Nested Knowledge project, confirm screening instructions/calibration, and begin abstract screening once setup is complete.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -37586,7 +37565,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41052,7 +41031,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41708,7 +41687,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -46473,7 +46452,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -51114,7 +51093,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -51328,7 +51307,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Data extraction phase; full-text screening outputs are feeding extraction and analysis setup</t>
+          <t>Data extraction remains underway. Blood Pressure Targets is expected to complete the Laser AI data-extraction stage during the week of 2026-08-10. Completed outputs will then be collected for analysis.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -51345,7 +51324,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Data extraction phase; full-text screening outputs are feeding extraction and analysis setup</t>
+          <t>Data extraction remains underway. Blood Pressure Targets is expected to complete the Laser AI data-extraction stage during the week of 2026-08-10. Completed outputs will then be collected for analysis.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -51362,7 +51341,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Continue data extraction and analysis preparation; reconcile full-text decisions and submit extraction outputs/time logs.</t>
+          <t>Complete data extraction, collect extraction outputs and time logs, and send the data-extraction usability survey once the stage is complete.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -51379,7 +51358,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>Week of 2026-08-10</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -51396,7 +51375,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>On track for full-text completion; data extraction setup next dependency</t>
+          <t>Data extraction is underway; completion is now expected during the week of 2026-08-10.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -51452,7 +51431,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56498,7 +56477,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -56712,7 +56691,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete; 10 studies are selected for data extraction. Conventional timing is now available: Emilie—abstract 3h36m10s and full text 12h; Robin—abstract 6h35m and full text 4h12m (corrected from 3h06m). Repeated Laser AI output issues remain: Run 10 appears incomplete and 44 citations in Runs 3–5 remain unevaluated.</t>
+          <t>Abstract and full-text screening are complete in the AI-assisted and conventional workflows. Ten studies are selected for data extraction. Conventional screening time-on-task is now complete; Robin's full-text time was corrected to 4h12. Repeated Laser AI run-validation issues remain provisional.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56729,7 +56708,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nested Knowledge abstract screening and AI-assisted full-text screening are complete; 10 studies are selected for data extraction. Conventional timing is now available: Emilie—abstract 3h36m10s and full text 12h; Robin—abstract 6h35m and full text 4h12m (corrected from 3h06m). Repeated Laser AI output issues remain: Run 10 appears incomplete and 44 citations in Runs 3–5 remain unevaluated.</t>
+          <t>Abstract and full-text screening are complete in the AI-assisted and conventional workflows. Ten studies are selected for data extraction. Conventional screening time-on-task is now complete; Robin's full-text time was corrected to 4h12. Repeated Laser AI run-validation issues remain provisional.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56746,7 +56725,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Finalise the Nested Knowledge data-extraction workflow; validate and consolidate conventional and AI-assisted time logs; correct Run 10 and resolve the 44 unevaluated citations; complete the interim comparison.</t>
+          <t>Finalise the Nested Knowledge data-extraction workflow; correct Run 10 and resolve the 44 unevaluated citations in Runs 3-5; complete the interim comparison.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56780,7 +56759,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Conventional timing has been received; repeated Laser AI output validation issues remain before final reporting.</t>
+          <t>Repeated Laser AI outputs still require validation before final reporting; conventional screening timing has now been received and updated.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -57239,10 +57218,10 @@
           <t>Setup / Coordination</t>
         </is>
       </c>
-      <c r="B42">
+      <c r="B42" t="n">
         <v>100</v>
       </c>
-      <c r="C42">
+      <c r="C42" t="n">
         <v>100</v>
       </c>
       <c r="D42" t="inlineStr">
@@ -57267,10 +57246,10 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43">
+      <c r="B43" t="n">
         <v>100</v>
       </c>
-      <c r="C43">
+      <c r="C43" t="n">
         <v>100</v>
       </c>
       <c r="D43" t="inlineStr">
@@ -57295,10 +57274,10 @@
           <t>Full-text Screening</t>
         </is>
       </c>
-      <c r="B44">
+      <c r="B44" t="n">
         <v>100</v>
       </c>
-      <c r="C44">
+      <c r="C44" t="n">
         <v>100</v>
       </c>
       <c r="D44" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboard last updated date
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2592,7 +2592,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13187,7 +13187,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27726,7 +27726,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32309,7 +32309,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -51431,7 +51431,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56815,7 +56815,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">

</xml_diff>

<commit_message>
Sync dashboard last updated date
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2592,7 +2592,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13187,7 +13187,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27726,7 +27726,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32309,7 +32309,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -51431,7 +51431,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56815,7 +56815,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">

</xml_diff>

<commit_message>
Add Oral Galactagogues review
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -25,6 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-08 Oral Galactagogues" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -22921,17 +22922,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Shortlisted</t>
+          <t>Converted to full sheet</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Onboarding confirmed for 2026-08-10 at 3:00 PM Malaysia time; full team and two Cochrane elective students will attend.</t>
+          <t>Converted to phase1-08 Oral Galactagogues; onboarding confirmed for 2026-08-10.</t>
         </is>
       </c>
       <c r="E30" s="17" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="F30" s="17" t="inlineStr">
@@ -22941,22 +22942,22 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Onboarding 2026-08-10; tool training and setup to follow.</t>
+          <t>Onboarding complete/confirmed; tool training and setup to follow.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Initial onboarding will cover the study and parallel workflow; tool training and setup will be scheduled afterward.</t>
+          <t>Converted to dashboard review phase1-08.</t>
         </is>
       </c>
       <c r="I30" s="17" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -27355,12 +27356,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>phase1-08</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -36764,13 +36770,4602 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M125"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <cols>
+    <col width="14" customWidth="1" style="29" min="1" max="1"/>
+    <col width="16" customWidth="1" style="29" min="2" max="2"/>
+    <col width="28" customWidth="1" style="29" min="3" max="3"/>
+    <col width="18" customWidth="1" style="29" min="4" max="4"/>
+    <col width="48" customWidth="1" style="29" min="5" max="5"/>
+    <col width="28" customWidth="1" style="29" min="6" max="6"/>
+    <col width="24" customWidth="1" style="29" min="7" max="8"/>
+    <col width="18" customWidth="1" style="29" min="9" max="10"/>
+    <col width="16" customWidth="1" style="29" min="11" max="11"/>
+    <col width="30" customWidth="1" style="29" min="12" max="12"/>
+    <col width="12" customWidth="1" style="29" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1" s="29">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>phase1-08 Oral Galactagogues | Dashboard Content Sheet</t>
+        </is>
+      </c>
+      <c r="K1" s="18" t="n"/>
+      <c r="L1" s="18" t="n"/>
+      <c r="M1" s="18" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Executive Review Card</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Card Field</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ReviewID</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>phase1-08</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ShortName</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Oral Galactagogues</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ReviewTitle</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Oral galactagogues (natural therapies or drugs) for increasing breast milk production in mothers of non-hospitalised term infants</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Onboarding confirmed</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tool</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CurrentStage</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Onboarding is confirmed for 2026-08-10 at 3:00 PM Malaysia time with the full review team and two Cochrane elective students. Tool training and setup will follow after onboarding.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CurrentUpdate</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Onboarding is confirmed for 2026-08-10 at 3:00 PM Malaysia time with the full review team and two Cochrane elective students. Tool training and setup will follow after onboarding.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>NextAction</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Complete onboarding, confirm tool allocation and team split, then schedule tool training and setup.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TargetDate</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>New Phase 1 review added from the onboarding pipeline; setup has not started yet.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DisplayInHTML</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Set to No if review should not appear in dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LastUpdated</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard Milestones</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="5" t="n"/>
+      <c r="I22" s="5" t="n"/>
+      <c r="J22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>TargetDate</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>onboarding</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>setup</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>fullText</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>analysis</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Files Displayed in Review Detail</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="5" t="n"/>
+      <c r="J31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>FileType</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G32" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>RIS</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>PDFs</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Criteria</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Extraction</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Time Log</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Stage Progress: Visual Tracker / Operations</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="5" t="n"/>
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="5" t="n"/>
+      <c r="G40" s="5" t="n"/>
+      <c r="H40" s="5" t="n"/>
+      <c r="I40" s="5" t="n"/>
+      <c r="J40" s="5" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>StageName</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>HumanProgress</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>AIProgress</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>TargetDate</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H41" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Setup / Coordination</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Onboarding confirmed; tool allocation and setup to follow.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Abstract Screening</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Full-text Screening</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Data Extraction / Analysis</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Review Workflow Status: Full 63 Actions</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n"/>
+      <c r="C47" s="5" t="n"/>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="5" t="n"/>
+      <c r="F47" s="5" t="n"/>
+      <c r="G47" s="5" t="n"/>
+      <c r="H47" s="5" t="n"/>
+      <c r="I47" s="5" t="n"/>
+      <c r="J47" s="5" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>ActionOrder</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>WorkflowStepID</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>WorkflowGroup</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>ShortName</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>Responsible</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>DependsOn</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>Blocks</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="K48" s="10" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="L48" s="10" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="M48" s="10" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>w01</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D49" s="18" t="inlineStr">
+        <is>
+          <t>Review selected</t>
+        </is>
+      </c>
+      <c r="E49" s="18" t="inlineStr">
+        <is>
+          <t>Selection of review - core team</t>
+        </is>
+      </c>
+      <c r="F49" s="18" t="inlineStr">
+        <is>
+          <t>Core Team</t>
+        </is>
+      </c>
+      <c r="G49" s="18" t="n"/>
+      <c r="H49" s="18" t="inlineStr">
+        <is>
+          <t>w02</t>
+        </is>
+      </c>
+      <c r="I49" s="18" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J49" s="18" t="inlineStr"/>
+      <c r="K49" s="18" t="inlineStr"/>
+      <c r="L49" s="18" t="n"/>
+      <c r="M49" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" s="18" t="inlineStr">
+        <is>
+          <t>w02</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D50" s="18" t="inlineStr">
+        <is>
+          <t>PM confirmation</t>
+        </is>
+      </c>
+      <c r="E50" s="18" t="inlineStr">
+        <is>
+          <t>Selection of review - project manager confirmation</t>
+        </is>
+      </c>
+      <c r="F50" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G50" s="18" t="inlineStr">
+        <is>
+          <t>w01</t>
+        </is>
+      </c>
+      <c r="H50" s="18" t="inlineStr">
+        <is>
+          <t>w03</t>
+        </is>
+      </c>
+      <c r="I50" s="18" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J50" s="18" t="inlineStr"/>
+      <c r="K50" s="18" t="inlineStr"/>
+      <c r="L50" s="18" t="n"/>
+      <c r="M50" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>w03</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D51" s="18" t="inlineStr">
+        <is>
+          <t>Final confirmation</t>
+        </is>
+      </c>
+      <c r="E51" s="18" t="inlineStr">
+        <is>
+          <t>Selection of review - final confirmation</t>
+        </is>
+      </c>
+      <c r="F51" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G51" s="18" t="inlineStr">
+        <is>
+          <t>w02</t>
+        </is>
+      </c>
+      <c r="H51" s="18" t="inlineStr">
+        <is>
+          <t>w04</t>
+        </is>
+      </c>
+      <c r="I51" s="18" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J51" s="18" t="inlineStr"/>
+      <c r="K51" s="18" t="inlineStr"/>
+      <c r="L51" s="18" t="n"/>
+      <c r="M51" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>w04</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>Tool allocated</t>
+        </is>
+      </c>
+      <c r="E52" s="18" t="inlineStr">
+        <is>
+          <t>Confirm allocated AI tool for review</t>
+        </is>
+      </c>
+      <c r="F52" s="18" t="inlineStr">
+        <is>
+          <t>Core Team</t>
+        </is>
+      </c>
+      <c r="G52" s="18" t="inlineStr">
+        <is>
+          <t>w03</t>
+        </is>
+      </c>
+      <c r="H52" s="18" t="inlineStr">
+        <is>
+          <t>w05,w07,w15,w30,w45</t>
+        </is>
+      </c>
+      <c r="I52" s="18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J52" s="18" t="inlineStr"/>
+      <c r="K52" s="18" t="inlineStr"/>
+      <c r="L52" s="18" t="inlineStr">
+        <is>
+          <t>Tool allocation to be confirmed after onboarding.</t>
+        </is>
+      </c>
+      <c r="M52" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="28" customHeight="1" s="29">
+      <c r="A53" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B53" s="18" t="inlineStr">
+        <is>
+          <t>w05</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D53" s="18" t="inlineStr">
+        <is>
+          <t>Team split</t>
+        </is>
+      </c>
+      <c r="E53" s="18" t="inlineStr">
+        <is>
+          <t>Confirm review team split: Human workflow and AI-assisted workflow</t>
+        </is>
+      </c>
+      <c r="F53" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Review Team</t>
+        </is>
+      </c>
+      <c r="G53" s="18" t="inlineStr">
+        <is>
+          <t>w04</t>
+        </is>
+      </c>
+      <c r="H53" s="18" t="inlineStr">
+        <is>
+          <t>w08,w09,w17,w32,w47</t>
+        </is>
+      </c>
+      <c r="I53" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J53" s="18" t="inlineStr"/>
+      <c r="K53" s="18" t="inlineStr"/>
+      <c r="L53" s="18" t="inlineStr"/>
+      <c r="M53" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B54" s="18" t="inlineStr">
+        <is>
+          <t>w06</t>
+        </is>
+      </c>
+      <c r="C54" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D54" s="18" t="inlineStr">
+        <is>
+          <t>Folder access</t>
+        </is>
+      </c>
+      <c r="E54" s="18" t="inlineStr">
+        <is>
+          <t>Confirm SharePoint/folder access for review team</t>
+        </is>
+      </c>
+      <c r="F54" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Review Team</t>
+        </is>
+      </c>
+      <c r="G54" s="18" t="inlineStr">
+        <is>
+          <t>w03</t>
+        </is>
+      </c>
+      <c r="H54" s="18" t="inlineStr">
+        <is>
+          <t>w10,w11,w12</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J54" s="18" t="inlineStr"/>
+      <c r="K54" s="18" t="inlineStr"/>
+      <c r="M54" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="28" customHeight="1" s="29">
+      <c r="A55" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B55" s="18" t="inlineStr">
+        <is>
+          <t>w07</t>
+        </is>
+      </c>
+      <c r="C55" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D55" s="18" t="inlineStr">
+        <is>
+          <t>Tool access</t>
+        </is>
+      </c>
+      <c r="E55" s="18" t="inlineStr">
+        <is>
+          <t>Confirm AI tool access for allocated users</t>
+        </is>
+      </c>
+      <c r="F55" s="18" t="inlineStr">
+        <is>
+          <t>Response Team / Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G55" s="18" t="inlineStr">
+        <is>
+          <t>w04</t>
+        </is>
+      </c>
+      <c r="H55" s="18" t="inlineStr">
+        <is>
+          <t>w15,w30,w45</t>
+        </is>
+      </c>
+      <c r="I55" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J55" s="18" t="inlineStr"/>
+      <c r="K55" s="18" t="inlineStr"/>
+      <c r="L55" s="18" t="inlineStr"/>
+      <c r="M55" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B56" s="18" t="inlineStr">
+        <is>
+          <t>w08</t>
+        </is>
+      </c>
+      <c r="C56" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D56" s="18" t="inlineStr">
+        <is>
+          <t>Blinding shared</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="inlineStr">
+        <is>
+          <t>Confirm blinding instructions shared with review teams</t>
+        </is>
+      </c>
+      <c r="F56" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Sean</t>
+        </is>
+      </c>
+      <c r="G56" s="18" t="inlineStr">
+        <is>
+          <t>w05</t>
+        </is>
+      </c>
+      <c r="H56" s="18" t="inlineStr">
+        <is>
+          <t>w17,w18,w32,w33,w47,w48</t>
+        </is>
+      </c>
+      <c r="I56" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J56" s="18" t="inlineStr"/>
+      <c r="K56" s="18" t="inlineStr"/>
+      <c r="L56" s="18" t="inlineStr"/>
+      <c r="M56" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
+          <t>w09</t>
+        </is>
+      </c>
+      <c r="C57" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D57" s="18" t="inlineStr">
+        <is>
+          <t>Time tracking</t>
+        </is>
+      </c>
+      <c r="E57" s="18" t="inlineStr">
+        <is>
+          <t>Confirm Clockify or alternate time-tracking setup</t>
+        </is>
+      </c>
+      <c r="F57" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G57" s="18" t="inlineStr">
+        <is>
+          <t>w05</t>
+        </is>
+      </c>
+      <c r="H57" s="18" t="inlineStr">
+        <is>
+          <t>w17,w18,w32,w33,w47,w48</t>
+        </is>
+      </c>
+      <c r="I57" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J57" s="18" t="inlineStr"/>
+      <c r="K57" s="18" t="inlineStr"/>
+      <c r="L57" s="18" t="inlineStr"/>
+      <c r="M57" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="28" customHeight="1" s="29">
+      <c r="A58" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="B58" s="18" t="inlineStr">
+        <is>
+          <t>w10</t>
+        </is>
+      </c>
+      <c r="C58" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="inlineStr">
+        <is>
+          <t>RIS files</t>
+        </is>
+      </c>
+      <c r="E58" s="18" t="inlineStr">
+        <is>
+          <t>Review team to share RIS files with setup team</t>
+        </is>
+      </c>
+      <c r="F58" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G58" s="18" t="inlineStr">
+        <is>
+          <t>w06</t>
+        </is>
+      </c>
+      <c r="H58" s="18" t="inlineStr">
+        <is>
+          <t>w15</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J58" s="18" t="inlineStr"/>
+      <c r="K58" s="18" t="inlineStr"/>
+      <c r="M58" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="28" customHeight="1" s="29">
+      <c r="A59" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>w11</t>
+        </is>
+      </c>
+      <c r="C59" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D59" s="18" t="inlineStr">
+        <is>
+          <t>Protocol &amp; criteria</t>
+        </is>
+      </c>
+      <c r="E59" s="18" t="inlineStr">
+        <is>
+          <t>Review team to share protocol and inclusion/exclusion criteria</t>
+        </is>
+      </c>
+      <c r="F59" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G59" s="18" t="inlineStr">
+        <is>
+          <t>w06</t>
+        </is>
+      </c>
+      <c r="H59" s="18" t="inlineStr">
+        <is>
+          <t>w12,w15,w29</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J59" s="18" t="inlineStr"/>
+      <c r="K59" s="18" t="inlineStr"/>
+      <c r="M59" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="28" customHeight="1" s="29">
+      <c r="A60" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="B60" s="18" t="inlineStr">
+        <is>
+          <t>w12</t>
+        </is>
+      </c>
+      <c r="C60" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D60" s="18" t="inlineStr">
+        <is>
+          <t>Data items</t>
+        </is>
+      </c>
+      <c r="E60" s="18" t="inlineStr">
+        <is>
+          <t>Finalise data items with Sean</t>
+        </is>
+      </c>
+      <c r="F60" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Sean</t>
+        </is>
+      </c>
+      <c r="G60" s="18" t="inlineStr">
+        <is>
+          <t>w11</t>
+        </is>
+      </c>
+      <c r="H60" s="18" t="inlineStr">
+        <is>
+          <t>w13,w14,w43,w44</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J60" s="18" t="inlineStr"/>
+      <c r="K60" s="18" t="inlineStr"/>
+      <c r="M60" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="28" customHeight="1" s="29">
+      <c r="A61" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>w13</t>
+        </is>
+      </c>
+      <c r="C61" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>Comparable DE</t>
+        </is>
+      </c>
+      <c r="E61" s="18" t="inlineStr">
+        <is>
+          <t>Confirm data extraction structure is comparable between Human and AI workflows</t>
+        </is>
+      </c>
+      <c r="F61" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Sean</t>
+        </is>
+      </c>
+      <c r="G61" s="18" t="inlineStr">
+        <is>
+          <t>w12</t>
+        </is>
+      </c>
+      <c r="H61" s="18" t="inlineStr">
+        <is>
+          <t>w14,w44</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J61" s="18" t="inlineStr"/>
+      <c r="K61" s="18" t="inlineStr"/>
+      <c r="M61" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="28" customHeight="1" s="29">
+      <c r="A62" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="B62" s="18" t="inlineStr">
+        <is>
+          <t>w14</t>
+        </is>
+      </c>
+      <c r="C62" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>Sean approval</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="inlineStr">
+        <is>
+          <t>Confirm extraction form/template is approved by Sean</t>
+        </is>
+      </c>
+      <c r="F62" s="18" t="inlineStr">
+        <is>
+          <t>Sean</t>
+        </is>
+      </c>
+      <c r="G62" s="18" t="inlineStr">
+        <is>
+          <t>w13</t>
+        </is>
+      </c>
+      <c r="H62" s="18" t="inlineStr">
+        <is>
+          <t>w43,w44,w45</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J62" s="18" t="inlineStr"/>
+      <c r="K62" s="18" t="inlineStr"/>
+      <c r="M62" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="28" customHeight="1" s="29">
+      <c r="A63" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t>w15</t>
+        </is>
+      </c>
+      <c r="C63" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D63" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup</t>
+        </is>
+      </c>
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup - allocated AI tool for abstract screening</t>
+        </is>
+      </c>
+      <c r="F63" s="18" t="inlineStr">
+        <is>
+          <t>Response Team / Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G63" s="18" t="inlineStr">
+        <is>
+          <t>w04,w07,w10,w11</t>
+        </is>
+      </c>
+      <c r="H63" s="18" t="inlineStr">
+        <is>
+          <t>w16</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J63" s="18" t="inlineStr"/>
+      <c r="K63" s="18" t="inlineStr"/>
+      <c r="M63" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="28" customHeight="1" s="29">
+      <c r="A64" s="18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B64" s="18" t="inlineStr">
+        <is>
+          <t>w16</t>
+        </is>
+      </c>
+      <c r="C64" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D64" s="18" t="inlineStr">
+        <is>
+          <t>Setup validated</t>
+        </is>
+      </c>
+      <c r="E64" s="18" t="inlineStr">
+        <is>
+          <t>Review team validates abstract screening setup before starting</t>
+        </is>
+      </c>
+      <c r="F64" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G64" s="18" t="inlineStr">
+        <is>
+          <t>w15</t>
+        </is>
+      </c>
+      <c r="H64" s="18" t="inlineStr">
+        <is>
+          <t>w17,w18</t>
+        </is>
+      </c>
+      <c r="I64" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J64" s="18" t="inlineStr"/>
+      <c r="K64" s="18" t="inlineStr"/>
+      <c r="L64" s="18" t="inlineStr"/>
+      <c r="M64" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B65" s="18" t="inlineStr">
+        <is>
+          <t>w17</t>
+        </is>
+      </c>
+      <c r="C65" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D65" s="18" t="inlineStr">
+        <is>
+          <t>Human screening</t>
+        </is>
+      </c>
+      <c r="E65" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening - Human workflow</t>
+        </is>
+      </c>
+      <c r="F65" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G65" s="18" t="inlineStr">
+        <is>
+          <t>w05,w08,w09,w16</t>
+        </is>
+      </c>
+      <c r="H65" s="18" t="inlineStr">
+        <is>
+          <t>w21,w24,w25</t>
+        </is>
+      </c>
+      <c r="I65" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J65" s="18" t="inlineStr"/>
+      <c r="K65" s="18" t="inlineStr"/>
+      <c r="L65" s="18" t="inlineStr"/>
+      <c r="M65" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="18" t="n">
+        <v>18</v>
+      </c>
+      <c r="B66" s="18" t="inlineStr">
+        <is>
+          <t>w18</t>
+        </is>
+      </c>
+      <c r="C66" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D66" s="18" t="inlineStr">
+        <is>
+          <t>AI screening</t>
+        </is>
+      </c>
+      <c r="E66" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening - allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F66" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G66" s="18" t="inlineStr">
+        <is>
+          <t>w07,w08,w09,w16</t>
+        </is>
+      </c>
+      <c r="H66" s="18" t="inlineStr">
+        <is>
+          <t>w19,w21,w24,w25</t>
+        </is>
+      </c>
+      <c r="I66" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J66" s="18" t="inlineStr"/>
+      <c r="K66" s="18" t="inlineStr"/>
+      <c r="L66" s="18" t="inlineStr"/>
+      <c r="M66" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="18" t="n">
+        <v>19</v>
+      </c>
+      <c r="B67" s="18" t="inlineStr">
+        <is>
+          <t>w19</t>
+        </is>
+      </c>
+      <c r="C67" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D67" s="18" t="inlineStr">
+        <is>
+          <t>Export AI output</t>
+        </is>
+      </c>
+      <c r="E67" s="18" t="inlineStr">
+        <is>
+          <t>Export abstract screening output from allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F67" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G67" s="18" t="inlineStr">
+        <is>
+          <t>w18</t>
+        </is>
+      </c>
+      <c r="H67" s="18" t="inlineStr">
+        <is>
+          <t>w20</t>
+        </is>
+      </c>
+      <c r="I67" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J67" s="18" t="inlineStr"/>
+      <c r="K67" s="18" t="inlineStr"/>
+      <c r="L67" s="18" t="inlineStr"/>
+      <c r="M67" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="B68" s="18" t="inlineStr">
+        <is>
+          <t>w20</t>
+        </is>
+      </c>
+      <c r="C68" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D68" s="18" t="inlineStr">
+        <is>
+          <t>Share output</t>
+        </is>
+      </c>
+      <c r="E68" s="18" t="inlineStr">
+        <is>
+          <t>Share abstract screening output with Sean / data manager</t>
+        </is>
+      </c>
+      <c r="F68" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Data Manager</t>
+        </is>
+      </c>
+      <c r="G68" s="18" t="inlineStr">
+        <is>
+          <t>w19</t>
+        </is>
+      </c>
+      <c r="H68" s="18" t="inlineStr">
+        <is>
+          <t>w24,w25</t>
+        </is>
+      </c>
+      <c r="I68" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J68" s="18" t="inlineStr"/>
+      <c r="K68" s="18" t="inlineStr"/>
+      <c r="L68" s="18" t="inlineStr"/>
+      <c r="M68" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="18" t="n">
+        <v>21</v>
+      </c>
+      <c r="B69" s="18" t="inlineStr">
+        <is>
+          <t>w21</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D69" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent</t>
+        </is>
+      </c>
+      <c r="E69" s="18" t="inlineStr">
+        <is>
+          <t>Share usability survey on abstract screening experience</t>
+        </is>
+      </c>
+      <c r="F69" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G69" s="18" t="inlineStr">
+        <is>
+          <t>w17,w18</t>
+        </is>
+      </c>
+      <c r="H69" s="18" t="inlineStr">
+        <is>
+          <t>w22</t>
+        </is>
+      </c>
+      <c r="I69" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J69" s="18" t="inlineStr"/>
+      <c r="K69" s="18" t="inlineStr"/>
+      <c r="L69" s="18" t="inlineStr"/>
+      <c r="M69" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="18" t="n">
+        <v>22</v>
+      </c>
+      <c r="B70" s="18" t="inlineStr">
+        <is>
+          <t>w22</t>
+        </is>
+      </c>
+      <c r="C70" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D70" s="18" t="inlineStr">
+        <is>
+          <t>Survey submitted</t>
+        </is>
+      </c>
+      <c r="E70" s="18" t="inlineStr">
+        <is>
+          <t>Submit usability survey on abstract screening experience</t>
+        </is>
+      </c>
+      <c r="F70" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G70" s="18" t="inlineStr">
+        <is>
+          <t>w21</t>
+        </is>
+      </c>
+      <c r="H70" s="18" t="inlineStr">
+        <is>
+          <t>w23</t>
+        </is>
+      </c>
+      <c r="I70" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J70" s="18" t="inlineStr"/>
+      <c r="K70" s="18" t="inlineStr"/>
+      <c r="L70" s="18" t="inlineStr"/>
+      <c r="M70" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="28" customHeight="1" s="29">
+      <c r="A71" s="18" t="n">
+        <v>23</v>
+      </c>
+      <c r="B71" s="18" t="inlineStr">
+        <is>
+          <t>w23</t>
+        </is>
+      </c>
+      <c r="C71" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
+        <is>
+          <t>Survey received</t>
+        </is>
+      </c>
+      <c r="E71" s="18" t="inlineStr">
+        <is>
+          <t>Confirm usability survey responses received for abstract screening</t>
+        </is>
+      </c>
+      <c r="F71" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G71" s="18" t="inlineStr">
+        <is>
+          <t>w22</t>
+        </is>
+      </c>
+      <c r="H71" s="18" t="inlineStr">
+        <is>
+          <t>w24</t>
+        </is>
+      </c>
+      <c r="I71" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J71" s="18" t="inlineStr"/>
+      <c r="K71" s="18" t="inlineStr"/>
+      <c r="L71" s="18" t="inlineStr"/>
+      <c r="M71" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="28" customHeight="1" s="29">
+      <c r="A72" s="18" t="n">
+        <v>24</v>
+      </c>
+      <c r="B72" s="18" t="inlineStr">
+        <is>
+          <t>w24</t>
+        </is>
+      </c>
+      <c r="C72" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
+        <is>
+          <t>Quality check</t>
+        </is>
+      </c>
+      <c r="E72" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness and quality check before abstract screening adjudication</t>
+        </is>
+      </c>
+      <c r="F72" s="18" t="inlineStr">
+        <is>
+          <t>Data Manager / Sean</t>
+        </is>
+      </c>
+      <c r="G72" s="18" t="inlineStr">
+        <is>
+          <t>w20,w23</t>
+        </is>
+      </c>
+      <c r="H72" s="18" t="inlineStr">
+        <is>
+          <t>w25</t>
+        </is>
+      </c>
+      <c r="I72" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J72" s="18" t="inlineStr"/>
+      <c r="K72" s="18" t="inlineStr"/>
+      <c r="L72" s="18" t="inlineStr"/>
+      <c r="M72" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="B73" s="18" t="inlineStr">
+        <is>
+          <t>w25</t>
+        </is>
+      </c>
+      <c r="C73" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
+        <is>
+          <t>Abstract adjudication</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication panel after abstract screening</t>
+        </is>
+      </c>
+      <c r="F73" s="18" t="inlineStr">
+        <is>
+          <t>Sean and Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="G73" s="18" t="inlineStr">
+        <is>
+          <t>w24</t>
+        </is>
+      </c>
+      <c r="H73" s="18" t="inlineStr">
+        <is>
+          <t>w26,w28,w30</t>
+        </is>
+      </c>
+      <c r="I73" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J73" s="18" t="inlineStr"/>
+      <c r="K73" s="18" t="inlineStr"/>
+      <c r="L73" s="18" t="inlineStr"/>
+      <c r="M73" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="18" t="n">
+        <v>26</v>
+      </c>
+      <c r="B74" s="18" t="inlineStr">
+        <is>
+          <t>w26</t>
+        </is>
+      </c>
+      <c r="C74" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D74" s="18" t="inlineStr">
+        <is>
+          <t>PDFs received</t>
+        </is>
+      </c>
+      <c r="E74" s="18" t="inlineStr">
+        <is>
+          <t>Review team to share PDF files with setup team</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G74" s="18" t="inlineStr">
+        <is>
+          <t>w25</t>
+        </is>
+      </c>
+      <c r="H74" s="18" t="inlineStr">
+        <is>
+          <t>w27,w29</t>
+        </is>
+      </c>
+      <c r="I74" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J74" s="18" t="inlineStr"/>
+      <c r="K74" s="18" t="inlineStr"/>
+      <c r="L74" s="18" t="inlineStr"/>
+      <c r="M74" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="18" t="n">
+        <v>27</v>
+      </c>
+      <c r="B75" s="18" t="inlineStr">
+        <is>
+          <t>w27</t>
+        </is>
+      </c>
+      <c r="C75" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D75" s="18" t="inlineStr">
+        <is>
+          <t>PDF issues logged</t>
+        </is>
+      </c>
+      <c r="E75" s="18" t="inlineStr">
+        <is>
+          <t>Confirm unavailable PDFs or access issues are logged</t>
+        </is>
+      </c>
+      <c r="F75" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Krishna</t>
+        </is>
+      </c>
+      <c r="G75" s="18" t="inlineStr">
+        <is>
+          <t>w26</t>
+        </is>
+      </c>
+      <c r="H75" s="18" t="inlineStr">
+        <is>
+          <t>w29</t>
+        </is>
+      </c>
+      <c r="I75" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J75" s="18" t="inlineStr"/>
+      <c r="K75" s="18" t="inlineStr"/>
+      <c r="L75" s="18" t="inlineStr"/>
+      <c r="M75" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="28" customHeight="1" s="29">
+      <c r="A76" s="18" t="n">
+        <v>28</v>
+      </c>
+      <c r="B76" s="18" t="inlineStr">
+        <is>
+          <t>w28</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D76" s="18" t="inlineStr">
+        <is>
+          <t>Check-in meeting</t>
+        </is>
+      </c>
+      <c r="E76" s="18" t="inlineStr">
+        <is>
+          <t>Meeting with Gerald, Amin, Susan, and optional review team members</t>
+        </is>
+      </c>
+      <c r="F76" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G76" s="18" t="inlineStr">
+        <is>
+          <t>w25</t>
+        </is>
+      </c>
+      <c r="H76" s="18" t="inlineStr">
+        <is>
+          <t>w29</t>
+        </is>
+      </c>
+      <c r="I76" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J76" s="18" t="inlineStr"/>
+      <c r="K76" s="18" t="inlineStr"/>
+      <c r="L76" s="18" t="inlineStr"/>
+      <c r="M76" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="18" t="n">
+        <v>29</v>
+      </c>
+      <c r="B77" s="18" t="inlineStr">
+        <is>
+          <t>w29</t>
+        </is>
+      </c>
+      <c r="C77" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D77" s="18" t="inlineStr">
+        <is>
+          <t>Criteria finalized</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="inlineStr">
+        <is>
+          <t>Confirm full-text screening criteria are finalized</t>
+        </is>
+      </c>
+      <c r="F77" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Sean</t>
+        </is>
+      </c>
+      <c r="G77" s="18" t="inlineStr">
+        <is>
+          <t>w11,w26,w27,w28</t>
+        </is>
+      </c>
+      <c r="H77" s="18" t="inlineStr">
+        <is>
+          <t>w30</t>
+        </is>
+      </c>
+      <c r="I77" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J77" s="18" t="inlineStr"/>
+      <c r="K77" s="18" t="inlineStr"/>
+      <c r="L77" s="18" t="inlineStr"/>
+      <c r="M77" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="28" customHeight="1" s="29">
+      <c r="A78" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="B78" s="18" t="inlineStr">
+        <is>
+          <t>w30</t>
+        </is>
+      </c>
+      <c r="C78" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D78" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup</t>
+        </is>
+      </c>
+      <c r="E78" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup - allocated AI tool for full-text screening</t>
+        </is>
+      </c>
+      <c r="F78" s="18" t="inlineStr">
+        <is>
+          <t>Response Team / Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G78" s="18" t="inlineStr">
+        <is>
+          <t>w04,w07,w29</t>
+        </is>
+      </c>
+      <c r="H78" s="18" t="inlineStr">
+        <is>
+          <t>w31</t>
+        </is>
+      </c>
+      <c r="I78" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J78" s="18" t="inlineStr"/>
+      <c r="K78" s="18" t="inlineStr"/>
+      <c r="L78" s="18" t="inlineStr"/>
+      <c r="M78" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="28" customHeight="1" s="29">
+      <c r="A79" s="18" t="n">
+        <v>31</v>
+      </c>
+      <c r="B79" s="18" t="inlineStr">
+        <is>
+          <t>w31</t>
+        </is>
+      </c>
+      <c r="C79" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D79" s="18" t="inlineStr">
+        <is>
+          <t>Setup validated</t>
+        </is>
+      </c>
+      <c r="E79" s="18" t="inlineStr">
+        <is>
+          <t>Review team validates full-text screening setup before starting</t>
+        </is>
+      </c>
+      <c r="F79" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G79" s="18" t="inlineStr">
+        <is>
+          <t>w30</t>
+        </is>
+      </c>
+      <c r="H79" s="18" t="inlineStr">
+        <is>
+          <t>w32,w33</t>
+        </is>
+      </c>
+      <c r="I79" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J79" s="18" t="inlineStr"/>
+      <c r="K79" s="18" t="inlineStr"/>
+      <c r="L79" s="18" t="inlineStr"/>
+      <c r="M79" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="18" t="n">
+        <v>32</v>
+      </c>
+      <c r="B80" s="18" t="inlineStr">
+        <is>
+          <t>w32</t>
+        </is>
+      </c>
+      <c r="C80" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D80" s="18" t="inlineStr">
+        <is>
+          <t>Human full text</t>
+        </is>
+      </c>
+      <c r="E80" s="18" t="inlineStr">
+        <is>
+          <t>Full-text screening - Human workflow</t>
+        </is>
+      </c>
+      <c r="F80" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G80" s="18" t="inlineStr">
+        <is>
+          <t>w05,w08,w09,w31</t>
+        </is>
+      </c>
+      <c r="H80" s="18" t="inlineStr">
+        <is>
+          <t>w36,w39,w40</t>
+        </is>
+      </c>
+      <c r="I80" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J80" s="18" t="inlineStr"/>
+      <c r="K80" s="18" t="inlineStr"/>
+      <c r="L80" s="18" t="inlineStr"/>
+      <c r="M80" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="18" t="n">
+        <v>33</v>
+      </c>
+      <c r="B81" s="18" t="inlineStr">
+        <is>
+          <t>w33</t>
+        </is>
+      </c>
+      <c r="C81" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D81" s="18" t="inlineStr">
+        <is>
+          <t>AI full text</t>
+        </is>
+      </c>
+      <c r="E81" s="18" t="inlineStr">
+        <is>
+          <t>Full-text screening - allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F81" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G81" s="18" t="inlineStr">
+        <is>
+          <t>w07,w08,w09,w31</t>
+        </is>
+      </c>
+      <c r="H81" s="18" t="inlineStr">
+        <is>
+          <t>w34,w36,w39,w40</t>
+        </is>
+      </c>
+      <c r="I81" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J81" s="18" t="inlineStr"/>
+      <c r="K81" s="18" t="inlineStr"/>
+      <c r="L81" s="18" t="inlineStr"/>
+      <c r="M81" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="18" t="n">
+        <v>34</v>
+      </c>
+      <c r="B82" s="18" t="inlineStr">
+        <is>
+          <t>w34</t>
+        </is>
+      </c>
+      <c r="C82" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D82" s="18" t="inlineStr">
+        <is>
+          <t>Export AI output</t>
+        </is>
+      </c>
+      <c r="E82" s="18" t="inlineStr">
+        <is>
+          <t>Export full-text screening output from allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F82" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G82" s="18" t="inlineStr">
+        <is>
+          <t>w33</t>
+        </is>
+      </c>
+      <c r="H82" s="18" t="inlineStr">
+        <is>
+          <t>w35</t>
+        </is>
+      </c>
+      <c r="I82" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J82" s="18" t="inlineStr"/>
+      <c r="K82" s="18" t="inlineStr"/>
+      <c r="L82" s="18" t="inlineStr"/>
+      <c r="M82" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="18" t="n">
+        <v>35</v>
+      </c>
+      <c r="B83" s="18" t="inlineStr">
+        <is>
+          <t>w35</t>
+        </is>
+      </c>
+      <c r="C83" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D83" s="18" t="inlineStr">
+        <is>
+          <t>Share output</t>
+        </is>
+      </c>
+      <c r="E83" s="18" t="inlineStr">
+        <is>
+          <t>Share full-text screening output with Sean / data manager</t>
+        </is>
+      </c>
+      <c r="F83" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Data Manager</t>
+        </is>
+      </c>
+      <c r="G83" s="18" t="inlineStr">
+        <is>
+          <t>w34</t>
+        </is>
+      </c>
+      <c r="H83" s="18" t="inlineStr">
+        <is>
+          <t>w39,w40</t>
+        </is>
+      </c>
+      <c r="I83" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J83" s="18" t="inlineStr"/>
+      <c r="K83" s="18" t="inlineStr"/>
+      <c r="L83" s="18" t="inlineStr"/>
+      <c r="M83" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="18" t="n">
+        <v>36</v>
+      </c>
+      <c r="B84" s="18" t="inlineStr">
+        <is>
+          <t>w36</t>
+        </is>
+      </c>
+      <c r="C84" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D84" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent</t>
+        </is>
+      </c>
+      <c r="E84" s="18" t="inlineStr">
+        <is>
+          <t>Share usability survey on full-text screening workflow</t>
+        </is>
+      </c>
+      <c r="F84" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G84" s="18" t="inlineStr">
+        <is>
+          <t>w32,w33</t>
+        </is>
+      </c>
+      <c r="H84" s="18" t="inlineStr">
+        <is>
+          <t>w37</t>
+        </is>
+      </c>
+      <c r="I84" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J84" s="18" t="inlineStr"/>
+      <c r="K84" s="18" t="inlineStr"/>
+      <c r="L84" s="18" t="inlineStr"/>
+      <c r="M84" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="18" t="n">
+        <v>37</v>
+      </c>
+      <c r="B85" s="18" t="inlineStr">
+        <is>
+          <t>w37</t>
+        </is>
+      </c>
+      <c r="C85" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D85" s="18" t="inlineStr">
+        <is>
+          <t>Survey submitted</t>
+        </is>
+      </c>
+      <c r="E85" s="18" t="inlineStr">
+        <is>
+          <t>Submit usability survey on full-text screening workflow</t>
+        </is>
+      </c>
+      <c r="F85" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G85" s="18" t="inlineStr">
+        <is>
+          <t>w36</t>
+        </is>
+      </c>
+      <c r="H85" s="18" t="inlineStr">
+        <is>
+          <t>w38</t>
+        </is>
+      </c>
+      <c r="I85" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J85" s="18" t="inlineStr"/>
+      <c r="K85" s="18" t="inlineStr"/>
+      <c r="L85" s="18" t="inlineStr"/>
+      <c r="M85" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="28" customHeight="1" s="29">
+      <c r="A86" s="18" t="n">
+        <v>38</v>
+      </c>
+      <c r="B86" s="18" t="inlineStr">
+        <is>
+          <t>w38</t>
+        </is>
+      </c>
+      <c r="C86" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D86" s="18" t="inlineStr">
+        <is>
+          <t>Survey received</t>
+        </is>
+      </c>
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>Confirm usability survey responses received for full-text screening</t>
+        </is>
+      </c>
+      <c r="F86" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G86" s="18" t="inlineStr">
+        <is>
+          <t>w37</t>
+        </is>
+      </c>
+      <c r="H86" s="18" t="inlineStr">
+        <is>
+          <t>w39</t>
+        </is>
+      </c>
+      <c r="I86" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J86" s="18" t="inlineStr"/>
+      <c r="K86" s="18" t="inlineStr"/>
+      <c r="L86" s="18" t="inlineStr"/>
+      <c r="M86" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="28" customHeight="1" s="29">
+      <c r="A87" s="18" t="n">
+        <v>39</v>
+      </c>
+      <c r="B87" s="18" t="inlineStr">
+        <is>
+          <t>w39</t>
+        </is>
+      </c>
+      <c r="C87" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D87" s="18" t="inlineStr">
+        <is>
+          <t>Quality check</t>
+        </is>
+      </c>
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness and quality check before full-text adjudication</t>
+        </is>
+      </c>
+      <c r="F87" s="18" t="inlineStr">
+        <is>
+          <t>Data Manager / Sean</t>
+        </is>
+      </c>
+      <c r="G87" s="18" t="inlineStr">
+        <is>
+          <t>w35,w38</t>
+        </is>
+      </c>
+      <c r="H87" s="18" t="inlineStr">
+        <is>
+          <t>w40</t>
+        </is>
+      </c>
+      <c r="I87" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J87" s="18" t="inlineStr"/>
+      <c r="K87" s="18" t="inlineStr"/>
+      <c r="L87" s="18" t="inlineStr"/>
+      <c r="M87" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="B88" s="18" t="inlineStr">
+        <is>
+          <t>w40</t>
+        </is>
+      </c>
+      <c r="C88" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D88" s="18" t="inlineStr">
+        <is>
+          <t>Full-text adjudication</t>
+        </is>
+      </c>
+      <c r="E88" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication panel after full-text screening</t>
+        </is>
+      </c>
+      <c r="F88" s="18" t="inlineStr">
+        <is>
+          <t>Sean and Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="G88" s="18" t="inlineStr">
+        <is>
+          <t>w39</t>
+        </is>
+      </c>
+      <c r="H88" s="18" t="inlineStr">
+        <is>
+          <t>w42,w43,w45</t>
+        </is>
+      </c>
+      <c r="I88" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J88" s="18" t="inlineStr"/>
+      <c r="K88" s="18" t="inlineStr"/>
+      <c r="L88" s="18" t="inlineStr"/>
+      <c r="M88" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="18" t="n">
+        <v>41</v>
+      </c>
+      <c r="B89" s="18" t="inlineStr">
+        <is>
+          <t>w41</t>
+        </is>
+      </c>
+      <c r="C89" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D89" s="18" t="inlineStr">
+        <is>
+          <t>Platform ready</t>
+        </is>
+      </c>
+      <c r="E89" s="18" t="inlineStr">
+        <is>
+          <t>Finalisation of Laser AI platform/server setup, if applicable</t>
+        </is>
+      </c>
+      <c r="F89" s="18" t="inlineStr">
+        <is>
+          <t>Core Team / Laser AI</t>
+        </is>
+      </c>
+      <c r="G89" s="18" t="inlineStr">
+        <is>
+          <t>w04,w07</t>
+        </is>
+      </c>
+      <c r="H89" s="18" t="inlineStr">
+        <is>
+          <t>w45</t>
+        </is>
+      </c>
+      <c r="I89" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J89" s="18" t="inlineStr"/>
+      <c r="K89" s="18" t="inlineStr"/>
+      <c r="L89" s="18" t="inlineStr"/>
+      <c r="M89" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="28" customHeight="1" s="29">
+      <c r="A90" s="18" t="n">
+        <v>42</v>
+      </c>
+      <c r="B90" s="18" t="inlineStr">
+        <is>
+          <t>w42</t>
+        </is>
+      </c>
+      <c r="C90" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D90" s="18" t="inlineStr">
+        <is>
+          <t>DE check-in</t>
+        </is>
+      </c>
+      <c r="E90" s="18" t="inlineStr">
+        <is>
+          <t>Meeting with Gerald and optional review team members before data extraction</t>
+        </is>
+      </c>
+      <c r="F90" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G90" s="18" t="inlineStr">
+        <is>
+          <t>w40</t>
+        </is>
+      </c>
+      <c r="H90" s="18" t="inlineStr">
+        <is>
+          <t>w43</t>
+        </is>
+      </c>
+      <c r="I90" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J90" s="18" t="inlineStr"/>
+      <c r="K90" s="18" t="inlineStr"/>
+      <c r="L90" s="18" t="inlineStr"/>
+      <c r="M90" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="18" t="n">
+        <v>43</v>
+      </c>
+      <c r="B91" s="18" t="inlineStr">
+        <is>
+          <t>w43</t>
+        </is>
+      </c>
+      <c r="C91" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D91" s="18" t="inlineStr">
+        <is>
+          <t>DE items confirmed</t>
+        </is>
+      </c>
+      <c r="E91" s="18" t="inlineStr">
+        <is>
+          <t>Confirm final data extraction items and definitions</t>
+        </is>
+      </c>
+      <c r="F91" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Sean</t>
+        </is>
+      </c>
+      <c r="G91" s="18" t="inlineStr">
+        <is>
+          <t>w12,w14,w40,w42</t>
+        </is>
+      </c>
+      <c r="H91" s="18" t="inlineStr">
+        <is>
+          <t>w44</t>
+        </is>
+      </c>
+      <c r="I91" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J91" s="18" t="inlineStr"/>
+      <c r="K91" s="18" t="inlineStr"/>
+      <c r="L91" s="18" t="inlineStr"/>
+      <c r="M91" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="18" t="n">
+        <v>44</v>
+      </c>
+      <c r="B92" s="18" t="inlineStr">
+        <is>
+          <t>w44</t>
+        </is>
+      </c>
+      <c r="C92" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D92" s="18" t="inlineStr">
+        <is>
+          <t>Form approved</t>
+        </is>
+      </c>
+      <c r="E92" s="18" t="inlineStr">
+        <is>
+          <t>Confirm extraction form/template is approved by Sean</t>
+        </is>
+      </c>
+      <c r="F92" s="18" t="inlineStr">
+        <is>
+          <t>Sean</t>
+        </is>
+      </c>
+      <c r="G92" s="18" t="inlineStr">
+        <is>
+          <t>w13,w14,w43</t>
+        </is>
+      </c>
+      <c r="H92" s="18" t="inlineStr">
+        <is>
+          <t>w45</t>
+        </is>
+      </c>
+      <c r="I92" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J92" s="18" t="inlineStr"/>
+      <c r="K92" s="18" t="inlineStr"/>
+      <c r="L92" s="18" t="inlineStr"/>
+      <c r="M92" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="28" customHeight="1" s="29">
+      <c r="A93" s="18" t="n">
+        <v>45</v>
+      </c>
+      <c r="B93" s="18" t="inlineStr">
+        <is>
+          <t>w45</t>
+        </is>
+      </c>
+      <c r="C93" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D93" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup</t>
+        </is>
+      </c>
+      <c r="E93" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup - allocated AI tool for data extraction</t>
+        </is>
+      </c>
+      <c r="F93" s="18" t="inlineStr">
+        <is>
+          <t>Response Team / Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G93" s="18" t="inlineStr">
+        <is>
+          <t>w41,w44</t>
+        </is>
+      </c>
+      <c r="H93" s="18" t="inlineStr">
+        <is>
+          <t>w46</t>
+        </is>
+      </c>
+      <c r="I93" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J93" s="18" t="inlineStr"/>
+      <c r="K93" s="18" t="inlineStr"/>
+      <c r="L93" s="18" t="inlineStr"/>
+      <c r="M93" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="28" customHeight="1" s="29">
+      <c r="A94" s="18" t="n">
+        <v>46</v>
+      </c>
+      <c r="B94" s="18" t="inlineStr">
+        <is>
+          <t>w46</t>
+        </is>
+      </c>
+      <c r="C94" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D94" s="18" t="inlineStr">
+        <is>
+          <t>Setup validated</t>
+        </is>
+      </c>
+      <c r="E94" s="18" t="inlineStr">
+        <is>
+          <t>Review team validates data extraction setup before starting</t>
+        </is>
+      </c>
+      <c r="F94" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G94" s="18" t="inlineStr">
+        <is>
+          <t>w45</t>
+        </is>
+      </c>
+      <c r="H94" s="18" t="inlineStr">
+        <is>
+          <t>w47,w48</t>
+        </is>
+      </c>
+      <c r="I94" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J94" s="18" t="inlineStr"/>
+      <c r="K94" s="18" t="inlineStr"/>
+      <c r="L94" s="18" t="inlineStr"/>
+      <c r="M94" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="18" t="n">
+        <v>47</v>
+      </c>
+      <c r="B95" s="18" t="inlineStr">
+        <is>
+          <t>w47</t>
+        </is>
+      </c>
+      <c r="C95" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D95" s="18" t="inlineStr">
+        <is>
+          <t>Human extraction</t>
+        </is>
+      </c>
+      <c r="E95" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction - Human workflow</t>
+        </is>
+      </c>
+      <c r="F95" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G95" s="18" t="inlineStr">
+        <is>
+          <t>w05,w08,w09,w46</t>
+        </is>
+      </c>
+      <c r="H95" s="18" t="inlineStr">
+        <is>
+          <t>w51,w54,w55</t>
+        </is>
+      </c>
+      <c r="I95" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J95" s="18" t="inlineStr"/>
+      <c r="K95" s="18" t="inlineStr"/>
+      <c r="L95" s="18" t="inlineStr"/>
+      <c r="M95" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="18" t="n">
+        <v>48</v>
+      </c>
+      <c r="B96" s="18" t="inlineStr">
+        <is>
+          <t>w48</t>
+        </is>
+      </c>
+      <c r="C96" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D96" s="18" t="inlineStr">
+        <is>
+          <t>AI extraction</t>
+        </is>
+      </c>
+      <c r="E96" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction - allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F96" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G96" s="18" t="inlineStr">
+        <is>
+          <t>w07,w08,w09,w46</t>
+        </is>
+      </c>
+      <c r="H96" s="18" t="inlineStr">
+        <is>
+          <t>w49,w51,w54,w55</t>
+        </is>
+      </c>
+      <c r="I96" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J96" s="18" t="inlineStr"/>
+      <c r="K96" s="18" t="inlineStr"/>
+      <c r="L96" s="18" t="inlineStr"/>
+      <c r="M96" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="18" t="n">
+        <v>49</v>
+      </c>
+      <c r="B97" s="18" t="inlineStr">
+        <is>
+          <t>w49</t>
+        </is>
+      </c>
+      <c r="C97" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D97" s="18" t="inlineStr">
+        <is>
+          <t>Export AI output</t>
+        </is>
+      </c>
+      <c r="E97" s="18" t="inlineStr">
+        <is>
+          <t>Export data extraction output from allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F97" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G97" s="18" t="inlineStr">
+        <is>
+          <t>w48</t>
+        </is>
+      </c>
+      <c r="H97" s="18" t="inlineStr">
+        <is>
+          <t>w50</t>
+        </is>
+      </c>
+      <c r="I97" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J97" s="18" t="inlineStr"/>
+      <c r="K97" s="18" t="inlineStr"/>
+      <c r="L97" s="18" t="inlineStr"/>
+      <c r="M97" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="B98" s="18" t="inlineStr">
+        <is>
+          <t>w50</t>
+        </is>
+      </c>
+      <c r="C98" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D98" s="18" t="inlineStr">
+        <is>
+          <t>Share output</t>
+        </is>
+      </c>
+      <c r="E98" s="18" t="inlineStr">
+        <is>
+          <t>Share data extraction output with Sean / data manager</t>
+        </is>
+      </c>
+      <c r="F98" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Data Manager</t>
+        </is>
+      </c>
+      <c r="G98" s="18" t="inlineStr">
+        <is>
+          <t>w49</t>
+        </is>
+      </c>
+      <c r="H98" s="18" t="inlineStr">
+        <is>
+          <t>w54,w55</t>
+        </is>
+      </c>
+      <c r="I98" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J98" s="18" t="inlineStr"/>
+      <c r="K98" s="18" t="inlineStr"/>
+      <c r="L98" s="18" t="inlineStr"/>
+      <c r="M98" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="18" t="n">
+        <v>51</v>
+      </c>
+      <c r="B99" s="18" t="inlineStr">
+        <is>
+          <t>w51</t>
+        </is>
+      </c>
+      <c r="C99" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D99" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent</t>
+        </is>
+      </c>
+      <c r="E99" s="18" t="inlineStr">
+        <is>
+          <t>Share usability survey on data extraction workflow</t>
+        </is>
+      </c>
+      <c r="F99" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G99" s="18" t="inlineStr">
+        <is>
+          <t>w47,w48</t>
+        </is>
+      </c>
+      <c r="H99" s="18" t="inlineStr">
+        <is>
+          <t>w52</t>
+        </is>
+      </c>
+      <c r="I99" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J99" s="18" t="inlineStr"/>
+      <c r="K99" s="18" t="inlineStr"/>
+      <c r="L99" s="18" t="inlineStr"/>
+      <c r="M99" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="18" t="n">
+        <v>52</v>
+      </c>
+      <c r="B100" s="18" t="inlineStr">
+        <is>
+          <t>w52</t>
+        </is>
+      </c>
+      <c r="C100" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D100" s="18" t="inlineStr">
+        <is>
+          <t>Survey submitted</t>
+        </is>
+      </c>
+      <c r="E100" s="18" t="inlineStr">
+        <is>
+          <t>Submit usability survey on data extraction workflow</t>
+        </is>
+      </c>
+      <c r="F100" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G100" s="18" t="inlineStr">
+        <is>
+          <t>w51</t>
+        </is>
+      </c>
+      <c r="H100" s="18" t="inlineStr">
+        <is>
+          <t>w53</t>
+        </is>
+      </c>
+      <c r="I100" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J100" s="18" t="inlineStr"/>
+      <c r="K100" s="18" t="inlineStr"/>
+      <c r="L100" s="18" t="inlineStr"/>
+      <c r="M100" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="28" customHeight="1" s="29">
+      <c r="A101" s="18" t="n">
+        <v>53</v>
+      </c>
+      <c r="B101" s="18" t="inlineStr">
+        <is>
+          <t>w53</t>
+        </is>
+      </c>
+      <c r="C101" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D101" s="18" t="inlineStr">
+        <is>
+          <t>Survey received</t>
+        </is>
+      </c>
+      <c r="E101" s="18" t="inlineStr">
+        <is>
+          <t>Confirm usability survey responses received for data extraction</t>
+        </is>
+      </c>
+      <c r="F101" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G101" s="18" t="inlineStr">
+        <is>
+          <t>w52</t>
+        </is>
+      </c>
+      <c r="H101" s="18" t="inlineStr">
+        <is>
+          <t>w54</t>
+        </is>
+      </c>
+      <c r="I101" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J101" s="18" t="inlineStr"/>
+      <c r="K101" s="18" t="inlineStr"/>
+      <c r="L101" s="18" t="inlineStr"/>
+      <c r="M101" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="28" customHeight="1" s="29">
+      <c r="A102" s="18" t="n">
+        <v>54</v>
+      </c>
+      <c r="B102" s="18" t="inlineStr">
+        <is>
+          <t>w54</t>
+        </is>
+      </c>
+      <c r="C102" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D102" s="18" t="inlineStr">
+        <is>
+          <t>Quality check</t>
+        </is>
+      </c>
+      <c r="E102" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness and quality check before data extraction adjudication</t>
+        </is>
+      </c>
+      <c r="F102" s="18" t="inlineStr">
+        <is>
+          <t>Data Manager / Sean</t>
+        </is>
+      </c>
+      <c r="G102" s="18" t="inlineStr">
+        <is>
+          <t>w50,w53</t>
+        </is>
+      </c>
+      <c r="H102" s="18" t="inlineStr">
+        <is>
+          <t>w55</t>
+        </is>
+      </c>
+      <c r="I102" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J102" s="18" t="inlineStr"/>
+      <c r="K102" s="18" t="inlineStr"/>
+      <c r="L102" s="18" t="inlineStr"/>
+      <c r="M102" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="18" t="n">
+        <v>55</v>
+      </c>
+      <c r="B103" s="18" t="inlineStr">
+        <is>
+          <t>w55</t>
+        </is>
+      </c>
+      <c r="C103" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D103" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication dataset</t>
+        </is>
+      </c>
+      <c r="E103" s="18" t="inlineStr">
+        <is>
+          <t>Prepare adjudication-ready dataset</t>
+        </is>
+      </c>
+      <c r="F103" s="18" t="inlineStr">
+        <is>
+          <t>Data Manager / Sean</t>
+        </is>
+      </c>
+      <c r="G103" s="18" t="inlineStr">
+        <is>
+          <t>w54</t>
+        </is>
+      </c>
+      <c r="H103" s="18" t="inlineStr">
+        <is>
+          <t>w56,w57,w58,w61,w62,w63</t>
+        </is>
+      </c>
+      <c r="I103" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J103" s="18" t="inlineStr"/>
+      <c r="K103" s="18" t="inlineStr"/>
+      <c r="L103" s="18" t="inlineStr"/>
+      <c r="M103" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="18" t="n">
+        <v>56</v>
+      </c>
+      <c r="B104" s="18" t="inlineStr">
+        <is>
+          <t>w56</t>
+        </is>
+      </c>
+      <c r="C104" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D104" s="18" t="inlineStr">
+        <is>
+          <t>DE adjudication</t>
+        </is>
+      </c>
+      <c r="E104" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication panel after data extraction</t>
+        </is>
+      </c>
+      <c r="F104" s="18" t="inlineStr">
+        <is>
+          <t>Sean and Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="G104" s="18" t="inlineStr">
+        <is>
+          <t>w55</t>
+        </is>
+      </c>
+      <c r="H104" s="18" t="inlineStr">
+        <is>
+          <t>w57,w60,w61,w62,w63</t>
+        </is>
+      </c>
+      <c r="I104" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J104" s="18" t="inlineStr"/>
+      <c r="K104" s="18" t="inlineStr"/>
+      <c r="L104" s="18" t="inlineStr"/>
+      <c r="M104" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="18" t="n">
+        <v>57</v>
+      </c>
+      <c r="B105" s="18" t="inlineStr">
+        <is>
+          <t>w57</t>
+        </is>
+      </c>
+      <c r="C105" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D105" s="18" t="inlineStr">
+        <is>
+          <t>Gerald closeout</t>
+        </is>
+      </c>
+      <c r="E105" s="18" t="inlineStr">
+        <is>
+          <t>Meeting with Gerald before analysis closeout</t>
+        </is>
+      </c>
+      <c r="F105" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G105" s="18" t="inlineStr">
+        <is>
+          <t>w56</t>
+        </is>
+      </c>
+      <c r="H105" s="18" t="inlineStr">
+        <is>
+          <t>w59,w63</t>
+        </is>
+      </c>
+      <c r="I105" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J105" s="18" t="inlineStr"/>
+      <c r="K105" s="18" t="inlineStr"/>
+      <c r="L105" s="18" t="inlineStr"/>
+      <c r="M105" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="18" t="n">
+        <v>58</v>
+      </c>
+      <c r="B106" s="18" t="inlineStr">
+        <is>
+          <t>w58</t>
+        </is>
+      </c>
+      <c r="C106" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D106" s="18" t="inlineStr">
+        <is>
+          <t>Stability study</t>
+        </is>
+      </c>
+      <c r="E106" s="18" t="inlineStr">
+        <is>
+          <t>Fully automated and stability study - Pawel and Noosheen</t>
+        </is>
+      </c>
+      <c r="F106" s="18" t="inlineStr">
+        <is>
+          <t>Pawel / Noosheen</t>
+        </is>
+      </c>
+      <c r="G106" s="18" t="inlineStr">
+        <is>
+          <t>w55</t>
+        </is>
+      </c>
+      <c r="H106" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I106" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J106" s="18" t="inlineStr"/>
+      <c r="K106" s="18" t="inlineStr"/>
+      <c r="L106" s="18" t="inlineStr"/>
+      <c r="M106" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="18" t="n">
+        <v>59</v>
+      </c>
+      <c r="B107" s="18" t="inlineStr">
+        <is>
+          <t>w59</t>
+        </is>
+      </c>
+      <c r="C107" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D107" s="18" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="E107" s="18" t="inlineStr">
+        <is>
+          <t>Follow-up and review</t>
+        </is>
+      </c>
+      <c r="F107" s="18" t="inlineStr">
+        <is>
+          <t>Core Team</t>
+        </is>
+      </c>
+      <c r="G107" s="18" t="inlineStr">
+        <is>
+          <t>w57</t>
+        </is>
+      </c>
+      <c r="H107" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I107" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J107" s="18" t="inlineStr"/>
+      <c r="K107" s="18" t="inlineStr"/>
+      <c r="L107" s="18" t="inlineStr"/>
+      <c r="M107" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="B108" s="18" t="inlineStr">
+        <is>
+          <t>w60</t>
+        </is>
+      </c>
+      <c r="C108" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D108" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication work</t>
+        </is>
+      </c>
+      <c r="E108" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication panel parallel work</t>
+        </is>
+      </c>
+      <c r="F108" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="G108" s="18" t="inlineStr">
+        <is>
+          <t>w25,w40,w56</t>
+        </is>
+      </c>
+      <c r="H108" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I108" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J108" s="18" t="inlineStr"/>
+      <c r="K108" s="18" t="inlineStr"/>
+      <c r="L108" s="18" t="inlineStr"/>
+      <c r="M108" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="18" t="n">
+        <v>61</v>
+      </c>
+      <c r="B109" s="18" t="inlineStr">
+        <is>
+          <t>w61</t>
+        </is>
+      </c>
+      <c r="C109" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D109" s="18" t="inlineStr">
+        <is>
+          <t>Afroditi analysis</t>
+        </is>
+      </c>
+      <c r="E109" s="18" t="inlineStr">
+        <is>
+          <t>Afroditi analysis</t>
+        </is>
+      </c>
+      <c r="F109" s="18" t="inlineStr">
+        <is>
+          <t>Afroditi</t>
+        </is>
+      </c>
+      <c r="G109" s="18" t="inlineStr">
+        <is>
+          <t>w55,w56</t>
+        </is>
+      </c>
+      <c r="H109" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I109" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J109" s="18" t="inlineStr"/>
+      <c r="K109" s="18" t="inlineStr"/>
+      <c r="L109" s="18" t="inlineStr"/>
+      <c r="M109" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="18" t="n">
+        <v>62</v>
+      </c>
+      <c r="B110" s="18" t="inlineStr">
+        <is>
+          <t>w62</t>
+        </is>
+      </c>
+      <c r="C110" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D110" s="18" t="inlineStr">
+        <is>
+          <t>Downstream errors</t>
+        </is>
+      </c>
+      <c r="E110" s="18" t="inlineStr">
+        <is>
+          <t>Downstream impact of errors research - Max and Joanna</t>
+        </is>
+      </c>
+      <c r="F110" s="18" t="inlineStr">
+        <is>
+          <t>Max / Joanna</t>
+        </is>
+      </c>
+      <c r="G110" s="18" t="inlineStr">
+        <is>
+          <t>w55,w56</t>
+        </is>
+      </c>
+      <c r="H110" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I110" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J110" s="18" t="inlineStr"/>
+      <c r="K110" s="18" t="inlineStr"/>
+      <c r="L110" s="18" t="inlineStr"/>
+      <c r="M110" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="18" t="n">
+        <v>63</v>
+      </c>
+      <c r="B111" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="C111" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D111" s="18" t="inlineStr">
+        <is>
+          <t>Final analysis</t>
+        </is>
+      </c>
+      <c r="E111" s="18" t="inlineStr">
+        <is>
+          <t>Final analysis</t>
+        </is>
+      </c>
+      <c r="F111" s="18" t="inlineStr">
+        <is>
+          <t>Analysis Team</t>
+        </is>
+      </c>
+      <c r="G111" s="18" t="inlineStr">
+        <is>
+          <t>w57,w58,w59,w60,w61,w62</t>
+        </is>
+      </c>
+      <c r="H111" s="18" t="n"/>
+      <c r="I111" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J111" s="18" t="inlineStr"/>
+      <c r="K111" s="18" t="inlineStr"/>
+      <c r="L111" s="18" t="inlineStr"/>
+      <c r="M111" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>Review Tasks Displayed in Dashboard</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="n"/>
+      <c r="C113" s="5" t="n"/>
+      <c r="D113" s="5" t="n"/>
+      <c r="E113" s="5" t="n"/>
+      <c r="F113" s="5" t="n"/>
+      <c r="G113" s="5" t="n"/>
+      <c r="H113" s="5" t="n"/>
+      <c r="I113" s="5" t="n"/>
+      <c r="J113" s="5" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>TaskID</t>
+        </is>
+      </c>
+      <c r="B114" s="1" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C114" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D114" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E114" s="1" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="F114" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="G114" s="1" t="inlineStr">
+        <is>
+          <t>Dependency</t>
+        </is>
+      </c>
+      <c r="H114" s="1" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="I114" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="J114" s="1" t="inlineStr">
+        <is>
+          <t>SourceDate</t>
+        </is>
+      </c>
+      <c r="K114" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>task-phase1-08-001</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Complete onboarding and confirm tool-training/setup plan</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Krishna / Siew Cheng Foong / Project Team</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Onboarding meeting</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Onboarding confirmed; tool training and setup to follow.</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Project tracking</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>Recent Mail / Communication Log Displayed in Dashboard</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="n"/>
+      <c r="C120" s="5" t="n"/>
+      <c r="D120" s="5" t="n"/>
+      <c r="E120" s="5" t="n"/>
+      <c r="F120" s="5" t="n"/>
+      <c r="G120" s="5" t="n"/>
+      <c r="H120" s="5" t="n"/>
+      <c r="I120" s="5" t="n"/>
+      <c r="J120" s="5" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="inlineStr">
+        <is>
+          <t>CommunicationID</t>
+        </is>
+      </c>
+      <c r="B121" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C121" s="1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="D121" s="1" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E121" s="1" t="inlineStr">
+        <is>
+          <t>Responsible</t>
+        </is>
+      </c>
+      <c r="F121" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="G121" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H121" s="1" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="I121" s="1" t="inlineStr">
+        <is>
+          <t>LinkedTaskID</t>
+        </is>
+      </c>
+      <c r="J121" s="1" t="inlineStr">
+        <is>
+          <t>LinkedAction</t>
+        </is>
+      </c>
+      <c r="K121" s="1" t="inlineStr">
+        <is>
+          <t>SourceType</t>
+        </is>
+      </c>
+      <c r="L121" s="1" t="inlineStr">
+        <is>
+          <t>SourceLink</t>
+        </is>
+      </c>
+      <c r="M121" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>comm-phase1-08-001</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Oral galactagogues onboarding confirmed</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong / review team / Cochrane elective students / project team</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Initial onboarding will cover the study and parallel workflow; tool training and setup will be scheduled afterward.</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>task-phase1-08-001</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Complete onboarding and confirm tool-training/setup plan</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Project tracking</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>Critical Items Displayed in Dashboard</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="n"/>
+      <c r="C124" s="5" t="n"/>
+      <c r="D124" s="5" t="n"/>
+      <c r="E124" s="5" t="n"/>
+      <c r="F124" s="5" t="n"/>
+      <c r="G124" s="5" t="n"/>
+      <c r="H124" s="5" t="n"/>
+      <c r="I124" s="5" t="n"/>
+      <c r="J124" s="5" t="n"/>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="inlineStr">
+        <is>
+          <t>CriticalItem</t>
+        </is>
+      </c>
+      <c r="B125" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C125" s="1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="D125" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E125" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="F125" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G125" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>SourceDate</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="18" customWidth="1" style="29" min="1" max="2"/>
@@ -37554,6 +42149,78 @@
       <c r="N11" t="inlineStr">
         <is>
           <t>phase1-07 Human Milk</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>phase1-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Oral Galactagogues</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Oral galactagogues (natural therapies or drugs) for increasing breast milk production in mothers of non-hospitalised term infants</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Onboarding confirmed</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Onboarding is confirmed for 2026-08-10 at 3:00 PM Malaysia time with the full review team and two Cochrane elective students. Tool training and setup will follow after onboarding.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Complete onboarding, confirm tool allocation and team split, then schedule tool training and setup.</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>phase1-08 Oral Galactagogues</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync Oral Galactagogues review
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -25,6 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-08 Oral Galactagogues" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -22921,17 +22922,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Shortlisted</t>
+          <t>Converted to full sheet</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Onboarding confirmed for 2026-08-10 at 3:00 PM Malaysia time; full team and two Cochrane elective students will attend.</t>
+          <t>Converted to phase1-08 Oral Galactagogues; onboarding confirmed for 2026-08-10.</t>
         </is>
       </c>
       <c r="E30" s="17" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="F30" s="17" t="inlineStr">
@@ -22941,22 +22942,22 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Onboarding 2026-08-10; tool training and setup to follow.</t>
+          <t>Onboarding complete/confirmed; tool training and setup to follow.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Initial onboarding will cover the study and parallel workflow; tool training and setup will be scheduled afterward.</t>
+          <t>Converted to dashboard review phase1-08.</t>
         </is>
       </c>
       <c r="I30" s="17" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -27355,12 +27356,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>phase1-08</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -36764,13 +36770,4602 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M125"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <cols>
+    <col width="14" customWidth="1" style="29" min="1" max="1"/>
+    <col width="16" customWidth="1" style="29" min="2" max="2"/>
+    <col width="28" customWidth="1" style="29" min="3" max="3"/>
+    <col width="18" customWidth="1" style="29" min="4" max="4"/>
+    <col width="48" customWidth="1" style="29" min="5" max="5"/>
+    <col width="28" customWidth="1" style="29" min="6" max="6"/>
+    <col width="24" customWidth="1" style="29" min="7" max="8"/>
+    <col width="18" customWidth="1" style="29" min="9" max="10"/>
+    <col width="16" customWidth="1" style="29" min="11" max="11"/>
+    <col width="30" customWidth="1" style="29" min="12" max="12"/>
+    <col width="12" customWidth="1" style="29" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1" s="29">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>phase1-08 Oral Galactagogues | Dashboard Content Sheet</t>
+        </is>
+      </c>
+      <c r="K1" s="18" t="n"/>
+      <c r="L1" s="18" t="n"/>
+      <c r="M1" s="18" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Executive Review Card</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Card Field</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ReviewID</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>phase1-08</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ShortName</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Oral Galactagogues</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ReviewTitle</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Oral galactagogues (natural therapies or drugs) for increasing breast milk production in mothers of non-hospitalised term infants</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Onboarding confirmed</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tool</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CurrentStage</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Onboarding is confirmed for 2026-08-10 at 3:00 PM Malaysia time with the full review team and two Cochrane elective students. Tool training and setup will follow after onboarding.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CurrentUpdate</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Onboarding is confirmed for 2026-08-10 at 3:00 PM Malaysia time with the full review team and two Cochrane elective students. Tool training and setup will follow after onboarding.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>NextAction</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Complete onboarding, confirm tool allocation and team split, then schedule tool training and setup.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TargetDate</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>New Phase 1 review added from the onboarding pipeline; setup has not started yet.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DisplayInHTML</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Set to No if review should not appear in dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LastUpdated</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard Milestones</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="5" t="n"/>
+      <c r="I22" s="5" t="n"/>
+      <c r="J22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>TargetDate</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>onboarding</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>setup</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>fullText</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>analysis</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Files Displayed in Review Detail</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="5" t="n"/>
+      <c r="J31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>FileType</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G32" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>RIS</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>PDFs</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Criteria</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Extraction</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Time Log</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Stage Progress: Visual Tracker / Operations</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="5" t="n"/>
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="5" t="n"/>
+      <c r="G40" s="5" t="n"/>
+      <c r="H40" s="5" t="n"/>
+      <c r="I40" s="5" t="n"/>
+      <c r="J40" s="5" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>StageName</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>HumanProgress</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>AIProgress</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>TargetDate</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H41" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Setup / Coordination</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Onboarding confirmed; tool allocation and setup to follow.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Abstract Screening</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Full-text Screening</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Data Extraction / Analysis</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Review Workflow Status: Full 63 Actions</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n"/>
+      <c r="C47" s="5" t="n"/>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="5" t="n"/>
+      <c r="F47" s="5" t="n"/>
+      <c r="G47" s="5" t="n"/>
+      <c r="H47" s="5" t="n"/>
+      <c r="I47" s="5" t="n"/>
+      <c r="J47" s="5" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>ActionOrder</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>WorkflowStepID</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>WorkflowGroup</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>ShortName</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>Responsible</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>DependsOn</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>Blocks</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="K48" s="10" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="L48" s="10" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="M48" s="10" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>w01</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D49" s="18" t="inlineStr">
+        <is>
+          <t>Review selected</t>
+        </is>
+      </c>
+      <c r="E49" s="18" t="inlineStr">
+        <is>
+          <t>Selection of review - core team</t>
+        </is>
+      </c>
+      <c r="F49" s="18" t="inlineStr">
+        <is>
+          <t>Core Team</t>
+        </is>
+      </c>
+      <c r="G49" s="18" t="n"/>
+      <c r="H49" s="18" t="inlineStr">
+        <is>
+          <t>w02</t>
+        </is>
+      </c>
+      <c r="I49" s="18" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J49" s="18" t="inlineStr"/>
+      <c r="K49" s="18" t="inlineStr"/>
+      <c r="L49" s="18" t="n"/>
+      <c r="M49" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" s="18" t="inlineStr">
+        <is>
+          <t>w02</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D50" s="18" t="inlineStr">
+        <is>
+          <t>PM confirmation</t>
+        </is>
+      </c>
+      <c r="E50" s="18" t="inlineStr">
+        <is>
+          <t>Selection of review - project manager confirmation</t>
+        </is>
+      </c>
+      <c r="F50" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G50" s="18" t="inlineStr">
+        <is>
+          <t>w01</t>
+        </is>
+      </c>
+      <c r="H50" s="18" t="inlineStr">
+        <is>
+          <t>w03</t>
+        </is>
+      </c>
+      <c r="I50" s="18" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J50" s="18" t="inlineStr"/>
+      <c r="K50" s="18" t="inlineStr"/>
+      <c r="L50" s="18" t="n"/>
+      <c r="M50" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>w03</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D51" s="18" t="inlineStr">
+        <is>
+          <t>Final confirmation</t>
+        </is>
+      </c>
+      <c r="E51" s="18" t="inlineStr">
+        <is>
+          <t>Selection of review - final confirmation</t>
+        </is>
+      </c>
+      <c r="F51" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G51" s="18" t="inlineStr">
+        <is>
+          <t>w02</t>
+        </is>
+      </c>
+      <c r="H51" s="18" t="inlineStr">
+        <is>
+          <t>w04</t>
+        </is>
+      </c>
+      <c r="I51" s="18" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J51" s="18" t="inlineStr"/>
+      <c r="K51" s="18" t="inlineStr"/>
+      <c r="L51" s="18" t="n"/>
+      <c r="M51" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>w04</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>Tool allocated</t>
+        </is>
+      </c>
+      <c r="E52" s="18" t="inlineStr">
+        <is>
+          <t>Confirm allocated AI tool for review</t>
+        </is>
+      </c>
+      <c r="F52" s="18" t="inlineStr">
+        <is>
+          <t>Core Team</t>
+        </is>
+      </c>
+      <c r="G52" s="18" t="inlineStr">
+        <is>
+          <t>w03</t>
+        </is>
+      </c>
+      <c r="H52" s="18" t="inlineStr">
+        <is>
+          <t>w05,w07,w15,w30,w45</t>
+        </is>
+      </c>
+      <c r="I52" s="18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J52" s="18" t="inlineStr"/>
+      <c r="K52" s="18" t="inlineStr"/>
+      <c r="L52" s="18" t="inlineStr">
+        <is>
+          <t>Tool allocation to be confirmed after onboarding.</t>
+        </is>
+      </c>
+      <c r="M52" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="28" customHeight="1" s="29">
+      <c r="A53" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B53" s="18" t="inlineStr">
+        <is>
+          <t>w05</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D53" s="18" t="inlineStr">
+        <is>
+          <t>Team split</t>
+        </is>
+      </c>
+      <c r="E53" s="18" t="inlineStr">
+        <is>
+          <t>Confirm review team split: Human workflow and AI-assisted workflow</t>
+        </is>
+      </c>
+      <c r="F53" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Review Team</t>
+        </is>
+      </c>
+      <c r="G53" s="18" t="inlineStr">
+        <is>
+          <t>w04</t>
+        </is>
+      </c>
+      <c r="H53" s="18" t="inlineStr">
+        <is>
+          <t>w08,w09,w17,w32,w47</t>
+        </is>
+      </c>
+      <c r="I53" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J53" s="18" t="inlineStr"/>
+      <c r="K53" s="18" t="inlineStr"/>
+      <c r="L53" s="18" t="inlineStr"/>
+      <c r="M53" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B54" s="18" t="inlineStr">
+        <is>
+          <t>w06</t>
+        </is>
+      </c>
+      <c r="C54" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D54" s="18" t="inlineStr">
+        <is>
+          <t>Folder access</t>
+        </is>
+      </c>
+      <c r="E54" s="18" t="inlineStr">
+        <is>
+          <t>Confirm SharePoint/folder access for review team</t>
+        </is>
+      </c>
+      <c r="F54" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Review Team</t>
+        </is>
+      </c>
+      <c r="G54" s="18" t="inlineStr">
+        <is>
+          <t>w03</t>
+        </is>
+      </c>
+      <c r="H54" s="18" t="inlineStr">
+        <is>
+          <t>w10,w11,w12</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J54" s="18" t="inlineStr"/>
+      <c r="K54" s="18" t="inlineStr"/>
+      <c r="M54" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="28" customHeight="1" s="29">
+      <c r="A55" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B55" s="18" t="inlineStr">
+        <is>
+          <t>w07</t>
+        </is>
+      </c>
+      <c r="C55" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D55" s="18" t="inlineStr">
+        <is>
+          <t>Tool access</t>
+        </is>
+      </c>
+      <c r="E55" s="18" t="inlineStr">
+        <is>
+          <t>Confirm AI tool access for allocated users</t>
+        </is>
+      </c>
+      <c r="F55" s="18" t="inlineStr">
+        <is>
+          <t>Response Team / Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G55" s="18" t="inlineStr">
+        <is>
+          <t>w04</t>
+        </is>
+      </c>
+      <c r="H55" s="18" t="inlineStr">
+        <is>
+          <t>w15,w30,w45</t>
+        </is>
+      </c>
+      <c r="I55" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J55" s="18" t="inlineStr"/>
+      <c r="K55" s="18" t="inlineStr"/>
+      <c r="L55" s="18" t="inlineStr"/>
+      <c r="M55" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B56" s="18" t="inlineStr">
+        <is>
+          <t>w08</t>
+        </is>
+      </c>
+      <c r="C56" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D56" s="18" t="inlineStr">
+        <is>
+          <t>Blinding shared</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="inlineStr">
+        <is>
+          <t>Confirm blinding instructions shared with review teams</t>
+        </is>
+      </c>
+      <c r="F56" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Sean</t>
+        </is>
+      </c>
+      <c r="G56" s="18" t="inlineStr">
+        <is>
+          <t>w05</t>
+        </is>
+      </c>
+      <c r="H56" s="18" t="inlineStr">
+        <is>
+          <t>w17,w18,w32,w33,w47,w48</t>
+        </is>
+      </c>
+      <c r="I56" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J56" s="18" t="inlineStr"/>
+      <c r="K56" s="18" t="inlineStr"/>
+      <c r="L56" s="18" t="inlineStr"/>
+      <c r="M56" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
+          <t>w09</t>
+        </is>
+      </c>
+      <c r="C57" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D57" s="18" t="inlineStr">
+        <is>
+          <t>Time tracking</t>
+        </is>
+      </c>
+      <c r="E57" s="18" t="inlineStr">
+        <is>
+          <t>Confirm Clockify or alternate time-tracking setup</t>
+        </is>
+      </c>
+      <c r="F57" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G57" s="18" t="inlineStr">
+        <is>
+          <t>w05</t>
+        </is>
+      </c>
+      <c r="H57" s="18" t="inlineStr">
+        <is>
+          <t>w17,w18,w32,w33,w47,w48</t>
+        </is>
+      </c>
+      <c r="I57" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J57" s="18" t="inlineStr"/>
+      <c r="K57" s="18" t="inlineStr"/>
+      <c r="L57" s="18" t="inlineStr"/>
+      <c r="M57" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="28" customHeight="1" s="29">
+      <c r="A58" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="B58" s="18" t="inlineStr">
+        <is>
+          <t>w10</t>
+        </is>
+      </c>
+      <c r="C58" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="inlineStr">
+        <is>
+          <t>RIS files</t>
+        </is>
+      </c>
+      <c r="E58" s="18" t="inlineStr">
+        <is>
+          <t>Review team to share RIS files with setup team</t>
+        </is>
+      </c>
+      <c r="F58" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G58" s="18" t="inlineStr">
+        <is>
+          <t>w06</t>
+        </is>
+      </c>
+      <c r="H58" s="18" t="inlineStr">
+        <is>
+          <t>w15</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J58" s="18" t="inlineStr"/>
+      <c r="K58" s="18" t="inlineStr"/>
+      <c r="M58" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="28" customHeight="1" s="29">
+      <c r="A59" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>w11</t>
+        </is>
+      </c>
+      <c r="C59" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D59" s="18" t="inlineStr">
+        <is>
+          <t>Protocol &amp; criteria</t>
+        </is>
+      </c>
+      <c r="E59" s="18" t="inlineStr">
+        <is>
+          <t>Review team to share protocol and inclusion/exclusion criteria</t>
+        </is>
+      </c>
+      <c r="F59" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G59" s="18" t="inlineStr">
+        <is>
+          <t>w06</t>
+        </is>
+      </c>
+      <c r="H59" s="18" t="inlineStr">
+        <is>
+          <t>w12,w15,w29</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J59" s="18" t="inlineStr"/>
+      <c r="K59" s="18" t="inlineStr"/>
+      <c r="M59" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="28" customHeight="1" s="29">
+      <c r="A60" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="B60" s="18" t="inlineStr">
+        <is>
+          <t>w12</t>
+        </is>
+      </c>
+      <c r="C60" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D60" s="18" t="inlineStr">
+        <is>
+          <t>Data items</t>
+        </is>
+      </c>
+      <c r="E60" s="18" t="inlineStr">
+        <is>
+          <t>Finalise data items with Sean</t>
+        </is>
+      </c>
+      <c r="F60" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Sean</t>
+        </is>
+      </c>
+      <c r="G60" s="18" t="inlineStr">
+        <is>
+          <t>w11</t>
+        </is>
+      </c>
+      <c r="H60" s="18" t="inlineStr">
+        <is>
+          <t>w13,w14,w43,w44</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J60" s="18" t="inlineStr"/>
+      <c r="K60" s="18" t="inlineStr"/>
+      <c r="M60" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="28" customHeight="1" s="29">
+      <c r="A61" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>w13</t>
+        </is>
+      </c>
+      <c r="C61" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>Comparable DE</t>
+        </is>
+      </c>
+      <c r="E61" s="18" t="inlineStr">
+        <is>
+          <t>Confirm data extraction structure is comparable between Human and AI workflows</t>
+        </is>
+      </c>
+      <c r="F61" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Sean</t>
+        </is>
+      </c>
+      <c r="G61" s="18" t="inlineStr">
+        <is>
+          <t>w12</t>
+        </is>
+      </c>
+      <c r="H61" s="18" t="inlineStr">
+        <is>
+          <t>w14,w44</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J61" s="18" t="inlineStr"/>
+      <c r="K61" s="18" t="inlineStr"/>
+      <c r="M61" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="28" customHeight="1" s="29">
+      <c r="A62" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="B62" s="18" t="inlineStr">
+        <is>
+          <t>w14</t>
+        </is>
+      </c>
+      <c r="C62" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>Sean approval</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="inlineStr">
+        <is>
+          <t>Confirm extraction form/template is approved by Sean</t>
+        </is>
+      </c>
+      <c r="F62" s="18" t="inlineStr">
+        <is>
+          <t>Sean</t>
+        </is>
+      </c>
+      <c r="G62" s="18" t="inlineStr">
+        <is>
+          <t>w13</t>
+        </is>
+      </c>
+      <c r="H62" s="18" t="inlineStr">
+        <is>
+          <t>w43,w44,w45</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J62" s="18" t="inlineStr"/>
+      <c r="K62" s="18" t="inlineStr"/>
+      <c r="M62" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="28" customHeight="1" s="29">
+      <c r="A63" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t>w15</t>
+        </is>
+      </c>
+      <c r="C63" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D63" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup</t>
+        </is>
+      </c>
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup - allocated AI tool for abstract screening</t>
+        </is>
+      </c>
+      <c r="F63" s="18" t="inlineStr">
+        <is>
+          <t>Response Team / Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G63" s="18" t="inlineStr">
+        <is>
+          <t>w04,w07,w10,w11</t>
+        </is>
+      </c>
+      <c r="H63" s="18" t="inlineStr">
+        <is>
+          <t>w16</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J63" s="18" t="inlineStr"/>
+      <c r="K63" s="18" t="inlineStr"/>
+      <c r="M63" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="28" customHeight="1" s="29">
+      <c r="A64" s="18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B64" s="18" t="inlineStr">
+        <is>
+          <t>w16</t>
+        </is>
+      </c>
+      <c r="C64" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D64" s="18" t="inlineStr">
+        <is>
+          <t>Setup validated</t>
+        </is>
+      </c>
+      <c r="E64" s="18" t="inlineStr">
+        <is>
+          <t>Review team validates abstract screening setup before starting</t>
+        </is>
+      </c>
+      <c r="F64" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G64" s="18" t="inlineStr">
+        <is>
+          <t>w15</t>
+        </is>
+      </c>
+      <c r="H64" s="18" t="inlineStr">
+        <is>
+          <t>w17,w18</t>
+        </is>
+      </c>
+      <c r="I64" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J64" s="18" t="inlineStr"/>
+      <c r="K64" s="18" t="inlineStr"/>
+      <c r="L64" s="18" t="inlineStr"/>
+      <c r="M64" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B65" s="18" t="inlineStr">
+        <is>
+          <t>w17</t>
+        </is>
+      </c>
+      <c r="C65" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D65" s="18" t="inlineStr">
+        <is>
+          <t>Human screening</t>
+        </is>
+      </c>
+      <c r="E65" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening - Human workflow</t>
+        </is>
+      </c>
+      <c r="F65" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G65" s="18" t="inlineStr">
+        <is>
+          <t>w05,w08,w09,w16</t>
+        </is>
+      </c>
+      <c r="H65" s="18" t="inlineStr">
+        <is>
+          <t>w21,w24,w25</t>
+        </is>
+      </c>
+      <c r="I65" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J65" s="18" t="inlineStr"/>
+      <c r="K65" s="18" t="inlineStr"/>
+      <c r="L65" s="18" t="inlineStr"/>
+      <c r="M65" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="18" t="n">
+        <v>18</v>
+      </c>
+      <c r="B66" s="18" t="inlineStr">
+        <is>
+          <t>w18</t>
+        </is>
+      </c>
+      <c r="C66" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D66" s="18" t="inlineStr">
+        <is>
+          <t>AI screening</t>
+        </is>
+      </c>
+      <c r="E66" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening - allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F66" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G66" s="18" t="inlineStr">
+        <is>
+          <t>w07,w08,w09,w16</t>
+        </is>
+      </c>
+      <c r="H66" s="18" t="inlineStr">
+        <is>
+          <t>w19,w21,w24,w25</t>
+        </is>
+      </c>
+      <c r="I66" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J66" s="18" t="inlineStr"/>
+      <c r="K66" s="18" t="inlineStr"/>
+      <c r="L66" s="18" t="inlineStr"/>
+      <c r="M66" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="18" t="n">
+        <v>19</v>
+      </c>
+      <c r="B67" s="18" t="inlineStr">
+        <is>
+          <t>w19</t>
+        </is>
+      </c>
+      <c r="C67" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D67" s="18" t="inlineStr">
+        <is>
+          <t>Export AI output</t>
+        </is>
+      </c>
+      <c r="E67" s="18" t="inlineStr">
+        <is>
+          <t>Export abstract screening output from allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F67" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G67" s="18" t="inlineStr">
+        <is>
+          <t>w18</t>
+        </is>
+      </c>
+      <c r="H67" s="18" t="inlineStr">
+        <is>
+          <t>w20</t>
+        </is>
+      </c>
+      <c r="I67" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J67" s="18" t="inlineStr"/>
+      <c r="K67" s="18" t="inlineStr"/>
+      <c r="L67" s="18" t="inlineStr"/>
+      <c r="M67" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="B68" s="18" t="inlineStr">
+        <is>
+          <t>w20</t>
+        </is>
+      </c>
+      <c r="C68" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D68" s="18" t="inlineStr">
+        <is>
+          <t>Share output</t>
+        </is>
+      </c>
+      <c r="E68" s="18" t="inlineStr">
+        <is>
+          <t>Share abstract screening output with Sean / data manager</t>
+        </is>
+      </c>
+      <c r="F68" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Data Manager</t>
+        </is>
+      </c>
+      <c r="G68" s="18" t="inlineStr">
+        <is>
+          <t>w19</t>
+        </is>
+      </c>
+      <c r="H68" s="18" t="inlineStr">
+        <is>
+          <t>w24,w25</t>
+        </is>
+      </c>
+      <c r="I68" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J68" s="18" t="inlineStr"/>
+      <c r="K68" s="18" t="inlineStr"/>
+      <c r="L68" s="18" t="inlineStr"/>
+      <c r="M68" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="18" t="n">
+        <v>21</v>
+      </c>
+      <c r="B69" s="18" t="inlineStr">
+        <is>
+          <t>w21</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D69" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent</t>
+        </is>
+      </c>
+      <c r="E69" s="18" t="inlineStr">
+        <is>
+          <t>Share usability survey on abstract screening experience</t>
+        </is>
+      </c>
+      <c r="F69" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G69" s="18" t="inlineStr">
+        <is>
+          <t>w17,w18</t>
+        </is>
+      </c>
+      <c r="H69" s="18" t="inlineStr">
+        <is>
+          <t>w22</t>
+        </is>
+      </c>
+      <c r="I69" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J69" s="18" t="inlineStr"/>
+      <c r="K69" s="18" t="inlineStr"/>
+      <c r="L69" s="18" t="inlineStr"/>
+      <c r="M69" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="18" t="n">
+        <v>22</v>
+      </c>
+      <c r="B70" s="18" t="inlineStr">
+        <is>
+          <t>w22</t>
+        </is>
+      </c>
+      <c r="C70" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D70" s="18" t="inlineStr">
+        <is>
+          <t>Survey submitted</t>
+        </is>
+      </c>
+      <c r="E70" s="18" t="inlineStr">
+        <is>
+          <t>Submit usability survey on abstract screening experience</t>
+        </is>
+      </c>
+      <c r="F70" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G70" s="18" t="inlineStr">
+        <is>
+          <t>w21</t>
+        </is>
+      </c>
+      <c r="H70" s="18" t="inlineStr">
+        <is>
+          <t>w23</t>
+        </is>
+      </c>
+      <c r="I70" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J70" s="18" t="inlineStr"/>
+      <c r="K70" s="18" t="inlineStr"/>
+      <c r="L70" s="18" t="inlineStr"/>
+      <c r="M70" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="28" customHeight="1" s="29">
+      <c r="A71" s="18" t="n">
+        <v>23</v>
+      </c>
+      <c r="B71" s="18" t="inlineStr">
+        <is>
+          <t>w23</t>
+        </is>
+      </c>
+      <c r="C71" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
+        <is>
+          <t>Survey received</t>
+        </is>
+      </c>
+      <c r="E71" s="18" t="inlineStr">
+        <is>
+          <t>Confirm usability survey responses received for abstract screening</t>
+        </is>
+      </c>
+      <c r="F71" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G71" s="18" t="inlineStr">
+        <is>
+          <t>w22</t>
+        </is>
+      </c>
+      <c r="H71" s="18" t="inlineStr">
+        <is>
+          <t>w24</t>
+        </is>
+      </c>
+      <c r="I71" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J71" s="18" t="inlineStr"/>
+      <c r="K71" s="18" t="inlineStr"/>
+      <c r="L71" s="18" t="inlineStr"/>
+      <c r="M71" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="28" customHeight="1" s="29">
+      <c r="A72" s="18" t="n">
+        <v>24</v>
+      </c>
+      <c r="B72" s="18" t="inlineStr">
+        <is>
+          <t>w24</t>
+        </is>
+      </c>
+      <c r="C72" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
+        <is>
+          <t>Quality check</t>
+        </is>
+      </c>
+      <c r="E72" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness and quality check before abstract screening adjudication</t>
+        </is>
+      </c>
+      <c r="F72" s="18" t="inlineStr">
+        <is>
+          <t>Data Manager / Sean</t>
+        </is>
+      </c>
+      <c r="G72" s="18" t="inlineStr">
+        <is>
+          <t>w20,w23</t>
+        </is>
+      </c>
+      <c r="H72" s="18" t="inlineStr">
+        <is>
+          <t>w25</t>
+        </is>
+      </c>
+      <c r="I72" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J72" s="18" t="inlineStr"/>
+      <c r="K72" s="18" t="inlineStr"/>
+      <c r="L72" s="18" t="inlineStr"/>
+      <c r="M72" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="B73" s="18" t="inlineStr">
+        <is>
+          <t>w25</t>
+        </is>
+      </c>
+      <c r="C73" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
+        <is>
+          <t>Abstract adjudication</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication panel after abstract screening</t>
+        </is>
+      </c>
+      <c r="F73" s="18" t="inlineStr">
+        <is>
+          <t>Sean and Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="G73" s="18" t="inlineStr">
+        <is>
+          <t>w24</t>
+        </is>
+      </c>
+      <c r="H73" s="18" t="inlineStr">
+        <is>
+          <t>w26,w28,w30</t>
+        </is>
+      </c>
+      <c r="I73" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J73" s="18" t="inlineStr"/>
+      <c r="K73" s="18" t="inlineStr"/>
+      <c r="L73" s="18" t="inlineStr"/>
+      <c r="M73" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="18" t="n">
+        <v>26</v>
+      </c>
+      <c r="B74" s="18" t="inlineStr">
+        <is>
+          <t>w26</t>
+        </is>
+      </c>
+      <c r="C74" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D74" s="18" t="inlineStr">
+        <is>
+          <t>PDFs received</t>
+        </is>
+      </c>
+      <c r="E74" s="18" t="inlineStr">
+        <is>
+          <t>Review team to share PDF files with setup team</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G74" s="18" t="inlineStr">
+        <is>
+          <t>w25</t>
+        </is>
+      </c>
+      <c r="H74" s="18" t="inlineStr">
+        <is>
+          <t>w27,w29</t>
+        </is>
+      </c>
+      <c r="I74" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J74" s="18" t="inlineStr"/>
+      <c r="K74" s="18" t="inlineStr"/>
+      <c r="L74" s="18" t="inlineStr"/>
+      <c r="M74" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="18" t="n">
+        <v>27</v>
+      </c>
+      <c r="B75" s="18" t="inlineStr">
+        <is>
+          <t>w27</t>
+        </is>
+      </c>
+      <c r="C75" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D75" s="18" t="inlineStr">
+        <is>
+          <t>PDF issues logged</t>
+        </is>
+      </c>
+      <c r="E75" s="18" t="inlineStr">
+        <is>
+          <t>Confirm unavailable PDFs or access issues are logged</t>
+        </is>
+      </c>
+      <c r="F75" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Krishna</t>
+        </is>
+      </c>
+      <c r="G75" s="18" t="inlineStr">
+        <is>
+          <t>w26</t>
+        </is>
+      </c>
+      <c r="H75" s="18" t="inlineStr">
+        <is>
+          <t>w29</t>
+        </is>
+      </c>
+      <c r="I75" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J75" s="18" t="inlineStr"/>
+      <c r="K75" s="18" t="inlineStr"/>
+      <c r="L75" s="18" t="inlineStr"/>
+      <c r="M75" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="28" customHeight="1" s="29">
+      <c r="A76" s="18" t="n">
+        <v>28</v>
+      </c>
+      <c r="B76" s="18" t="inlineStr">
+        <is>
+          <t>w28</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D76" s="18" t="inlineStr">
+        <is>
+          <t>Check-in meeting</t>
+        </is>
+      </c>
+      <c r="E76" s="18" t="inlineStr">
+        <is>
+          <t>Meeting with Gerald, Amin, Susan, and optional review team members</t>
+        </is>
+      </c>
+      <c r="F76" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G76" s="18" t="inlineStr">
+        <is>
+          <t>w25</t>
+        </is>
+      </c>
+      <c r="H76" s="18" t="inlineStr">
+        <is>
+          <t>w29</t>
+        </is>
+      </c>
+      <c r="I76" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J76" s="18" t="inlineStr"/>
+      <c r="K76" s="18" t="inlineStr"/>
+      <c r="L76" s="18" t="inlineStr"/>
+      <c r="M76" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="18" t="n">
+        <v>29</v>
+      </c>
+      <c r="B77" s="18" t="inlineStr">
+        <is>
+          <t>w29</t>
+        </is>
+      </c>
+      <c r="C77" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D77" s="18" t="inlineStr">
+        <is>
+          <t>Criteria finalized</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="inlineStr">
+        <is>
+          <t>Confirm full-text screening criteria are finalized</t>
+        </is>
+      </c>
+      <c r="F77" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Sean</t>
+        </is>
+      </c>
+      <c r="G77" s="18" t="inlineStr">
+        <is>
+          <t>w11,w26,w27,w28</t>
+        </is>
+      </c>
+      <c r="H77" s="18" t="inlineStr">
+        <is>
+          <t>w30</t>
+        </is>
+      </c>
+      <c r="I77" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J77" s="18" t="inlineStr"/>
+      <c r="K77" s="18" t="inlineStr"/>
+      <c r="L77" s="18" t="inlineStr"/>
+      <c r="M77" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="28" customHeight="1" s="29">
+      <c r="A78" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="B78" s="18" t="inlineStr">
+        <is>
+          <t>w30</t>
+        </is>
+      </c>
+      <c r="C78" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D78" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup</t>
+        </is>
+      </c>
+      <c r="E78" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup - allocated AI tool for full-text screening</t>
+        </is>
+      </c>
+      <c r="F78" s="18" t="inlineStr">
+        <is>
+          <t>Response Team / Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G78" s="18" t="inlineStr">
+        <is>
+          <t>w04,w07,w29</t>
+        </is>
+      </c>
+      <c r="H78" s="18" t="inlineStr">
+        <is>
+          <t>w31</t>
+        </is>
+      </c>
+      <c r="I78" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J78" s="18" t="inlineStr"/>
+      <c r="K78" s="18" t="inlineStr"/>
+      <c r="L78" s="18" t="inlineStr"/>
+      <c r="M78" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="28" customHeight="1" s="29">
+      <c r="A79" s="18" t="n">
+        <v>31</v>
+      </c>
+      <c r="B79" s="18" t="inlineStr">
+        <is>
+          <t>w31</t>
+        </is>
+      </c>
+      <c r="C79" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D79" s="18" t="inlineStr">
+        <is>
+          <t>Setup validated</t>
+        </is>
+      </c>
+      <c r="E79" s="18" t="inlineStr">
+        <is>
+          <t>Review team validates full-text screening setup before starting</t>
+        </is>
+      </c>
+      <c r="F79" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G79" s="18" t="inlineStr">
+        <is>
+          <t>w30</t>
+        </is>
+      </c>
+      <c r="H79" s="18" t="inlineStr">
+        <is>
+          <t>w32,w33</t>
+        </is>
+      </c>
+      <c r="I79" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J79" s="18" t="inlineStr"/>
+      <c r="K79" s="18" t="inlineStr"/>
+      <c r="L79" s="18" t="inlineStr"/>
+      <c r="M79" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="18" t="n">
+        <v>32</v>
+      </c>
+      <c r="B80" s="18" t="inlineStr">
+        <is>
+          <t>w32</t>
+        </is>
+      </c>
+      <c r="C80" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D80" s="18" t="inlineStr">
+        <is>
+          <t>Human full text</t>
+        </is>
+      </c>
+      <c r="E80" s="18" t="inlineStr">
+        <is>
+          <t>Full-text screening - Human workflow</t>
+        </is>
+      </c>
+      <c r="F80" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G80" s="18" t="inlineStr">
+        <is>
+          <t>w05,w08,w09,w31</t>
+        </is>
+      </c>
+      <c r="H80" s="18" t="inlineStr">
+        <is>
+          <t>w36,w39,w40</t>
+        </is>
+      </c>
+      <c r="I80" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J80" s="18" t="inlineStr"/>
+      <c r="K80" s="18" t="inlineStr"/>
+      <c r="L80" s="18" t="inlineStr"/>
+      <c r="M80" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="18" t="n">
+        <v>33</v>
+      </c>
+      <c r="B81" s="18" t="inlineStr">
+        <is>
+          <t>w33</t>
+        </is>
+      </c>
+      <c r="C81" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D81" s="18" t="inlineStr">
+        <is>
+          <t>AI full text</t>
+        </is>
+      </c>
+      <c r="E81" s="18" t="inlineStr">
+        <is>
+          <t>Full-text screening - allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F81" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G81" s="18" t="inlineStr">
+        <is>
+          <t>w07,w08,w09,w31</t>
+        </is>
+      </c>
+      <c r="H81" s="18" t="inlineStr">
+        <is>
+          <t>w34,w36,w39,w40</t>
+        </is>
+      </c>
+      <c r="I81" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J81" s="18" t="inlineStr"/>
+      <c r="K81" s="18" t="inlineStr"/>
+      <c r="L81" s="18" t="inlineStr"/>
+      <c r="M81" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="18" t="n">
+        <v>34</v>
+      </c>
+      <c r="B82" s="18" t="inlineStr">
+        <is>
+          <t>w34</t>
+        </is>
+      </c>
+      <c r="C82" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D82" s="18" t="inlineStr">
+        <is>
+          <t>Export AI output</t>
+        </is>
+      </c>
+      <c r="E82" s="18" t="inlineStr">
+        <is>
+          <t>Export full-text screening output from allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F82" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G82" s="18" t="inlineStr">
+        <is>
+          <t>w33</t>
+        </is>
+      </c>
+      <c r="H82" s="18" t="inlineStr">
+        <is>
+          <t>w35</t>
+        </is>
+      </c>
+      <c r="I82" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J82" s="18" t="inlineStr"/>
+      <c r="K82" s="18" t="inlineStr"/>
+      <c r="L82" s="18" t="inlineStr"/>
+      <c r="M82" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="18" t="n">
+        <v>35</v>
+      </c>
+      <c r="B83" s="18" t="inlineStr">
+        <is>
+          <t>w35</t>
+        </is>
+      </c>
+      <c r="C83" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D83" s="18" t="inlineStr">
+        <is>
+          <t>Share output</t>
+        </is>
+      </c>
+      <c r="E83" s="18" t="inlineStr">
+        <is>
+          <t>Share full-text screening output with Sean / data manager</t>
+        </is>
+      </c>
+      <c r="F83" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Data Manager</t>
+        </is>
+      </c>
+      <c r="G83" s="18" t="inlineStr">
+        <is>
+          <t>w34</t>
+        </is>
+      </c>
+      <c r="H83" s="18" t="inlineStr">
+        <is>
+          <t>w39,w40</t>
+        </is>
+      </c>
+      <c r="I83" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J83" s="18" t="inlineStr"/>
+      <c r="K83" s="18" t="inlineStr"/>
+      <c r="L83" s="18" t="inlineStr"/>
+      <c r="M83" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="18" t="n">
+        <v>36</v>
+      </c>
+      <c r="B84" s="18" t="inlineStr">
+        <is>
+          <t>w36</t>
+        </is>
+      </c>
+      <c r="C84" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D84" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent</t>
+        </is>
+      </c>
+      <c r="E84" s="18" t="inlineStr">
+        <is>
+          <t>Share usability survey on full-text screening workflow</t>
+        </is>
+      </c>
+      <c r="F84" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G84" s="18" t="inlineStr">
+        <is>
+          <t>w32,w33</t>
+        </is>
+      </c>
+      <c r="H84" s="18" t="inlineStr">
+        <is>
+          <t>w37</t>
+        </is>
+      </c>
+      <c r="I84" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J84" s="18" t="inlineStr"/>
+      <c r="K84" s="18" t="inlineStr"/>
+      <c r="L84" s="18" t="inlineStr"/>
+      <c r="M84" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="18" t="n">
+        <v>37</v>
+      </c>
+      <c r="B85" s="18" t="inlineStr">
+        <is>
+          <t>w37</t>
+        </is>
+      </c>
+      <c r="C85" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D85" s="18" t="inlineStr">
+        <is>
+          <t>Survey submitted</t>
+        </is>
+      </c>
+      <c r="E85" s="18" t="inlineStr">
+        <is>
+          <t>Submit usability survey on full-text screening workflow</t>
+        </is>
+      </c>
+      <c r="F85" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G85" s="18" t="inlineStr">
+        <is>
+          <t>w36</t>
+        </is>
+      </c>
+      <c r="H85" s="18" t="inlineStr">
+        <is>
+          <t>w38</t>
+        </is>
+      </c>
+      <c r="I85" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J85" s="18" t="inlineStr"/>
+      <c r="K85" s="18" t="inlineStr"/>
+      <c r="L85" s="18" t="inlineStr"/>
+      <c r="M85" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="28" customHeight="1" s="29">
+      <c r="A86" s="18" t="n">
+        <v>38</v>
+      </c>
+      <c r="B86" s="18" t="inlineStr">
+        <is>
+          <t>w38</t>
+        </is>
+      </c>
+      <c r="C86" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D86" s="18" t="inlineStr">
+        <is>
+          <t>Survey received</t>
+        </is>
+      </c>
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>Confirm usability survey responses received for full-text screening</t>
+        </is>
+      </c>
+      <c r="F86" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G86" s="18" t="inlineStr">
+        <is>
+          <t>w37</t>
+        </is>
+      </c>
+      <c r="H86" s="18" t="inlineStr">
+        <is>
+          <t>w39</t>
+        </is>
+      </c>
+      <c r="I86" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J86" s="18" t="inlineStr"/>
+      <c r="K86" s="18" t="inlineStr"/>
+      <c r="L86" s="18" t="inlineStr"/>
+      <c r="M86" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="28" customHeight="1" s="29">
+      <c r="A87" s="18" t="n">
+        <v>39</v>
+      </c>
+      <c r="B87" s="18" t="inlineStr">
+        <is>
+          <t>w39</t>
+        </is>
+      </c>
+      <c r="C87" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D87" s="18" t="inlineStr">
+        <is>
+          <t>Quality check</t>
+        </is>
+      </c>
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness and quality check before full-text adjudication</t>
+        </is>
+      </c>
+      <c r="F87" s="18" t="inlineStr">
+        <is>
+          <t>Data Manager / Sean</t>
+        </is>
+      </c>
+      <c r="G87" s="18" t="inlineStr">
+        <is>
+          <t>w35,w38</t>
+        </is>
+      </c>
+      <c r="H87" s="18" t="inlineStr">
+        <is>
+          <t>w40</t>
+        </is>
+      </c>
+      <c r="I87" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J87" s="18" t="inlineStr"/>
+      <c r="K87" s="18" t="inlineStr"/>
+      <c r="L87" s="18" t="inlineStr"/>
+      <c r="M87" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="B88" s="18" t="inlineStr">
+        <is>
+          <t>w40</t>
+        </is>
+      </c>
+      <c r="C88" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D88" s="18" t="inlineStr">
+        <is>
+          <t>Full-text adjudication</t>
+        </is>
+      </c>
+      <c r="E88" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication panel after full-text screening</t>
+        </is>
+      </c>
+      <c r="F88" s="18" t="inlineStr">
+        <is>
+          <t>Sean and Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="G88" s="18" t="inlineStr">
+        <is>
+          <t>w39</t>
+        </is>
+      </c>
+      <c r="H88" s="18" t="inlineStr">
+        <is>
+          <t>w42,w43,w45</t>
+        </is>
+      </c>
+      <c r="I88" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J88" s="18" t="inlineStr"/>
+      <c r="K88" s="18" t="inlineStr"/>
+      <c r="L88" s="18" t="inlineStr"/>
+      <c r="M88" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="18" t="n">
+        <v>41</v>
+      </c>
+      <c r="B89" s="18" t="inlineStr">
+        <is>
+          <t>w41</t>
+        </is>
+      </c>
+      <c r="C89" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D89" s="18" t="inlineStr">
+        <is>
+          <t>Platform ready</t>
+        </is>
+      </c>
+      <c r="E89" s="18" t="inlineStr">
+        <is>
+          <t>Finalisation of Laser AI platform/server setup, if applicable</t>
+        </is>
+      </c>
+      <c r="F89" s="18" t="inlineStr">
+        <is>
+          <t>Core Team / Laser AI</t>
+        </is>
+      </c>
+      <c r="G89" s="18" t="inlineStr">
+        <is>
+          <t>w04,w07</t>
+        </is>
+      </c>
+      <c r="H89" s="18" t="inlineStr">
+        <is>
+          <t>w45</t>
+        </is>
+      </c>
+      <c r="I89" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J89" s="18" t="inlineStr"/>
+      <c r="K89" s="18" t="inlineStr"/>
+      <c r="L89" s="18" t="inlineStr"/>
+      <c r="M89" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="28" customHeight="1" s="29">
+      <c r="A90" s="18" t="n">
+        <v>42</v>
+      </c>
+      <c r="B90" s="18" t="inlineStr">
+        <is>
+          <t>w42</t>
+        </is>
+      </c>
+      <c r="C90" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D90" s="18" t="inlineStr">
+        <is>
+          <t>DE check-in</t>
+        </is>
+      </c>
+      <c r="E90" s="18" t="inlineStr">
+        <is>
+          <t>Meeting with Gerald and optional review team members before data extraction</t>
+        </is>
+      </c>
+      <c r="F90" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G90" s="18" t="inlineStr">
+        <is>
+          <t>w40</t>
+        </is>
+      </c>
+      <c r="H90" s="18" t="inlineStr">
+        <is>
+          <t>w43</t>
+        </is>
+      </c>
+      <c r="I90" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J90" s="18" t="inlineStr"/>
+      <c r="K90" s="18" t="inlineStr"/>
+      <c r="L90" s="18" t="inlineStr"/>
+      <c r="M90" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="18" t="n">
+        <v>43</v>
+      </c>
+      <c r="B91" s="18" t="inlineStr">
+        <is>
+          <t>w43</t>
+        </is>
+      </c>
+      <c r="C91" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D91" s="18" t="inlineStr">
+        <is>
+          <t>DE items confirmed</t>
+        </is>
+      </c>
+      <c r="E91" s="18" t="inlineStr">
+        <is>
+          <t>Confirm final data extraction items and definitions</t>
+        </is>
+      </c>
+      <c r="F91" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Sean</t>
+        </is>
+      </c>
+      <c r="G91" s="18" t="inlineStr">
+        <is>
+          <t>w12,w14,w40,w42</t>
+        </is>
+      </c>
+      <c r="H91" s="18" t="inlineStr">
+        <is>
+          <t>w44</t>
+        </is>
+      </c>
+      <c r="I91" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J91" s="18" t="inlineStr"/>
+      <c r="K91" s="18" t="inlineStr"/>
+      <c r="L91" s="18" t="inlineStr"/>
+      <c r="M91" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="18" t="n">
+        <v>44</v>
+      </c>
+      <c r="B92" s="18" t="inlineStr">
+        <is>
+          <t>w44</t>
+        </is>
+      </c>
+      <c r="C92" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D92" s="18" t="inlineStr">
+        <is>
+          <t>Form approved</t>
+        </is>
+      </c>
+      <c r="E92" s="18" t="inlineStr">
+        <is>
+          <t>Confirm extraction form/template is approved by Sean</t>
+        </is>
+      </c>
+      <c r="F92" s="18" t="inlineStr">
+        <is>
+          <t>Sean</t>
+        </is>
+      </c>
+      <c r="G92" s="18" t="inlineStr">
+        <is>
+          <t>w13,w14,w43</t>
+        </is>
+      </c>
+      <c r="H92" s="18" t="inlineStr">
+        <is>
+          <t>w45</t>
+        </is>
+      </c>
+      <c r="I92" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J92" s="18" t="inlineStr"/>
+      <c r="K92" s="18" t="inlineStr"/>
+      <c r="L92" s="18" t="inlineStr"/>
+      <c r="M92" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="28" customHeight="1" s="29">
+      <c r="A93" s="18" t="n">
+        <v>45</v>
+      </c>
+      <c r="B93" s="18" t="inlineStr">
+        <is>
+          <t>w45</t>
+        </is>
+      </c>
+      <c r="C93" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D93" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup</t>
+        </is>
+      </c>
+      <c r="E93" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup - allocated AI tool for data extraction</t>
+        </is>
+      </c>
+      <c r="F93" s="18" t="inlineStr">
+        <is>
+          <t>Response Team / Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G93" s="18" t="inlineStr">
+        <is>
+          <t>w41,w44</t>
+        </is>
+      </c>
+      <c r="H93" s="18" t="inlineStr">
+        <is>
+          <t>w46</t>
+        </is>
+      </c>
+      <c r="I93" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J93" s="18" t="inlineStr"/>
+      <c r="K93" s="18" t="inlineStr"/>
+      <c r="L93" s="18" t="inlineStr"/>
+      <c r="M93" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="28" customHeight="1" s="29">
+      <c r="A94" s="18" t="n">
+        <v>46</v>
+      </c>
+      <c r="B94" s="18" t="inlineStr">
+        <is>
+          <t>w46</t>
+        </is>
+      </c>
+      <c r="C94" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D94" s="18" t="inlineStr">
+        <is>
+          <t>Setup validated</t>
+        </is>
+      </c>
+      <c r="E94" s="18" t="inlineStr">
+        <is>
+          <t>Review team validates data extraction setup before starting</t>
+        </is>
+      </c>
+      <c r="F94" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G94" s="18" t="inlineStr">
+        <is>
+          <t>w45</t>
+        </is>
+      </c>
+      <c r="H94" s="18" t="inlineStr">
+        <is>
+          <t>w47,w48</t>
+        </is>
+      </c>
+      <c r="I94" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J94" s="18" t="inlineStr"/>
+      <c r="K94" s="18" t="inlineStr"/>
+      <c r="L94" s="18" t="inlineStr"/>
+      <c r="M94" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="18" t="n">
+        <v>47</v>
+      </c>
+      <c r="B95" s="18" t="inlineStr">
+        <is>
+          <t>w47</t>
+        </is>
+      </c>
+      <c r="C95" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D95" s="18" t="inlineStr">
+        <is>
+          <t>Human extraction</t>
+        </is>
+      </c>
+      <c r="E95" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction - Human workflow</t>
+        </is>
+      </c>
+      <c r="F95" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G95" s="18" t="inlineStr">
+        <is>
+          <t>w05,w08,w09,w46</t>
+        </is>
+      </c>
+      <c r="H95" s="18" t="inlineStr">
+        <is>
+          <t>w51,w54,w55</t>
+        </is>
+      </c>
+      <c r="I95" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J95" s="18" t="inlineStr"/>
+      <c r="K95" s="18" t="inlineStr"/>
+      <c r="L95" s="18" t="inlineStr"/>
+      <c r="M95" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="18" t="n">
+        <v>48</v>
+      </c>
+      <c r="B96" s="18" t="inlineStr">
+        <is>
+          <t>w48</t>
+        </is>
+      </c>
+      <c r="C96" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D96" s="18" t="inlineStr">
+        <is>
+          <t>AI extraction</t>
+        </is>
+      </c>
+      <c r="E96" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction - allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F96" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G96" s="18" t="inlineStr">
+        <is>
+          <t>w07,w08,w09,w46</t>
+        </is>
+      </c>
+      <c r="H96" s="18" t="inlineStr">
+        <is>
+          <t>w49,w51,w54,w55</t>
+        </is>
+      </c>
+      <c r="I96" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J96" s="18" t="inlineStr"/>
+      <c r="K96" s="18" t="inlineStr"/>
+      <c r="L96" s="18" t="inlineStr"/>
+      <c r="M96" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="18" t="n">
+        <v>49</v>
+      </c>
+      <c r="B97" s="18" t="inlineStr">
+        <is>
+          <t>w49</t>
+        </is>
+      </c>
+      <c r="C97" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D97" s="18" t="inlineStr">
+        <is>
+          <t>Export AI output</t>
+        </is>
+      </c>
+      <c r="E97" s="18" t="inlineStr">
+        <is>
+          <t>Export data extraction output from allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F97" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G97" s="18" t="inlineStr">
+        <is>
+          <t>w48</t>
+        </is>
+      </c>
+      <c r="H97" s="18" t="inlineStr">
+        <is>
+          <t>w50</t>
+        </is>
+      </c>
+      <c r="I97" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J97" s="18" t="inlineStr"/>
+      <c r="K97" s="18" t="inlineStr"/>
+      <c r="L97" s="18" t="inlineStr"/>
+      <c r="M97" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="B98" s="18" t="inlineStr">
+        <is>
+          <t>w50</t>
+        </is>
+      </c>
+      <c r="C98" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D98" s="18" t="inlineStr">
+        <is>
+          <t>Share output</t>
+        </is>
+      </c>
+      <c r="E98" s="18" t="inlineStr">
+        <is>
+          <t>Share data extraction output with Sean / data manager</t>
+        </is>
+      </c>
+      <c r="F98" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Data Manager</t>
+        </is>
+      </c>
+      <c r="G98" s="18" t="inlineStr">
+        <is>
+          <t>w49</t>
+        </is>
+      </c>
+      <c r="H98" s="18" t="inlineStr">
+        <is>
+          <t>w54,w55</t>
+        </is>
+      </c>
+      <c r="I98" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J98" s="18" t="inlineStr"/>
+      <c r="K98" s="18" t="inlineStr"/>
+      <c r="L98" s="18" t="inlineStr"/>
+      <c r="M98" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="18" t="n">
+        <v>51</v>
+      </c>
+      <c r="B99" s="18" t="inlineStr">
+        <is>
+          <t>w51</t>
+        </is>
+      </c>
+      <c r="C99" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D99" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent</t>
+        </is>
+      </c>
+      <c r="E99" s="18" t="inlineStr">
+        <is>
+          <t>Share usability survey on data extraction workflow</t>
+        </is>
+      </c>
+      <c r="F99" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G99" s="18" t="inlineStr">
+        <is>
+          <t>w47,w48</t>
+        </is>
+      </c>
+      <c r="H99" s="18" t="inlineStr">
+        <is>
+          <t>w52</t>
+        </is>
+      </c>
+      <c r="I99" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J99" s="18" t="inlineStr"/>
+      <c r="K99" s="18" t="inlineStr"/>
+      <c r="L99" s="18" t="inlineStr"/>
+      <c r="M99" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="18" t="n">
+        <v>52</v>
+      </c>
+      <c r="B100" s="18" t="inlineStr">
+        <is>
+          <t>w52</t>
+        </is>
+      </c>
+      <c r="C100" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D100" s="18" t="inlineStr">
+        <is>
+          <t>Survey submitted</t>
+        </is>
+      </c>
+      <c r="E100" s="18" t="inlineStr">
+        <is>
+          <t>Submit usability survey on data extraction workflow</t>
+        </is>
+      </c>
+      <c r="F100" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G100" s="18" t="inlineStr">
+        <is>
+          <t>w51</t>
+        </is>
+      </c>
+      <c r="H100" s="18" t="inlineStr">
+        <is>
+          <t>w53</t>
+        </is>
+      </c>
+      <c r="I100" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J100" s="18" t="inlineStr"/>
+      <c r="K100" s="18" t="inlineStr"/>
+      <c r="L100" s="18" t="inlineStr"/>
+      <c r="M100" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="28" customHeight="1" s="29">
+      <c r="A101" s="18" t="n">
+        <v>53</v>
+      </c>
+      <c r="B101" s="18" t="inlineStr">
+        <is>
+          <t>w53</t>
+        </is>
+      </c>
+      <c r="C101" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D101" s="18" t="inlineStr">
+        <is>
+          <t>Survey received</t>
+        </is>
+      </c>
+      <c r="E101" s="18" t="inlineStr">
+        <is>
+          <t>Confirm usability survey responses received for data extraction</t>
+        </is>
+      </c>
+      <c r="F101" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G101" s="18" t="inlineStr">
+        <is>
+          <t>w52</t>
+        </is>
+      </c>
+      <c r="H101" s="18" t="inlineStr">
+        <is>
+          <t>w54</t>
+        </is>
+      </c>
+      <c r="I101" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J101" s="18" t="inlineStr"/>
+      <c r="K101" s="18" t="inlineStr"/>
+      <c r="L101" s="18" t="inlineStr"/>
+      <c r="M101" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="28" customHeight="1" s="29">
+      <c r="A102" s="18" t="n">
+        <v>54</v>
+      </c>
+      <c r="B102" s="18" t="inlineStr">
+        <is>
+          <t>w54</t>
+        </is>
+      </c>
+      <c r="C102" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D102" s="18" t="inlineStr">
+        <is>
+          <t>Quality check</t>
+        </is>
+      </c>
+      <c r="E102" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness and quality check before data extraction adjudication</t>
+        </is>
+      </c>
+      <c r="F102" s="18" t="inlineStr">
+        <is>
+          <t>Data Manager / Sean</t>
+        </is>
+      </c>
+      <c r="G102" s="18" t="inlineStr">
+        <is>
+          <t>w50,w53</t>
+        </is>
+      </c>
+      <c r="H102" s="18" t="inlineStr">
+        <is>
+          <t>w55</t>
+        </is>
+      </c>
+      <c r="I102" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J102" s="18" t="inlineStr"/>
+      <c r="K102" s="18" t="inlineStr"/>
+      <c r="L102" s="18" t="inlineStr"/>
+      <c r="M102" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="18" t="n">
+        <v>55</v>
+      </c>
+      <c r="B103" s="18" t="inlineStr">
+        <is>
+          <t>w55</t>
+        </is>
+      </c>
+      <c r="C103" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D103" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication dataset</t>
+        </is>
+      </c>
+      <c r="E103" s="18" t="inlineStr">
+        <is>
+          <t>Prepare adjudication-ready dataset</t>
+        </is>
+      </c>
+      <c r="F103" s="18" t="inlineStr">
+        <is>
+          <t>Data Manager / Sean</t>
+        </is>
+      </c>
+      <c r="G103" s="18" t="inlineStr">
+        <is>
+          <t>w54</t>
+        </is>
+      </c>
+      <c r="H103" s="18" t="inlineStr">
+        <is>
+          <t>w56,w57,w58,w61,w62,w63</t>
+        </is>
+      </c>
+      <c r="I103" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J103" s="18" t="inlineStr"/>
+      <c r="K103" s="18" t="inlineStr"/>
+      <c r="L103" s="18" t="inlineStr"/>
+      <c r="M103" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="18" t="n">
+        <v>56</v>
+      </c>
+      <c r="B104" s="18" t="inlineStr">
+        <is>
+          <t>w56</t>
+        </is>
+      </c>
+      <c r="C104" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D104" s="18" t="inlineStr">
+        <is>
+          <t>DE adjudication</t>
+        </is>
+      </c>
+      <c r="E104" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication panel after data extraction</t>
+        </is>
+      </c>
+      <c r="F104" s="18" t="inlineStr">
+        <is>
+          <t>Sean and Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="G104" s="18" t="inlineStr">
+        <is>
+          <t>w55</t>
+        </is>
+      </c>
+      <c r="H104" s="18" t="inlineStr">
+        <is>
+          <t>w57,w60,w61,w62,w63</t>
+        </is>
+      </c>
+      <c r="I104" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J104" s="18" t="inlineStr"/>
+      <c r="K104" s="18" t="inlineStr"/>
+      <c r="L104" s="18" t="inlineStr"/>
+      <c r="M104" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="18" t="n">
+        <v>57</v>
+      </c>
+      <c r="B105" s="18" t="inlineStr">
+        <is>
+          <t>w57</t>
+        </is>
+      </c>
+      <c r="C105" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D105" s="18" t="inlineStr">
+        <is>
+          <t>Gerald closeout</t>
+        </is>
+      </c>
+      <c r="E105" s="18" t="inlineStr">
+        <is>
+          <t>Meeting with Gerald before analysis closeout</t>
+        </is>
+      </c>
+      <c r="F105" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G105" s="18" t="inlineStr">
+        <is>
+          <t>w56</t>
+        </is>
+      </c>
+      <c r="H105" s="18" t="inlineStr">
+        <is>
+          <t>w59,w63</t>
+        </is>
+      </c>
+      <c r="I105" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J105" s="18" t="inlineStr"/>
+      <c r="K105" s="18" t="inlineStr"/>
+      <c r="L105" s="18" t="inlineStr"/>
+      <c r="M105" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="18" t="n">
+        <v>58</v>
+      </c>
+      <c r="B106" s="18" t="inlineStr">
+        <is>
+          <t>w58</t>
+        </is>
+      </c>
+      <c r="C106" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D106" s="18" t="inlineStr">
+        <is>
+          <t>Stability study</t>
+        </is>
+      </c>
+      <c r="E106" s="18" t="inlineStr">
+        <is>
+          <t>Fully automated and stability study - Pawel and Noosheen</t>
+        </is>
+      </c>
+      <c r="F106" s="18" t="inlineStr">
+        <is>
+          <t>Pawel / Noosheen</t>
+        </is>
+      </c>
+      <c r="G106" s="18" t="inlineStr">
+        <is>
+          <t>w55</t>
+        </is>
+      </c>
+      <c r="H106" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I106" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J106" s="18" t="inlineStr"/>
+      <c r="K106" s="18" t="inlineStr"/>
+      <c r="L106" s="18" t="inlineStr"/>
+      <c r="M106" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="18" t="n">
+        <v>59</v>
+      </c>
+      <c r="B107" s="18" t="inlineStr">
+        <is>
+          <t>w59</t>
+        </is>
+      </c>
+      <c r="C107" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D107" s="18" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="E107" s="18" t="inlineStr">
+        <is>
+          <t>Follow-up and review</t>
+        </is>
+      </c>
+      <c r="F107" s="18" t="inlineStr">
+        <is>
+          <t>Core Team</t>
+        </is>
+      </c>
+      <c r="G107" s="18" t="inlineStr">
+        <is>
+          <t>w57</t>
+        </is>
+      </c>
+      <c r="H107" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I107" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J107" s="18" t="inlineStr"/>
+      <c r="K107" s="18" t="inlineStr"/>
+      <c r="L107" s="18" t="inlineStr"/>
+      <c r="M107" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="B108" s="18" t="inlineStr">
+        <is>
+          <t>w60</t>
+        </is>
+      </c>
+      <c r="C108" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D108" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication work</t>
+        </is>
+      </c>
+      <c r="E108" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication panel parallel work</t>
+        </is>
+      </c>
+      <c r="F108" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="G108" s="18" t="inlineStr">
+        <is>
+          <t>w25,w40,w56</t>
+        </is>
+      </c>
+      <c r="H108" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I108" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J108" s="18" t="inlineStr"/>
+      <c r="K108" s="18" t="inlineStr"/>
+      <c r="L108" s="18" t="inlineStr"/>
+      <c r="M108" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="18" t="n">
+        <v>61</v>
+      </c>
+      <c r="B109" s="18" t="inlineStr">
+        <is>
+          <t>w61</t>
+        </is>
+      </c>
+      <c r="C109" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D109" s="18" t="inlineStr">
+        <is>
+          <t>Afroditi analysis</t>
+        </is>
+      </c>
+      <c r="E109" s="18" t="inlineStr">
+        <is>
+          <t>Afroditi analysis</t>
+        </is>
+      </c>
+      <c r="F109" s="18" t="inlineStr">
+        <is>
+          <t>Afroditi</t>
+        </is>
+      </c>
+      <c r="G109" s="18" t="inlineStr">
+        <is>
+          <t>w55,w56</t>
+        </is>
+      </c>
+      <c r="H109" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I109" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J109" s="18" t="inlineStr"/>
+      <c r="K109" s="18" t="inlineStr"/>
+      <c r="L109" s="18" t="inlineStr"/>
+      <c r="M109" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="18" t="n">
+        <v>62</v>
+      </c>
+      <c r="B110" s="18" t="inlineStr">
+        <is>
+          <t>w62</t>
+        </is>
+      </c>
+      <c r="C110" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D110" s="18" t="inlineStr">
+        <is>
+          <t>Downstream errors</t>
+        </is>
+      </c>
+      <c r="E110" s="18" t="inlineStr">
+        <is>
+          <t>Downstream impact of errors research - Max and Joanna</t>
+        </is>
+      </c>
+      <c r="F110" s="18" t="inlineStr">
+        <is>
+          <t>Max / Joanna</t>
+        </is>
+      </c>
+      <c r="G110" s="18" t="inlineStr">
+        <is>
+          <t>w55,w56</t>
+        </is>
+      </c>
+      <c r="H110" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I110" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J110" s="18" t="inlineStr"/>
+      <c r="K110" s="18" t="inlineStr"/>
+      <c r="L110" s="18" t="inlineStr"/>
+      <c r="M110" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="18" t="n">
+        <v>63</v>
+      </c>
+      <c r="B111" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="C111" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D111" s="18" t="inlineStr">
+        <is>
+          <t>Final analysis</t>
+        </is>
+      </c>
+      <c r="E111" s="18" t="inlineStr">
+        <is>
+          <t>Final analysis</t>
+        </is>
+      </c>
+      <c r="F111" s="18" t="inlineStr">
+        <is>
+          <t>Analysis Team</t>
+        </is>
+      </c>
+      <c r="G111" s="18" t="inlineStr">
+        <is>
+          <t>w57,w58,w59,w60,w61,w62</t>
+        </is>
+      </c>
+      <c r="H111" s="18" t="n"/>
+      <c r="I111" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J111" s="18" t="inlineStr"/>
+      <c r="K111" s="18" t="inlineStr"/>
+      <c r="L111" s="18" t="inlineStr"/>
+      <c r="M111" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>Review Tasks Displayed in Dashboard</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="n"/>
+      <c r="C113" s="5" t="n"/>
+      <c r="D113" s="5" t="n"/>
+      <c r="E113" s="5" t="n"/>
+      <c r="F113" s="5" t="n"/>
+      <c r="G113" s="5" t="n"/>
+      <c r="H113" s="5" t="n"/>
+      <c r="I113" s="5" t="n"/>
+      <c r="J113" s="5" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>TaskID</t>
+        </is>
+      </c>
+      <c r="B114" s="1" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C114" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D114" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E114" s="1" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="F114" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="G114" s="1" t="inlineStr">
+        <is>
+          <t>Dependency</t>
+        </is>
+      </c>
+      <c r="H114" s="1" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="I114" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="J114" s="1" t="inlineStr">
+        <is>
+          <t>SourceDate</t>
+        </is>
+      </c>
+      <c r="K114" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>task-phase1-08-001</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Complete onboarding and confirm tool-training/setup plan</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Krishna / Siew Cheng Foong / Project Team</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Onboarding meeting</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Onboarding confirmed; tool training and setup to follow.</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Project tracking</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>Recent Mail / Communication Log Displayed in Dashboard</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="n"/>
+      <c r="C120" s="5" t="n"/>
+      <c r="D120" s="5" t="n"/>
+      <c r="E120" s="5" t="n"/>
+      <c r="F120" s="5" t="n"/>
+      <c r="G120" s="5" t="n"/>
+      <c r="H120" s="5" t="n"/>
+      <c r="I120" s="5" t="n"/>
+      <c r="J120" s="5" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="inlineStr">
+        <is>
+          <t>CommunicationID</t>
+        </is>
+      </c>
+      <c r="B121" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C121" s="1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="D121" s="1" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E121" s="1" t="inlineStr">
+        <is>
+          <t>Responsible</t>
+        </is>
+      </c>
+      <c r="F121" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="G121" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H121" s="1" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="I121" s="1" t="inlineStr">
+        <is>
+          <t>LinkedTaskID</t>
+        </is>
+      </c>
+      <c r="J121" s="1" t="inlineStr">
+        <is>
+          <t>LinkedAction</t>
+        </is>
+      </c>
+      <c r="K121" s="1" t="inlineStr">
+        <is>
+          <t>SourceType</t>
+        </is>
+      </c>
+      <c r="L121" s="1" t="inlineStr">
+        <is>
+          <t>SourceLink</t>
+        </is>
+      </c>
+      <c r="M121" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>comm-phase1-08-001</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Oral galactagogues onboarding confirmed</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong / review team / Cochrane elective students / project team</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Initial onboarding will cover the study and parallel workflow; tool training and setup will be scheduled afterward.</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>task-phase1-08-001</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Complete onboarding and confirm tool-training/setup plan</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Project tracking</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>Critical Items Displayed in Dashboard</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="n"/>
+      <c r="C124" s="5" t="n"/>
+      <c r="D124" s="5" t="n"/>
+      <c r="E124" s="5" t="n"/>
+      <c r="F124" s="5" t="n"/>
+      <c r="G124" s="5" t="n"/>
+      <c r="H124" s="5" t="n"/>
+      <c r="I124" s="5" t="n"/>
+      <c r="J124" s="5" t="n"/>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="inlineStr">
+        <is>
+          <t>CriticalItem</t>
+        </is>
+      </c>
+      <c r="B125" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C125" s="1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="D125" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E125" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="F125" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G125" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>SourceDate</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="18" customWidth="1" style="29" min="1" max="2"/>
@@ -37554,6 +42149,78 @@
       <c r="N11" t="inlineStr">
         <is>
           <t>phase1-07 Human Milk</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>phase1-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Oral Galactagogues</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Oral galactagogues (natural therapies or drugs) for increasing breast milk production in mothers of non-hospitalised term infants</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Onboarding confirmed</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Onboarding is confirmed for 2026-08-10 at 3:00 PM Malaysia time with the full review team and two Cochrane elective students. Tool training and setup will follow after onboarding.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Complete onboarding, confirm tool allocation and team split, then schedule tool training and setup.</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>phase1-08 Oral Galactagogues</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update August review status dashboard
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text screening preparation</t>
+          <t>AI-assisted abstract screening restarting</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AI-assisted and conventional abstract screening are complete. Fifteen April/May records are moving to full text, and 128 prior-search records will also be added to both arms. Shared-folder access for PDFs is in place.</t>
+          <t>Laser AI work has restarted. AI-assisted abstract screening is expected to recommence; confirmation of actual commencement is pending.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AI-assisted and conventional abstract screening are complete. Fifteen April/May records are moving to full text, and 128 prior-search records will also be added to both arms. Shared-folder access for PDFs is in place.</t>
+          <t>Laser AI work has restarted. AI-assisted abstract screening is expected to recommence; confirmation of actual commencement is pending.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Consolidate the final full-text record set and DOIs, upload PDFs, finalise any full-text decision-flow amendments, and proceed with full-text screening in both arms.</t>
+          <t>Confirm commencement of AI-assisted abstract screening and continue tracking time separately for both workflows.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abstract screening is complete; the current dependency is consolidating the full-text set and PDFs, including the additional 128 prior-search records.</t>
+          <t>Restart approved; actual commencement and current screening progress still require confirmation.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Complete - both workflows</t>
+          <t>Restarting - commencement to be confirmed</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3027,12 +3027,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Conventional and Laser AI abstract screening complete; AI workflow moved 15 records to full text.</t>
+          <t>Conventional screening commenced; AI-assisted screening restart is being confirmed.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
@@ -4117,7 +4117,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
@@ -22922,17 +22922,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Converted to full sheet</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Converted to phase1-08 Oral Galactagogues; onboarding confirmed for 2026-08-10.</t>
+          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
         </is>
       </c>
       <c r="E30" s="17" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="F30" s="17" t="inlineStr">
@@ -22942,22 +22942,22 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Onboarding complete/confirmed; tool training and setup to follow.</t>
+          <t>Not participating</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Converted to dashboard review phase1-08.</t>
+          <t>Rerun search produced 377 records, but all relevant studies had already been processed. Team formally declined on 2026-08-11.</t>
         </is>
       </c>
       <c r="I30" s="17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -36701,7 +36701,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>2026-07-30 phase status recheck: BP Targets moved to Data Extraction / Analysis; Psoriasis moved to Full-text Screening; Fruit &amp; Veg marked Abstract Screening Complete; Probiotics AAD and Human Milk set to Setup phase.</t>
+          <t>2026-08-13 updates: Fruit &amp; Veg Laser AI restart noted; Oral Galactagogues withdrawn after 2026-08-11 team decline; BP Targets extraction completion confirmation overdue; Psoriasis date marked overdue/confirmation required.</t>
         </is>
       </c>
     </row>
@@ -36916,7 +36916,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Onboarding confirmed</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -36984,7 +36984,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Onboarding is confirmed for 2026-08-10 at 3:00 PM Malaysia time with the full review team and two Cochrane elective students. Tool training and setup will follow after onboarding.</t>
+          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -37001,7 +37001,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Onboarding is confirmed for 2026-08-10 at 3:00 PM Malaysia time with the full review team and two Cochrane elective students. Tool training and setup will follow after onboarding.</t>
+          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -37018,7 +37018,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete onboarding, confirm tool allocation and team split, then schedule tool training and setup.</t>
+          <t>Retain as withdrawn/historical record; no active onboarding or tool setup required.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -37052,7 +37052,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>New Phase 1 review added from the onboarding pipeline; setup has not started yet.</t>
+          <t>Rerun search produced 377 records, but all relevant studies had already been processed. Team formally declined on 2026-08-11.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -37069,7 +37069,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -37108,7 +37108,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -37200,6 +37200,11 @@
           <t>abstract</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Withdrawn - not participating</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37210,6 +37215,11 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>fullText</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Rerun search produced 377 records, but all relevant studies had already been processed. Team formally declined on 2026-08-11.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -37499,7 +37509,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -37527,7 +37537,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -37550,7 +37560,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -37573,7 +37583,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -41624,17 +41634,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Data extraction remains underway. Blood Pressure Targets is expected to complete the Laser AI data-extraction stage during the week of 2026-08-10. Completed outputs will then be collected for analysis.</t>
+          <t>Data extraction is underway in both workflows. Completion was expected during the week of 2026-08-03, but final completion has not yet been confirmed.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Complete data extraction, collect extraction outputs and time logs, and send the data-extraction usability survey once the stage is complete.</t>
+          <t>Confirm whether both workflows have completed data extraction; collect outputs, time logs and usability-survey responses.</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>Week of 2026-08-10</t>
+          <t>Completion confirmation overdue</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -41706,7 +41716,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Overdue / confirmation required</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -41748,7 +41758,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Full-text screening preparation</t>
+          <t>AI-assisted abstract screening restarting</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -41768,12 +41778,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>AI-assisted and conventional abstract screening are complete. Fifteen April/May records are moving to full text, and 128 prior-search records will also be added to both arms. Shared-folder access for PDFs is in place.</t>
+          <t>Laser AI work has restarted. AI-assisted abstract screening is expected to recommence; confirmation of actual commencement is pending.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Consolidate the final full-text record set and DOIs, upload PDFs, finalise any full-text decision-flow amendments, and proceed with full-text screening in both arms.</t>
+          <t>Confirm commencement of AI-assisted abstract screening and continue tracking conventional and AI-assisted screening time separately.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -42175,7 +42185,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Onboarding confirmed</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -42195,22 +42205,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Onboarding is confirmed for 2026-08-10 at 3:00 PM Malaysia time with the full review team and two Cochrane elective students. Tool training and setup will follow after onboarding.</t>
+          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Complete onboarding, confirm tool allocation and team split, then schedule tool training and setup.</t>
+          <t>Retain as withdrawn/historical record; no active onboarding or tool setup required.</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -46094,7 +46104,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>To Be Updated</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Laser AI work restarted; Fruit &amp; Veg screening restart pending confirmation.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -55974,7 +55989,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Data extraction remains underway. Blood Pressure Targets is expected to complete the Laser AI data-extraction stage during the week of 2026-08-10. Completed outputs will then be collected for analysis.</t>
+          <t>Data extraction is underway in both workflows; final completion has not yet been confirmed.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -55991,7 +56006,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Data extraction remains underway. Blood Pressure Targets is expected to complete the Laser AI data-extraction stage during the week of 2026-08-10. Completed outputs will then be collected for analysis.</t>
+          <t>Completion was expected during the week of 2026-08-03; confirmation remains pending.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56008,7 +56023,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete data extraction, collect extraction outputs and time logs, and send the data-extraction usability survey once the stage is complete.</t>
+          <t>Confirm completion of both extraction workflows and collect outputs, time logs and usability-survey responses.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56025,7 +56040,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Week of 2026-08-10</t>
+          <t>Completion confirmation overdue</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56098,7 +56113,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -61409,7 +61424,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Overdue / confirmation required</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -61482,7 +61497,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">

</xml_diff>

<commit_message>
Update live August review statuses
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text screening preparation</t>
+          <t>AI-assisted abstract screening restarting</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AI-assisted and conventional abstract screening are complete. Fifteen April/May records are moving to full text, and 128 prior-search records will also be added to both arms. Shared-folder access for PDFs is in place.</t>
+          <t>Laser AI work has restarted. AI-assisted abstract screening is expected to recommence; confirmation of actual commencement is pending.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AI-assisted and conventional abstract screening are complete. Fifteen April/May records are moving to full text, and 128 prior-search records will also be added to both arms. Shared-folder access for PDFs is in place.</t>
+          <t>Laser AI work has restarted. AI-assisted abstract screening is expected to recommence; confirmation of actual commencement is pending.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Consolidate the final full-text record set and DOIs, upload PDFs, finalise any full-text decision-flow amendments, and proceed with full-text screening in both arms.</t>
+          <t>Confirm commencement of AI-assisted abstract screening and continue tracking time separately for both workflows.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abstract screening is complete; the current dependency is consolidating the full-text set and PDFs, including the additional 128 prior-search records.</t>
+          <t>Restart approved; actual commencement and current screening progress still require confirmation.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Complete - both workflows</t>
+          <t>Restarting - commencement to be confirmed</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3027,12 +3027,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Conventional and Laser AI abstract screening complete; AI workflow moved 15 records to full text.</t>
+          <t>Conventional screening commenced; AI-assisted screening restart is being confirmed.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
@@ -4117,7 +4117,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
@@ -22922,17 +22922,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Converted to full sheet</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Converted to phase1-08 Oral Galactagogues; onboarding confirmed for 2026-08-10.</t>
+          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
         </is>
       </c>
       <c r="E30" s="17" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="F30" s="17" t="inlineStr">
@@ -22942,22 +22942,22 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Onboarding complete/confirmed; tool training and setup to follow.</t>
+          <t>Not participating</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Converted to dashboard review phase1-08.</t>
+          <t>Rerun search produced 377 records, but all relevant studies had already been processed. Team formally declined on 2026-08-11.</t>
         </is>
       </c>
       <c r="I30" s="17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -36701,7 +36701,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>2026-07-30 phase status recheck: BP Targets moved to Data Extraction / Analysis; Psoriasis moved to Full-text Screening; Fruit &amp; Veg marked Abstract Screening Complete; Probiotics AAD and Human Milk set to Setup phase.</t>
+          <t>2026-08-13 updates: Fruit &amp; Veg Laser AI restart noted; Oral Galactagogues withdrawn after 2026-08-11 team decline; BP Targets extraction completion confirmation overdue; Psoriasis date marked overdue/confirmation required.</t>
         </is>
       </c>
     </row>
@@ -36916,7 +36916,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Onboarding confirmed</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -36984,7 +36984,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Onboarding is confirmed for 2026-08-10 at 3:00 PM Malaysia time with the full review team and two Cochrane elective students. Tool training and setup will follow after onboarding.</t>
+          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -37001,7 +37001,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Onboarding is confirmed for 2026-08-10 at 3:00 PM Malaysia time with the full review team and two Cochrane elective students. Tool training and setup will follow after onboarding.</t>
+          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -37018,7 +37018,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete onboarding, confirm tool allocation and team split, then schedule tool training and setup.</t>
+          <t>Retain as withdrawn/historical record; no active onboarding or tool setup required.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -37052,7 +37052,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>New Phase 1 review added from the onboarding pipeline; setup has not started yet.</t>
+          <t>Rerun search produced 377 records, but all relevant studies had already been processed. Team formally declined on 2026-08-11.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -37069,7 +37069,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -37108,7 +37108,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -37200,6 +37200,11 @@
           <t>abstract</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Withdrawn - not participating</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37210,6 +37215,11 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>fullText</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Rerun search produced 377 records, but all relevant studies had already been processed. Team formally declined on 2026-08-11.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -37499,7 +37509,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -37527,7 +37537,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -37550,7 +37560,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -37573,7 +37583,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -41624,17 +41634,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Data extraction remains underway. Blood Pressure Targets is expected to complete the Laser AI data-extraction stage during the week of 2026-08-10. Completed outputs will then be collected for analysis.</t>
+          <t>Data extraction is underway in both workflows. Completion was expected during the week of 2026-08-03, but final completion has not yet been confirmed.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Complete data extraction, collect extraction outputs and time logs, and send the data-extraction usability survey once the stage is complete.</t>
+          <t>Confirm whether both workflows have completed data extraction; collect outputs, time logs and usability-survey responses.</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>Week of 2026-08-10</t>
+          <t>Completion confirmation overdue</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -41706,7 +41716,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Overdue / confirmation required</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -41748,7 +41758,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Full-text screening preparation</t>
+          <t>AI-assisted abstract screening restarting</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -41768,12 +41778,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>AI-assisted and conventional abstract screening are complete. Fifteen April/May records are moving to full text, and 128 prior-search records will also be added to both arms. Shared-folder access for PDFs is in place.</t>
+          <t>Laser AI work has restarted. AI-assisted abstract screening is expected to recommence; confirmation of actual commencement is pending.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Consolidate the final full-text record set and DOIs, upload PDFs, finalise any full-text decision-flow amendments, and proceed with full-text screening in both arms.</t>
+          <t>Confirm commencement of AI-assisted abstract screening and continue tracking conventional and AI-assisted screening time separately.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -42175,7 +42185,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Onboarding confirmed</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -42195,22 +42205,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Onboarding is confirmed for 2026-08-10 at 3:00 PM Malaysia time with the full review team and two Cochrane elective students. Tool training and setup will follow after onboarding.</t>
+          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Complete onboarding, confirm tool allocation and team split, then schedule tool training and setup.</t>
+          <t>Retain as withdrawn/historical record; no active onboarding or tool setup required.</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -46094,7 +46104,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>To Be Updated</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Laser AI work restarted; Fruit &amp; Veg screening restart pending confirmation.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -55974,7 +55989,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Data extraction remains underway. Blood Pressure Targets is expected to complete the Laser AI data-extraction stage during the week of 2026-08-10. Completed outputs will then be collected for analysis.</t>
+          <t>Data extraction is underway in both workflows; final completion has not yet been confirmed.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -55991,7 +56006,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Data extraction remains underway. Blood Pressure Targets is expected to complete the Laser AI data-extraction stage during the week of 2026-08-10. Completed outputs will then be collected for analysis.</t>
+          <t>Completion was expected during the week of 2026-08-03; confirmation remains pending.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56008,7 +56023,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete data extraction, collect extraction outputs and time logs, and send the data-extraction usability survey once the stage is complete.</t>
+          <t>Confirm completion of both extraction workflows and collect outputs, time logs and usability-survey responses.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56025,7 +56040,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Week of 2026-08-10</t>
+          <t>Completion confirmation overdue</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56098,7 +56113,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -61409,7 +61424,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Overdue / confirmation required</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -61482,7 +61497,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">

</xml_diff>

<commit_message>
Update August review dashboard snapshot
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2287,6 +2287,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2401,7 +2402,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AI-assisted abstract screening restarting</t>
+          <t>Full-text workflow decision pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2469,7 +2470,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Laser AI work has restarted. AI-assisted abstract screening is expected to recommence; confirmation of actual commencement is pending.</t>
+          <t>Screening substantially complete; decision pending for 128 studies and 3 abstracts</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2486,7 +2487,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Laser AI work has restarted. AI-assisted abstract screening is expected to recommence; confirmation of actual commencement is pending.</t>
+          <t>Screening substantially complete; decision pending for 128 studies and 3 abstracts</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2503,7 +2504,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm commencement of AI-assisted abstract screening and continue tracking time separately for both workflows.</t>
+          <t>Obtain team’s selected option and finish 3 abstracts</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2520,7 +2521,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD - after full-text set reconciliation</t>
+          <t>Awaiting review team</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2537,7 +2538,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Restart approved; actual commencement and current screening progress still require confirmation.</t>
+          <t>Full-text work held pending workflow decision</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2554,7 +2555,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2593,7 +2594,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2692,7 +2693,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Restarting - commencement to be confirmed</t>
+          <t>Substantially complete—3 abstracts pending</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2709,7 +2710,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Decision pending for 128 studies</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3027,7 +3028,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Substantially complete—3 abstracts pending</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3055,7 +3056,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Blocked—workflow option pending</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -4060,7 +4061,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
@@ -4117,7 +4118,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
@@ -7858,6 +7859,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -8159,7 +8161,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -12882,6 +12884,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -12996,7 +12999,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup in progress - search strategy/access issue</t>
+          <t>Laser AI setup scheduled/confirmation pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -13064,7 +13067,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
+          <t>Documents re-forwarded; setup planned for August 18</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13081,7 +13084,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
+          <t>Documents re-forwarded; setup planned for August 18</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13098,7 +13101,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Clarify wildcard use, complete accessible searches, document LILACS/IBECS limitations, finalise Laser AI setup, and confirm the screening start.</t>
+          <t>Confirm setup, access, documents and start date</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13115,7 +13118,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -13132,7 +13135,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Most setup materials are available; search-strategy clarification and database-access issues remain before screening can start.</t>
+          <t>Documents re-shared; setup/access confirmation pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -13149,7 +13152,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -13188,7 +13191,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13270,7 +13273,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Setup scheduled for August 18; confirmation pending</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -13584,7 +13587,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>In Progress—setup confirmation pending</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -14545,7 +14548,7 @@
       </c>
       <c r="I63" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
@@ -14602,7 +14605,7 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
@@ -17672,6 +17675,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -17978,7 +17982,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -22408,12 +22412,12 @@
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Under Shortlisting</t>
+          <t>Shortlisted</t>
         </is>
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>Search by July 2026</t>
+          <t>Laser AI setup preparation; confirmation pending</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
@@ -22421,9 +22425,21 @@
           <t>Phase 1</t>
         </is>
       </c>
-      <c r="F14" s="17" t="n"/>
-      <c r="G14" s="17" t="n"/>
-      <c r="H14" s="17" t="n"/>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>Syeda Kanza Naqvi/Jai Das</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>Setup requested 2026-08-17</t>
+        </is>
+      </c>
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>Initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending</t>
+        </is>
+      </c>
       <c r="I14" s="17" t="inlineStr">
         <is>
           <t>No</t>
@@ -22927,7 +22943,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
+          <t>Withdrawn—conventional work completed; blinding not feasible</t>
         </is>
       </c>
       <c r="E30" s="17" t="inlineStr">
@@ -22942,12 +22958,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Not participating</t>
+          <t>No further action</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Rerun search produced 377 records, but all relevant studies had already been processed. Team formally declined on 2026-08-11.</t>
+          <t>Not suitable because work was already completed and blinding was impossible</t>
         </is>
       </c>
       <c r="I30" s="17" t="inlineStr">
@@ -27426,6 +27442,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -27540,7 +27557,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract screening underway</t>
+          <t>Conventional screening complete; NK screening underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -27608,7 +27625,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Setup phase underway; template revisions and project configuration remain before screening begins</t>
+          <t>Calibration and conventional screening complete; NK screening continuing</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27625,7 +27642,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Setup phase underway; template revisions and project configuration remain before screening begins</t>
+          <t>Calibration and conventional screening complete; NK screening continuing</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27642,7 +27659,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Continue conventional and AI-assisted abstract screening; monitor progress and time logs; then prepare the full-text screening stage.</t>
+          <t>Complete NK screening/time capture, then begin full text</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27676,7 +27693,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Project configuration and screening depend on final data extraction template revisions</t>
+          <t>Conventional workflow ahead; full text awaits both workflows</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -27732,7 +27749,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27831,7 +27848,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Conventional complete; NK in progress</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -27844,6 +27861,11 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>fullText</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Hold until both abstract-screening arms complete</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -28142,9 +28164,14 @@
           <t>Abstract Screening</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Conventional complete; NK in progress</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -28161,7 +28188,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Not Started—sequencing dependency</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -29155,7 +29182,7 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
@@ -29208,7 +29235,7 @@
       </c>
       <c r="I66" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
@@ -32009,6 +32036,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -32123,7 +32151,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup in progress</t>
+          <t>Nested Knowledge setup confirmation pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32191,7 +32219,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Onboarding/training are complete. The team has supplied a deduplicated RIS file with 2,053 records, 35 selected data items, and Study Protocol Info containing inclusion/exclusion/PICOS details. Nested Knowledge configuration can proceed.</t>
+          <t>Search results and data items received; awaiting setup confirmation</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32208,7 +32236,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Onboarding/training are complete. The team has supplied a deduplicated RIS file with 2,053 records, 35 selected data items, and Study Protocol Info containing inclusion/exclusion/PICOS details. Nested Knowledge configuration can proceed.</t>
+          <t>Search results and data items received; awaiting setup confirmation</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32225,7 +32253,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Configure the Nested Knowledge project, confirm screening instructions/calibration, and begin abstract screening once setup is complete.</t>
+          <t>Obtain setup/access/start confirmation</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32242,7 +32270,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD - after setup validation</t>
+          <t>Awaiting setup confirmation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -32259,7 +32287,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Key setup inputs are now received; Nested Knowledge configuration is the next step. Full-text PDFs can be assembled later for the full-text stage.</t>
+          <t>Files available; setup confirmation/document check pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32276,7 +32304,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -32315,7 +32343,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32397,7 +32425,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Waiting on Meghan confirmation</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -32520,7 +32548,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Deduplicated RIS/search file received - 2,053 records.</t>
+          <t>Deduplicated search results received August 3</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -32559,12 +32587,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>To confirm</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Inclusion/exclusion criteria and PICOS received in Study Protocol Info.</t>
+          <t>Final setup-document check pending</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -32586,7 +32614,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>35 selected data-extraction items received.</t>
+          <t>Selected data items received/shared</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -32603,12 +32631,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>To confirm</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Protocol / Study Protocol Info received.</t>
+          <t>Final setup-document check pending</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -32705,7 +32733,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>In Progress—setup confirmation pending</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -33656,7 +33684,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
@@ -36802,6 +36830,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -37108,7 +37137,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -41614,12 +41643,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Data extraction underway</t>
+          <t>Extraction complete; Laser AI access pending</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -41634,22 +41663,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Data extraction is underway in both workflows. Completion was expected during the week of 2026-08-03, but final completion has not yet been confirmed.</t>
+          <t>Both workflow extractions complete; conventional files and time logs received; Laser AI outputs awaiting access</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Confirm whether both workflows have completed data extraction; collect outputs, time logs and usability-survey responses.</t>
+          <t>Resolve Laser AI access, download outputs and begin comparison/adjudication</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>Completion confirmation overdue</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Needs Action</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -41686,12 +41715,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data extraction underway</t>
+          <t>Data-extraction confirmation pending</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -41706,22 +41735,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Abstract and full-text screening are complete in the AI-assisted and conventional workflows. Ten studies are selected for data extraction. Conventional screening time-on-task is now complete; Robin's full-text time was corrected to 4h12. Repeated Laser AI run-validation issues remain provisional.</t>
+          <t>Screening complete; awaiting final extraction files and time records</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Finalise the Nested Knowledge data-extraction workflow; correct Run 10 and resolve the 44 unevaluated citations in Runs 3-5; complete the interim comparison.</t>
+          <t>Obtain final extraction files/time records and complete validation</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Overdue / confirmation required</t>
+          <t>Awaiting review team</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -41758,7 +41787,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AI-assisted abstract screening restarting</t>
+          <t>Full-text workflow decision pending</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -41778,22 +41807,22 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Laser AI work has restarted. AI-assisted abstract screening is expected to recommence; confirmation of actual commencement is pending.</t>
+          <t>Screening substantially complete; decision needed for 128 studies and final 3 abstracts</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Confirm commencement of AI-assisted abstract screening and continue tracking conventional and AI-assisted screening time separately.</t>
+          <t>Obtain team’s preferred option and complete final 3 abstracts</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>TBD - after full-text set reconciliation</t>
+          <t>Awaiting review team</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -41897,7 +41926,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Setup in progress - search strategy/access issue</t>
+          <t>Laser AI setup scheduled/confirmation pending</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -41917,22 +41946,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
+          <t>Documents re-forwarded; setup planned for August 18</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Clarify wildcard use, complete accessible searches, document LILACS/IBECS limitations, finalise Laser AI setup, and confirm the screening start.</t>
+          <t>Confirm setup, access, additional documents and screening start</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -41989,17 +42018,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Future batch planning</t>
+          <t>Planning based on results through mid-October</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Keep placeholders until Phase 1 stabilizes.</t>
+          <t>Review results after mid-October and decide next phase/tool strategy</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>After mid-October 2026</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -42041,7 +42070,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Abstract screening underway</t>
+          <t>Conventional abstract screening complete; NK screening underway</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -42061,12 +42090,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Setup phase underway; template revisions and project configuration remain before screening begins</t>
+          <t>Calibration complete; conventional screening complete; NK screening continuing</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Continue conventional and AI-assisted abstract screening; monitor progress and time logs; then prepare the full-text screening stage.</t>
+          <t>Complete NK screening, record time and then start full text</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -42113,7 +42142,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Setup in progress</t>
+          <t>Nested Knowledge setup confirmation pending</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -42133,22 +42162,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Onboarding/training are complete. The team has supplied a deduplicated RIS file with 2,053 records, 35 selected data items, and Study Protocol Info containing inclusion/exclusion/PICOS details. Nested Knowledge configuration can proceed.</t>
+          <t>Search results and data items received; awaiting Meghan’s setup confirmation</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Configure the Nested Knowledge project, confirm screening instructions/calibration, and begin abstract screening once setup is complete.</t>
+          <t>Obtain setup/access/start confirmation</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>TBD - after setup validation</t>
+          <t>Awaiting setup confirmation</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -45812,12 +45841,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mid April to End June</t>
+          <t>Mid April to mid-October 2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Current Focus</t>
+          <t>Laser AI continues; onboarding active</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -45839,12 +45868,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>End June</t>
+          <t>July–December 2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Decision Gate</t>
+          <t>In progress; CESAR-FM extension initiated</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -45866,12 +45895,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Start July to End September</t>
+          <t>Decision after mid-October results</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Pending results-based decision</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -45893,12 +45922,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>December 2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Final report/project closeout</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -46401,6 +46430,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -46702,7 +46732,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -51166,6 +51196,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -51467,7 +51498,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -55807,6 +55838,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -55921,7 +55953,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data extraction underway</t>
+          <t>Extraction complete; Laser AI access pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -55938,7 +55970,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -55989,7 +56021,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Data extraction is underway in both workflows; final completion has not yet been confirmed.</t>
+          <t>Both extractions complete; conventional outputs received; Laser AI retrieval pending</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56006,7 +56038,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Completion was expected during the week of 2026-08-03; confirmation remains pending.</t>
+          <t>Both extractions complete; conventional outputs received; Laser AI retrieval pending</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56023,7 +56055,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm completion of both extraction workflows and collect outputs, time logs and usability-survey responses.</t>
+          <t>Resolve access, download outputs and begin comparison</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56040,7 +56072,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Completion confirmation overdue</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56057,7 +56089,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Data extraction is underway; completion is now expected during the week of 2026-08-10.</t>
+          <t>Extraction complete; analysis delayed by access</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56074,7 +56106,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Needs Action</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -56113,7 +56145,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56246,7 +56278,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete—outputs submitted</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -56259,6 +56291,11 @@
       <c r="A29" t="inlineStr">
         <is>
           <t>analysis</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Blocked—Laser AI access pending</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -56399,7 +56436,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Conventional extraction received; Laser AI download pending</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -56438,12 +56475,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Conventional and AI time reports received</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -56516,11 +56553,15 @@
           <t>Setup / Coordination</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>0</v>
-      </c>
-      <c r="C42" t="n">
-        <v>0</v>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -56539,11 +56580,15 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43" t="n">
-        <v>0</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0</v>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -56562,11 +56607,15 @@
           <t>Full-text Screening</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>0</v>
-      </c>
-      <c r="C44" t="n">
-        <v>0</v>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -56585,15 +56634,19 @@
           <t>Data Extraction / Analysis</t>
         </is>
       </c>
-      <c r="B45" t="n">
-        <v>0</v>
-      </c>
-      <c r="C45" t="n">
-        <v>0</v>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Extraction complete; analysis access-blocked</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -59160,7 +59213,7 @@
       </c>
       <c r="I95" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J95" s="18" t="n"/>
@@ -59213,7 +59266,7 @@
       </c>
       <c r="I96" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J96" s="18" t="n"/>
@@ -59266,7 +59319,7 @@
       </c>
       <c r="I97" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J97" s="18" t="n"/>
@@ -59319,7 +59372,7 @@
       </c>
       <c r="I98" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J98" s="18" t="n"/>
@@ -61191,6 +61244,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -61305,7 +61359,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data extraction underway</t>
+          <t>Data-extraction confirmation pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -61322,7 +61376,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -61373,7 +61427,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abstract and full-text screening are complete in the AI-assisted and conventional workflows. Ten studies are selected for data extraction. Conventional screening time-on-task is now complete; Robin's full-text time was corrected to 4h12. Repeated Laser AI run-validation issues remain provisional.</t>
+          <t>Screening complete; awaiting final extraction files and times</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -61390,7 +61444,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abstract and full-text screening are complete in the AI-assisted and conventional workflows. Ten studies are selected for data extraction. Conventional screening time-on-task is now complete; Robin's full-text time was corrected to 4h12. Repeated Laser AI run-validation issues remain provisional.</t>
+          <t>Screening complete; awaiting final extraction files and times</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -61407,7 +61461,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Finalise the Nested Knowledge data-extraction workflow; correct Run 10 and resolve the 44 unevaluated citations in Runs 3-5; complete the interim comparison.</t>
+          <t>Obtain final extraction files/times and complete validation</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -61424,7 +61478,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Overdue / confirmation required</t>
+          <t>Awaiting review team</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -61441,7 +61495,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Repeated Laser AI outputs still require validation before final reporting; conventional screening timing has now been received and updated.</t>
+          <t>Final extraction completion and timing unconfirmed</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -61458,7 +61512,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -61497,7 +61551,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -61630,7 +61684,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Status requested 2026-08-17</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -61643,6 +61697,11 @@
       <c r="A29" t="inlineStr">
         <is>
           <t>analysis</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Provisional comparison available; final validation pending</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -61822,12 +61881,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Conventional timing received: Emilie abstract 3h36m10s, full text 12h; Robin abstract 6h35m, full text 4h12m (corrected from 3h06m).</t>
+          <t>Screening times received; extraction time records pending</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -61928,11 +61987,15 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43" t="n">
-        <v>100</v>
-      </c>
-      <c r="C43" t="n">
-        <v>100</v>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -61956,11 +62019,15 @@
           <t>Full-text Screening</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>100</v>
-      </c>
-      <c r="C44" t="n">
-        <v>100</v>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -61992,7 +62059,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Extraction status awaiting review team</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -64564,7 +64631,7 @@
       </c>
       <c r="I95" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J95" s="18" t="n"/>
@@ -64617,7 +64684,7 @@
       </c>
       <c r="I96" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J96" s="18" t="n"/>

</xml_diff>

<commit_message>
Replace Oral Galactagogues with LNS review
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -25,7 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-08 Oral Galactagogues" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-08 LNS" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -2287,7 +2287,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -7859,7 +7858,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -12884,7 +12882,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -17675,7 +17672,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -22412,12 +22408,12 @@
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Shortlisted</t>
+          <t>Converted to full sheet</t>
         </is>
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>Laser AI setup preparation; confirmation pending</t>
+          <t>Converted to phase1-08; Laser AI setup preparation and confirmation pending</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
@@ -22427,7 +22423,7 @@
       </c>
       <c r="F14" s="17" t="inlineStr">
         <is>
-          <t>Syeda Kanza Naqvi/Jai Das</t>
+          <t>Syeda Kanza Naqvi / Jai Das</t>
         </is>
       </c>
       <c r="G14" s="17" t="inlineStr">
@@ -22437,17 +22433,17 @@
       </c>
       <c r="H14" s="17" t="inlineStr">
         <is>
-          <t>Initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending</t>
+          <t>Converted to phase1-08 LNS; initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending</t>
         </is>
       </c>
       <c r="I14" s="17" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -27442,7 +27438,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -32036,7 +32031,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -36823,7 +36817,7 @@
     <row r="1" ht="18" customHeight="1" s="29">
       <c r="A1" s="28" t="inlineStr">
         <is>
-          <t>phase1-08 Oral Galactagogues | Dashboard Content Sheet</t>
+          <t>phase1-08 LNS | Dashboard Content Sheet</t>
         </is>
       </c>
       <c r="K1" s="18" t="n"/>
@@ -36894,7 +36888,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Oral Galactagogues</t>
+          <t>LNS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -36911,7 +36905,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Oral galactagogues (natural therapies or drugs) for increasing breast milk production in mothers of non-hospitalised term infants</t>
+          <t>Preventive lipid-based nutrient supplements given with complementary foods to infants and young children 6 to 23 months of age for health, nutrition, and developmental outcomes</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -36945,7 +36939,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Laser AI setup preparation; confirmation pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -36979,7 +36973,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Laser AI</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -36996,7 +36990,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Siew Cheng Foong</t>
+          <t>Syeda Kanza Naqvi / Jai Das</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -37013,7 +37007,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
+          <t>Initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -37030,7 +37024,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
+          <t>Initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -37047,7 +37041,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Retain as withdrawn/historical record; no active onboarding or tool setup required.</t>
+          <t>Confirm Laser AI setup preparation, complete setup confirmation, and agree screening start plan.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -37064,7 +37058,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>Setup requested 2026-08-17</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -37081,7 +37075,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Rerun search produced 377 records, but all relevant studies had already been processed. Team formally declined on 2026-08-11.</t>
+          <t>Laser AI setup preparation is active; setup confirmation is still pending.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -37098,7 +37092,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -37202,7 +37196,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -37217,6 +37211,11 @@
           <t>setup</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Setup requested 2026-08-17</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37231,7 +37230,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Withdrawn - not participating</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -37248,7 +37247,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rerun search produced 377 records, but all relevant studies had already been processed. Team formally declined on 2026-08-11.</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -37263,6 +37262,11 @@
           <t>extraction</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37273,6 +37277,11 @@
       <c r="A29" t="inlineStr">
         <is>
           <t>analysis</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -37347,7 +37356,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Initial files received</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -37391,7 +37400,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Protocol/eligibility confirmation pending</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -37413,7 +37422,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Data items/setup confirmation pending</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -37435,7 +37444,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Protocol/criteria confirmation pending</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -37538,7 +37547,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>In Progress - setup confirmation pending</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -37566,7 +37575,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -37589,7 +37598,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -37612,7 +37621,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -37957,7 +37966,7 @@
       </c>
       <c r="I53" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J53" s="18" t="inlineStr"/>
@@ -38010,7 +38019,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J54" s="18" t="inlineStr"/>
@@ -38062,7 +38071,7 @@
       </c>
       <c r="I55" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J55" s="18" t="inlineStr"/>
@@ -38115,7 +38124,7 @@
       </c>
       <c r="I56" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J56" s="18" t="inlineStr"/>
@@ -38168,7 +38177,7 @@
       </c>
       <c r="I57" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J57" s="18" t="inlineStr"/>
@@ -38221,7 +38230,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J58" s="18" t="inlineStr"/>
@@ -38273,7 +38282,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J59" s="18" t="inlineStr"/>
@@ -38325,7 +38334,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J60" s="18" t="inlineStr"/>
@@ -38377,7 +38386,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J61" s="18" t="inlineStr"/>
@@ -38429,7 +38438,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J62" s="18" t="inlineStr"/>
@@ -38481,7 +38490,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J63" s="18" t="inlineStr"/>
@@ -42199,12 +42208,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Oral Galactagogues</t>
+          <t>LNS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Oral galactagogues (natural therapies or drugs) for increasing breast milk production in mothers of non-hospitalised term infants</t>
+          <t>Preventive lipid-based nutrient supplements given with complementary foods to infants and young children 6 to 23 months of age for health, nutrition, and developmental outcomes</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -42214,7 +42223,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Laser AI setup preparation; confirmation pending</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -42224,32 +42233,32 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Laser AI</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Siew Cheng Foong</t>
+          <t>Syeda Kanza Naqvi / Jai Das</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
+          <t>Initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Retain as withdrawn/historical record; no active onboarding or tool setup required.</t>
+          <t>Confirm Laser AI setup preparation, complete setup confirmation, and agree screening start plan.</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>Setup requested 2026-08-17</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -42259,7 +42268,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>phase1-08 Oral Galactagogues</t>
+          <t>phase1-08 LNS</t>
         </is>
       </c>
     </row>
@@ -46430,7 +46439,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -51196,7 +51204,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -55838,7 +55845,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -61244,7 +61250,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update dashboard through August 20
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text workflow decision pending</t>
+          <t>Abstract screening complete; full-text setup underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Screening substantially complete; decision pending for 128 studies and 3 abstracts</t>
+          <t>Abstract-screening discrepancies resolved; PDFs for 145 full-text records uploaded</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Screening substantially complete; decision pending for 128 studies and 3 abstracts</t>
+          <t>Abstract-screening discrepancies resolved; PDFs for 145 full-text records uploaded</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Obtain team’s selected option and finish 3 abstracts</t>
+          <t>Confirm full-text setup and commence both screening arms</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2520,7 +2520,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting review team</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Full-text work held pending workflow decision</t>
+          <t>Full-text setup awaiting final confirmation</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Substantially complete—3 abstracts pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Decision pending for 128 studies</t>
+          <t>Setup underway-145 records</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2825,12 +2825,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Shared folder provided; PDFs being collected/uploaded for full-text screening.</t>
+          <t>PDFs for 17 plus 128 records uploaded to SharePoint</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Full-text decision flow and eligibility criteria configured; minor amendments under review.</t>
+          <t>Updated full-text decision flow submitted</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3027,12 +3027,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Substantially complete—3 abstracts pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Conventional screening commenced; AI-assisted screening restart is being confirmed.</t>
+          <t>Both title/abstract arms complete; discrepant records reconciled</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3055,12 +3055,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Blocked—workflow option pending</t>
+          <t>Setup in progress</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Awaiting conventional export/DOIs, decision on 128 prior records, PDF-sharing method and final decision flow.</t>
+          <t>Superset confirmed; 145 PDFs uploaded; awaiting project readiness confirmation</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
@@ -4060,14 +4060,14 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
       <c r="K65" s="18" t="n"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Conventional abstract screening complete; export and DOIs awaited.</t>
+          <t>Conventional abstract screening complete</t>
         </is>
       </c>
       <c r="M65" s="18" t="inlineStr">
@@ -4451,14 +4451,14 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J72" s="18" t="n"/>
       <c r="K72" s="18" t="n"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Reconcile conventional export with AI output and determine treatment of 128 prior records.</t>
+          <t>Superset principle confirmed and discrepancies reconciled</t>
         </is>
       </c>
       <c r="M72" s="18" t="inlineStr">
@@ -4561,14 +4561,14 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>PDF-sharing method and complete full-text record set are being confirmed.</t>
+          <t>PDFs for 145 records uploaded on 10 August</t>
         </is>
       </c>
       <c r="M74" s="18" t="inlineStr">
@@ -4781,14 +4781,14 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Full-text workflow setup awaits record/PDF reconciliation and final criteria.</t>
+          <t>Full-text project being prepared using the combined record set</t>
         </is>
       </c>
       <c r="M78" s="18" t="inlineStr">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="D120" s="23" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete / No longer required</t>
         </is>
       </c>
       <c r="E120" s="23" t="inlineStr">
@@ -6969,7 +6969,7 @@
       </c>
       <c r="D121" s="23" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete / No longer required</t>
         </is>
       </c>
       <c r="E121" s="23" t="inlineStr">
@@ -7024,7 +7024,7 @@
       </c>
       <c r="D122" s="23" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete / No longer required</t>
         </is>
       </c>
       <c r="E122" s="23" t="inlineStr">
@@ -7700,7 +7700,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Methodology re-onboarding still pending</t>
+          <t>Re-onboarding no longer required</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -7720,7 +7720,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -7737,7 +7737,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Human abstract screening status not confirmed</t>
+          <t>Human abstract screening confirmed complete</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -7757,7 +7757,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -7774,7 +7774,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Updated search completion not confirmed</t>
+          <t>Updated search confirmed complete</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -7794,7 +7794,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -12996,7 +12996,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Laser AI setup scheduled/confirmation pending</t>
+          <t>Laser AI setup complete; decision-flow approval pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -13064,7 +13064,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Documents re-forwarded; setup planned for August 18</t>
+          <t>Laser AI project created with 3,486 deduplicated references</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13081,7 +13081,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Documents re-forwarded; setup planned for August 18</t>
+          <t>Laser AI project created with 3,486 deduplicated references</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13098,7 +13098,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm setup, access, documents and start date</t>
+          <t>Review team to approve decision flow; then provide access and start screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13115,7 +13115,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>Awaiting review team approval</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -13132,7 +13132,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Documents re-shared; setup/access confirmation pending</t>
+          <t>Setup complete; screening awaits validation</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -13188,7 +13188,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13270,7 +13270,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Setup scheduled for August 18; confirmation pending</t>
+          <t>Complete-3,486 references uploaded</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -13283,6 +13283,11 @@
       <c r="A26" t="inlineStr">
         <is>
           <t>abstract</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Awaiting decision-flow approval</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -13388,12 +13393,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Search/RIS files partly available; additional searches await wildcard clarification; LILACS/IBECS remain inaccessible.</t>
+          <t>3,486 deduplicated references uploaded to Laser AI</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -13432,12 +13437,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Eligibility criteria received in protocol</t>
+          <t>Decision flow prepared; review-team approval pending</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -13454,12 +13459,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Selected data items finalized and saved to SharePoint</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -13476,12 +13481,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Protocol available in SharePoint</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -13584,12 +13589,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>In Progress—setup confirmation pending</t>
+          <t>Setup complete-validation pending</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Protocol and data items complete; search strategy/database access issues remain.</t>
+          <t>Project configured; decision flow awaiting team approval</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -14264,12 +14269,16 @@
       </c>
       <c r="I58" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J58" s="18" t="n"/>
       <c r="K58" s="18" t="n"/>
-      <c r="L58" s="18" t="n"/>
+      <c r="L58" s="18" t="inlineStr">
+        <is>
+          <t>3,486 deduplicated references uploaded</t>
+        </is>
+      </c>
       <c r="M58" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14545,14 +14554,14 @@
       </c>
       <c r="I63" s="18" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Laser AI setup awaits final search set and search-strategy resolution.</t>
+          <t>Laser AI abstract-screening project configured</t>
         </is>
       </c>
       <c r="M63" s="18" t="inlineStr">
@@ -14607,7 +14616,11 @@
       </c>
       <c r="J64" s="18" t="n"/>
       <c r="K64" s="18" t="n"/>
-      <c r="L64" s="18" t="n"/>
+      <c r="L64" s="18" t="inlineStr">
+        <is>
+          <t>Awaiting review-team approval of decision flow</t>
+        </is>
+      </c>
       <c r="M64" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -17182,17 +17195,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Identify additional eligible review</t>
+          <t>Approve Vitamin C decision flow</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Core Team</t>
+          <t>Syeda Kanza Naqvi / Jai Das</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -17202,27 +17215,27 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>Awaiting review team approval</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Candidate pool</t>
+          <t>Laser AI setup complete</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Shortlist review options.</t>
+          <t>Decision flow prepared; approval required before screening begins.</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Project tracking</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -17239,37 +17252,37 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Confirm team availability after candidate selection</t>
+          <t>Provide Laser AI access to allocated users</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Krishna / Review Team</t>
+          <t>Response Team / Laser AI</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>After decision-flow approval</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Review identification</t>
+          <t>Decision-flow approval</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Contact review team once candidate is selected.</t>
+          <t>Provide reviewer access after the team approves the configured flow.</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -17279,7 +17292,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -17296,12 +17309,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Assign allocated AI tool after candidate selection</t>
+          <t>Start parallel abstract screening and time tracking</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Core Team</t>
+          <t>Review Team / Krishna</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -17316,17 +17329,17 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>After access</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Tool allocation</t>
+          <t>Tool access and team readiness</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Assign one tool only after a review is selected.</t>
+          <t>Begin both screening arms and confirm time-tracking method.</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -17336,7 +17349,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -17353,37 +17366,37 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Hold onboarding until review is confirmed</t>
+          <t>Confirm finalized SharePoint package</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Krishna / Response Team</t>
+          <t>Krishna / Review Team</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>After confirmation</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Review and tool confirmation</t>
+          <t>Protocol, criteria and data items</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Start onboarding only after candidate and tool are confirmed.</t>
+          <t>Confirm the SharePoint package contains final protocol, criteria and selected data items.</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -17393,7 +17406,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -17402,6 +17415,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -17479,11 +17493,7 @@
           <t>SourceLink</t>
         </is>
       </c>
-      <c r="M121" s="1" t="inlineStr">
-        <is>
-          <t>Display</t>
-        </is>
-      </c>
+      <c r="M121" s="1" t="n"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -17493,37 +17503,37 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Additional Phase 1 review slot</t>
+          <t>Vitamin C setup completed</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Core Team</t>
+          <t>Krishna / Response Team / Review Team</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Krishna / Core Team</t>
+          <t>Review Team</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>Awaiting review team approval</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>One additional eligible review still needs to be identified or confirmed for Phase 1.</t>
+          <t>Laser AI project created with 3,486 deduplicated references; decision-flow approval is the next gating step.</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -17533,20 +17543,16 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Identify additional eligible review</t>
+          <t>Approve Vitamin C decision flow</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Project tracking</t>
-        </is>
-      </c>
-      <c r="M122" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -17603,7 +17609,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Open Phase 1 review slot</t>
+          <t>Decision-flow approval pending</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -17611,9 +17617,24 @@
           <t>High</t>
         </is>
       </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Syeda Kanza Naqvi / Jai Das</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Awaiting review team approval</t>
+        </is>
+      </c>
       <c r="E126" t="inlineStr">
         <is>
           <t>Open</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Screening cannot start until the configured decision flow is approved.</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -22309,7 +22330,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Converted to phase1-07; setup inputs complete and Nested Knowledge configuration underway</t>
+          <t>Converted to phase1-07; Nested Knowledge setup complete and criteria approval pending</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22319,12 +22340,12 @@
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>Mohan Pammi</t>
+          <t>Mohan Pammi / Murali</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Configuration and setup validation underway</t>
+          <t>Awaiting Murali's screening-criteria approval</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -22351,7 +22372,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>Amanda Cross ? Interventions for improving medication-taking ability and adherence in older adults prescribed multiple medications</t>
+          <t>Amanda Cross - Interventions for improving medication-taking ability and adherence in older adults prescribed multiple medications</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
@@ -22413,7 +22434,7 @@
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-08; Laser AI setup preparation and confirmation pending</t>
+          <t>Converted to phase1-08; Laser AI setup started with four database searches outstanding</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
@@ -22428,7 +22449,7 @@
       </c>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>Setup requested 2026-08-17</t>
+          <t>Awaiting four searches</t>
         </is>
       </c>
       <c r="H14" s="17" t="inlineStr">
@@ -22465,7 +22486,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Protocol, criteria and 35 data items received; accessible searches underway; wildcard and LILACS/IBECS issues remain</t>
+          <t>Converted to phase1-05; Laser AI setup completed with 3,486 references; decision-flow approval pending</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
@@ -22480,7 +22501,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Setup in progress; screening awaits final search resolution</t>
+          <t>Awaiting review team approval</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -22835,7 +22856,7 @@
       </c>
       <c r="D28" s="17" t="inlineStr">
         <is>
-          <t>Onboarding and tool training completed; awaiting final template revisions</t>
+          <t>Converted to phase1-06; conventional screening complete, Nested Knowledge screening underway and full text deliberately paused</t>
         </is>
       </c>
       <c r="E28" s="17" t="inlineStr">
@@ -22850,7 +22871,7 @@
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>Awaiting final template revisions</t>
+          <t>Full text paused until Nested Knowledge abstract screening complete</t>
         </is>
       </c>
       <c r="H28" s="17" t="inlineStr">
@@ -23130,15 +23151,56 @@
       </c>
     </row>
     <row r="34" ht="24" customHeight="1" s="29">
-      <c r="A34" s="17" t="n"/>
-      <c r="B34" s="17" t="n"/>
-      <c r="C34" s="17" t="n"/>
-      <c r="D34" s="17" t="n"/>
-      <c r="E34" s="17" t="n"/>
-      <c r="F34" s="17" t="n"/>
-      <c r="G34" s="17" t="n"/>
-      <c r="H34" s="17" t="n"/>
-      <c r="I34" s="17" t="n"/>
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>new-23</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>Michelle Butler - Hospital nurse staffing review</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>Under Shortlisting</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>Interested; search expected to be completed and screening ready at the end of September</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>Phase 1 / timeline assessment</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>Michelle Butler</t>
+        </is>
+      </c>
+      <c r="G34" s="17" t="inlineStr">
+        <is>
+          <t>End of September 2026</t>
+        </is>
+      </c>
+      <c r="H34" s="17" t="inlineStr">
+        <is>
+          <t>Standard eligibility and workflow questions sent; awaiting detailed response</t>
+        </is>
+      </c>
+      <c r="I34" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="24" customHeight="1" s="29">
       <c r="A35" s="17" t="n"/>
@@ -27149,7 +27211,7 @@
       </c>
       <c r="J5" s="25" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>No longer required</t>
         </is>
       </c>
       <c r="K5" s="25" t="inlineStr">
@@ -27160,7 +27222,7 @@
       <c r="L5" s="25" t="n"/>
       <c r="M5" s="25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -27170,7 +27232,11 @@
           <t>mtg-06</t>
         </is>
       </c>
-      <c r="B6" s="25" t="n"/>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
       <c r="C6" s="25" t="n"/>
       <c r="D6" s="25" t="n"/>
       <c r="E6" s="25" t="inlineStr">
@@ -27200,7 +27266,7 @@
       </c>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="K6" s="25" t="inlineStr">
@@ -27211,7 +27277,7 @@
       <c r="L6" s="25" t="n"/>
       <c r="M6" s="25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -27221,7 +27287,11 @@
           <t>mtg-07</t>
         </is>
       </c>
-      <c r="B7" s="25" t="n"/>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="C7" s="25" t="n"/>
       <c r="D7" s="25" t="n"/>
       <c r="E7" s="25" t="inlineStr">
@@ -27251,7 +27321,7 @@
       </c>
       <c r="J7" s="25" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="K7" s="25" t="inlineStr">
@@ -27262,7 +27332,7 @@
       <c r="L7" s="25" t="n"/>
       <c r="M7" s="25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -27373,17 +27443,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Scheduled</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>phase1-08</t>
+          <t>Completed; team subsequently withdrew</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -27744,7 +27809,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27860,7 +27925,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Hold until both abstract-screening arms complete</t>
+          <t>On hold until Nested Knowledge abstract screening is complete</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -28186,6 +28251,11 @@
           <t>Not Started—sequencing dependency</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Team confirmed that Covidence full-text screening will remain paused</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -31699,52 +31769,52 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>task-phase1-05-001</t>
+          <t>task-phase1-06-001</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Identify additional eligible review</t>
+          <t>Complete Nested Knowledge abstract screening</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Core Team</t>
+          <t>Review Team / Nested Knowledge</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Candidate pool</t>
+          <t>NK screening completion</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Shortlist review options.</t>
+          <t>Continue NK abstract screening before full-text work resumes.</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Project tracking</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -31756,52 +31826,52 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>task-phase1-05-002</t>
+          <t>task-phase1-06-002</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Confirm team availability after candidate selection</t>
+          <t>Keep Covidence full-text screening paused</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Krishna / Review Team</t>
+          <t>Jeremy Steen / Bradley Johnston</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Review identification</t>
+          <t>Parallel workflow sequencing</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Contact review team once candidate is selected.</t>
+          <t>Conventional full-text screening will remain paused until NK abstract screening finishes.</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Project tracking</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -31813,12 +31883,42 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>task-phase1-05-003</t>
+          <t>task-phase1-06-003</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Confirm NK screening completion and export</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Review Team / Response Team</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>After NK screening</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>NK abstract screening</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Assign one tool only after a review is selected.</t>
+          <t>Export output once NK screening is complete.</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -31828,7 +31928,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -31840,12 +31940,42 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>task-phase1-05-004</t>
+          <t>task-phase1-06-004</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Start full-text screening after both arms align</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Review Team / Response Team</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>After abstract-screening closeout</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>NK and conventional abstract-screening completion</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Start onboarding only after candidate and tool are confirmed.</t>
+          <t>Resume full-text workflow only after abstract-screening outputs are ready.</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -31855,7 +31985,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -31864,6 +31994,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -31886,12 +32017,36 @@
           <t>CommunicationID</t>
         </is>
       </c>
-      <c r="B121" s="1" t="n"/>
-      <c r="C121" s="1" t="n"/>
-      <c r="D121" s="1" t="n"/>
-      <c r="E121" s="1" t="n"/>
-      <c r="F121" s="1" t="n"/>
-      <c r="G121" s="1" t="n"/>
+      <c r="B121" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C121" s="1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="D121" s="1" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E121" s="1" t="inlineStr">
+        <is>
+          <t>Responsible</t>
+        </is>
+      </c>
+      <c r="F121" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="G121" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
       <c r="H121" s="1" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -31917,44 +32072,66 @@
           <t>SourceLink</t>
         </is>
       </c>
-      <c r="M121" s="1" t="inlineStr">
-        <is>
-          <t>Display</t>
-        </is>
-      </c>
+      <c r="M121" s="1" t="n"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>comm-phase1-05-001</t>
+          <t>comm-phase1-06-001</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Probiotics full text paused</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Jeremy Steen / Bradley Johnston / Krishna</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>After NK abstract screening</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>One additional eligible review still needs to be identified or confirmed for Phase 1.</t>
+          <t>Team confirmed Covidence full-text screening will remain paused until Nested Knowledge abstract screening is complete.</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>task-phase1-05-001</t>
+          <t>task-phase1-06-001</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Identify additional eligible review</t>
+          <t>Complete Nested Knowledge abstract screening</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Project tracking</t>
-        </is>
-      </c>
-      <c r="M122" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -31977,17 +32154,71 @@
           <t>CriticalItem</t>
         </is>
       </c>
-      <c r="B125" s="1" t="n"/>
-      <c r="C125" s="1" t="n"/>
-      <c r="D125" s="1" t="n"/>
-      <c r="E125" s="1" t="n"/>
-      <c r="F125" s="1" t="n"/>
-      <c r="G125" s="1" t="n"/>
+      <c r="B125" s="1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="C125" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D125" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="E125" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F125" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G125" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Open Phase 1 review slot</t>
+          <t>Full-text screening deliberately paused</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>After NK abstract screening</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Sequencing dependency is intentional and should be monitored.</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -32145,7 +32376,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Nested Knowledge setup confirmation pending</t>
+          <t>Nested Knowledge setup complete; criteria validation pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32213,7 +32444,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Search results and data items received; awaiting setup confirmation</t>
+          <t>NK project created with 2,024 references; awaiting Murali's screening-criteria approval</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32230,7 +32461,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Search results and data items received; awaiting setup confirmation</t>
+          <t>NK project created with 2,024 references; awaiting Murali's screening-criteria approval</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32247,7 +32478,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Obtain setup/access/start confirmation</t>
+          <t>Confirm access and approve abstract/full-text criteria before screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32264,7 +32495,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting setup confirmation</t>
+          <t>Awaiting review team approval</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -32281,7 +32512,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Files available; setup confirmation/document check pending</t>
+          <t>Setup complete; screening not yet started</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32337,7 +32568,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32419,7 +32650,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Waiting on Meghan confirmation</t>
+          <t>Complete-validation pending</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -32432,6 +32663,11 @@
       <c r="A26" t="inlineStr">
         <is>
           <t>abstract</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Awaiting criteria approval</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -32581,12 +32817,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>To confirm</t>
+          <t>Pending approval</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Final setup-document check pending</t>
+          <t>Abstract and full-text criteria configured; Murali review pending</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -32625,12 +32861,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>To confirm</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Final setup-document check pending</t>
+          <t>Published review accepted in lieu of a separate protocol</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -32727,12 +32963,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>In Progress—setup confirmation pending</t>
+          <t>Setup complete-validation pending</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Setup inputs are complete; Nested Knowledge configuration and validation are next.</t>
+          <t>NK project contains 2,024 references; screening criteria awaiting approval</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -33234,12 +33470,16 @@
       </c>
       <c r="I55" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J55" s="18" t="n"/>
       <c r="K55" s="18" t="n"/>
-      <c r="L55" s="18" t="n"/>
+      <c r="L55" s="18" t="inlineStr">
+        <is>
+          <t>Murali invited using both email addresses; access confirmation pending</t>
+        </is>
+      </c>
       <c r="M55" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33678,14 +33918,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Nested Knowledge configuration is the next operational step.</t>
+          <t>Initial NK project setup completed with 2,024 references</t>
         </is>
       </c>
       <c r="M63" s="18" t="inlineStr">
@@ -33735,12 +33975,16 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
       <c r="K64" s="18" t="n"/>
-      <c r="L64" s="18" t="n"/>
+      <c r="L64" s="18" t="inlineStr">
+        <is>
+          <t>Murali to approve abstract and full-text criteria</t>
+        </is>
+      </c>
       <c r="M64" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -36310,17 +36554,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>task-phase1-05-001</t>
+          <t>task-phase1-07-001</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Identify additional eligible review</t>
+          <t>Confirm Murali's Nested Knowledge access</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Core Team</t>
+          <t>Murali / Response Team</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -36335,27 +36579,27 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>Awaiting review team approval</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Candidate pool</t>
+          <t>NK invitation</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Shortlist review options.</t>
+          <t>Murali invited using both email addresses; access confirmation pending.</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Project tracking</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -36367,42 +36611,42 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>task-phase1-05-002</t>
+          <t>task-phase1-07-002</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Confirm team availability after candidate selection</t>
+          <t>Approve abstract and full-text criteria</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Krishna / Review Team</t>
+          <t>Murali / Review Team</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Awaiting review team approval</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Review identification</t>
+          <t>NK project setup</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Contact review team once candidate is selected.</t>
+          <t>Screening criteria configured and awaiting Murali's approval.</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -36412,7 +36656,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -36424,12 +36668,42 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>task-phase1-05-003</t>
+          <t>task-phase1-07-003</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Begin Nested Knowledge screening after validation</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Review Team / Nested Knowledge</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>After criteria approval</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Access and criteria approval</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Assign one tool only after a review is selected.</t>
+          <t>Start screening once access and criteria validation are confirmed.</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -36439,7 +36713,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -36451,12 +36725,42 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>task-phase1-05-004</t>
+          <t>task-phase1-07-004</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Confirm published review/protocol package</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Krishna / Review Team</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Protocol replacement</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Start onboarding only after candidate and tool are confirmed.</t>
+          <t>Published review accepted in lieu of a separate protocol.</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -36466,7 +36770,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -36475,6 +36779,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -36497,12 +36802,36 @@
           <t>CommunicationID</t>
         </is>
       </c>
-      <c r="B121" s="1" t="n"/>
-      <c r="C121" s="1" t="n"/>
-      <c r="D121" s="1" t="n"/>
-      <c r="E121" s="1" t="n"/>
-      <c r="F121" s="1" t="n"/>
-      <c r="G121" s="1" t="n"/>
+      <c r="B121" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C121" s="1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="D121" s="1" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E121" s="1" t="inlineStr">
+        <is>
+          <t>Responsible</t>
+        </is>
+      </c>
+      <c r="F121" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="G121" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
       <c r="H121" s="1" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -36528,44 +36857,66 @@
           <t>SourceLink</t>
         </is>
       </c>
-      <c r="M121" s="1" t="inlineStr">
-        <is>
-          <t>Display</t>
-        </is>
-      </c>
+      <c r="M121" s="1" t="n"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>comm-phase1-05-001</t>
+          <t>comm-phase1-07-001</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Human Milk NK setup complete</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Krishna / Murali / Response Team</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Murali / Review Team</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Awaiting review team approval</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>One additional eligible review still needs to be identified or confirmed for Phase 1.</t>
+          <t>NK project contains 2,024 references; Murali's access and screening-criteria approval remain the next actions.</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>task-phase1-05-001</t>
+          <t>task-phase1-07-002</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Identify additional eligible review</t>
+          <t>Approve abstract and full-text criteria</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Project tracking</t>
-        </is>
-      </c>
-      <c r="M122" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -36588,17 +36939,71 @@
           <t>CriticalItem</t>
         </is>
       </c>
-      <c r="B125" s="1" t="n"/>
-      <c r="C125" s="1" t="n"/>
-      <c r="D125" s="1" t="n"/>
-      <c r="E125" s="1" t="n"/>
-      <c r="F125" s="1" t="n"/>
-      <c r="G125" s="1" t="n"/>
+      <c r="B125" s="1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="C125" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D125" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="E125" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F125" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G125" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Open Phase 1 review slot</t>
+          <t>Criteria approval pending</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Murali / Review Team</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Awaiting review team approval</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Abstract and full-text screening should not start until criteria are approved.</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -36824,7 +37229,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -36939,7 +37343,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Laser AI setup preparation; confirmation pending</t>
+          <t>Laser AI setup started; four searches outstanding</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -37007,7 +37411,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending.</t>
+          <t>Initial setup started; selected data items finalized; completion awaits four database searches</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -37024,7 +37428,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending.</t>
+          <t>Initial setup started; selected data items finalized; completion awaits four database searches</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -37041,7 +37445,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm Laser AI setup preparation, complete setup confirmation, and agree screening start plan.</t>
+          <t>Obtain four remaining searches, complete upload and validate decision flow</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -37058,7 +37462,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Setup requested 2026-08-17</t>
+          <t>Awaiting four searches</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -37075,7 +37479,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Laser AI setup preparation is active; setup confirmation is still pending.</t>
+          <t>Setup partially complete; final search set unavailable</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -37131,7 +37535,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -37213,7 +37617,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Setup requested 2026-08-17</t>
+          <t>In progress-four searches outstanding</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -37351,12 +37755,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Initial files received</t>
+          <t>Initial files received; four database searches outstanding</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -37417,12 +37821,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Data items/setup confirmation pending</t>
+          <t>Selected data items saved with minor clarifications</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -37547,12 +37951,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>In Progress - setup confirmation pending</t>
+          <t>In progress-search set incomplete</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Onboarding confirmed; tool allocation and setup to follow.</t>
+          <t>Laser AI setup started; cannot be completed until four remaining searches arrive</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -38334,11 +38738,16 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J60" s="18" t="inlineStr"/>
       <c r="K60" s="18" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Selected data items finalized and saved</t>
+        </is>
+      </c>
       <c r="M60" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -38490,11 +38899,16 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J63" s="18" t="inlineStr"/>
       <c r="K63" s="18" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Initial setup started; final upload awaits four searches</t>
+        </is>
+      </c>
       <c r="M63" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -41122,17 +41536,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Complete onboarding and confirm tool-training/setup plan</t>
+          <t>Obtain four outstanding database searches</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Krishna / Siew Cheng Foong / Project Team</t>
+          <t>Syeda Kanza Naqvi / Jai Das</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -41142,17 +41556,17 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>Awaiting four searches</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Onboarding meeting</t>
+          <t>Search completion</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Onboarding confirmed; tool training and setup to follow.</t>
+          <t>Four remaining database searches are needed before final upload and validation can complete.</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -41162,7 +41576,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -41262,37 +41676,37 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Oral galactagogues onboarding confirmed</t>
+          <t>LNS Laser AI setup started</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Siew Cheng Foong / review team / Cochrane elective students / project team</t>
+          <t>Syeda Kanza Naqvi / Jai Das / Krishna</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Krishna</t>
+          <t>Review Team</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>Awaiting four searches</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Initial onboarding will cover the study and parallel workflow; tool training and setup will be scheduled afterward.</t>
+          <t>Initial setup started and selected data items saved; final upload awaits four outstanding database searches.</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -41302,7 +41716,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Complete onboarding and confirm tool-training/setup plan</t>
+          <t>Obtain four outstanding database searches</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -41652,7 +42066,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Extraction complete; Laser AI access pending</t>
+          <t>Extraction complete; analysis access partially restored</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -41672,12 +42086,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Both workflow extractions complete; conventional files and time logs received; Laser AI outputs awaiting access</t>
+          <t>Both extractions complete; Krishna's Laser AI access restored; project visibility, Sean's access and output retrieval require confirmation</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Resolve Laser AI access, download outputs and begin comparison/adjudication</t>
+          <t>Verify BP project access, download Laser AI outputs and begin comparison</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
@@ -41796,7 +42210,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Full-text workflow decision pending</t>
+          <t>Abstract screening complete; full-text setup underway</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -41816,22 +42230,22 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Screening substantially complete; decision needed for 128 studies and final 3 abstracts</t>
+          <t>Screening discrepancy resolved; PDFs for 145 records uploaded; full-text setup awaiting confirmation</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Obtain team’s preferred option and complete final 3 abstracts</t>
+          <t>Confirm full-text project readiness and commence parallel full-text screening</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Awaiting review team</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -41935,7 +42349,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Laser AI setup scheduled/confirmation pending</t>
+          <t>Laser AI setup complete; decision-flow approval pending</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -41955,17 +42369,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Documents re-forwarded; setup planned for August 18</t>
+          <t>Laser AI project created with 3,486 deduplicated references</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Confirm setup, access, additional documents and screening start</t>
+          <t>Obtain decision-flow approval, provide reviewer access and begin screening</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>Awaiting review team approval</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -42151,7 +42565,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Nested Knowledge setup confirmation pending</t>
+          <t>Nested Knowledge setup complete; criteria validation pending</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -42171,17 +42585,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Search results and data items received; awaiting Meghan’s setup confirmation</t>
+          <t>NK project created with 2,024 references; documents uploaded; awaiting Murali's screening-criteria approval</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Obtain setup/access/start confirmation</t>
+          <t>Confirm Murali's access and criteria approval, then begin screening</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Awaiting setup confirmation</t>
+          <t>Awaiting review team approval</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -42223,7 +42637,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Laser AI setup preparation; confirmation pending</t>
+          <t>Laser AI setup started; four searches outstanding</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -42243,17 +42657,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending.</t>
+          <t>Initial setup started; selected data items saved; completion awaits results from four remaining database searches</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Confirm Laser AI setup preparation, complete setup confirmation, and agree screening start plan.</t>
+          <t>Obtain four outstanding searches, complete upload and validate the decision flow</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Setup requested 2026-08-17</t>
+          <t>Awaiting four searches</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -55959,7 +56373,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Extraction complete; Laser AI access pending</t>
+          <t>Extraction complete; analysis access partially restored</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56027,7 +56441,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Both extractions complete; conventional outputs received; Laser AI retrieval pending</t>
+          <t>Both extractions complete; Krishna's Laser AI access restored; output retrieval and Sean's access require confirmation</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56044,7 +56458,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Both extractions complete; conventional outputs received; Laser AI retrieval pending</t>
+          <t>Both extractions complete; Krishna's Laser AI access restored; output retrieval and Sean's access require confirmation</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56061,7 +56475,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Resolve access, download outputs and begin comparison</t>
+          <t>Verify project visibility, download Laser AI outputs and begin comparison</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56095,7 +56509,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Extraction complete; analysis delayed by access</t>
+          <t>Extraction complete; analysis pending output retrieval</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56151,7 +56565,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56301,7 +56715,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Blocked—Laser AI access pending</t>
+          <t>Access restored for Krishna; output retrieval and Sean access to confirm</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -56442,7 +56856,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Conventional extraction received; Laser AI download pending</t>
+          <t>Conventional extraction received; Laser AI output retrieval pending</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -57099,12 +57513,16 @@
       </c>
       <c r="I55" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J55" s="18" t="n"/>
       <c r="K55" s="18" t="n"/>
-      <c r="L55" s="18" t="n"/>
+      <c r="L55" s="18" t="inlineStr">
+        <is>
+          <t>Krishna can log in; confirm BP project visibility and Sean's access</t>
+        </is>
+      </c>
       <c r="M55" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -57629,7 +58047,7 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
@@ -60500,7 +60918,7 @@
       </c>
       <c r="D121" s="23" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E121" s="23" t="inlineStr">
@@ -60555,7 +60973,7 @@
       </c>
       <c r="D122" s="23" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E122" s="23" t="inlineStr">
@@ -60955,7 +61373,7 @@
       </c>
       <c r="G134" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="H134" s="23" t="inlineStr">
@@ -61016,7 +61434,7 @@
       </c>
       <c r="G135" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="H135" s="23" t="inlineStr">
@@ -61129,7 +61547,7 @@
     <row r="145" ht="56" customHeight="1" s="29">
       <c r="A145" s="23" t="inlineStr">
         <is>
-          <t>Human abstract screening status not yet confirmed</t>
+          <t>Conventional workflow completed</t>
         </is>
       </c>
       <c r="B145" s="23" t="inlineStr">
@@ -61149,7 +61567,7 @@
       </c>
       <c r="E145" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F145" s="23" t="inlineStr">
@@ -61166,7 +61584,7 @@
     <row r="146" ht="42" customHeight="1" s="29">
       <c r="A146" s="23" t="inlineStr">
         <is>
-          <t>Abstract screening time log pending</t>
+          <t>Time logs received</t>
         </is>
       </c>
       <c r="B146" s="23" t="inlineStr">
@@ -61186,7 +61604,7 @@
       </c>
       <c r="E146" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F146" s="23" t="inlineStr">
@@ -61556,7 +61974,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">

</xml_diff>

<commit_message>
Fix current phase milestones
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract screening complete; full-text setup underway</t>
+          <t>Full-text setup underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abstract-screening discrepancies resolved; PDFs for 145 full-text records uploaded</t>
+          <t>Abstract screening complete; full-text setup underway with 145 uploaded records</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abstract-screening discrepancies resolved; PDFs for 145 full-text records uploaded</t>
+          <t>Abstract screening complete; full-text setup underway with 145 uploaded records</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm full-text setup and commence both screening arms</t>
+          <t>Confirm full-text project readiness and commence both screening arms</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Setup underway-145 records</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -17415,7 +17415,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -17552,7 +17551,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -31994,7 +31992,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -32131,7 +32128,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -36779,7 +36775,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -36916,7 +36911,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -42066,7 +42060,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Extraction complete; analysis access partially restored</t>
+          <t>Analysis in progress; access partially restored</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -56373,7 +56367,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Extraction complete; analysis access partially restored</t>
+          <t>Analysis in progress; access partially restored</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56509,7 +56503,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Extraction complete; analysis pending output retrieval</t>
+          <t>Analysis pending Laser AI output retrieval</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56698,7 +56692,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Complete—outputs submitted</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -56715,7 +56709,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Access restored for Krishna; output retrieval and Sean access to confirm</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">

</xml_diff>

<commit_message>
Update BP and Psoriasis August 24 status
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -34,7 +34,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="9">
     <font>
       <name val="Carlito"/>
@@ -167,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -248,6 +250,9 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -42060,7 +42065,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Analysis in progress; access partially restored</t>
+          <t>Analysis underway; reference-standard clarification pending</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -42080,22 +42085,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Both extractions complete; Krishna's Laser AI access restored; project visibility, Sean's access and output retrieval require confirmation</t>
+          <t>Both extraction outputs received; Sean is analysing the results and awaiting clarification of the final reference standard</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Verify BP project access, download Laser AI outputs and begin comparison</t>
+          <t>Obtain Doreen's clarification, confirm the final reference standard and continue comparison</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>Immediate</t>
+          <t>Awaiting review-team clarification</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -42132,7 +42137,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data-extraction confirmation pending</t>
+          <t>Data extraction complete; validation underway</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -42152,22 +42157,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Screening complete; awaiting final extraction files and time records</t>
+          <t>Conventional and AI extraction files received; times recorded as 2h45 and 2h10 respectively</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Obtain final extraction files/time records and complete validation</t>
+          <t>Validate both extraction outputs and prepare the comparison/adjudication dataset</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Awaiting review team</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -56367,7 +56372,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Analysis in progress; access partially restored</t>
+          <t>Analysis underway; reference-standard clarification pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56435,7 +56440,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Both extractions complete; Krishna's Laser AI access restored; output retrieval and Sean's access require confirmation</t>
+          <t>Both extraction outputs received; Sean is analysing the results and awaiting reference-standard clarification</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56452,7 +56457,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Both extractions complete; Krishna's Laser AI access restored; output retrieval and Sean's access require confirmation</t>
+          <t>Sean has begun analysing the project data; clarification requested from Doreen on the Study Tree file</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56469,7 +56474,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify project visibility, download Laser AI outputs and begin comparison</t>
+          <t>Confirm whether the Study Tree represents the final post-extraction reference standard, then continue comparison</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56486,7 +56491,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Immediate</t>
+          <t>Awaiting review-team clarification</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56503,7 +56508,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Analysis pending Laser AI output retrieval</t>
+          <t>Analysis underway; final reference standard not yet confirmed</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56520,7 +56525,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -56559,7 +56564,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56850,7 +56855,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Conventional extraction received; Laser AI output retrieval pending</t>
+          <t>Conventional and Laser AI extraction outputs received</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -57060,7 +57065,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Extraction complete; analysis access-blocked</t>
+          <t>Extraction complete; analysis underway</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -57507,14 +57512,14 @@
       </c>
       <c r="I55" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J55" s="18" t="n"/>
       <c r="K55" s="18" t="n"/>
       <c r="L55" s="18" t="inlineStr">
         <is>
-          <t>Krishna can log in; confirm BP project visibility and Sean's access</t>
+          <t>Project data available to Sean for analysis</t>
         </is>
       </c>
       <c r="M55" s="18" t="inlineStr">
@@ -59313,7 +59318,7 @@
       </c>
       <c r="I89" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J89" s="18" t="n"/>
@@ -59366,7 +59371,7 @@
       </c>
       <c r="I90" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J90" s="18" t="n"/>
@@ -59419,7 +59424,7 @@
       </c>
       <c r="I91" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J91" s="18" t="n"/>
@@ -59472,7 +59477,7 @@
       </c>
       <c r="I92" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J92" s="18" t="n"/>
@@ -59525,7 +59530,7 @@
       </c>
       <c r="I93" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J93" s="18" t="n"/>
@@ -59578,7 +59583,7 @@
       </c>
       <c r="I94" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J94" s="18" t="n"/>
@@ -59737,7 +59742,7 @@
       </c>
       <c r="I97" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J97" s="18" t="n"/>
@@ -59790,7 +59795,7 @@
       </c>
       <c r="I98" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J98" s="18" t="n"/>
@@ -60002,12 +60007,16 @@
       </c>
       <c r="I102" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J102" s="18" t="n"/>
       <c r="K102" s="18" t="n"/>
-      <c r="L102" s="18" t="n"/>
+      <c r="L102" s="18" t="inlineStr">
+        <is>
+          <t>Sean is reviewing discrepancies; final reference-standard definition pending</t>
+        </is>
+      </c>
       <c r="M102" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -60055,12 +60064,16 @@
       </c>
       <c r="I103" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J103" s="18" t="n"/>
       <c r="K103" s="18" t="n"/>
-      <c r="L103" s="18" t="n"/>
+      <c r="L103" s="18" t="inlineStr">
+        <is>
+          <t>Prepare after Doreen confirms the final included-study reference standard</t>
+        </is>
+      </c>
       <c r="M103" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -61776,7 +61789,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data-extraction confirmation pending</t>
+          <t>Data extraction complete; validation underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -61844,7 +61857,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Screening complete; awaiting final extraction files and times</t>
+          <t>Conventional and AI extraction files received; validation can begin</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -61861,7 +61874,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Screening complete; awaiting final extraction files and times</t>
+          <t>Sivem provided both extraction files; conventional time 2h45 and AI time 2h10</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -61878,7 +61891,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Obtain final extraction files/times and complete validation</t>
+          <t>Validate extraction outputs and prepare the comparison/adjudication dataset</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -61895,7 +61908,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting review team</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -61912,7 +61925,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Final extraction completion and timing unconfirmed</t>
+          <t>Extraction complete; comparison and adjudication remain</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -61929,7 +61942,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -61968,7 +61981,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -62101,7 +62114,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Status requested 2026-08-17</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -62118,7 +62131,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Provisional comparison available; final validation pending</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -62254,12 +62267,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Conventional and AI extraction files received</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -62298,12 +62311,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Screening times received; extraction time records pending</t>
+          <t>Extraction times received: conventional 2h45; AI 2h10</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -62469,19 +62482,19 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Extraction status awaiting review team</t>
+          <t>Extraction complete; validation underway</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Nested Knowledge data-extraction setup and repeated-run validation analysis are underway.</t>
+          <t>Both extraction outputs received; comparison and quality validation are next</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -64730,7 +64743,7 @@
       </c>
       <c r="I89" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J89" s="18" t="n"/>
@@ -64783,7 +64796,7 @@
       </c>
       <c r="I90" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J90" s="18" t="n"/>
@@ -64836,7 +64849,7 @@
       </c>
       <c r="I91" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J91" s="18" t="n"/>
@@ -64889,7 +64902,7 @@
       </c>
       <c r="I92" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J92" s="18" t="n"/>
@@ -64942,7 +64955,7 @@
       </c>
       <c r="I93" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J93" s="18" t="n"/>
@@ -64995,7 +65008,7 @@
       </c>
       <c r="I94" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J94" s="18" t="n"/>
@@ -65048,7 +65061,7 @@
       </c>
       <c r="I95" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J95" s="18" t="n"/>
@@ -65101,7 +65114,7 @@
       </c>
       <c r="I96" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J96" s="18" t="n"/>
@@ -65154,7 +65167,7 @@
       </c>
       <c r="I97" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J97" s="18" t="n"/>
@@ -65207,7 +65220,7 @@
       </c>
       <c r="I98" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J98" s="18" t="n"/>
@@ -65419,12 +65432,16 @@
       </c>
       <c r="I102" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J102" s="18" t="n"/>
       <c r="K102" s="18" t="n"/>
-      <c r="L102" s="18" t="n"/>
+      <c r="L102" s="18" t="inlineStr">
+        <is>
+          <t>Validate conventional and AI extraction files</t>
+        </is>
+      </c>
       <c r="M102" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -65472,7 +65489,7 @@
       </c>
       <c r="I103" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J103" s="18" t="n"/>
@@ -66329,7 +66346,7 @@
       </c>
       <c r="D121" s="23" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E121" s="23" t="inlineStr">
@@ -66347,7 +66364,7 @@
       </c>
       <c r="H121" s="23" t="inlineStr">
         <is>
-          <t>Meghan confirmed she would start entering data fields into NK</t>
+          <t>Nested Knowledge extraction setup and AI extraction completed</t>
         </is>
       </c>
       <c r="I121" s="23" t="inlineStr">
@@ -66382,7 +66399,7 @@
       </c>
       <c r="D122" s="23" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E122" s="23" t="inlineStr">
@@ -66400,7 +66417,7 @@
       </c>
       <c r="H122" s="23" t="inlineStr">
         <is>
-          <t>Conventional team clarified expected Excel and Word outputs</t>
+          <t>Conventional extraction file received</t>
         </is>
       </c>
       <c r="I122" s="23" t="inlineStr">
@@ -66435,7 +66452,7 @@
       </c>
       <c r="D123" s="23" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E123" s="23" t="inlineStr">
@@ -66455,7 +66472,7 @@
       </c>
       <c r="H123" s="23" t="inlineStr">
         <is>
-          <t>Sean asked extractors to follow agreed instructions before AI extraction begins</t>
+          <t>Extraction completed using the agreed definitions</t>
         </is>
       </c>
       <c r="I123" s="23" t="inlineStr">
@@ -66745,301 +66762,306 @@
       </c>
     </row>
     <row r="133" ht="56" customHeight="1" s="29">
-      <c r="B133" s="23" t="inlineStr">
+      <c r="A133" t="inlineStr">
         <is>
           <t>comm-phase1-02-004</t>
         </is>
       </c>
-      <c r="C133" s="27" t="n">
+      <c r="B133" s="33" t="n">
         <v>46161</v>
       </c>
+      <c r="C133" s="27" t="inlineStr">
+        <is>
+          <t>Psoriasis / NK survey responses</t>
+        </is>
+      </c>
       <c r="D133" s="23" t="inlineStr">
         <is>
-          <t>Psoriasis / NK survey responses</t>
+          <t>Susan / Krishna</t>
         </is>
       </c>
       <c r="E133" s="23" t="inlineStr">
         <is>
-          <t>Susan / Krishna</t>
-        </is>
-      </c>
-      <c r="F133" s="23" t="inlineStr">
-        <is>
           <t>Susan / Ursula</t>
         </is>
       </c>
-      <c r="G133" s="27" t="n">
+      <c r="F133" s="33" t="n">
         <v>46161</v>
       </c>
+      <c r="G133" s="27" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
       <c r="H133" s="23" t="inlineStr">
         <is>
+          <t>Two new NK title and abstract screening survey responses received</t>
+        </is>
+      </c>
+      <c r="I133" s="23" t="inlineStr">
+        <is>
+          <t>task-phase1-02-005</t>
+        </is>
+      </c>
+      <c r="J133" s="23" t="inlineStr">
+        <is>
+          <t>Confirm survey responses</t>
+        </is>
+      </c>
+      <c r="K133" s="23" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="L133" s="23" t="n"/>
+      <c r="M133" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N133" s="23" t="n"/>
+    </row>
+    <row r="134" ht="70" customHeight="1" s="29">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>comm-phase1-02-005</t>
+        </is>
+      </c>
+      <c r="B134" s="33" t="n">
+        <v>46162</v>
+      </c>
+      <c r="C134" s="27" t="inlineStr">
+        <is>
+          <t>Psoriasis NK data field setup</t>
+        </is>
+      </c>
+      <c r="D134" s="23" t="inlineStr">
+        <is>
+          <t>Meghan / Sivem / Sean</t>
+        </is>
+      </c>
+      <c r="E134" s="23" t="inlineStr">
+        <is>
+          <t>Meghan</t>
+        </is>
+      </c>
+      <c r="F134" s="33" t="n">
+        <v>46173</v>
+      </c>
+      <c r="G134" s="27" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H134" s="23" t="inlineStr">
+        <is>
+          <t>Meghan confirmed she would start entering data fields into Nested Knowledge</t>
+        </is>
+      </c>
+      <c r="I134" s="23" t="inlineStr">
+        <is>
+          <t>task-phase1-02-007</t>
+        </is>
+      </c>
+      <c r="J134" s="23" t="inlineStr">
+        <is>
+          <t>Enter NK data fields</t>
+        </is>
+      </c>
+      <c r="K134" s="23" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="L134" s="23" t="n"/>
+      <c r="M134" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N134" s="23" t="n"/>
+    </row>
+    <row r="135" ht="42" customHeight="1" s="29">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>comm-phase1-02-006</t>
+        </is>
+      </c>
+      <c r="B135" s="33" t="n">
+        <v>46167</v>
+      </c>
+      <c r="C135" s="27" t="inlineStr">
+        <is>
+          <t>Psoriasis updated data item list</t>
+        </is>
+      </c>
+      <c r="D135" s="23" t="inlineStr">
+        <is>
+          <t>Sean / Sivem / Meghan</t>
+        </is>
+      </c>
+      <c r="E135" s="23" t="inlineStr">
+        <is>
+          <t>Sean / Meghan</t>
+        </is>
+      </c>
+      <c r="F135" s="33" t="n">
+        <v>46167</v>
+      </c>
+      <c r="G135" s="27" t="inlineStr">
+        <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I133" s="23" t="inlineStr">
-        <is>
-          <t>Two new NK title and abstract screening survey responses received</t>
-        </is>
-      </c>
-      <c r="J133" s="23" t="inlineStr">
-        <is>
-          <t>task-phase1-02-005</t>
-        </is>
-      </c>
-      <c r="K133" s="23" t="inlineStr">
-        <is>
-          <t>Confirm survey responses</t>
-        </is>
-      </c>
-      <c r="L133" s="23" t="inlineStr">
+      <c r="H135" s="23" t="inlineStr">
+        <is>
+          <t>Updated data item list uploaded to shared folder</t>
+        </is>
+      </c>
+      <c r="I135" s="23" t="inlineStr">
+        <is>
+          <t>task-phase1-02-006</t>
+        </is>
+      </c>
+      <c r="J135" s="23" t="inlineStr">
+        <is>
+          <t>Finalize data items</t>
+        </is>
+      </c>
+      <c r="K135" s="23" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="M133" s="23" t="n"/>
-      <c r="N133" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="134" ht="70" customHeight="1" s="29">
-      <c r="B134" s="23" t="inlineStr">
-        <is>
-          <t>comm-phase1-02-005</t>
-        </is>
-      </c>
-      <c r="C134" s="27" t="n">
-        <v>46162</v>
-      </c>
-      <c r="D134" s="23" t="inlineStr">
-        <is>
-          <t>Psoriasis NK data field setup</t>
-        </is>
-      </c>
-      <c r="E134" s="23" t="inlineStr">
-        <is>
-          <t>Meghan / Sivem / Sean</t>
-        </is>
-      </c>
-      <c r="F134" s="23" t="inlineStr">
-        <is>
-          <t>Meghan</t>
-        </is>
-      </c>
-      <c r="G134" s="27" t="n">
+      <c r="L135" s="23" t="n"/>
+      <c r="M135" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N135" s="23" t="n"/>
+    </row>
+    <row r="136" ht="56" customHeight="1" s="29">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>comm-phase1-02-007</t>
+        </is>
+      </c>
+      <c r="B136" s="33" t="n">
+        <v>46168</v>
+      </c>
+      <c r="C136" s="27" t="inlineStr">
+        <is>
+          <t>Psoriasis conventional extraction format</t>
+        </is>
+      </c>
+      <c r="D136" s="23" t="inlineStr">
+        <is>
+          <t>Emilie / Sean / Meghan</t>
+        </is>
+      </c>
+      <c r="E136" s="23" t="inlineStr">
+        <is>
+          <t>Emilie / Robin</t>
+        </is>
+      </c>
+      <c r="F136" s="33" t="n">
         <v>46173</v>
       </c>
-      <c r="H134" s="23" t="inlineStr">
+      <c r="G136" s="27" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="I134" s="23" t="inlineStr">
-        <is>
-          <t>Meghan confirmed she would start entering data fields into Nested Knowledge</t>
-        </is>
-      </c>
-      <c r="J134" s="23" t="inlineStr">
-        <is>
-          <t>task-phase1-02-007</t>
-        </is>
-      </c>
-      <c r="K134" s="23" t="inlineStr">
-        <is>
-          <t>Enter NK data fields</t>
-        </is>
-      </c>
-      <c r="L134" s="23" t="inlineStr">
+      <c r="H136" s="23" t="inlineStr">
+        <is>
+          <t>Conventional team clarified planned Excel and Word outputs</t>
+        </is>
+      </c>
+      <c r="I136" s="23" t="inlineStr">
+        <is>
+          <t>task-phase1-02-008</t>
+        </is>
+      </c>
+      <c r="J136" s="23" t="inlineStr">
+        <is>
+          <t>Confirm conventional extraction format</t>
+        </is>
+      </c>
+      <c r="K136" s="23" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="M134" s="23" t="n"/>
-      <c r="N134" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" ht="42" customHeight="1" s="29">
-      <c r="B135" s="23" t="inlineStr">
-        <is>
-          <t>comm-phase1-02-006</t>
-        </is>
-      </c>
-      <c r="C135" s="27" t="n">
-        <v>46167</v>
-      </c>
-      <c r="D135" s="23" t="inlineStr">
-        <is>
-          <t>Psoriasis updated data item list</t>
-        </is>
-      </c>
-      <c r="E135" s="23" t="inlineStr">
-        <is>
-          <t>Sean / Sivem / Meghan</t>
-        </is>
-      </c>
-      <c r="F135" s="23" t="inlineStr">
-        <is>
-          <t>Sean / Meghan</t>
-        </is>
-      </c>
-      <c r="G135" s="27" t="n">
-        <v>46167</v>
-      </c>
-      <c r="H135" s="23" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="I135" s="23" t="inlineStr">
-        <is>
-          <t>Updated data item list uploaded to shared folder</t>
-        </is>
-      </c>
-      <c r="J135" s="23" t="inlineStr">
-        <is>
-          <t>task-phase1-02-006</t>
-        </is>
-      </c>
-      <c r="K135" s="23" t="inlineStr">
-        <is>
-          <t>Finalize data items</t>
-        </is>
-      </c>
-      <c r="L135" s="23" t="inlineStr">
+      <c r="L136" s="23" t="n"/>
+      <c r="M136" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N136" s="23" t="n"/>
+    </row>
+    <row r="137" ht="70" customHeight="1" s="29">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>comm-phase1-02-008</t>
+        </is>
+      </c>
+      <c r="B137" s="33" t="n">
+        <v>46169</v>
+      </c>
+      <c r="C137" s="27" t="inlineStr">
+        <is>
+          <t>Psoriasis extraction definitions</t>
+        </is>
+      </c>
+      <c r="D137" s="23" t="inlineStr">
+        <is>
+          <t>Sean / Emilie / Meghan / Sivem</t>
+        </is>
+      </c>
+      <c r="E137" s="23" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="F137" s="23" t="inlineStr">
+        <is>
+          <t>Immediate</t>
+        </is>
+      </c>
+      <c r="G137" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H137" s="23" t="inlineStr">
+        <is>
+          <t>Sean asked extractors to follow agreed definitions before AI extraction begins</t>
+        </is>
+      </c>
+      <c r="I137" s="23" t="inlineStr">
+        <is>
+          <t>task-phase1-02-009</t>
+        </is>
+      </c>
+      <c r="J137" s="23" t="inlineStr">
+        <is>
+          <t>Confirm no further changes</t>
+        </is>
+      </c>
+      <c r="K137" s="23" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="M135" s="23" t="n"/>
-      <c r="N135" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="136" ht="56" customHeight="1" s="29">
-      <c r="B136" s="23" t="inlineStr">
-        <is>
-          <t>comm-phase1-02-007</t>
-        </is>
-      </c>
-      <c r="C136" s="27" t="n">
-        <v>46168</v>
-      </c>
-      <c r="D136" s="23" t="inlineStr">
-        <is>
-          <t>Psoriasis conventional extraction format</t>
-        </is>
-      </c>
-      <c r="E136" s="23" t="inlineStr">
-        <is>
-          <t>Emilie / Sean / Meghan</t>
-        </is>
-      </c>
-      <c r="F136" s="23" t="inlineStr">
-        <is>
-          <t>Emilie / Robin</t>
-        </is>
-      </c>
-      <c r="G136" s="27" t="n">
-        <v>46173</v>
-      </c>
-      <c r="H136" s="23" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="I136" s="23" t="inlineStr">
-        <is>
-          <t>Conventional team clarified planned Excel and Word outputs</t>
-        </is>
-      </c>
-      <c r="J136" s="23" t="inlineStr">
-        <is>
-          <t>task-phase1-02-008</t>
-        </is>
-      </c>
-      <c r="K136" s="23" t="inlineStr">
-        <is>
-          <t>Confirm conventional extraction format</t>
-        </is>
-      </c>
-      <c r="L136" s="23" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="M136" s="23" t="n"/>
-      <c r="N136" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="137" ht="70" customHeight="1" s="29">
-      <c r="B137" s="23" t="inlineStr">
-        <is>
-          <t>comm-phase1-02-008</t>
-        </is>
-      </c>
-      <c r="C137" s="27" t="n">
-        <v>46169</v>
-      </c>
-      <c r="D137" s="23" t="inlineStr">
-        <is>
-          <t>Psoriasis extraction definitions</t>
-        </is>
-      </c>
-      <c r="E137" s="23" t="inlineStr">
-        <is>
-          <t>Sean / Emilie / Meghan / Sivem</t>
-        </is>
-      </c>
-      <c r="F137" s="23" t="inlineStr">
-        <is>
-          <t>Review Team</t>
-        </is>
-      </c>
-      <c r="G137" s="23" t="inlineStr">
-        <is>
-          <t>Immediate</t>
-        </is>
-      </c>
-      <c r="H137" s="23" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I137" s="23" t="inlineStr">
-        <is>
-          <t>Sean asked extractors to follow agreed definitions before AI extraction begins</t>
-        </is>
-      </c>
-      <c r="J137" s="23" t="inlineStr">
-        <is>
-          <t>task-phase1-02-009</t>
-        </is>
-      </c>
-      <c r="K137" s="23" t="inlineStr">
-        <is>
-          <t>Confirm no further changes</t>
-        </is>
-      </c>
-      <c r="L137" s="23" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="M137" s="23" t="n"/>
-      <c r="N137" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="L137" s="23" t="n"/>
+      <c r="M137" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N137" s="23" t="n"/>
     </row>
     <row r="138" s="29"/>
     <row r="139" s="29"/>
@@ -67163,12 +67185,12 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Needed before AI-assisted data extraction begins in NK</t>
+          <t>Resolved; AI-assisted extraction completed</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -67198,12 +67220,12 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Conventional outputs need to match agreed standalone data item structure</t>
+          <t>Conventional extraction output received</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboard through August 27
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2406,7 +2406,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text setup underway</t>
+          <t>Full-text workflow testing underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abstract screening complete; full-text setup underway with 145 uploaded records</t>
+          <t>Abstract screening complete; combined full-text project prepared with 144 records</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abstract screening complete; full-text setup underway with 145 uploaded records</t>
+          <t>Duplicate removed; translated PDF received; AI-command testing pending</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm full-text project readiness and commence both screening arms</t>
+          <t>Upload the translated PDF, complete AI-command testing and open both screening arms</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Full-text setup awaiting final confirmation</t>
+          <t>Full-text setup nearly complete; screening not yet started</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PDFs for 17 plus 128 records uploaded to SharePoint</t>
+          <t>Full-text set reduced to 144; translated PDF received; one inaccessible study retained</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Updated full-text decision flow submitted</t>
+          <t>Full-text workflow updated; AI-command testing pending</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Superset confirmed; 145 PDFs uploaded; awaiting project readiness confirmation</t>
+          <t>Combined project contains 144 records; translated PDF received; workflow testing pending</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4573,7 +4573,7 @@
       <c r="K74" s="18" t="n"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>PDFs for 145 records uploaded on 10 August</t>
+          <t>Full-text set reduced to 144 after duplicate removal; translated PDF received</t>
         </is>
       </c>
       <c r="M74" s="18" t="inlineStr">
@@ -4623,12 +4623,16 @@
       </c>
       <c r="I75" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J75" s="18" t="n"/>
       <c r="K75" s="18" t="n"/>
-      <c r="L75" s="18" t="n"/>
+      <c r="L75" s="18" t="inlineStr">
+        <is>
+          <t>Missing-PDF approach agreed: retain the study and exclude as unable to access</t>
+        </is>
+      </c>
       <c r="M75" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4736,7 +4740,7 @@
       <c r="K77" s="18" t="n"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Full-text decision flow requires final amendments.</t>
+          <t>Full-text workflow updated; AI-command testing pending</t>
         </is>
       </c>
       <c r="M77" s="18" t="inlineStr">
@@ -4793,7 +4797,7 @@
       <c r="K78" s="18" t="n"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Full-text project being prepared using the combined record set</t>
+          <t>Combined Laser AI project prepared with 144 records</t>
         </is>
       </c>
       <c r="M78" s="18" t="inlineStr">
@@ -17810,7 +17814,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -17878,7 +17882,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Future batch planning</t>
+          <t>Future-phase placeholder; not active</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -17895,7 +17899,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>No update recorded.</t>
+          <t>No further AI-tool onboarding under the current project</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -17912,7 +17916,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Keep placeholders until Phase 1 stabilizes.</t>
+          <t>Retain for future consideration; no current action</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -17963,7 +17967,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -17980,7 +17984,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -18002,7 +18006,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -22333,7 +22337,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Converted to phase1-07; Nested Knowledge setup complete and criteria approval pending</t>
+          <t>Converted to phase1-07; criteria approved and abstract screening ready to start</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22348,12 +22352,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Awaiting Murali's screening-criteria approval</t>
+          <t>Ready for abstract screening</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Converted to phase1-07 Human Milk; RIS, criteria, protocol information and 35 data items received</t>
+          <t>Criteria approved; AI responses generated; project opened for abstract screening</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -23166,17 +23170,17 @@
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>Under Shortlisting</t>
+          <t>Future Phase</t>
         </is>
       </c>
       <c r="D34" s="17" t="inlineStr">
         <is>
-          <t>Interested; search expected to be completed and screening ready at the end of September</t>
+          <t>Interested; retain for a future phase because no further current-project onboarding is planned</t>
         </is>
       </c>
       <c r="E34" s="17" t="inlineStr">
         <is>
-          <t>Phase 1 / timeline assessment</t>
+          <t>Future phase</t>
         </is>
       </c>
       <c r="F34" s="17" t="inlineStr">
@@ -23191,7 +23195,7 @@
       </c>
       <c r="H34" s="17" t="inlineStr">
         <is>
-          <t>Standard eligibility and workflow questions sent; awaiting detailed response</t>
+          <t>Questions sent; no detailed response received; retain for future consideration</t>
         </is>
       </c>
       <c r="I34" s="17" t="inlineStr">
@@ -32377,7 +32381,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Nested Knowledge setup complete; criteria validation pending</t>
+          <t>Criteria approved; abstract screening ready to start</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32445,7 +32449,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NK project created with 2,024 references; awaiting Murali's screening-criteria approval</t>
+          <t>Criteria approved; AI responses generated; abstract screening open</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32462,7 +32466,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NK project created with 2,024 references; awaiting Murali's screening-criteria approval</t>
+          <t>Full-text criteria revised and approved; team cleared to begin abstract screening</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32479,7 +32483,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm access and approve abstract/full-text criteria before screening</t>
+          <t>Begin parallel abstract screening and record time</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32496,7 +32500,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting review team approval</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -32513,7 +32517,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Setup complete; screening not yet started</t>
+          <t>Setup validated; screening ready to start</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32530,7 +32534,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -32569,7 +32573,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32651,7 +32655,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Complete-validation pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -32668,7 +32672,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Awaiting criteria approval</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -32818,12 +32822,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Pending approval</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Abstract and full-text criteria configured; Murali review pending</t>
+          <t>Abstract and full-text criteria approved; AI responses generated</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -32964,12 +32968,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Setup complete-validation pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>NK project contains 2,024 references; screening criteria awaiting approval</t>
+          <t>NK project contains 2,024 references; criteria approved and AI configuration completed</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -32986,7 +32990,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -33478,7 +33482,7 @@
       <c r="K55" s="18" t="n"/>
       <c r="L55" s="18" t="inlineStr">
         <is>
-          <t>Murali invited using both email addresses; access confirmation pending</t>
+          <t>Murali accessed NK and approved the criteria; confirm access for remaining reviewers</t>
         </is>
       </c>
       <c r="M55" s="18" t="inlineStr">
@@ -33976,14 +33980,14 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
       <c r="K64" s="18" t="n"/>
       <c r="L64" s="18" t="inlineStr">
         <is>
-          <t>Murali to approve abstract and full-text criteria</t>
+          <t>Criteria approved and AI responses generated on 26 August</t>
         </is>
       </c>
       <c r="M64" s="18" t="inlineStr">
@@ -34033,12 +34037,16 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
       <c r="K65" s="18" t="n"/>
-      <c r="L65" s="18" t="n"/>
+      <c r="L65" s="18" t="inlineStr">
+        <is>
+          <t>Conventional team can begin abstract screening</t>
+        </is>
+      </c>
       <c r="M65" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34086,12 +34094,16 @@
       </c>
       <c r="I66" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
       <c r="K66" s="18" t="n"/>
-      <c r="L66" s="18" t="n"/>
+      <c r="L66" s="18" t="inlineStr">
+        <is>
+          <t>AI-assisted team can begin abstract screening</t>
+        </is>
+      </c>
       <c r="M66" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -42065,7 +42077,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Analysis underway; reference-standard clarification pending</t>
+          <t>Reference standard clarified; adjudication preparation underway</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -42085,22 +42097,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Both extraction outputs received; Sean is analysing the results and awaiting clarification of the final reference standard</t>
+          <t>Reference standard confirmed as four reports; screening results finalized and adjudication sheet in preparation</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Obtain Doreen's clarification, confirm the final reference standard and continue comparison</t>
+          <t>Finalize the data-extraction adjudication sheet and begin adjudication</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>Awaiting review-team clarification</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -42137,7 +42149,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data extraction complete; validation underway</t>
+          <t>Data extraction complete; AI/NK output export pending</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -42157,12 +42169,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Conventional and AI extraction files received; times recorded as 2h45 and 2h10 respectively</t>
+          <t>Both extractions completed; conventional file received; AI/NK output not yet shared with the data manager</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Validate both extraction outputs and prepare the comparison/adjudication dataset</t>
+          <t>Export and share the AI/NK extraction output with Sean, then begin validation</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -42172,7 +42184,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Needs Action</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -42209,7 +42221,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Abstract screening complete; full-text setup underway</t>
+          <t>Abstract screening complete; full-text workflow testing underway</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -42229,12 +42241,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Screening discrepancy resolved; PDFs for 145 records uploaded; full-text setup awaiting confirmation</t>
+          <t>Combined full-text project prepared with 144 records; translated PDF received; AI-command testing pending</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Confirm full-text project readiness and commence parallel full-text screening</t>
+          <t>Upload the translated PDF, complete AI-command testing and open both full-text screening arms</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -42420,7 +42432,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Deferred-no further AI-tool onboarding in the current project</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -42440,27 +42452,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Planning based on results through mid-October</t>
+          <t>Retained only as a future-phase placeholder</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Review results after mid-October and decide next phase/tool strategy</t>
+          <t>No current-project action</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>After mid-October 2026</t>
+          <t>Not applicable</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -42564,7 +42576,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Nested Knowledge setup complete; criteria validation pending</t>
+          <t>Criteria approved; abstract screening ready to start</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -42584,22 +42596,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>NK project created with 2,024 references; documents uploaded; awaiting Murali's screening-criteria approval</t>
+          <t>Criteria approved; AI responses generated; review team cleared to begin abstract screening</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Confirm Murali's access and criteria approval, then begin screening</t>
+          <t>Begin parallel abstract screening and record time</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Awaiting review team approval</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -46268,7 +46280,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Laser AI continues; onboarding active</t>
+          <t>Laser AI continues; focus on completing current reviews</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -46322,7 +46334,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Pending results-based decision</t>
+          <t>Deferred; no further onboarding under the current project</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -46560,7 +46572,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Laser AI work restarted; Fruit &amp; Veg screening restart pending confirmation.</t>
+          <t>Laser AI operational; Fruit &amp; Veg full-text workflow testing underway</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -46685,7 +46697,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Completed; team subsequently withdrew</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -46695,7 +46707,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -46722,7 +46734,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -46749,7 +46761,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -46776,7 +46788,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -46803,7 +46815,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -56372,7 +56384,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Analysis underway; reference-standard clarification pending</t>
+          <t>Reference standard clarified; adjudication preparation underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56440,7 +56452,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Both extraction outputs received; Sean is analysing the results and awaiting reference-standard clarification</t>
+          <t>Screening results finalized; reference standard confirmed as four reports; quality review underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56457,7 +56469,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sean has begun analysing the project data; clarification requested from Doreen on the Study Tree file</t>
+          <t>Thirty-one reports passed conventional full text; four entered harmonized extraction; conventional title/abstract screening detected 3/4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56474,7 +56486,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm whether the Study Tree represents the final post-extraction reference standard, then continue comparison</t>
+          <t>Finalize the data-extraction adjudication sheet and begin adjudication</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56491,7 +56503,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting review-team clarification</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56508,7 +56520,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Analysis underway; final reference standard not yet confirmed</t>
+          <t>Reference-standard issue resolved; adjudication dataset in preparation</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56525,7 +56537,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -56564,7 +56576,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -57065,7 +57077,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Extraction complete; analysis underway</t>
+          <t>Extraction complete; adjudication preparation underway</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Reference standard confirmed as four reports; adjudication sheet in preparation</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -60014,7 +60031,7 @@
       <c r="K102" s="18" t="n"/>
       <c r="L102" s="18" t="inlineStr">
         <is>
-          <t>Sean is reviewing discrepancies; final reference-standard definition pending</t>
+          <t>Reference standard confirmed; Sean is completing the data-quality review</t>
         </is>
       </c>
       <c r="M102" s="18" t="inlineStr">
@@ -60064,14 +60081,14 @@
       </c>
       <c r="I103" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J103" s="18" t="n"/>
       <c r="K103" s="18" t="n"/>
       <c r="L103" s="18" t="inlineStr">
         <is>
-          <t>Prepare after Doreen confirms the final included-study reference standard</t>
+          <t>Sean is preparing the adjudication-ready data-extraction sheet</t>
         </is>
       </c>
       <c r="M103" s="18" t="inlineStr">
@@ -61789,7 +61806,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data extraction complete; validation underway</t>
+          <t>Data extraction complete; AI/NK output export pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -61857,7 +61874,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Conventional and AI extraction files received; validation can begin</t>
+          <t>Both extractions complete; conventional file received; AI/NK output awaiting export</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -61874,7 +61891,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sivem provided both extraction files; conventional time 2h45 and AI time 2h10</t>
+          <t>Conventional file received; conventional time 2h45 and AI extraction time 2h10 confirmed</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -61891,7 +61908,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Validate extraction outputs and prepare the comparison/adjudication dataset</t>
+          <t>Export the AI/NK output, share it with Sean and begin validation</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -61925,7 +61942,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Extraction complete; comparison and adjudication remain</t>
+          <t>Extraction complete; AI/NK output export and validation pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -61942,7 +61959,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Needs Action</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -61981,7 +61998,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -62131,7 +62148,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -62267,12 +62284,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Conventional and AI extraction files received</t>
+          <t>Conventional file received; AI/NK extraction output pending</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -62489,12 +62506,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Extraction complete; validation underway</t>
+          <t>Extraction complete; AI/NK output export pending</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Both extraction outputs received; comparison and quality validation are next</t>
+          <t>Conventional output received; AI/NK export must be shared before validation</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -65167,12 +65184,16 @@
       </c>
       <c r="I97" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J97" s="18" t="n"/>
       <c r="K97" s="18" t="n"/>
-      <c r="L97" s="18" t="n"/>
+      <c r="L97" s="18" t="inlineStr">
+        <is>
+          <t>Export the final AI/NK extraction output</t>
+        </is>
+      </c>
       <c r="M97" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -65220,12 +65241,16 @@
       </c>
       <c r="I98" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J98" s="18" t="n"/>
       <c r="K98" s="18" t="n"/>
-      <c r="L98" s="18" t="n"/>
+      <c r="L98" s="18" t="inlineStr">
+        <is>
+          <t>Share the AI/NK output with Sean after export</t>
+        </is>
+      </c>
       <c r="M98" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -65432,14 +65457,14 @@
       </c>
       <c r="I102" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J102" s="18" t="n"/>
       <c r="K102" s="18" t="n"/>
       <c r="L102" s="18" t="inlineStr">
         <is>
-          <t>Validate conventional and AI extraction files</t>
+          <t>Awaiting AI/NK extraction output</t>
         </is>
       </c>
       <c r="M102" s="18" t="inlineStr">
@@ -65489,12 +65514,16 @@
       </c>
       <c r="I103" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J103" s="18" t="n"/>
       <c r="K103" s="18" t="n"/>
-      <c r="L103" s="18" t="n"/>
+      <c r="L103" s="18" t="inlineStr">
+        <is>
+          <t>Prepare after output validation</t>
+        </is>
+      </c>
       <c r="M103" s="18" t="inlineStr">
         <is>
           <t>Yes</t>

</xml_diff>

<commit_message>
Update dashboard through September 1
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2406,7 +2406,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text workflow testing underway</t>
+          <t>Full-text screening ready to start</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abstract screening complete; combined full-text project prepared with 144 records</t>
+          <t>Abstract screening complete; combined 144-record project ready</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Duplicate removed; translated PDF received; AI-command testing pending</t>
+          <t>Translated PDF uploaded; AI workflow tested and issue resolved</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Upload the translated PDF, complete AI-command testing and open both screening arms</t>
+          <t>Begin both full-text screening arms and record time</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Full-text setup nearly complete; screening not yet started</t>
+          <t>Setup validated; screening not yet confirmed started</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Full-text workflow updated; AI-command testing pending</t>
+          <t>Full-text criteria and AI decision workflow validated</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3060,12 +3060,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Setup in progress</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Combined project contains 144 records; translated PDF received; workflow testing pending</t>
+          <t>Combined project ready; translated PDF uploaded and AI workflow issue resolved</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4733,14 +4733,14 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J77" s="18" t="n"/>
       <c r="K77" s="18" t="n"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Full-text workflow updated; AI-command testing pending</t>
+          <t>Full-text workflow validated on 1 September</t>
         </is>
       </c>
       <c r="M77" s="18" t="inlineStr">
@@ -4790,14 +4790,14 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Combined Laser AI project prepared with 144 records</t>
+          <t>Combined 144-record project configured and ready</t>
         </is>
       </c>
       <c r="M78" s="18" t="inlineStr">
@@ -4847,12 +4847,16 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
-      <c r="L79" s="18" t="n"/>
+      <c r="L79" s="18" t="inlineStr">
+        <is>
+          <t>AI decision workflow tested successfully</t>
+        </is>
+      </c>
       <c r="M79" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4900,12 +4904,16 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
-      <c r="L80" s="18" t="n"/>
+      <c r="L80" s="18" t="inlineStr">
+        <is>
+          <t>Conventional team cleared to begin full-text screening</t>
+        </is>
+      </c>
       <c r="M80" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4953,12 +4961,16 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
-      <c r="L81" s="18" t="n"/>
+      <c r="L81" s="18" t="inlineStr">
+        <is>
+          <t>Laser AI team cleared to begin full-text screening</t>
+        </is>
+      </c>
       <c r="M81" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13005,7 +13017,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Laser AI setup complete; decision-flow approval pending</t>
+          <t>Decision flow approved; abstract screening ready to start</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -13073,7 +13085,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Laser AI project created with 3,486 deduplicated references</t>
+          <t>Project approved with 3,486 references; screening ready</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13090,7 +13102,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Laser AI project created with 3,486 deduplicated references</t>
+          <t>Project approved with 3,486 references; screening ready</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13107,7 +13119,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Review team to approve decision flow; then provide access and start screening</t>
+          <t>Begin parallel abstract screening and record time</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13124,7 +13136,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting review team approval</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -13141,7 +13153,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Setup complete; screening awaits validation</t>
+          <t>Setup validated; screening not yet confirmed started</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -13158,7 +13170,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -13197,7 +13209,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13296,7 +13308,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Awaiting decision-flow approval</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -13451,7 +13463,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Decision flow prepared; review-team approval pending</t>
+          <t>Decision flow approved after protocol review on 28 August</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -13598,12 +13610,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Setup complete-validation pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Project configured; decision flow awaiting team approval</t>
+          <t>Project validated and ready for abstract screening</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -14119,12 +14131,16 @@
       </c>
       <c r="I55" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J55" s="18" t="n"/>
       <c r="K55" s="18" t="n"/>
-      <c r="L55" s="18" t="n"/>
+      <c r="L55" s="18" t="inlineStr">
+        <is>
+          <t>Reviewer access and screening instructions provided</t>
+        </is>
+      </c>
       <c r="M55" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14620,14 +14636,14 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
       <c r="K64" s="18" t="n"/>
       <c r="L64" s="18" t="inlineStr">
         <is>
-          <t>Awaiting review-team approval of decision flow</t>
+          <t>Decision flow approved on 28 August</t>
         </is>
       </c>
       <c r="M64" s="18" t="inlineStr">
@@ -14677,12 +14693,16 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
       <c r="K65" s="18" t="n"/>
-      <c r="L65" s="18" t="n"/>
+      <c r="L65" s="18" t="inlineStr">
+        <is>
+          <t>Conventional abstract screening ready to begin</t>
+        </is>
+      </c>
       <c r="M65" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14730,12 +14750,16 @@
       </c>
       <c r="I66" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
       <c r="K66" s="18" t="n"/>
-      <c r="L66" s="18" t="n"/>
+      <c r="L66" s="18" t="inlineStr">
+        <is>
+          <t>Laser AI abstract screening ready to begin</t>
+        </is>
+      </c>
       <c r="M66" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -17214,7 +17238,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -17224,7 +17248,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Awaiting review team approval</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -17234,7 +17258,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Decision flow prepared; approval required before screening begins.</t>
+          <t>Decision flow approved after review against the protocol</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -17244,7 +17268,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -17271,7 +17295,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -17281,7 +17305,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>After decision-flow approval</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -17291,7 +17315,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Provide reviewer access after the team approves the configured flow.</t>
+          <t>Project opened and screening instructions provided</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -17301,7 +17325,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -17328,7 +17352,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -17338,12 +17362,12 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>After access</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Tool access and team readiness</t>
+          <t>Access provided and setup validated</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -17616,7 +17640,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Decision-flow approval pending</t>
+          <t>Abstract screening ready to start</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -17631,17 +17655,17 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Awaiting review team approval</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Screening cannot start until the configured decision flow is approved.</t>
+          <t>Decision flow approved; project ready for screening</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -22441,7 +22465,7 @@
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-08; Laser AI setup started with four database searches outstanding</t>
+          <t>Converted to phase1-08; setup approved with 14,743 references before four final searches</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
@@ -22456,12 +22480,12 @@
       </c>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>Awaiting four searches</t>
+          <t>Awaiting count confirmation and four searches</t>
         </is>
       </c>
       <c r="H14" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-08 LNS; initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending</t>
+          <t>Decision flow approved; confirm expected count and provide four final searches</t>
         </is>
       </c>
       <c r="I14" s="17" t="inlineStr">
@@ -22493,7 +22517,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Converted to phase1-05; Laser AI setup completed with 3,486 references; decision-flow approval pending</t>
+          <t>Converted to phase1-05; decision flow approved and abstract screening ready</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
@@ -22508,12 +22532,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Awaiting review team approval</t>
+          <t>Ready for abstract screening</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Converted to phase1-05 Vitamin C; search strategy/database access issues remain before screening</t>
+          <t>Project validated with 3,486 references; reviewer instructions provided</t>
         </is>
       </c>
       <c r="I15" s="17" t="inlineStr">
@@ -37354,7 +37378,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Laser AI setup started; four searches outstanding</t>
+          <t>Laser AI setup ready; reference-count confirmation pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -37422,7 +37446,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Initial setup started; selected data items finalized; completion awaits four database searches</t>
+          <t>Decision flow approved; 14,743 references loaded before the final four searches</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -37439,7 +37463,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Initial setup started; selected data items finalized; completion awaits four database searches</t>
+          <t>Decision flow approved; 14,743 references loaded before the final four searches</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -37456,7 +37480,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Obtain four remaining searches, complete upload and validate decision flow</t>
+          <t>Confirm the 14,743-reference count and provide the final four searches</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -37473,7 +37497,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting four searches</t>
+          <t>Awaiting review-team confirmation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -37490,7 +37514,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Setup partially complete; final search set unavailable</t>
+          <t>Setup ready; final reference set not yet confirmed</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -37546,7 +37570,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -37611,7 +37635,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -37628,7 +37652,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>In progress-four searches outstanding</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -37645,7 +37669,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -37771,7 +37795,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Initial files received; four database searches outstanding</t>
+          <t>14,743 deduplicated references loaded; four searches still outstanding</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -37810,12 +37834,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Protocol/eligibility confirmation pending</t>
+          <t>Decision flow approved on 28 August</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -37854,12 +37878,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Protocol/criteria confirmation pending</t>
+          <t>Protocol and criteria reviewed; setup approved</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -37962,12 +37986,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>In progress-search set incomplete</t>
+          <t>Complete / Under Review</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Laser AI setup started; cannot be completed until four remaining searches arrive</t>
+          <t>Project ready with 14,743 records; awaiting count confirmation and four final searches</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -38324,14 +38348,14 @@
       </c>
       <c r="I52" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J52" s="18" t="inlineStr"/>
       <c r="K52" s="18" t="inlineStr"/>
       <c r="L52" s="18" t="inlineStr">
         <is>
-          <t>Tool allocation to be confirmed after onboarding.</t>
+          <t>Laser AI allocated</t>
         </is>
       </c>
       <c r="M52" s="18" t="inlineStr">
@@ -38697,11 +38721,16 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J59" s="18" t="inlineStr"/>
       <c r="K59" s="18" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Protocol and criteria reviewed; decision flow approved</t>
+        </is>
+      </c>
       <c r="M59" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -38910,14 +38939,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete / Under Review</t>
         </is>
       </c>
       <c r="J63" s="18" t="inlineStr"/>
       <c r="K63" s="18" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Initial setup started; final upload awaits four searches</t>
+          <t>Project ready with 14,743 references; four search additions pending</t>
         </is>
       </c>
       <c r="M63" s="18" t="inlineStr">
@@ -38967,12 +38996,16 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J64" s="18" t="inlineStr"/>
       <c r="K64" s="18" t="inlineStr"/>
-      <c r="L64" s="18" t="inlineStr"/>
+      <c r="L64" s="18" t="inlineStr">
+        <is>
+          <t>Confirm expected reference count before distributing citations</t>
+        </is>
+      </c>
       <c r="M64" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -41577,7 +41610,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Four remaining database searches are needed before final upload and validation can complete.</t>
+          <t>Project currently contains 14,743 references; confirm expected count and provide four final searches</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -41587,7 +41620,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -41687,12 +41720,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>LNS Laser AI setup started</t>
+          <t>LNS project ready; count confirmation pending</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -41702,12 +41735,12 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Review Team</t>
+          <t>Syeda Kanza Naqvi / Jai Das</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Awaiting four searches</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -41717,7 +41750,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Initial setup started and selected data items saved; final upload awaits four outstanding database searches.</t>
+          <t>Project ready with 14,743 references before the four remaining searches</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -41727,7 +41760,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Obtain four outstanding database searches</t>
+          <t>Confirm count and provide four outstanding searches</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -42077,7 +42110,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Reference standard clarified; adjudication preparation underway</t>
+          <t>Adjudication dataset ready; panel catch-up pending</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -42097,17 +42130,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Reference standard confirmed as four reports; screening results finalized and adjudication sheet in preparation</t>
+          <t>Reference standard confirmed; randomized adjudication spreadsheet prepared and first dataset received</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Finalize the data-extraction adjudication sheet and begin adjudication</t>
+          <t>Reschedule the adjudication-panel catch-up and begin adjudication</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>TBD - reschedule panel call</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -42149,12 +42182,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data extraction complete; AI/NK output export pending</t>
+          <t>Corrective full-text cross-screening setup underway</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -42169,12 +42202,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Both extractions completed; conventional file received; AI/NK output not yet shared with the data manager</t>
+          <t>Both extraction outputs received; comparison identified 139 AI-only and 25 conventional-only full-text records</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Export and share the AI/NK extraction output with Sean, then begin validation</t>
+          <t>Send the 139-record list, configure 25 records in NK and complete corrective cross-screening</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -42184,7 +42217,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -42221,7 +42254,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Abstract screening complete; full-text workflow testing underway</t>
+          <t>Full-text screening cleared to begin</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -42241,12 +42274,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Combined full-text project prepared with 144 records; translated PDF received; AI-command testing pending</t>
+          <t>Combined 144-record project ready; translated PDF uploaded and AI workflow issue resolved</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Upload the translated PDF, complete AI-command testing and open both full-text screening arms</t>
+          <t>Begin both full-text screening arms and record time</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -42256,7 +42289,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -42360,7 +42393,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Laser AI setup complete; decision-flow approval pending</t>
+          <t>Decision flow approved; abstract screening ready to start</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -42380,22 +42413,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Laser AI project created with 3,486 deduplicated references</t>
+          <t>Review team approved the 3,486-reference project; screening can begin</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Obtain decision-flow approval, provide reviewer access and begin screening</t>
+          <t>Begin parallel abstract screening and record time</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Awaiting review team approval</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -42648,7 +42681,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Laser AI setup started; four searches outstanding</t>
+          <t>Laser AI setup ready; reference-count confirmation pending</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -42668,17 +42701,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Initial setup started; selected data items saved; completion awaits results from four remaining database searches</t>
+          <t>Decision flow approved; 14,743 references loaded before the four remaining searches</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Obtain four outstanding searches, complete upload and validate the decision flow</t>
+          <t>Confirm the 14,743-reference count and provide the four remaining searches before screening</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Awaiting four searches</t>
+          <t>Awaiting review-team confirmation</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -46307,7 +46340,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>In progress; CESAR-FM extension initiated</t>
+          <t>All five review groups consented; model and data-governance finalization underway</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -46572,7 +46605,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Laser AI operational; Fruit &amp; Veg full-text workflow testing underway</t>
+          <t>Laser AI operational; Fruit &amp; Veg full-text workflow validated and ready to screen</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -56384,7 +56417,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Reference standard clarified; adjudication preparation underway</t>
+          <t>Adjudication dataset ready; panel catch-up pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56452,7 +56485,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Screening results finalized; reference standard confirmed as four reports; quality review underway</t>
+          <t>Reference standard confirmed; randomized adjudication dataset prepared</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56469,7 +56502,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Thirty-one reports passed conventional full text; four entered harmonized extraction; conventional title/abstract screening detected 3/4</t>
+          <t>First dataset ready for adjudication; panel call requires rescheduling</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56486,7 +56519,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Finalize the data-extraction adjudication sheet and begin adjudication</t>
+          <t>Reschedule the adjudication-panel catch-up and begin adjudication</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56503,7 +56536,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>TBD - reschedule panel call</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56520,7 +56553,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Reference-standard issue resolved; adjudication dataset in preparation</t>
+          <t>Adjudication data ready; panel meeting not yet held</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56576,7 +56609,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56818,12 +56851,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Four reference-standard PDFs shared with Gerald and the extension team</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -57077,12 +57110,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Extraction complete; adjudication preparation underway</t>
+          <t>Extraction complete; adjudication dataset ready</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Reference standard confirmed as four reports; adjudication sheet in preparation</t>
+          <t>Randomized adjudication spreadsheet prepared; panel catch-up to be rescheduled</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -60024,14 +60057,14 @@
       </c>
       <c r="I102" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J102" s="18" t="n"/>
       <c r="K102" s="18" t="n"/>
       <c r="L102" s="18" t="inlineStr">
         <is>
-          <t>Reference standard confirmed; Sean is completing the data-quality review</t>
+          <t>Data-quality review completed; adjudication dataset prepared</t>
         </is>
       </c>
       <c r="M102" s="18" t="inlineStr">
@@ -60081,14 +60114,14 @@
       </c>
       <c r="I103" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J103" s="18" t="n"/>
       <c r="K103" s="18" t="n"/>
       <c r="L103" s="18" t="inlineStr">
         <is>
-          <t>Sean is preparing the adjudication-ready data-extraction sheet</t>
+          <t>Randomized adjudication-ready spreadsheet prepared and shared</t>
         </is>
       </c>
       <c r="M103" s="18" t="inlineStr">
@@ -60138,12 +60171,16 @@
       </c>
       <c r="I104" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J104" s="18" t="n"/>
       <c r="K104" s="18" t="n"/>
-      <c r="L104" s="18" t="n"/>
+      <c r="L104" s="18" t="inlineStr">
+        <is>
+          <t>Panel catch-up to be rescheduled; no advance pilot required</t>
+        </is>
+      </c>
       <c r="M104" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -61806,7 +61843,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data extraction complete; AI/NK output export pending</t>
+          <t>Corrective full-text cross-screening setup underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -61823,7 +61860,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -61874,7 +61911,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Both extractions complete; conventional file received; AI/NK output awaiting export</t>
+          <t>Both extraction outputs received; screening comparison identified unmatched full-text records</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -61891,7 +61928,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Conventional file received; conventional time 2h45 and AI extraction time 2h10 confirmed</t>
+          <t>139 records require conventional screening and 25 require AI/NK screening</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -61908,7 +61945,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Export the AI/NK output, share it with Sean and begin validation</t>
+          <t>Send the 139-record list, configure 25 records in NK and complete corrective screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -61942,7 +61979,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Extraction complete; AI/NK output export and validation pending</t>
+          <t>Analysis paused pending corrective cross-screening</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -61959,7 +61996,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -61998,7 +62035,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -62114,7 +62151,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -62148,7 +62185,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -62240,12 +62277,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>PDFs for the 10 extracted studies received and shared with Sean</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -62262,12 +62299,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Existing full-text criteria applicable to corrective screening</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -62284,12 +62321,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Conventional file received; AI/NK extraction output pending</t>
+          <t>Conventional and AI/NK extraction data received</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -62478,12 +62515,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Conventional and AI-assisted full-text screening complete; 10 studies selected.</t>
+          <t>Original screening complete; 139 conventional and 25 AI/NK records require corrective cross-screening</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -62506,12 +62543,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Extraction complete; AI/NK output export pending</t>
+          <t>Extraction complete; validation blocked by corrective screening</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Conventional output received; AI/NK export must be shared before validation</t>
+          <t>Both extraction outputs received; final analysis awaits corrective screening</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -63488,12 +63525,16 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
       <c r="K65" s="18" t="n"/>
-      <c r="L65" s="18" t="n"/>
+      <c r="L65" s="18" t="inlineStr">
+        <is>
+          <t>Original conventional title/abstract screening complete</t>
+        </is>
+      </c>
       <c r="M65" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -63965,12 +64006,16 @@
       </c>
       <c r="I74" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
-      <c r="L74" s="18" t="n"/>
+      <c r="L74" s="18" t="inlineStr">
+        <is>
+          <t>Ten selected-study PDFs shared with Sean</t>
+        </is>
+      </c>
       <c r="M74" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -64124,12 +64169,16 @@
       </c>
       <c r="I77" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J77" s="18" t="n"/>
       <c r="K77" s="18" t="n"/>
-      <c r="L77" s="18" t="n"/>
+      <c r="L77" s="18" t="inlineStr">
+        <is>
+          <t>Full-text criteria finalized and retained for corrective screening</t>
+        </is>
+      </c>
       <c r="M77" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -64177,12 +64226,16 @@
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
-      <c r="L78" s="18" t="n"/>
+      <c r="L78" s="18" t="inlineStr">
+        <is>
+          <t>Nested Knowledge setup decision pending for the 25 unmatched records</t>
+        </is>
+      </c>
       <c r="M78" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -64230,12 +64283,16 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
-      <c r="L79" s="18" t="n"/>
+      <c r="L79" s="18" t="inlineStr">
+        <is>
+          <t>Validate the corrective NK project before screening</t>
+        </is>
+      </c>
       <c r="M79" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -64283,12 +64340,16 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
-      <c r="L80" s="18" t="n"/>
+      <c r="L80" s="18" t="inlineStr">
+        <is>
+          <t>Conventional team to screen 139 unmatched records</t>
+        </is>
+      </c>
       <c r="M80" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -64336,12 +64397,16 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
-      <c r="L81" s="18" t="n"/>
+      <c r="L81" s="18" t="inlineStr">
+        <is>
+          <t>AI/NK team to screen 25 unmatched records</t>
+        </is>
+      </c>
       <c r="M81" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -65184,14 +65249,14 @@
       </c>
       <c r="I97" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J97" s="18" t="n"/>
       <c r="K97" s="18" t="n"/>
       <c r="L97" s="18" t="inlineStr">
         <is>
-          <t>Export the final AI/NK extraction output</t>
+          <t>AI/NK extracted data received by Sean</t>
         </is>
       </c>
       <c r="M97" s="18" t="inlineStr">
@@ -65241,14 +65306,14 @@
       </c>
       <c r="I98" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J98" s="18" t="n"/>
       <c r="K98" s="18" t="n"/>
       <c r="L98" s="18" t="inlineStr">
         <is>
-          <t>Share the AI/NK output with Sean after export</t>
+          <t>AI/NK extracted data shared with Sean</t>
         </is>
       </c>
       <c r="M98" s="18" t="inlineStr">
@@ -65457,14 +65522,14 @@
       </c>
       <c r="I102" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="J102" s="18" t="n"/>
       <c r="K102" s="18" t="n"/>
       <c r="L102" s="18" t="inlineStr">
         <is>
-          <t>Awaiting AI/NK extraction output</t>
+          <t>Validation blocked until corrective screening is complete</t>
         </is>
       </c>
       <c r="M102" s="18" t="inlineStr">
@@ -65514,14 +65579,14 @@
       </c>
       <c r="I103" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="J103" s="18" t="n"/>
       <c r="K103" s="18" t="n"/>
       <c r="L103" s="18" t="inlineStr">
         <is>
-          <t>Prepare after output validation</t>
+          <t>Prepare after corrected full-text sets are finalized</t>
         </is>
       </c>
       <c r="M103" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboard through September 3
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -22361,7 +22361,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Converted to phase1-07; criteria approved and abstract screening ready to start</t>
+          <t>Converted to phase1-07; abstract screening underway</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22376,12 +22376,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Ready for abstract screening</t>
+          <t>Abstract screening expected to finish this week</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Criteria approved; AI responses generated; project opened for abstract screening</t>
+          <t>Murali and Michelle started screening; full-text screening planned next week</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -32405,7 +32405,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Criteria approved; abstract screening ready to start</t>
+          <t>Abstract screening underway; expected completion this week; full-text screening planned next week</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32473,7 +32473,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Criteria approved; AI responses generated; abstract screening open</t>
+          <t>Murali and Michelle are screening abstracts; completion expected this week</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32490,7 +32490,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Full-text criteria revised and approved; team cleared to begin abstract screening</t>
+          <t>Abstract screening started; Mohan also confirmed likely project access</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32507,7 +32507,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Begin parallel abstract screening and record time</t>
+          <t>Complete abstract screening, notify the project team, circulate the survey and set up full-text screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32524,7 +32524,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Immediate</t>
+          <t>2026-09-06 (expected)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -32541,7 +32541,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Setup validated; screening ready to start</t>
+          <t>Abstract screening underway; full-text setup planned next</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32558,7 +32558,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -32597,7 +32597,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32711,6 +32711,11 @@
           <t>fullText</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33014,7 +33019,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Murali and Michelle are screening; completion expected this week</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -33031,7 +33041,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Full-text screening planned for next week after the survey and project setup</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -33499,14 +33514,14 @@
       </c>
       <c r="I55" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete / Under Review</t>
         </is>
       </c>
       <c r="J55" s="18" t="n"/>
       <c r="K55" s="18" t="n"/>
       <c r="L55" s="18" t="inlineStr">
         <is>
-          <t>Murali accessed NK and approved the criteria; confirm access for remaining reviewers</t>
+          <t>Murali and Michelle are actively screening; Mohan likely confirmed access through mohanv@bcm.edu; Gautham’s access remains unconfirmed</t>
         </is>
       </c>
       <c r="M55" s="18" t="inlineStr">
@@ -34061,14 +34076,14 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
       <c r="K65" s="18" t="n"/>
       <c r="L65" s="18" t="inlineStr">
         <is>
-          <t>Conventional team can begin abstract screening</t>
+          <t>Conventional abstract screening underway</t>
         </is>
       </c>
       <c r="M65" s="18" t="inlineStr">
@@ -34118,14 +34133,14 @@
       </c>
       <c r="I66" s="18" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
       <c r="K66" s="18" t="n"/>
       <c r="L66" s="18" t="inlineStr">
         <is>
-          <t>AI-assisted team can begin abstract screening</t>
+          <t>AI-assisted abstract screening underway</t>
         </is>
       </c>
       <c r="M66" s="18" t="inlineStr">
@@ -34286,7 +34301,11 @@
       </c>
       <c r="J69" s="18" t="n"/>
       <c r="K69" s="18" t="n"/>
-      <c r="L69" s="18" t="n"/>
+      <c r="L69" s="18" t="inlineStr">
+        <is>
+          <t>Send the short usability survey once abstract screening is complete</t>
+        </is>
+      </c>
       <c r="M69" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34705,12 +34724,16 @@
       </c>
       <c r="I77" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J77" s="18" t="n"/>
       <c r="K77" s="18" t="n"/>
-      <c r="L77" s="18" t="n"/>
+      <c r="L77" s="18" t="inlineStr">
+        <is>
+          <t>Full-text criteria revised and approved on 26 August</t>
+        </is>
+      </c>
       <c r="M77" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -36606,7 +36629,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -36616,7 +36639,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Awaiting review team approval</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -36626,7 +36649,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Murali invited using both email addresses; access confirmation pending.</t>
+          <t>Murali’s access confirmed through active screening</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -36636,7 +36659,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -36663,7 +36686,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -36673,7 +36696,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Awaiting review team approval</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -36683,7 +36706,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Screening criteria configured and awaiting Murali's approval.</t>
+          <t>Abstract and full-text criteria approved; AI responses generated</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -36693,7 +36716,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -36710,7 +36733,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Begin Nested Knowledge screening after validation</t>
+          <t>Complete abstract screening and notify the project team</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -36720,7 +36743,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -36730,17 +36753,17 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>After criteria approval</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Access and criteria approval</t>
+          <t>Abstract screening underway</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Start screening once access and criteria validation are confirmed.</t>
+          <t>Screening underway; circulate the survey and prepare full-text setup after completion</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -36750,7 +36773,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -36903,47 +36926,47 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Human Milk NK setup complete</t>
+          <t>Human Milk abstract screening underway</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Krishna / Murali / Response Team</t>
+          <t>Murali / Michelle / Mohan / Krishna / Meghan</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Murali / Review Team</t>
+          <t>Murali / Michelle / Krishna</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Awaiting review team approval</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>NK project contains 2,024 references; Murali's access and screening-criteria approval remain the next actions.</t>
+          <t>Murali and Michelle started abstract screening; completion expected this week and full-text screening planned next week</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>task-phase1-07-002</t>
+          <t>task-phase1-07-003</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Approve abstract and full-text criteria</t>
+          <t>Complete abstract screening, circulate survey and prepare full-text setup</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -37008,32 +37031,32 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Criteria approval pending</t>
+          <t>Complete abstract screening and prepare full-text setup</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Murali / Review Team</t>
+          <t>Review Team / Krishna / Nested Knowledge</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Awaiting review team approval</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Abstract and full-text screening should not start until criteria are approved.</t>
+          <t>Screening underway; notify Krishna after completion so the survey and full-text setup can proceed</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -42110,7 +42133,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Adjudication dataset ready; panel catch-up pending</t>
+          <t>Adjudication dataset ready; panel meeting scheduled</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -42130,17 +42153,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Reference standard confirmed; randomized adjudication spreadsheet prepared and first dataset received</t>
+          <t>Reference standard confirmed; randomized adjudication dataset prepared; panel invitation sent</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Reschedule the adjudication-panel catch-up and begin adjudication</t>
+          <t>Hold the scheduled panel meeting and begin adjudication; resolve CESAR extension PDF/mapping gap</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>TBD - reschedule panel call</t>
+          <t>Scheduled — see calendar invitation</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -42202,12 +42225,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Both extraction outputs received; comparison identified 139 AI-only and 25 conventional-only full-text records</t>
+          <t>The 139-record RIS/PDF package was sent to the conventional team; the existing NK project was selected for the 25 AI records</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Send the 139-record list, configure 25 records in NK and complete corrective cross-screening</t>
+          <t>Add 25 records to the existing NK project, complete both corrective screening arms and rerun the comparison</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -42609,7 +42632,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Criteria approved; abstract screening ready to start</t>
+          <t>Abstract screening underway; expected completion this week; full-text screening planned next week</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -42629,22 +42652,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Criteria approved; AI responses generated; review team cleared to begin abstract screening</t>
+          <t>Murali and Michelle have started abstract screening; completion expected this week</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Begin parallel abstract screening and record time</t>
+          <t>Complete abstract screening, circulate the short survey and set up full-text screening</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Immediate</t>
+          <t>2026-09-06 (expected)</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -46340,7 +46363,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>All five review groups consented; model and data-governance finalization underway</t>
+          <t>All five groups consented; model/data-governance work continues; the BP automated run awaits the complete PDF package, mapping and supplementary-material decision</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -56417,7 +56440,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Adjudication dataset ready; panel catch-up pending</t>
+          <t>Adjudication dataset ready; panel meeting scheduled</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56485,7 +56508,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Reference standard confirmed; randomized adjudication dataset prepared</t>
+          <t>Reference standard confirmed; randomized adjudication dataset prepared; panel invitation sent</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56502,7 +56525,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>First dataset ready for adjudication; panel call requires rescheduling</t>
+          <t>Panel invitation sent; no advance pilot is required</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56519,7 +56542,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Reschedule the adjudication-panel catch-up and begin adjudication</t>
+          <t>Hold the panel meeting and begin adjudication; complete the CESAR extension PDF/mapping package</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56536,7 +56559,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD - reschedule panel call</t>
+          <t>Scheduled — see calendar invitation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56553,7 +56576,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Adjudication data ready; panel meeting not yet held</t>
+          <t>Panel meeting scheduled; CESAR extension input gap remains</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56609,7 +56632,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56856,7 +56879,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Four reference-standard PDFs shared with Gerald and the extension team</t>
+          <t>Only 4 of 19 full-text PDFs are visible to the extension team; complete mapping and supplementary-material scope are pending</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -57110,12 +57133,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Extraction complete; adjudication dataset ready</t>
+          <t>Extraction complete; adjudication ready; CESAR extension inputs incomplete</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Randomized adjudication spreadsheet prepared; panel catch-up to be rescheduled</t>
+          <t>Adjudication meeting scheduled; extension screening awaits the complete PDF/mapping package</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -60171,14 +60194,14 @@
       </c>
       <c r="I104" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="J104" s="18" t="n"/>
       <c r="K104" s="18" t="n"/>
       <c r="L104" s="18" t="inlineStr">
         <is>
-          <t>Panel catch-up to be rescheduled; no advance pilot required</t>
+          <t>Meeting invitation sent; no advance pilot required</t>
         </is>
       </c>
       <c r="M104" s="18" t="inlineStr">
@@ -60281,12 +60304,16 @@
       </c>
       <c r="I106" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="J106" s="18" t="n"/>
       <c r="K106" s="18" t="n"/>
-      <c r="L106" s="18" t="n"/>
+      <c r="L106" s="18" t="inlineStr">
+        <is>
+          <t>Automated run blocked pending all 19 PDFs, record-to-PDF mapping and a supplementary-material decision</t>
+        </is>
+      </c>
       <c r="M106" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -61911,7 +61938,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Both extraction outputs received; screening comparison identified unmatched full-text records</t>
+          <t>Corrective screening preparation underway; the conventional package was sent and the existing NK project selected</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -61928,7 +61955,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>139 records require conventional screening and 25 require AI/NK screening</t>
+          <t>The 139-record RIS/PDF package was sent; addition of 25 records to the existing NK project is pending</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -61945,7 +61972,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Send the 139-record list, configure 25 records in NK and complete corrective screening</t>
+          <t>Add 25 records to the existing NK project and complete both corrective screening arms</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -62035,7 +62062,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -62185,7 +62212,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Risk</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -62282,7 +62309,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PDFs for the 10 extracted studies received and shared with Sean</t>
+          <t>Corrective-screening PDFs for 139 records are available in the shared folder; ten extracted-study PDFs were shared with Sean</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -62520,7 +62547,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Original screening complete; 139 conventional and 25 AI/NK records require corrective cross-screening</t>
+          <t>The 139-record package was sent to the conventional team; the 25-record NK setup remains pending</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -64233,7 +64260,7 @@
       <c r="K78" s="18" t="n"/>
       <c r="L78" s="18" t="inlineStr">
         <is>
-          <t>Nested Knowledge setup decision pending for the 25 unmatched records</t>
+          <t>Sean selected the existing NK project; Meghan to add the 25 records</t>
         </is>
       </c>
       <c r="M78" s="18" t="inlineStr">
@@ -64290,7 +64317,7 @@
       <c r="K79" s="18" t="n"/>
       <c r="L79" s="18" t="inlineStr">
         <is>
-          <t>Validate the corrective NK project before screening</t>
+          <t>Validate the existing project after the 25 records are added</t>
         </is>
       </c>
       <c r="M79" s="18" t="inlineStr">
@@ -64347,7 +64374,7 @@
       <c r="K80" s="18" t="n"/>
       <c r="L80" s="18" t="inlineStr">
         <is>
-          <t>Conventional team to screen 139 unmatched records</t>
+          <t>The 139-record RIS and PDF location were sent; screening completion pending</t>
         </is>
       </c>
       <c r="M80" s="18" t="inlineStr">
@@ -64404,7 +64431,7 @@
       <c r="K81" s="18" t="n"/>
       <c r="L81" s="18" t="inlineStr">
         <is>
-          <t>AI/NK team to screen 25 unmatched records</t>
+          <t>Add 25 records to the existing NK project and complete AI-assisted screening</t>
         </is>
       </c>
       <c r="M81" s="18" t="inlineStr">
@@ -66106,7 +66133,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -66126,7 +66153,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Nested Knowledge commented on unavailable or paywalled records; confirm whether review team can source remaining files.</t>
+          <t>Original full-text access issues were handled before screening completion</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -66163,7 +66190,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -66183,7 +66210,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Trial registry and multi-abstract PDF issues were addressed by Nested Knowledge; remaining access gaps need confirmation.</t>
+          <t>Original full-text setup and screening completed</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -66220,7 +66247,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -66240,7 +66267,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Confirm criteria before full-text AI setup proceeds.</t>
+          <t>Full-text criteria finalized and retained for corrective screening</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -66277,7 +66304,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -66297,7 +66324,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Send survey when abstract screening is confirmed complete.</t>
+          <t>Survey sent; NK abstract-screening responses received</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -66944,12 +66971,12 @@
       </c>
       <c r="G134" s="27" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H134" s="23" t="inlineStr">
         <is>
-          <t>Meghan confirmed she would start entering data fields into Nested Knowledge</t>
+          <t>NK data-field setup and AI extraction completed</t>
         </is>
       </c>
       <c r="I134" s="23" t="inlineStr">
@@ -67064,12 +67091,12 @@
       </c>
       <c r="G136" s="27" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H136" s="23" t="inlineStr">
         <is>
-          <t>Conventional team clarified planned Excel and Word outputs</t>
+          <t>Conventional extraction output received</t>
         </is>
       </c>
       <c r="I136" s="23" t="inlineStr">
@@ -67126,12 +67153,12 @@
       </c>
       <c r="G137" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="H137" s="23" t="inlineStr">
         <is>
-          <t>Sean asked extractors to follow agreed definitions before AI extraction begins</t>
+          <t>Definitions confirmed and extraction completed</t>
         </is>
       </c>
       <c r="I137" s="23" t="inlineStr">

</xml_diff>